<commit_message>
Dossier comptable : contrôle des G50 IMPORT mars à août 2026
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XYis4EzVZMNdoYCxmLrRh4
</commit_message>
<xml_diff>
--- a/DOSSIER_COMPTABLE_SARL_DPR_COMPAGNY_2026.xlsx
+++ b/DOSSIER_COMPTABLE_SARL_DPR_COMPAGNY_2026.xlsx
@@ -202,7 +202,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -245,6 +245,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="166" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -1108,11 +1109,11 @@
     <row r="36">
       <c r="A36" s="12" t="inlineStr">
         <is>
-          <t>G50 juin/août : total déclaré = recalculé</t>
+          <t>G50 mars–août : totaux et report de précompte</t>
         </is>
       </c>
       <c r="B36" s="4">
-        <f>IF(AND(ABS('G50 2026'!B26)&lt;1,ABS('G50 2026'!C26)&lt;1),"OK","ÉCART")</f>
+        <f>IF(AND(SUMPRODUCT(ABS('G50 2026'!B29:G29))&lt;1,SUMPRODUCT(ABS('G50 2026'!C16:G16))&lt;1),"OK","ÉCART")</f>
         <v/>
       </c>
     </row>
@@ -1254,7 +1255,7 @@
       </c>
       <c r="B48" s="12" t="inlineStr">
         <is>
-          <t>Contrôle TVA / IRG / TA des G50 IMPORT juin et août</t>
+          <t>Contrôle TVA / IRG / timbre / TA des G50 IMPORT mars–août</t>
         </is>
       </c>
       <c r="C48" s="17" t="n"/>
@@ -4014,7 +4015,7 @@
         <f>SUM(D5:D7)-SUM(D8:D15)</f>
         <v/>
       </c>
-      <c r="E16" s="36">
+      <c r="E16" s="37">
         <f>IF(C16=0,"",D16/C16-1)</f>
         <v/>
       </c>
@@ -4717,7 +4718,7 @@
           <t>A01</t>
         </is>
       </c>
-      <c r="B5" s="37" t="n">
+      <c r="B5" s="38" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="29" t="inlineStr">
@@ -4735,7 +4736,7 @@
           <t>Déclaration CNAS de février 2026 non fournie (assiette paie 952 475,81 ; 7 STC payés).</t>
         </is>
       </c>
-      <c r="F5" s="38">
+      <c r="F5" s="39">
         <f>'Rappro CNAS'!J6</f>
         <v/>
       </c>
@@ -4744,8 +4745,8 @@
           <t>Fournir la déclaration de février + EMS avec 7 sorties ; à défaut, la déposer (pénalités de retard).</t>
         </is>
       </c>
-      <c r="H5" s="39" t="n"/>
-      <c r="I5" s="39" t="inlineStr">
+      <c r="H5" s="40" t="n"/>
+      <c r="I5" s="40" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -4757,7 +4758,7 @@
           <t>A02</t>
         </is>
       </c>
-      <c r="B6" s="37" t="n">
+      <c r="B6" s="38" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="29" t="inlineStr">
@@ -4775,7 +4776,7 @@
           <t>Centralisateur de mars 2026 absent (onglet vide) alors que la CNAS de mars déclare 368 389,93 d'assiette, 5 salariés.</t>
         </is>
       </c>
-      <c r="F6" s="38">
+      <c r="F6" s="39">
         <f>'Rappro CNAS'!K7</f>
         <v/>
       </c>
@@ -4784,8 +4785,8 @@
           <t>Obtenir le livre de paie de mars et le saisir dans « Paie IMPORT » col. E ; comptabiliser la paie de mars.</t>
         </is>
       </c>
-      <c r="H6" s="39" t="n"/>
-      <c r="I6" s="39" t="inlineStr">
+      <c r="H6" s="40" t="n"/>
+      <c r="I6" s="40" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -4797,7 +4798,7 @@
           <t>A03</t>
         </is>
       </c>
-      <c r="B7" s="37" t="n">
+      <c r="B7" s="38" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="29" t="inlineStr">
@@ -4815,7 +4816,7 @@
           <t>Prime de ponctualité (R540) imposée à l'IRG mais exclue du salaire de poste (assiette CNAS) chaque mois.</t>
         </is>
       </c>
-      <c r="F7" s="38">
+      <c r="F7" s="39">
         <f>'Rappro CNAS'!V13</f>
         <v/>
       </c>
@@ -4824,8 +4825,8 @@
           <t>Vérifier le paramétrage de la rubrique R540 (soumise SS) ; régulariser les déclarations concernées.</t>
         </is>
       </c>
-      <c r="H7" s="39" t="n"/>
-      <c r="I7" s="39" t="inlineStr">
+      <c r="H7" s="40" t="n"/>
+      <c r="I7" s="40" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -4837,7 +4838,7 @@
           <t>A04</t>
         </is>
       </c>
-      <c r="B8" s="40" t="n">
+      <c r="B8" s="41" t="n">
         <v>2</v>
       </c>
       <c r="C8" s="29" t="inlineStr">
@@ -4855,14 +4856,14 @@
           <t>Effectif déclaré au T1 = 2 alors que 3 salariés sont inscrits ; T2 déclare 1 sortie et un effectif final de 2 ⇒ T1 aurait dû être 3.</t>
         </is>
       </c>
-      <c r="F8" s="41" t="n"/>
+      <c r="F8" s="42" t="n"/>
       <c r="G8" s="29" t="inlineStr">
         <is>
           <t>Rectifier l'effectif du T1 auprès de la CNAS.</t>
         </is>
       </c>
-      <c r="H8" s="39" t="n"/>
-      <c r="I8" s="39" t="inlineStr">
+      <c r="H8" s="40" t="n"/>
+      <c r="I8" s="40" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -4874,7 +4875,7 @@
           <t>A05</t>
         </is>
       </c>
-      <c r="B9" s="40" t="n">
+      <c r="B9" s="41" t="n">
         <v>2</v>
       </c>
       <c r="C9" s="29" t="inlineStr">
@@ -4892,14 +4893,14 @@
           <t>Salarié totalement absent (non rémunéré) en juillet, disparu de la paie en août sans STC ni sortie déclarée.</t>
         </is>
       </c>
-      <c r="F9" s="41" t="n"/>
+      <c r="F9" s="42" t="n"/>
       <c r="G9" s="29" t="inlineStr">
         <is>
           <t>Établir le STC et déclarer la sortie dans l'EMS du T3 (échéance 30/10/2026).</t>
         </is>
       </c>
-      <c r="H9" s="39" t="n"/>
-      <c r="I9" s="39" t="inlineStr">
+      <c r="H9" s="40" t="n"/>
+      <c r="I9" s="40" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -4911,7 +4912,7 @@
           <t>A06</t>
         </is>
       </c>
-      <c r="B10" s="40" t="n">
+      <c r="B10" s="41" t="n">
         <v>2</v>
       </c>
       <c r="C10" s="29" t="inlineStr">
@@ -4929,14 +4930,14 @@
           <t>STC de 2 237,40 en août : une sortie à déclarer au T3.</t>
         </is>
       </c>
-      <c r="F10" s="41" t="n"/>
+      <c r="F10" s="42" t="n"/>
       <c r="G10" s="29" t="inlineStr">
         <is>
           <t>Déclarer la sortie dans l'EMS du T3.</t>
         </is>
       </c>
-      <c r="H10" s="39" t="n"/>
-      <c r="I10" s="39" t="inlineStr">
+      <c r="H10" s="40" t="n"/>
+      <c r="I10" s="40" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -4948,7 +4949,7 @@
           <t>A07</t>
         </is>
       </c>
-      <c r="B11" s="40" t="n">
+      <c r="B11" s="41" t="n">
         <v>2</v>
       </c>
       <c r="C11" s="29" t="inlineStr">
@@ -4966,7 +4967,7 @@
           <t>Déclarations T3 2026 (juil–sept) à établir ; paie de septembre non fournie.</t>
         </is>
       </c>
-      <c r="F11" s="38">
+      <c r="F11" s="39">
         <f>'Rappro CNAS'!J9+'Rappro CNAS'!J12</f>
         <v/>
       </c>
@@ -4975,8 +4976,8 @@
           <t>Transmettre les centralisateurs de septembre ; déposer et payer avant le 30/10/2026.</t>
         </is>
       </c>
-      <c r="H11" s="39" t="n"/>
-      <c r="I11" s="39" t="inlineStr">
+      <c r="H11" s="40" t="n"/>
+      <c r="I11" s="40" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -4988,7 +4989,7 @@
           <t>A08</t>
         </is>
       </c>
-      <c r="B12" s="42" t="n">
+      <c r="B12" s="43" t="n">
         <v>3</v>
       </c>
       <c r="C12" s="29" t="inlineStr">
@@ -5006,14 +5007,14 @@
           <t>Avril = mai et juillet = août strictement identiques (mêmes absences, heures sup., IRG) : variables probablement non saisies.</t>
         </is>
       </c>
-      <c r="F12" s="41" t="n"/>
+      <c r="F12" s="42" t="n"/>
       <c r="G12" s="29" t="inlineStr">
         <is>
           <t>Contrôler les pointages et bulletins de mai et août.</t>
         </is>
       </c>
-      <c r="H12" s="39" t="n"/>
-      <c r="I12" s="39" t="inlineStr">
+      <c r="H12" s="40" t="n"/>
+      <c r="I12" s="40" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5025,7 +5026,7 @@
           <t>A09</t>
         </is>
       </c>
-      <c r="B13" s="42" t="n">
+      <c r="B13" s="43" t="n">
         <v>3</v>
       </c>
       <c r="C13" s="29" t="inlineStr">
@@ -5043,7 +5044,7 @@
           <t>Frais de mission élevés (avril 41 615 ; mai 49 115, soit 47–55 % de l'assiette), non soumis à cotisations.</t>
         </is>
       </c>
-      <c r="F13" s="38">
+      <c r="F13" s="39">
         <f>'Paie TPM'!K26</f>
         <v/>
       </c>
@@ -5052,8 +5053,8 @@
           <t>Conserver ordres de mission et justificatifs ; risque de requalification en salaire.</t>
         </is>
       </c>
-      <c r="H13" s="39" t="n"/>
-      <c r="I13" s="39" t="inlineStr">
+      <c r="H13" s="40" t="n"/>
+      <c r="I13" s="40" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5065,7 +5066,7 @@
           <t>A10</t>
         </is>
       </c>
-      <c r="B14" s="42" t="n">
+      <c r="B14" s="43" t="n">
         <v>3</v>
       </c>
       <c r="C14" s="29" t="inlineStr">
@@ -5083,14 +5084,14 @@
           <t>Prime de responsabilité de 5,00 DA (janv.) et 1,14 DA (févr.) : paramètre vraisemblablement erroné (5 au lieu de 5 %).</t>
         </is>
       </c>
-      <c r="F14" s="41" t="n"/>
+      <c r="F14" s="42" t="n"/>
       <c r="G14" s="29" t="inlineStr">
         <is>
           <t>Corriger le paramètre B291 ; régulariser le rappel éventuel.</t>
         </is>
       </c>
-      <c r="H14" s="39" t="n"/>
-      <c r="I14" s="39" t="inlineStr">
+      <c r="H14" s="40" t="n"/>
+      <c r="I14" s="40" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5102,7 +5103,7 @@
           <t>A11</t>
         </is>
       </c>
-      <c r="B15" s="40" t="n">
+      <c r="B15" s="41" t="n">
         <v>2</v>
       </c>
       <c r="C15" s="29" t="inlineStr">
@@ -5120,7 +5121,7 @@
           <t>Bordereaux de versement CNAS à « 0,00 » : aucune preuve de paiement des cotisations dans le dossier.</t>
         </is>
       </c>
-      <c r="F15" s="38">
+      <c r="F15" s="39">
         <f>'Rappro CNAS'!K13</f>
         <v/>
       </c>
@@ -5129,8 +5130,8 @@
           <t>Joindre les quittances CNAS / avis de virement ; comptabiliser les règlements (débit 431).</t>
         </is>
       </c>
-      <c r="H15" s="39" t="n"/>
-      <c r="I15" s="39" t="inlineStr">
+      <c r="H15" s="40" t="n"/>
+      <c r="I15" s="40" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5142,7 +5143,7 @@
           <t>A12</t>
         </is>
       </c>
-      <c r="B16" s="40" t="n">
+      <c r="B16" s="41" t="n">
         <v>2</v>
       </c>
       <c r="C16" s="29" t="inlineStr">
@@ -5157,10 +5158,10 @@
       </c>
       <c r="E16" s="29" t="inlineStr">
         <is>
-          <t>IRG IMPORT : G50 juin et août conformes à la paie (écart d'arrondi ≤ 3 DA). G50 IMPORT janv.–mai et juillet, et toutes les G50 TPM, non fournies.</t>
-        </is>
-      </c>
-      <c r="F16" s="38">
+          <t>IRG IMPORT : G50 d'avril à août conformes à la paie (écarts d'arrondi ≤ 3 DA ; juillet : 2,30 DA retenus non reversés). Mars non vérifiable (paie absente). G50 janv.–févr. IMPORT et toutes les G50 TPM non fournies.</t>
+        </is>
+      </c>
+      <c r="F16" s="39">
         <f>'Échéancier IRG-CNAS'!G13</f>
         <v/>
       </c>
@@ -5169,8 +5170,8 @@
           <t>Fournir les G50 manquantes et compléter la colonne I de l'échéancier.</t>
         </is>
       </c>
-      <c r="H16" s="39" t="n"/>
-      <c r="I16" s="39" t="inlineStr">
+      <c r="H16" s="40" t="n"/>
+      <c r="I16" s="40" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5182,7 +5183,7 @@
           <t>A13</t>
         </is>
       </c>
-      <c r="B17" s="42" t="n">
+      <c r="B17" s="43" t="n">
         <v>3</v>
       </c>
       <c r="C17" s="29" t="inlineStr">
@@ -5200,14 +5201,14 @@
           <t>Paie paramétrée CACOBATPH (taux X504) mais aucune déclaration CACOBATPH (congés payés / intempéries) dans le dossier.</t>
         </is>
       </c>
-      <c r="F17" s="41" t="n"/>
+      <c r="F17" s="42" t="n"/>
       <c r="G17" s="29" t="inlineStr">
         <is>
           <t>Fournir les déclarations et paiements CACOBATPH 2026.</t>
         </is>
       </c>
-      <c r="H17" s="39" t="n"/>
-      <c r="I17" s="39" t="inlineStr">
+      <c r="H17" s="40" t="n"/>
+      <c r="I17" s="40" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5219,7 +5220,7 @@
           <t>A14</t>
         </is>
       </c>
-      <c r="B18" s="42" t="n">
+      <c r="B18" s="43" t="n">
         <v>3</v>
       </c>
       <c r="C18" s="29" t="inlineStr">
@@ -5237,14 +5238,14 @@
           <t>Libellés divergents : « D.P.R.COMPAGNY » / « DPR COMPAGNY » ; en-tête de paie TPM à l'adresse VGE TIZI alors que l'affiliation TPM est à TISSA.</t>
         </is>
       </c>
-      <c r="F18" s="41" t="n"/>
+      <c r="F18" s="42" t="n"/>
       <c r="G18" s="29" t="inlineStr">
         <is>
           <t>Harmoniser raison sociale et adresse dans le logiciel de paie.</t>
         </is>
       </c>
-      <c r="H18" s="39" t="n"/>
-      <c r="I18" s="39" t="inlineStr">
+      <c r="H18" s="40" t="n"/>
+      <c r="I18" s="40" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5256,7 +5257,7 @@
           <t>A15</t>
         </is>
       </c>
-      <c r="B19" s="42" t="n">
+      <c r="B19" s="43" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="29" t="inlineStr">
@@ -5274,14 +5275,14 @@
           <t>Périodicité mixte : déclarations mensuelles (janv., mars) puis trimestrielle (T2).</t>
         </is>
       </c>
-      <c r="F19" s="41" t="n"/>
+      <c r="F19" s="42" t="n"/>
       <c r="G19" s="29" t="inlineStr">
         <is>
           <t>Confirmer auprès de la CNAS le passage au trimestriel après la baisse d'effectif (12 → 5).</t>
         </is>
       </c>
-      <c r="H19" s="39" t="n"/>
-      <c r="I19" s="39" t="inlineStr">
+      <c r="H19" s="40" t="n"/>
+      <c r="I19" s="40" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5293,7 +5294,7 @@
           <t>A16</t>
         </is>
       </c>
-      <c r="B20" s="42" t="n">
+      <c r="B20" s="43" t="n">
         <v>3</v>
       </c>
       <c r="C20" s="29" t="inlineStr">
@@ -5311,14 +5312,14 @@
           <t>IRG non vérifiable salarié par salarié (centralisateurs uniquement).</t>
         </is>
       </c>
-      <c r="F20" s="41" t="n"/>
+      <c r="F20" s="42" t="n"/>
       <c r="G20" s="29" t="inlineStr">
         <is>
           <t>Fournir le livre de paie individuel / bulletins.</t>
         </is>
       </c>
-      <c r="H20" s="39" t="n"/>
-      <c r="I20" s="39" t="inlineStr">
+      <c r="H20" s="40" t="n"/>
+      <c r="I20" s="40" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5330,7 +5331,7 @@
           <t>A17</t>
         </is>
       </c>
-      <c r="B21" s="37" t="n">
+      <c r="B21" s="38" t="n">
         <v>1</v>
       </c>
       <c r="C21" s="29" t="inlineStr">
@@ -5348,7 +5349,7 @@
           <t>TVA collectée TPM (44537) et location (44527) jamais soldées : 58,9 M DA cumulés au 31/12/2025. En 2025, 4 839 300 de TVA TPM générée, seuls 391 208 passés en G50 (déc.).</t>
         </is>
       </c>
-      <c r="F21" s="38">
+      <c r="F21" s="39">
         <f>-('Balance 2024-2025'!D48+'Balance 2024-2025'!D47)</f>
         <v/>
       </c>
@@ -5357,8 +5358,8 @@
           <t>Rapprocher avec les G50 TPM 2023–2025 ; si TVA non déclarée, régulariser ; sinon passer les écritures de G50 manquantes.</t>
         </is>
       </c>
-      <c r="H21" s="39" t="n"/>
-      <c r="I21" s="39" t="inlineStr">
+      <c r="H21" s="40" t="n"/>
+      <c r="I21" s="40" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5370,7 +5371,7 @@
           <t>A18</t>
         </is>
       </c>
-      <c r="B22" s="37" t="n">
+      <c r="B22" s="38" t="n">
         <v>1</v>
       </c>
       <c r="C22" s="29" t="inlineStr">
@@ -5385,20 +5386,20 @@
       </c>
       <c r="E22" s="29" t="inlineStr">
         <is>
-          <t>G50 juin et août 2026 annotées « CA 03/2026 à déclarer pour manque TVA à récupérer » : le CA de mars 2026 est déclaré par fractions sur des mois ultérieurs (10 479 294 + 4 413 684 ; reste TVA noté 5 417 538).</t>
-        </is>
-      </c>
-      <c r="F22" s="38">
-        <f>'G50 2026'!B35</f>
+          <t>CA de mars 2026 réalisé 27 006 870 (annotation G50), mais seulement 3 445 200 déclarés en mars « pour manque TVA à récupérer » : 23 561 670 de CA reportés sur avril–août. En avril, le CA annoté (13 157 894,74) est calculé pour obtenir 2 500 000 de TVA. Le CA déclaré mensuellement est ajusté à la TVA déductible disponible.</t>
+        </is>
+      </c>
+      <c r="F22" s="39">
+        <f>'G50 2026'!B40</f>
         <v/>
       </c>
       <c r="G22" s="29" t="inlineStr">
         <is>
-          <t>Déclarer le CA au titre du mois de réalisation ; chiffrer et régulariser le retard sur mars 2026 (pénalités et majorations).</t>
-        </is>
-      </c>
-      <c r="H22" s="39" t="n"/>
-      <c r="I22" s="39" t="inlineStr">
+          <t>Déclarer le CA au titre du mois de réalisation ; rapprocher le CA déclaré du journal des ventes 2026 ; chiffrer les pénalités de retard sur la TVA différée.</t>
+        </is>
+      </c>
+      <c r="H22" s="40" t="n"/>
+      <c r="I22" s="40" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5410,7 +5411,7 @@
           <t>A19</t>
         </is>
       </c>
-      <c r="B23" s="40" t="n">
+      <c r="B23" s="41" t="n">
         <v>2</v>
       </c>
       <c r="C23" s="29" t="inlineStr">
@@ -5425,11 +5426,11 @@
       </c>
       <c r="E23" s="29" t="inlineStr">
         <is>
-          <t>IRG retenu sur les salariés TPM absent des G50 IMPORT (juin, août).</t>
-        </is>
-      </c>
-      <c r="F23" s="38">
-        <f>'G50 2026'!B21+'G50 2026'!C21</f>
+          <t>IRG retenu sur les salariés TPM (mars–août) absent des G50 IMPORT.</t>
+        </is>
+      </c>
+      <c r="F23" s="39">
+        <f>'G50 2026'!H22</f>
         <v/>
       </c>
       <c r="G23" s="29" t="inlineStr">
@@ -5437,8 +5438,8 @@
           <t>Fournir les G50 TPM 2026 ou régulariser.</t>
         </is>
       </c>
-      <c r="H23" s="39" t="n"/>
-      <c r="I23" s="39" t="inlineStr">
+      <c r="H23" s="40" t="n"/>
+      <c r="I23" s="40" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5450,7 +5451,7 @@
           <t>A20</t>
         </is>
       </c>
-      <c r="B24" s="40" t="n">
+      <c r="B24" s="41" t="n">
         <v>2</v>
       </c>
       <c r="C24" s="29" t="inlineStr">
@@ -5468,7 +5469,7 @@
           <t>Écriture du 31/12/2025 « POUR SOLDE PRCT EXE 2025 » passée en sens inverse (D 44410 / C 444, 3 074 299) : dette IBS 9,79 M et acomptes 6,15 M au lieu d'un net de 3 642 951.</t>
         </is>
       </c>
-      <c r="F24" s="38" t="n">
+      <c r="F24" s="39" t="n">
         <v>3074299</v>
       </c>
       <c r="G24" s="29" t="inlineStr">
@@ -5476,8 +5477,8 @@
           <t>Contrepasser et compenser (D 444 / C 44410) ; vérifier le paiement du solde IBS 2025 en 2026.</t>
         </is>
       </c>
-      <c r="H24" s="39" t="n"/>
-      <c r="I24" s="39" t="inlineStr">
+      <c r="H24" s="40" t="n"/>
+      <c r="I24" s="40" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5489,7 +5490,7 @@
           <t>A21</t>
         </is>
       </c>
-      <c r="B25" s="40" t="n">
+      <c r="B25" s="41" t="n">
         <v>2</v>
       </c>
       <c r="C25" s="29" t="inlineStr">
@@ -5507,7 +5508,7 @@
           <t>Solde IBS 2024 réglé le 03/07/2025 ; IBS 2025 net à liquider de 3 642 951 (précomptes douane déduits).</t>
         </is>
       </c>
-      <c r="F25" s="38" t="n">
+      <c r="F25" s="39" t="n">
         <v>3642951</v>
       </c>
       <c r="G25" s="29" t="inlineStr">
@@ -5515,8 +5516,8 @@
           <t>Vérifier les dates d'échéance de liquidation, les pénalités éventuelles et la preuve de paiement 2026.</t>
         </is>
       </c>
-      <c r="H25" s="39" t="n"/>
-      <c r="I25" s="39" t="inlineStr">
+      <c r="H25" s="40" t="n"/>
+      <c r="I25" s="40" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5528,7 +5529,7 @@
           <t>A22</t>
         </is>
       </c>
-      <c r="B26" s="40" t="n">
+      <c r="B26" s="41" t="n">
         <v>2</v>
       </c>
       <c r="C26" s="29" t="inlineStr">
@@ -5546,7 +5547,7 @@
           <t>Caisse de 12,1 M au 31/12/2025 (pic de 22,5 M) ; remboursement en espèces de 6 800 000 à SARL DPR AXXAM le 06/12/2025.</t>
         </is>
       </c>
-      <c r="F26" s="38">
+      <c r="F26" s="39">
         <f>'Balance 2024-2025'!D67</f>
         <v/>
       </c>
@@ -5555,8 +5556,8 @@
           <t>PV de caisse au 31/12 ; respecter l'obligation de paiement scriptural au-delà des seuils réglementaires.</t>
         </is>
       </c>
-      <c r="H26" s="39" t="n"/>
-      <c r="I26" s="39" t="inlineStr">
+      <c r="H26" s="40" t="n"/>
+      <c r="I26" s="40" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5568,7 +5569,7 @@
           <t>A23</t>
         </is>
       </c>
-      <c r="B27" s="40" t="n">
+      <c r="B27" s="41" t="n">
         <v>2</v>
       </c>
       <c r="C27" s="29" t="inlineStr">
@@ -5586,7 +5587,7 @@
           <t>100 % du CA TPM 2025 (25,47 M) facturé à SARL DPR AXXAM BRIQUETERIE ; aucune facturation TPM d'oct. à déc. 2025 alors que du personnel TPM reste payé.</t>
         </is>
       </c>
-      <c r="F27" s="38">
+      <c r="F27" s="39">
         <f>-'Balance 2024-2025'!D100</f>
         <v/>
       </c>
@@ -5595,8 +5596,8 @@
           <t>Documenter les conventions intra-groupe et la facturation d'oct.–déc. 2025.</t>
         </is>
       </c>
-      <c r="H27" s="39" t="n"/>
-      <c r="I27" s="39" t="inlineStr">
+      <c r="H27" s="40" t="n"/>
+      <c r="I27" s="40" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5608,7 +5609,7 @@
           <t>A24</t>
         </is>
       </c>
-      <c r="B28" s="40" t="n">
+      <c r="B28" s="41" t="n">
         <v>2</v>
       </c>
       <c r="C28" s="29" t="inlineStr">
@@ -5626,7 +5627,7 @@
           <t>Compte d'attente 47000 non soldé (« SARL FAHAS ?? », « TRESORERIE BEJAIA ?? », chèques).</t>
         </is>
       </c>
-      <c r="F28" s="38">
+      <c r="F28" s="39">
         <f>'Balance 2024-2025'!D59</f>
         <v/>
       </c>
@@ -5635,8 +5636,8 @@
           <t>Identifier et apurer avant clôture.</t>
         </is>
       </c>
-      <c r="H28" s="39" t="n"/>
-      <c r="I28" s="39" t="inlineStr">
+      <c r="H28" s="40" t="n"/>
+      <c r="I28" s="40" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5648,7 +5649,7 @@
           <t>A25</t>
         </is>
       </c>
-      <c r="B29" s="40" t="n">
+      <c r="B29" s="41" t="n">
         <v>2</v>
       </c>
       <c r="C29" s="29" t="inlineStr">
@@ -5666,7 +5667,7 @@
           <t>Compte 63120 « prime imposable » non soumise à cotisation : 957 406 en 2025 et 1 139 275 en 2024 (même mécanisme que A03).</t>
         </is>
       </c>
-      <c r="F29" s="38">
+      <c r="F29" s="39">
         <f>'États 2024-2025'!C24+'États 2024-2025'!D24</f>
         <v/>
       </c>
@@ -5675,8 +5676,8 @@
           <t>Analyser les primes concernées ; régulariser si elles sont cotisables.</t>
         </is>
       </c>
-      <c r="H29" s="39" t="n"/>
-      <c r="I29" s="39" t="inlineStr">
+      <c r="H29" s="40" t="n"/>
+      <c r="I29" s="40" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5688,7 +5689,7 @@
           <t>A26</t>
         </is>
       </c>
-      <c r="B30" s="42" t="n">
+      <c r="B30" s="43" t="n">
         <v>3</v>
       </c>
       <c r="C30" s="29" t="inlineStr">
@@ -5706,7 +5707,7 @@
           <t>Banque CPA El Kseur (51220) créditrice de 12,43 M au 31/12/2025 : découvert présenté en banque.</t>
         </is>
       </c>
-      <c r="F30" s="38">
+      <c r="F30" s="39">
         <f>ABS('Balance 2024-2025'!D63)</f>
         <v/>
       </c>
@@ -5715,8 +5716,8 @@
           <t>Reclasser en 519 ; vérifier les agios (aucune charge 661 en 2025).</t>
         </is>
       </c>
-      <c r="H30" s="39" t="n"/>
-      <c r="I30" s="39" t="inlineStr">
+      <c r="H30" s="40" t="n"/>
+      <c r="I30" s="40" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5728,7 +5729,7 @@
           <t>A27</t>
         </is>
       </c>
-      <c r="B31" s="42" t="n">
+      <c r="B31" s="43" t="n">
         <v>3</v>
       </c>
       <c r="C31" s="29" t="inlineStr">
@@ -5746,7 +5747,7 @@
           <t>Reversements IRG 2025 parfois partiels (févr., juin) et rattrapés le mois suivant ; amendes 2025 : douane 100 000, CNAS 1 746.</t>
         </is>
       </c>
-      <c r="F31" s="38">
+      <c r="F31" s="39">
         <f>'Balance 2024-2025'!D93</f>
         <v/>
       </c>
@@ -5755,8 +5756,8 @@
           <t>Reverser l'IRG en totalité chaque mois.</t>
         </is>
       </c>
-      <c r="H31" s="39" t="n"/>
-      <c r="I31" s="39" t="inlineStr">
+      <c r="H31" s="40" t="n"/>
+      <c r="I31" s="40" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5768,7 +5769,7 @@
           <t>A28</t>
         </is>
       </c>
-      <c r="B32" s="42" t="n">
+      <c r="B32" s="43" t="n">
         <v>3</v>
       </c>
       <c r="C32" s="29" t="inlineStr">
@@ -5783,17 +5784,17 @@
       </c>
       <c r="E32" s="29" t="inlineStr">
         <is>
-          <t>Modèle G50 non mis à jour : dates de signature 2022, onglet de saisie figé (mai, TVA 17 %) ; libellés de comptes de TVA à 17 %.</t>
-        </is>
-      </c>
-      <c r="F32" s="41" t="n"/>
+          <t>Modèle G50 non mis à jour : dates de signature imprimées de 2021–2022 sur toutes les G50 2026, onglet de saisie figé (mai, TVA 17 %) ; libellés de comptes de TVA à 17 %.</t>
+        </is>
+      </c>
+      <c r="F32" s="42" t="n"/>
       <c r="G32" s="29" t="inlineStr">
         <is>
           <t>Mettre à jour le modèle et les libellés (TVA 19 %).</t>
         </is>
       </c>
-      <c r="H32" s="39" t="n"/>
-      <c r="I32" s="39" t="inlineStr">
+      <c r="H32" s="40" t="n"/>
+      <c r="I32" s="40" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5805,7 +5806,7 @@
           <t>A29</t>
         </is>
       </c>
-      <c r="B33" s="42" t="n">
+      <c r="B33" s="43" t="n">
         <v>3</v>
       </c>
       <c r="C33" s="29" t="inlineStr">
@@ -5823,8 +5824,8 @@
           <t>Taxe d'apprentissage de 44 091 (août 2026) sur une base de 4 409 079 à justifier.</t>
         </is>
       </c>
-      <c r="F33" s="38">
-        <f>'G50 2026'!C23</f>
+      <c r="F33" s="39">
+        <f>'G50 2026'!G26</f>
         <v/>
       </c>
       <c r="G33" s="29" t="inlineStr">
@@ -5832,8 +5833,8 @@
           <t>Justifier la base (1 % de la masse salariale de référence).</t>
         </is>
       </c>
-      <c r="H33" s="39" t="n"/>
-      <c r="I33" s="39" t="inlineStr">
+      <c r="H33" s="40" t="n"/>
+      <c r="I33" s="40" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5845,7 +5846,7 @@
           <t>A30</t>
         </is>
       </c>
-      <c r="B34" s="42" t="n">
+      <c r="B34" s="43" t="n">
         <v>3</v>
       </c>
       <c r="C34" s="29" t="inlineStr">
@@ -5860,20 +5861,20 @@
       </c>
       <c r="E34" s="29" t="inlineStr">
         <is>
-          <t>Précompte TVA de juin 2026 (178 353) non repris en août ; G50 de juillet non fournie.</t>
-        </is>
-      </c>
-      <c r="F34" s="38">
-        <f>'G50 2026'!B15</f>
+          <t>Droit de timbre : même base (177 058) en avril et mai, mais 8 944 puis 3 173 ; aucun timbre les autres mois.</t>
+        </is>
+      </c>
+      <c r="F34" s="39">
+        <f>'G50 2026'!H24</f>
         <v/>
       </c>
       <c r="G34" s="29" t="inlineStr">
         <is>
-          <t>Vérifier l'imputation en juillet.</t>
-        </is>
-      </c>
-      <c r="H34" s="39" t="n"/>
-      <c r="I34" s="39" t="inlineStr">
+          <t>Justifier la base (ventes en espèces) et le taux appliqué.</t>
+        </is>
+      </c>
+      <c r="H34" s="40" t="n"/>
+      <c r="I34" s="40" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5885,7 +5886,7 @@
           <t>A31</t>
         </is>
       </c>
-      <c r="B35" s="42" t="n">
+      <c r="B35" s="43" t="n">
         <v>3</v>
       </c>
       <c r="C35" s="29" t="inlineStr">
@@ -5903,14 +5904,14 @@
           <t>Clients débiteurs 387,1 M et avances clients 314,6 M ; fournisseurs débiteurs 46,2 M au 31/12/2025.</t>
         </is>
       </c>
-      <c r="F35" s="41" t="n"/>
+      <c r="F35" s="42" t="n"/>
       <c r="G35" s="29" t="inlineStr">
         <is>
           <t>Lettrer les comptes clients/fournisseurs et compenser les avances soldées.</t>
         </is>
       </c>
-      <c r="H35" s="39" t="n"/>
-      <c r="I35" s="39" t="inlineStr">
+      <c r="H35" s="40" t="n"/>
+      <c r="I35" s="40" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5936,7 +5937,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6012,7 +6013,7 @@
           <t>Janv–août 2026</t>
         </is>
       </c>
-      <c r="E5" s="43" t="inlineStr">
+      <c r="E5" s="44" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6042,7 +6043,7 @@
           <t>Janv–août 2026</t>
         </is>
       </c>
-      <c r="E6" s="43" t="inlineStr">
+      <c r="E6" s="44" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6068,7 +6069,7 @@
           <t>Janvier 2026</t>
         </is>
       </c>
-      <c r="E7" s="43" t="inlineStr">
+      <c r="E7" s="44" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6098,7 +6099,7 @@
           <t>Mars 2026</t>
         </is>
       </c>
-      <c r="E8" s="43" t="inlineStr">
+      <c r="E8" s="44" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6128,7 +6129,7 @@
           <t>T2 2026</t>
         </is>
       </c>
-      <c r="E9" s="43" t="inlineStr">
+      <c r="E9" s="44" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6158,7 +6159,7 @@
           <t>T1 2026</t>
         </is>
       </c>
-      <c r="E10" s="43" t="inlineStr">
+      <c r="E10" s="44" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6188,7 +6189,7 @@
           <t>T2 2026</t>
         </is>
       </c>
-      <c r="E11" s="43" t="inlineStr">
+      <c r="E11" s="44" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6218,7 +6219,7 @@
           <t>Février 2026</t>
         </is>
       </c>
-      <c r="E12" s="44" t="inlineStr">
+      <c r="E12" s="45" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
@@ -6248,7 +6249,7 @@
           <t>Mars 2026</t>
         </is>
       </c>
-      <c r="E13" s="44" t="inlineStr">
+      <c r="E13" s="45" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
@@ -6274,7 +6275,7 @@
           <t>Septembre 2026</t>
         </is>
       </c>
-      <c r="E14" s="44" t="inlineStr">
+      <c r="E14" s="45" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
@@ -6304,7 +6305,7 @@
           <t>T3 2026</t>
         </is>
       </c>
-      <c r="E15" s="44" t="inlineStr">
+      <c r="E15" s="45" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
@@ -6334,7 +6335,7 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="E16" s="44" t="inlineStr">
+      <c r="E16" s="45" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
@@ -6364,7 +6365,7 @@
           <t>Juin 2026</t>
         </is>
       </c>
-      <c r="E17" s="43" t="inlineStr">
+      <c r="E17" s="44" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6394,7 +6395,7 @@
           <t>Août 2026</t>
         </is>
       </c>
-      <c r="E18" s="43" t="inlineStr">
+      <c r="E18" s="44" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6424,7 +6425,7 @@
           <t>Exercice 2024</t>
         </is>
       </c>
-      <c r="E19" s="43" t="inlineStr">
+      <c r="E19" s="44" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6454,7 +6455,7 @@
           <t>Exercice 2025</t>
         </is>
       </c>
-      <c r="E20" s="43" t="inlineStr">
+      <c r="E20" s="44" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6471,7 +6472,7 @@
       </c>
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>G50 IMPORT janv.–mai, juil., sept. 2026</t>
+          <t>G50_ARL_DPR_COMPANY_IMPORT_03/04/05/07-2026.xls</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
@@ -6481,15 +6482,19 @@
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>Mars, avril, mai, juillet 2026</t>
         </is>
       </c>
       <c r="E21" s="44" t="inlineStr">
         <is>
-          <t>Manquante</t>
-        </is>
-      </c>
-      <c r="F21" s="12" t="inlineStr"/>
+          <t>Reçue</t>
+        </is>
+      </c>
+      <c r="F21" s="12" t="inlineStr">
+        <is>
+          <t>Série mars–août complète</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="12" t="n">
@@ -6497,29 +6502,25 @@
       </c>
       <c r="B22" s="12" t="inlineStr">
         <is>
-          <t>G50 TPM 2026 (et rapprochement TVA TPM 2023–2025)</t>
+          <t>G50 IMPORT janvier, février et septembre 2026</t>
         </is>
       </c>
       <c r="C22" s="12" t="inlineStr">
         <is>
-          <t>TPM</t>
+          <t>IMPORT</t>
         </is>
       </c>
       <c r="D22" s="12" t="inlineStr">
         <is>
-          <t>2023–2026</t>
-        </is>
-      </c>
-      <c r="E22" s="44" t="inlineStr">
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E22" s="45" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
       </c>
-      <c r="F22" s="12" t="inlineStr">
-        <is>
-          <t>Voir A17, A19</t>
-        </is>
-      </c>
+      <c r="F22" s="12" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="12" t="n">
@@ -6527,12 +6528,12 @@
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>Journal comptable 2026 (PCCOMPTA)</t>
+          <t>Journal des ventes / factures 2026</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>Société</t>
+          <t>IMPORT</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
@@ -6540,14 +6541,14 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="E23" s="44" t="inlineStr">
+      <c r="E23" s="45" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
       </c>
       <c r="F23" s="12" t="inlineStr">
         <is>
-          <t>Pour rapprocher paie et G50 avec la comptabilité</t>
+          <t>Voir A18 : CA réel par mois</t>
         </is>
       </c>
     </row>
@@ -6557,27 +6558,27 @@
       </c>
       <c r="B24" s="12" t="inlineStr">
         <is>
-          <t>Liasse fiscale / bilan 2025 déposé et preuve de paiement IBS</t>
+          <t>G50 TPM 2026 (et rapprochement TVA TPM 2023–2025)</t>
         </is>
       </c>
       <c r="C24" s="12" t="inlineStr">
         <is>
-          <t>Société</t>
+          <t>TPM</t>
         </is>
       </c>
       <c r="D24" s="12" t="inlineStr">
         <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="E24" s="44" t="inlineStr">
+          <t>2023–2026</t>
+        </is>
+      </c>
+      <c r="E24" s="45" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
       </c>
       <c r="F24" s="12" t="inlineStr">
         <is>
-          <t>Voir A20, A21</t>
+          <t>Voir A17, A19</t>
         </is>
       </c>
     </row>
@@ -6587,7 +6588,7 @@
       </c>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>PV de caisse au 31/12/2025</t>
+          <t>Journal comptable 2026 (PCCOMPTA)</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
@@ -6597,17 +6598,17 @@
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="E25" s="44" t="inlineStr">
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E25" s="45" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
       </c>
       <c r="F25" s="12" t="inlineStr">
         <is>
-          <t>Voir A22</t>
+          <t>Pour rapprocher paie et G50 avec la comptabilité</t>
         </is>
       </c>
     </row>
@@ -6617,25 +6618,29 @@
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>Déclarations et paiements CACOBATPH</t>
+          <t>Liasse fiscale / bilan 2025 déposé et preuve de paiement IBS</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>Les deux</t>
+          <t>Société</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="E26" s="44" t="inlineStr">
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E26" s="45" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
       </c>
-      <c r="F26" s="12" t="inlineStr"/>
+      <c r="F26" s="12" t="inlineStr">
+        <is>
+          <t>Voir A20, A21</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="12" t="n">
@@ -6643,27 +6648,27 @@
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>Livre de paie individuel / bulletins</t>
+          <t>PV de caisse au 31/12/2025</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>Les deux</t>
+          <t>Société</t>
         </is>
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="E27" s="44" t="inlineStr">
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E27" s="45" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
       </c>
       <c r="F27" s="12" t="inlineStr">
         <is>
-          <t>Pour contrôle IRG</t>
+          <t>Voir A22</t>
         </is>
       </c>
     </row>
@@ -6673,12 +6678,12 @@
       </c>
       <c r="B28" s="12" t="inlineStr">
         <is>
-          <t>Ordres de mission et justificatifs de frais</t>
+          <t>Déclarations et paiements CACOBATPH</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
         <is>
-          <t>TPM</t>
+          <t>Les deux</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
@@ -6686,16 +6691,12 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="E28" s="44" t="inlineStr">
+      <c r="E28" s="45" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
       </c>
-      <c r="F28" s="12" t="inlineStr">
-        <is>
-          <t>Frais de mission élevés</t>
-        </is>
-      </c>
+      <c r="F28" s="12" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="12" t="n">
@@ -6703,25 +6704,85 @@
       </c>
       <c r="B29" s="12" t="inlineStr">
         <is>
+          <t>Livre de paie individuel / bulletins</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>Les deux</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E29" s="45" t="inlineStr">
+        <is>
+          <t>Manquante</t>
+        </is>
+      </c>
+      <c r="F29" s="12" t="inlineStr">
+        <is>
+          <t>Pour contrôle IRG</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>Ordres de mission et justificatifs de frais</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>TPM</t>
+        </is>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E30" s="45" t="inlineStr">
+        <is>
+          <t>Manquante</t>
+        </is>
+      </c>
+      <c r="F30" s="12" t="inlineStr">
+        <is>
+          <t>Frais de mission élevés</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
           <t>Relevés bancaires — virements de salaires</t>
         </is>
       </c>
-      <c r="C29" s="12" t="inlineStr">
+      <c r="C31" s="12" t="inlineStr">
         <is>
           <t>Les deux</t>
         </is>
       </c>
-      <c r="D29" s="12" t="inlineStr">
+      <c r="D31" s="12" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="E29" s="44" t="inlineStr">
+      <c r="E31" s="45" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
       </c>
-      <c r="F29" s="12" t="inlineStr">
+      <c r="F31" s="12" t="inlineStr">
         <is>
           <t>Pour lettrage du 421</t>
         </is>
@@ -15574,7 +15635,7 @@
       </c>
       <c r="I5" s="33" t="n"/>
       <c r="J5" s="30">
-        <f>IF(I5="","",I5-E5)</f>
+        <f>IF(I5="","",IF(E5=0,"paie absente",I5-E5))</f>
         <v/>
       </c>
       <c r="K5" s="6">
@@ -15631,7 +15692,7 @@
       </c>
       <c r="I6" s="33" t="n"/>
       <c r="J6" s="30">
-        <f>IF(I6="","",I6-E6)</f>
+        <f>IF(I6="","",IF(E6=0,"paie absente",I6-E6))</f>
         <v/>
       </c>
       <c r="K6" s="6">
@@ -15686,9 +15747,12 @@
           <t>20/04/2026</t>
         </is>
       </c>
-      <c r="I7" s="33" t="n"/>
+      <c r="I7" s="6">
+        <f>'G50 2026'!B19</f>
+        <v/>
+      </c>
       <c r="J7" s="30">
-        <f>IF(I7="","",I7-E7)</f>
+        <f>IF(I7="","",IF(E7=0,"paie absente",I7-E7))</f>
         <v/>
       </c>
       <c r="K7" s="6">
@@ -15743,9 +15807,12 @@
           <t>20/05/2026</t>
         </is>
       </c>
-      <c r="I8" s="33" t="n"/>
+      <c r="I8" s="6">
+        <f>'G50 2026'!C19</f>
+        <v/>
+      </c>
       <c r="J8" s="30">
-        <f>IF(I8="","",I8-E8)</f>
+        <f>IF(I8="","",IF(E8=0,"paie absente",I8-E8))</f>
         <v/>
       </c>
       <c r="K8" s="6">
@@ -15800,9 +15867,12 @@
           <t>20/06/2026</t>
         </is>
       </c>
-      <c r="I9" s="33" t="n"/>
+      <c r="I9" s="6">
+        <f>'G50 2026'!D19</f>
+        <v/>
+      </c>
       <c r="J9" s="30">
-        <f>IF(I9="","",I9-E9)</f>
+        <f>IF(I9="","",IF(E9=0,"paie absente",I9-E9))</f>
         <v/>
       </c>
       <c r="K9" s="6">
@@ -15858,11 +15928,11 @@
         </is>
       </c>
       <c r="I10" s="6">
-        <f>'G50 2026'!B18</f>
+        <f>'G50 2026'!E19</f>
         <v/>
       </c>
       <c r="J10" s="30">
-        <f>IF(I10="","",I10-E10)</f>
+        <f>IF(I10="","",IF(E10=0,"paie absente",I10-E10))</f>
         <v/>
       </c>
       <c r="K10" s="6">
@@ -15917,9 +15987,12 @@
           <t>20/08/2026</t>
         </is>
       </c>
-      <c r="I11" s="33" t="n"/>
+      <c r="I11" s="6">
+        <f>'G50 2026'!F19</f>
+        <v/>
+      </c>
       <c r="J11" s="30">
-        <f>IF(I11="","",I11-E11)</f>
+        <f>IF(I11="","",IF(E11=0,"paie absente",I11-E11))</f>
         <v/>
       </c>
       <c r="K11" s="6">
@@ -15975,11 +16048,11 @@
         </is>
       </c>
       <c r="I12" s="6">
-        <f>'G50 2026'!C18</f>
+        <f>'G50 2026'!G19</f>
         <v/>
       </c>
       <c r="J12" s="30">
-        <f>IF(I12="","",I12-E12)</f>
+        <f>IF(I12="","",IF(E12=0,"paie absente",I12-E12))</f>
         <v/>
       </c>
       <c r="K12" s="6">
@@ -16045,7 +16118,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Colonne I : G50 IMPORT juin et août reçues (liées à « G50 2026 ») ; autres mois en jaune à compléter. Écart IRG = G50 − IRG paie IMPORT. L'IRG TPM (colonne F) doit figurer sur une G50 TPM distincte (non fournie).</t>
+          <t>Colonne I : G50 IMPORT mars à août reçues (liées à « G50 2026 ») ; janvier et février en jaune à compléter. Écart IRG = G50 − IRG paie IMPORT. L'IRG TPM (colonne F) doit figurer sur une G50 TPM distincte (non fournie).</t>
         </is>
       </c>
     </row>
@@ -16061,13 +16134,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="55" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -16080,7 +16158,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Sources : G50_ARL_DPR_COMPANY_IMPORT_06-2026.xls et _08-2026_.xls (feuilles G.50-1/2/3). Valeurs en bleu = lues sur les G50.</t>
+          <t>Sources : fichiers G50_ARL_DPR_COMPANY_IMPORT_03 à 08-2026.xls (feuilles G.50-1/2/3). Valeurs en bleu = lues sur les G50.</t>
         </is>
       </c>
     </row>
@@ -16095,7 +16173,7 @@
       </c>
       <c r="C4" s="21" t="inlineStr">
         <is>
-          <t>Taux porté sur la G50 (ligne E3B22)</t>
+          <t>Taux porté sur les G50 (ligne E3B22)</t>
         </is>
       </c>
     </row>
@@ -16107,15 +16185,40 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
+          <t>Mars 2026</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>Avr 2026</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>Mai 2026</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
           <t>Juin 2026</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>Juil 2026</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="inlineStr">
         <is>
           <t>Août 2026</t>
         </is>
       </c>
-      <c r="D6" s="11" t="inlineStr">
+      <c r="H6" s="11" t="inlineStr">
+        <is>
+          <t>Cumul</t>
+        </is>
+      </c>
+      <c r="I6" s="11" t="inlineStr">
         <is>
           <t>Commentaire</t>
         </is>
@@ -16128,14 +16231,30 @@
         </is>
       </c>
       <c r="B7" s="25" t="n">
+        <v>3445200</v>
+      </c>
+      <c r="C7" s="25" t="n">
+        <v>23988307</v>
+      </c>
+      <c r="D7" s="25" t="n">
+        <v>16671298</v>
+      </c>
+      <c r="E7" s="25" t="n">
         <v>10479294</v>
       </c>
-      <c r="C7" s="25" t="n">
+      <c r="F7" s="25" t="n">
+        <v>7604135</v>
+      </c>
+      <c r="G7" s="25" t="n">
         <v>4413684</v>
       </c>
-      <c r="D7" s="35" t="inlineStr">
-        <is>
-          <t>Annoté sur la G50 : « TOTAL CA 03/2026 » / « CA A DECLARER 03/2026 POUR MANQUE TVA A RECUPERER »</t>
+      <c r="H7" s="7">
+        <f>SUM(B7:G7)</f>
+        <v/>
+      </c>
+      <c r="I7" s="35" t="inlineStr">
+        <is>
+          <t>Revente en l'état</t>
         </is>
       </c>
     </row>
@@ -16146,12 +16265,28 @@
         </is>
       </c>
       <c r="B8" s="25" t="n">
+        <v>654588</v>
+      </c>
+      <c r="C8" s="25" t="n">
+        <v>4557778</v>
+      </c>
+      <c r="D8" s="25" t="n">
+        <v>3167547</v>
+      </c>
+      <c r="E8" s="25" t="n">
         <v>1991066</v>
       </c>
-      <c r="C8" s="25" t="n">
+      <c r="F8" s="25" t="n">
+        <v>1444786</v>
+      </c>
+      <c r="G8" s="25" t="n">
         <v>838600</v>
       </c>
-      <c r="D8" s="35" t="inlineStr"/>
+      <c r="H8" s="7">
+        <f>SUM(B8:G8)</f>
+        <v/>
+      </c>
+      <c r="I8" s="35" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -16167,7 +16302,27 @@
         <f>ROUND(C7*$B$4,0)</f>
         <v/>
       </c>
-      <c r="D9" s="35" t="inlineStr">
+      <c r="D9" s="30">
+        <f>ROUND(D7*$B$4,0)</f>
+        <v/>
+      </c>
+      <c r="E9" s="30">
+        <f>ROUND(E7*$B$4,0)</f>
+        <v/>
+      </c>
+      <c r="F9" s="30">
+        <f>ROUND(F7*$B$4,0)</f>
+        <v/>
+      </c>
+      <c r="G9" s="30">
+        <f>ROUND(G7*$B$4,0)</f>
+        <v/>
+      </c>
+      <c r="H9" s="7">
+        <f>SUM(B9:G9)</f>
+        <v/>
+      </c>
+      <c r="I9" s="35" t="inlineStr">
         <is>
           <t>Calcul</t>
         </is>
@@ -16187,7 +16342,27 @@
         <f>C8-C9</f>
         <v/>
       </c>
-      <c r="D10" s="35" t="inlineStr">
+      <c r="D10" s="30">
+        <f>D8-D9</f>
+        <v/>
+      </c>
+      <c r="E10" s="30">
+        <f>E8-E9</f>
+        <v/>
+      </c>
+      <c r="F10" s="30">
+        <f>F8-F9</f>
+        <v/>
+      </c>
+      <c r="G10" s="30">
+        <f>G8-G9</f>
+        <v/>
+      </c>
+      <c r="H10" s="7">
+        <f>SUM(B10:G10)</f>
+        <v/>
+      </c>
+      <c r="I10" s="35" t="inlineStr">
         <is>
           <t>Arrondi admis ±1</t>
         </is>
@@ -16200,16 +16375,28 @@
         </is>
       </c>
       <c r="B11" s="25" t="n">
-        <v>386205</v>
+        <v>0</v>
       </c>
       <c r="C11" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="D11" s="35" t="inlineStr">
-        <is>
-          <t>Août : aucun précompte repris (G50 juillet non fournie)</t>
-        </is>
-      </c>
+      <c r="D11" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="25" t="n">
+        <v>386205</v>
+      </c>
+      <c r="F11" s="25" t="n">
+        <v>178353</v>
+      </c>
+      <c r="G11" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="7">
+        <f>SUM(B11:G11)</f>
+        <v/>
+      </c>
+      <c r="I11" s="35" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
@@ -16218,12 +16405,28 @@
         </is>
       </c>
       <c r="B12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="25" t="n">
+        <v>3919465</v>
+      </c>
+      <c r="D12" s="25" t="n">
+        <v>3553752</v>
+      </c>
+      <c r="E12" s="25" t="n">
         <v>1783214</v>
       </c>
-      <c r="C12" s="25" t="n">
+      <c r="F12" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="D12" s="35" t="inlineStr"/>
+      <c r="G12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="7">
+        <f>SUM(B12:G12)</f>
+        <v/>
+      </c>
+      <c r="I12" s="35" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -16239,7 +16442,27 @@
         <f>C11+C12</f>
         <v/>
       </c>
-      <c r="D13" s="35" t="inlineStr">
+      <c r="D13" s="30">
+        <f>D11+D12</f>
+        <v/>
+      </c>
+      <c r="E13" s="30">
+        <f>E11+E12</f>
+        <v/>
+      </c>
+      <c r="F13" s="30">
+        <f>F11+F12</f>
+        <v/>
+      </c>
+      <c r="G13" s="30">
+        <f>G11+G12</f>
+        <v/>
+      </c>
+      <c r="H13" s="7">
+        <f>SUM(B13:G13)</f>
+        <v/>
+      </c>
+      <c r="I13" s="35" t="inlineStr">
         <is>
           <t>Calcul</t>
         </is>
@@ -16259,7 +16482,27 @@
         <f>MAX(0,C8-C13)</f>
         <v/>
       </c>
-      <c r="D14" s="35" t="inlineStr">
+      <c r="D14" s="30">
+        <f>MAX(0,D8-D13)</f>
+        <v/>
+      </c>
+      <c r="E14" s="30">
+        <f>MAX(0,E8-E13)</f>
+        <v/>
+      </c>
+      <c r="F14" s="30">
+        <f>MAX(0,F8-F13)</f>
+        <v/>
+      </c>
+      <c r="G14" s="30">
+        <f>MAX(0,G8-G13)</f>
+        <v/>
+      </c>
+      <c r="H14" s="7">
+        <f>SUM(B14:G14)</f>
+        <v/>
+      </c>
+      <c r="I14" s="35" t="inlineStr">
         <is>
           <t>Calcul</t>
         </is>
@@ -16279,242 +16522,883 @@
         <f>MAX(0,C13-C8)</f>
         <v/>
       </c>
-      <c r="D15" s="35" t="inlineStr">
-        <is>
-          <t>Juin : 178 353 à reporter sur juillet</t>
+      <c r="D15" s="30">
+        <f>MAX(0,D13-D8)</f>
+        <v/>
+      </c>
+      <c r="E15" s="30">
+        <f>MAX(0,E13-E8)</f>
+        <v/>
+      </c>
+      <c r="F15" s="30">
+        <f>MAX(0,F13-F8)</f>
+        <v/>
+      </c>
+      <c r="G15" s="30">
+        <f>MAX(0,G13-G8)</f>
+        <v/>
+      </c>
+      <c r="H15" s="27" t="n"/>
+      <c r="I15" s="35" t="inlineStr">
+        <is>
+          <t>Calcul</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="inlineStr">
-        <is>
-          <t>IRG salaires — base déclarée (E1L20)</t>
-        </is>
-      </c>
-      <c r="B16" s="25" t="n">
-        <v>325645</v>
-      </c>
-      <c r="C16" s="25" t="n">
-        <v>300000</v>
-      </c>
-      <c r="D16" s="35" t="inlineStr"/>
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Contrôle report : précompte repris − reporté le mois précédent</t>
+        </is>
+      </c>
+      <c r="B16" s="22" t="n"/>
+      <c r="C16" s="30">
+        <f>C11-B15</f>
+        <v/>
+      </c>
+      <c r="D16" s="30">
+        <f>D11-C15</f>
+        <v/>
+      </c>
+      <c r="E16" s="30">
+        <f>E11-D15</f>
+        <v/>
+      </c>
+      <c r="F16" s="30">
+        <f>F11-E15</f>
+        <v/>
+      </c>
+      <c r="G16" s="30">
+        <f>G11-F15</f>
+        <v/>
+      </c>
+      <c r="H16" s="27" t="n"/>
+      <c r="I16" s="35" t="inlineStr">
+        <is>
+          <t>Doit être 0 (chaîne mai → juin → juillet)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>IRG salaires — base paie IMPORT (R650)</t>
-        </is>
-      </c>
-      <c r="B17" s="6">
-        <f>'Paie IMPORT'!H24</f>
-        <v/>
-      </c>
-      <c r="C17" s="6">
-        <f>'Paie IMPORT'!J24</f>
-        <v/>
-      </c>
-      <c r="D17" s="35" t="inlineStr">
-        <is>
-          <t>Lien paie</t>
-        </is>
-      </c>
+          <t>IRG salaires — base déclarée (E1L20)</t>
+        </is>
+      </c>
+      <c r="B17" s="25" t="n">
+        <v>365763</v>
+      </c>
+      <c r="C17" s="25" t="n">
+        <v>404385</v>
+      </c>
+      <c r="D17" s="25" t="n">
+        <v>426576</v>
+      </c>
+      <c r="E17" s="25" t="n">
+        <v>325645</v>
+      </c>
+      <c r="F17" s="25" t="n">
+        <v>286954</v>
+      </c>
+      <c r="G17" s="25" t="n">
+        <v>300000</v>
+      </c>
+      <c r="H17" s="7">
+        <f>SUM(B17:G17)</f>
+        <v/>
+      </c>
+      <c r="I17" s="35" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>IRG salaires — montant déclaré</t>
-        </is>
-      </c>
-      <c r="B18" s="25" t="n">
-        <v>59018</v>
-      </c>
-      <c r="C18" s="25" t="n">
-        <v>49670</v>
-      </c>
-      <c r="D18" s="35" t="inlineStr"/>
+          <t>IRG salaires — base paie IMPORT (R650)</t>
+        </is>
+      </c>
+      <c r="B18" s="6">
+        <f>'Paie IMPORT'!E24</f>
+        <v/>
+      </c>
+      <c r="C18" s="6">
+        <f>'Paie IMPORT'!F24</f>
+        <v/>
+      </c>
+      <c r="D18" s="6">
+        <f>'Paie IMPORT'!G24</f>
+        <v/>
+      </c>
+      <c r="E18" s="6">
+        <f>'Paie IMPORT'!H24</f>
+        <v/>
+      </c>
+      <c r="F18" s="6">
+        <f>'Paie IMPORT'!I24</f>
+        <v/>
+      </c>
+      <c r="G18" s="6">
+        <f>'Paie IMPORT'!J24</f>
+        <v/>
+      </c>
+      <c r="H18" s="7">
+        <f>SUM(B18:G18)</f>
+        <v/>
+      </c>
+      <c r="I18" s="35" t="inlineStr">
+        <is>
+          <t>Lien paie (mars : centralisateur absent)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
+          <t>IRG salaires — montant déclaré</t>
+        </is>
+      </c>
+      <c r="B19" s="25" t="n">
+        <v>60932</v>
+      </c>
+      <c r="C19" s="25" t="n">
+        <v>72478</v>
+      </c>
+      <c r="D19" s="25" t="n">
+        <v>79138</v>
+      </c>
+      <c r="E19" s="25" t="n">
+        <v>59018</v>
+      </c>
+      <c r="F19" s="25" t="n">
+        <v>42610</v>
+      </c>
+      <c r="G19" s="25" t="n">
+        <v>49670</v>
+      </c>
+      <c r="H19" s="7">
+        <f>SUM(B19:G19)</f>
+        <v/>
+      </c>
+      <c r="I19" s="35" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
           <t>IRG salaires — retenu en paie IMPORT (R660)</t>
         </is>
       </c>
-      <c r="B19" s="6">
+      <c r="B20" s="6">
+        <f>'Paie IMPORT'!E25</f>
+        <v/>
+      </c>
+      <c r="C20" s="6">
+        <f>'Paie IMPORT'!F25</f>
+        <v/>
+      </c>
+      <c r="D20" s="6">
+        <f>'Paie IMPORT'!G25</f>
+        <v/>
+      </c>
+      <c r="E20" s="6">
         <f>'Paie IMPORT'!H25</f>
         <v/>
       </c>
-      <c r="C19" s="6">
+      <c r="F20" s="6">
+        <f>'Paie IMPORT'!I25</f>
+        <v/>
+      </c>
+      <c r="G20" s="6">
         <f>'Paie IMPORT'!J25</f>
         <v/>
       </c>
-      <c r="D19" s="35" t="inlineStr">
+      <c r="H20" s="7">
+        <f>SUM(B20:G20)</f>
+        <v/>
+      </c>
+      <c r="I20" s="35" t="inlineStr">
         <is>
           <t>Lien paie</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Écart IRG déclaré − paie</t>
         </is>
       </c>
-      <c r="B20" s="30">
-        <f>B18-B19</f>
-        <v/>
-      </c>
-      <c r="C20" s="30">
-        <f>C18-C19</f>
-        <v/>
-      </c>
-      <c r="D20" s="35" t="inlineStr">
-        <is>
-          <t>Arrondi à la dizaine : conforme si |écart| &lt; 10</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="12" t="inlineStr">
-        <is>
-          <t>IRG retenu en paie TPM (non repris sur ces G50)</t>
-        </is>
-      </c>
-      <c r="B21" s="6">
-        <f>'Paie TPM'!H25</f>
-        <v/>
-      </c>
-      <c r="C21" s="6">
-        <f>'Paie TPM'!J25</f>
-        <v/>
-      </c>
-      <c r="D21" s="35" t="inlineStr">
-        <is>
-          <t>À déclarer sur une G50 TPM (non fournie)</t>
+      <c r="B21" s="30">
+        <f>IF(B20=0,"paie absente",B19-B20)</f>
+        <v/>
+      </c>
+      <c r="C21" s="30">
+        <f>IF(C20=0,"paie absente",C19-C20)</f>
+        <v/>
+      </c>
+      <c r="D21" s="30">
+        <f>IF(D20=0,"paie absente",D19-D20)</f>
+        <v/>
+      </c>
+      <c r="E21" s="30">
+        <f>IF(E20=0,"paie absente",E19-E20)</f>
+        <v/>
+      </c>
+      <c r="F21" s="30">
+        <f>IF(F20=0,"paie absente",F19-F20)</f>
+        <v/>
+      </c>
+      <c r="G21" s="30">
+        <f>IF(G20=0,"paie absente",G19-G20)</f>
+        <v/>
+      </c>
+      <c r="H21" s="27" t="n"/>
+      <c r="I21" s="35" t="inlineStr">
+        <is>
+          <t>Négatif = IRG retenu non reversé</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>Taxe d'apprentissage — base</t>
-        </is>
-      </c>
-      <c r="B22" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="C22" s="25" t="n">
-        <v>4409079</v>
-      </c>
-      <c r="D22" s="35" t="inlineStr">
-        <is>
-          <t>Base à justifier (1 % de la masse salariale)</t>
+          <t>IRG retenu en paie TPM (non repris sur ces G50)</t>
+        </is>
+      </c>
+      <c r="B22" s="6">
+        <f>'Paie TPM'!E25</f>
+        <v/>
+      </c>
+      <c r="C22" s="6">
+        <f>'Paie TPM'!F25</f>
+        <v/>
+      </c>
+      <c r="D22" s="6">
+        <f>'Paie TPM'!G25</f>
+        <v/>
+      </c>
+      <c r="E22" s="6">
+        <f>'Paie TPM'!H25</f>
+        <v/>
+      </c>
+      <c r="F22" s="6">
+        <f>'Paie TPM'!I25</f>
+        <v/>
+      </c>
+      <c r="G22" s="6">
+        <f>'Paie TPM'!J25</f>
+        <v/>
+      </c>
+      <c r="H22" s="7">
+        <f>SUM(B22:G22)</f>
+        <v/>
+      </c>
+      <c r="I22" s="35" t="inlineStr">
+        <is>
+          <t>À déclarer sur une G50 TPM (non fournie)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>Taxe d'apprentissage — montant</t>
+          <t>Droit de timbre — base</t>
         </is>
       </c>
       <c r="B23" s="25" t="n">
         <v>0</v>
       </c>
       <c r="C23" s="25" t="n">
+        <v>177058</v>
+      </c>
+      <c r="D23" s="25" t="n">
+        <v>177058</v>
+      </c>
+      <c r="E23" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="7">
+        <f>SUM(B23:G23)</f>
+        <v/>
+      </c>
+      <c r="I23" s="35" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>Droit de timbre — montant</t>
+        </is>
+      </c>
+      <c r="B24" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="25" t="n">
+        <v>8944</v>
+      </c>
+      <c r="D24" s="25" t="n">
+        <v>3173</v>
+      </c>
+      <c r="E24" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="7">
+        <f>SUM(B24:G24)</f>
+        <v/>
+      </c>
+      <c r="I24" s="35" t="inlineStr">
+        <is>
+          <t>Même base, montants différents : à justifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>Taxe d'apprentissage — base</t>
+        </is>
+      </c>
+      <c r="B25" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="25" t="n">
+        <v>4409079</v>
+      </c>
+      <c r="H25" s="7">
+        <f>SUM(B25:G25)</f>
+        <v/>
+      </c>
+      <c r="I25" s="35" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>Taxe d'apprentissage — montant</t>
+        </is>
+      </c>
+      <c r="B26" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="25" t="n">
         <v>44091</v>
       </c>
-      <c r="D23" s="35" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+      <c r="H26" s="7">
+        <f>SUM(B26:G26)</f>
+        <v/>
+      </c>
+      <c r="I26" s="35" t="inlineStr">
+        <is>
+          <t>1 % ; base à justifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>Total à payer déclaré</t>
         </is>
       </c>
-      <c r="B24" s="25" t="n">
+      <c r="B27" s="25" t="n">
+        <v>715520</v>
+      </c>
+      <c r="C27" s="25" t="n">
+        <v>719735</v>
+      </c>
+      <c r="D27" s="25" t="n">
+        <v>82311</v>
+      </c>
+      <c r="E27" s="25" t="n">
         <v>59018</v>
       </c>
-      <c r="C24" s="25" t="n">
+      <c r="F27" s="25" t="n">
+        <v>1309043</v>
+      </c>
+      <c r="G27" s="25" t="n">
         <v>932361</v>
       </c>
-      <c r="D24" s="35" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>Total recalculé (TVA + IRG + TA)</t>
-        </is>
-      </c>
-      <c r="B25" s="30">
-        <f>B14+B18+B23</f>
-        <v/>
-      </c>
-      <c r="C25" s="30">
-        <f>C14+C18+C23</f>
-        <v/>
-      </c>
-      <c r="D25" s="35" t="inlineStr">
+      <c r="H27" s="7">
+        <f>SUM(B27:G27)</f>
+        <v/>
+      </c>
+      <c r="I27" s="35" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Total recalculé (TVA + IRG + timbre + TA)</t>
+        </is>
+      </c>
+      <c r="B28" s="30">
+        <f>B14+B19+B24+B26</f>
+        <v/>
+      </c>
+      <c r="C28" s="30">
+        <f>C14+C19+C24+C26</f>
+        <v/>
+      </c>
+      <c r="D28" s="30">
+        <f>D14+D19+D24+D26</f>
+        <v/>
+      </c>
+      <c r="E28" s="30">
+        <f>E14+E19+E24+E26</f>
+        <v/>
+      </c>
+      <c r="F28" s="30">
+        <f>F14+F19+F24+F26</f>
+        <v/>
+      </c>
+      <c r="G28" s="30">
+        <f>G14+G19+G24+G26</f>
+        <v/>
+      </c>
+      <c r="H28" s="7">
+        <f>SUM(B28:G28)</f>
+        <v/>
+      </c>
+      <c r="I28" s="35" t="inlineStr">
         <is>
           <t>Calcul</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>Écart total</t>
         </is>
       </c>
-      <c r="B26" s="30">
-        <f>B24-B25</f>
-        <v/>
-      </c>
-      <c r="C26" s="30">
-        <f>C24-C25</f>
-        <v/>
-      </c>
-      <c r="D26" s="35" t="inlineStr">
+      <c r="B29" s="30">
+        <f>B27-B28</f>
+        <v/>
+      </c>
+      <c r="C29" s="30">
+        <f>C27-C28</f>
+        <v/>
+      </c>
+      <c r="D29" s="30">
+        <f>D27-D28</f>
+        <v/>
+      </c>
+      <c r="E29" s="30">
+        <f>E27-E28</f>
+        <v/>
+      </c>
+      <c r="F29" s="30">
+        <f>F27-F28</f>
+        <v/>
+      </c>
+      <c r="G29" s="30">
+        <f>G27-G28</f>
+        <v/>
+      </c>
+      <c r="H29" s="7">
+        <f>SUM(B29:G29)</f>
+        <v/>
+      </c>
+      <c r="I29" s="35" t="inlineStr">
         <is>
           <t>Doit être 0</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="12" t="inlineStr">
-        <is>
-          <t>Date de signature imprimée sur la G50</t>
-        </is>
-      </c>
-      <c r="B27" s="22" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>Date de signature imprimée</t>
+        </is>
+      </c>
+      <c r="B30" s="22" t="inlineStr">
+        <is>
+          <t>17/04/2021</t>
+        </is>
+      </c>
+      <c r="C30" s="22" t="inlineStr">
+        <is>
+          <t>18/05/2022</t>
+        </is>
+      </c>
+      <c r="D30" s="22" t="inlineStr">
+        <is>
+          <t>18/06/2022</t>
+        </is>
+      </c>
+      <c r="E30" s="22" t="inlineStr">
         <is>
           <t>28/07/2022</t>
         </is>
       </c>
-      <c r="C27" s="22" t="inlineStr">
+      <c r="F30" s="22" t="inlineStr">
         <is>
           <t>19/08/2022</t>
         </is>
       </c>
-      <c r="D27" s="35" t="inlineStr">
-        <is>
-          <t>Dates obsolètes (modèle 2022 non mis à jour)</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="40" customHeight="1">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>Cumul CA « 03/2026 » déclaré en juin + août</t>
-        </is>
-      </c>
-      <c r="B35" s="7">
-        <f>B7+C7</f>
-        <v/>
-      </c>
-      <c r="D35" s="35" t="inlineStr">
-        <is>
-          <t>Annotation G50 août : « RESTE A DECLARER TVA 5 417 538 — 08/2026 TVA RECU ». Le CA de mars 2026 est déclaré par fractions sur des mois ultérieurs (anomalie A18).</t>
-        </is>
+      <c r="G30" s="22" t="inlineStr">
+        <is>
+          <t>19/08/2022</t>
+        </is>
+      </c>
+      <c r="H30" s="27" t="n"/>
+      <c r="I30" s="35" t="inlineStr">
+        <is>
+          <t>Dates obsolètes : modèle non mis à jour</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Annotations portées en marge des G50 (suivi du CA de mars 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t>Rubrique</t>
+        </is>
+      </c>
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>Montant</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="inlineStr"/>
+      <c r="D34" s="11" t="inlineStr"/>
+      <c r="E34" s="11" t="inlineStr"/>
+      <c r="F34" s="11" t="inlineStr"/>
+      <c r="G34" s="11" t="inlineStr"/>
+      <c r="H34" s="11" t="inlineStr"/>
+      <c r="I34" s="11" t="inlineStr">
+        <is>
+          <t>Commentaire</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="29" t="inlineStr">
+        <is>
+          <t>CA réalisé en mars 2026 (« TOTAL CA 03/2026 », G50 mars)</t>
+        </is>
+      </c>
+      <c r="B35" s="25" t="n">
+        <v>27006870</v>
+      </c>
+      <c r="I35" s="35" t="inlineStr">
+        <is>
+          <t>Annotation G50 mars et avril</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="29" t="inlineStr">
+        <is>
+          <t>TVA correspondante (« TOTAL TVA 03/2026 »)</t>
+        </is>
+      </c>
+      <c r="B36" s="25" t="n">
+        <v>5131305</v>
+      </c>
+      <c r="I36" s="35" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="29" t="inlineStr">
+        <is>
+          <t>TVA recalculée sur le CA de mars</t>
+        </is>
+      </c>
+      <c r="B37" s="30">
+        <f>ROUND(B35*$B$4,0)</f>
+        <v/>
+      </c>
+      <c r="I37" s="35" t="inlineStr">
+        <is>
+          <t>Contrôle</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="29" t="inlineStr">
+        <is>
+          <t>CA de mars effectivement déclaré en mars</t>
+        </is>
+      </c>
+      <c r="B38" s="30">
+        <f>B7</f>
+        <v/>
+      </c>
+      <c r="I38" s="35" t="inlineStr">
+        <is>
+          <t>G50 mars</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="29" t="inlineStr">
+        <is>
+          <t>CA de mars reporté sur les mois suivants</t>
+        </is>
+      </c>
+      <c r="B39" s="36">
+        <f>B35-B38</f>
+        <v/>
+      </c>
+      <c r="I39" s="35" t="inlineStr">
+        <is>
+          <t>Annoté « RESTE A DECLARER CA » 23 561 670</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="29" t="inlineStr">
+        <is>
+          <t>TVA de mars payée en retard</t>
+        </is>
+      </c>
+      <c r="B40" s="36">
+        <f>ROUND(B39*$B$4,0)</f>
+        <v/>
+      </c>
+      <c r="I40" s="35" t="inlineStr">
+        <is>
+          <t>Annoté « RESTE A DECLARER TVA » 4 476 717</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="29" t="inlineStr">
+        <is>
+          <t>« CA DECLARE 04/2026 » annoté en avril</t>
+        </is>
+      </c>
+      <c r="B41" s="25" t="n">
+        <v>13157894.74</v>
+      </c>
+      <c r="I41" s="35" t="inlineStr">
+        <is>
+          <t>Soit 2 500 000 / 19 % : CA calculé à partir d'un objectif de TVA</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="29" t="inlineStr">
+        <is>
+          <t>TVA cible correspondante</t>
+        </is>
+      </c>
+      <c r="B42" s="30">
+        <f>ROUND(B41*$B$4,2)</f>
+        <v/>
+      </c>
+      <c r="I42" s="35" t="inlineStr">
+        <is>
+          <t>Contrôle</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="29" t="inlineStr">
+        <is>
+          <t>« RESTE A DECLARER TVA » annoté en juillet et août</t>
+        </is>
+      </c>
+      <c r="B43" s="25" t="n">
+        <v>5417538</v>
+      </c>
+      <c r="I43" s="35" t="inlineStr">
+        <is>
+          <t>Montant restant selon le suivi interne</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Comparaison avec le CA IMPORT 2025 des mêmes mois (compte 70001, journal 2025)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="11" t="inlineStr">
+        <is>
+          <t>Rubrique</t>
+        </is>
+      </c>
+      <c r="B46" s="11" t="inlineStr">
+        <is>
+          <t>Mars</t>
+        </is>
+      </c>
+      <c r="C46" s="11" t="inlineStr">
+        <is>
+          <t>Avr</t>
+        </is>
+      </c>
+      <c r="D46" s="11" t="inlineStr">
+        <is>
+          <t>Mai</t>
+        </is>
+      </c>
+      <c r="E46" s="11" t="inlineStr">
+        <is>
+          <t>Juin</t>
+        </is>
+      </c>
+      <c r="F46" s="11" t="inlineStr">
+        <is>
+          <t>Juil</t>
+        </is>
+      </c>
+      <c r="G46" s="11" t="inlineStr">
+        <is>
+          <t>Août</t>
+        </is>
+      </c>
+      <c r="H46" s="11" t="inlineStr">
+        <is>
+          <t>Cumul</t>
+        </is>
+      </c>
+      <c r="I46" s="11" t="inlineStr">
+        <is>
+          <t>Commentaire</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="12" t="inlineStr">
+        <is>
+          <t>CA 2025 (journal comptable)</t>
+        </is>
+      </c>
+      <c r="B47" s="25" t="n">
+        <v>31947529</v>
+      </c>
+      <c r="C47" s="25" t="n">
+        <v>29534571</v>
+      </c>
+      <c r="D47" s="25" t="n">
+        <v>41310810</v>
+      </c>
+      <c r="E47" s="25" t="n">
+        <v>28042831</v>
+      </c>
+      <c r="F47" s="25" t="n">
+        <v>23178604</v>
+      </c>
+      <c r="G47" s="25" t="n">
+        <v>15524844</v>
+      </c>
+      <c r="H47" s="7">
+        <f>SUM(B47:G47)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="12" t="inlineStr">
+        <is>
+          <t>CA 2026 déclaré sur G50</t>
+        </is>
+      </c>
+      <c r="B48" s="30">
+        <f>B7</f>
+        <v/>
+      </c>
+      <c r="C48" s="30">
+        <f>C7</f>
+        <v/>
+      </c>
+      <c r="D48" s="30">
+        <f>D7</f>
+        <v/>
+      </c>
+      <c r="E48" s="30">
+        <f>E7</f>
+        <v/>
+      </c>
+      <c r="F48" s="30">
+        <f>F7</f>
+        <v/>
+      </c>
+      <c r="G48" s="30">
+        <f>G7</f>
+        <v/>
+      </c>
+      <c r="H48" s="7">
+        <f>SUM(B48:G48)</f>
+        <v/>
+      </c>
+      <c r="I48" s="35" t="inlineStr">
+        <is>
+          <t>Le CA 2026 déclaré mois par mois ne reflète pas le CA réalisé (voir annotations) : rapprocher avec le journal des ventes 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="12" t="inlineStr">
+        <is>
+          <t>Variation 2026 / 2025</t>
+        </is>
+      </c>
+      <c r="B49" s="19">
+        <f>IF(B47=0,"",B48/B47-1)</f>
+        <v/>
+      </c>
+      <c r="C49" s="19">
+        <f>IF(C47=0,"",C48/C47-1)</f>
+        <v/>
+      </c>
+      <c r="D49" s="19">
+        <f>IF(D47=0,"",D48/D47-1)</f>
+        <v/>
+      </c>
+      <c r="E49" s="19">
+        <f>IF(E47=0,"",E48/E47-1)</f>
+        <v/>
+      </c>
+      <c r="F49" s="19">
+        <f>IF(F47=0,"",F48/F47-1)</f>
+        <v/>
+      </c>
+      <c r="G49" s="19">
+        <f>IF(G47=0,"",G48/G47-1)</f>
+        <v/>
+      </c>
+      <c r="H49" s="37">
+        <f>H48/H47-1</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Dossier comptable : G50 IMPORT janvier-février et G50 TPM juillet-août 2026
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XYis4EzVZMNdoYCxmLrRh4
</commit_message>
<xml_diff>
--- a/DOSSIER_COMPTABLE_SARL_DPR_COMPAGNY_2026.xlsx
+++ b/DOSSIER_COMPTABLE_SARL_DPR_COMPAGNY_2026.xlsx
@@ -18,13 +18,14 @@
     <sheet name="G50 2026" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Balance 2024-2025" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="États 2024-2025" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Anomalies &amp; actions" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Pièces" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="G50 TPM 2026" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Anomalies &amp; actions" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Pièces" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Journal paie'!$A$4:$G$140</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Balance 2024-2025'!$A$4:$E$104</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Anomalies &amp; actions'!$A$4:$I$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Anomalies &amp; actions'!$A$4:$I$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -202,7 +203,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -245,6 +246,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="10" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -676,7 +678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D58"/>
+  <dimension ref="A1:D60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1109,21 +1111,32 @@
     <row r="36">
       <c r="A36" s="12" t="inlineStr">
         <is>
-          <t>G50 mars–août : totaux et report de précompte</t>
+          <t>G50 IMPORT janv.–août : totaux et report de précompte</t>
         </is>
       </c>
       <c r="B36" s="4">
-        <f>IF(AND(SUMPRODUCT(ABS('G50 2026'!B29:G29))&lt;1,SUMPRODUCT(ABS('G50 2026'!C16:G16))&lt;1),"OK","ÉCART")</f>
+        <f>IF(AND(SUMPRODUCT(ABS('G50 2026'!B29:I29))&lt;1,SUMPRODUCT(ABS('G50 2026'!C16:I16))&lt;1),"OK","ÉCART")</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="12" t="inlineStr">
         <is>
+          <t>G50 TPM juil.–août : totaux</t>
+        </is>
+      </c>
+      <c r="B37" s="4">
+        <f>IF(AND(ABS('G50 TPM 2026'!B21)&lt;1,ABS('G50 TPM 2026'!C21)&lt;1),"OK","ÉCART")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="12" t="inlineStr">
+        <is>
           <t>Paie TPM : éléments soumis hors assiette</t>
         </is>
       </c>
-      <c r="B37" s="4">
+      <c r="B38" s="4">
         <f>IF(ABS('Paie TPM'!K37)&lt;0.01,"OK","ÉCART")</f>
         <v/>
       </c>
@@ -1255,7 +1268,7 @@
       </c>
       <c r="B48" s="12" t="inlineStr">
         <is>
-          <t>Contrôle TVA / IRG / timbre / TA des G50 IMPORT mars–août</t>
+          <t>Contrôle TVA / IRG / timbre / TA des G50 IMPORT janv.–août</t>
         </is>
       </c>
       <c r="C48" s="17" t="n"/>
@@ -1264,12 +1277,12 @@
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>Balance 2024-2025</t>
+          <t>G50 TPM 2026</t>
         </is>
       </c>
       <c r="B49" s="12" t="inlineStr">
         <is>
-          <t>Balance générale issue des journaux PCCOMPTA</t>
+          <t>Contrôle des G50 TPM et location (juil., août)</t>
         </is>
       </c>
       <c r="C49" s="17" t="n"/>
@@ -1278,103 +1291,79 @@
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>États 2024-2025</t>
+          <t>Balance 2024-2025</t>
         </is>
       </c>
       <c r="B50" s="12" t="inlineStr">
         <is>
-          <t>Compte de résultat et bilan simplifiés, indicateurs</t>
+          <t>Balance générale issue des journaux PCCOMPTA</t>
         </is>
       </c>
       <c r="C50" s="17" t="n"/>
       <c r="D50" s="18" t="n"/>
     </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>États 2024-2025</t>
+        </is>
+      </c>
+      <c r="B51" s="12" t="inlineStr">
+        <is>
+          <t>Compte de résultat et bilan simplifiés, indicateurs</t>
+        </is>
+      </c>
+      <c r="C51" s="17" t="n"/>
+      <c r="D51" s="18" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>Légende : bleu = saisie depuis une pièce ; vert = lien vers une autre feuille ; noir = calcul ; fond jaune = à compléter.</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="10" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="10" t="inlineStr">
         <is>
           <t>Exercices comptables</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="11" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="11" t="inlineStr">
         <is>
           <t>Indicateur</t>
         </is>
       </c>
-      <c r="B55" s="11" t="inlineStr">
+      <c r="B57" s="11" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="C55" s="11" t="inlineStr">
+      <c r="C57" s="11" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D55" s="11" t="inlineStr">
+      <c r="D57" s="11" t="inlineStr">
         <is>
           <t>Variation</t>
         </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="4" t="inlineStr">
-        <is>
-          <t>Chiffre d'affaires</t>
-        </is>
-      </c>
-      <c r="B56" s="6">
-        <f>'États 2024-2025'!C5</f>
-        <v/>
-      </c>
-      <c r="C56" s="6">
-        <f>'États 2024-2025'!D5</f>
-        <v/>
-      </c>
-      <c r="D56" s="19">
-        <f>IF(B56=0,"",C56/B56-1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="4" t="inlineStr">
-        <is>
-          <t>Charges de personnel</t>
-        </is>
-      </c>
-      <c r="B57" s="6">
-        <f>'États 2024-2025'!C10</f>
-        <v/>
-      </c>
-      <c r="C57" s="6">
-        <f>'États 2024-2025'!D10</f>
-        <v/>
-      </c>
-      <c r="D57" s="19">
-        <f>IF(B57=0,"",C57/B57-1)</f>
-        <v/>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>Résultat net</t>
+          <t>Chiffre d'affaires</t>
         </is>
       </c>
       <c r="B58" s="6">
-        <f>'États 2024-2025'!C16</f>
+        <f>'États 2024-2025'!C5</f>
         <v/>
       </c>
       <c r="C58" s="6">
-        <f>'États 2024-2025'!D16</f>
+        <f>'États 2024-2025'!D5</f>
         <v/>
       </c>
       <c r="D58" s="19">
@@ -1382,8 +1371,46 @@
         <v/>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>Charges de personnel</t>
+        </is>
+      </c>
+      <c r="B59" s="6">
+        <f>'États 2024-2025'!C10</f>
+        <v/>
+      </c>
+      <c r="C59" s="6">
+        <f>'États 2024-2025'!D10</f>
+        <v/>
+      </c>
+      <c r="D59" s="19">
+        <f>IF(B59=0,"",C59/B59-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>Résultat net</t>
+        </is>
+      </c>
+      <c r="B60" s="6">
+        <f>'États 2024-2025'!C16</f>
+        <v/>
+      </c>
+      <c r="C60" s="6">
+        <f>'États 2024-2025'!D16</f>
+        <v/>
+      </c>
+      <c r="D60" s="19">
+        <f>IF(B60=0,"",C60/B60-1)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="12">
     <mergeCell ref="B42:D42"/>
     <mergeCell ref="B45:D45"/>
     <mergeCell ref="B46:D46"/>
@@ -1393,6 +1420,7 @@
     <mergeCell ref="B40:D40"/>
     <mergeCell ref="B44:D44"/>
     <mergeCell ref="B43:D43"/>
+    <mergeCell ref="B51:D51"/>
     <mergeCell ref="B47:D47"/>
     <mergeCell ref="B48:D48"/>
   </mergeCells>
@@ -4015,7 +4043,7 @@
         <f>SUM(D5:D7)-SUM(D8:D15)</f>
         <v/>
       </c>
-      <c r="E16" s="37">
+      <c r="E16" s="38">
         <f>IF(C16=0,"",D16/C16-1)</f>
         <v/>
       </c>
@@ -4632,6 +4660,373 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:D25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="54" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Contrôle des G50 « TPM et location » consolidées 2026 (même NIF 000306018423274)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Sources : G50_07-2026_TPM_ET_LOCATION_CONSOLIDE_-.xls et G50_08-2026_TPM_ET_LOCATION_CONSOLIDE.xls. Activité portée : transport et distribution de toutes marchandises.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Rubrique</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>Juillet 2026</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>Août 2026</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>Commentaire</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Mois imprimé sur la G50</t>
+        </is>
+      </c>
+      <c r="B5" s="22" t="inlineStr">
+        <is>
+          <t>AVRIL</t>
+        </is>
+      </c>
+      <c r="C5" s="22" t="inlineStr">
+        <is>
+          <t>AOUT</t>
+        </is>
+      </c>
+      <c r="D5" s="35" t="inlineStr">
+        <is>
+          <t>Fichier « 07-2026 » mais mois imprimé « AVRIL »</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>CA imposable déclaré</t>
+        </is>
+      </c>
+      <c r="B6" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="35" t="inlineStr">
+        <is>
+          <t>Aucun CA TPM / location déclaré</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>TVA collectée déclarée</t>
+        </is>
+      </c>
+      <c r="B7" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="35" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Précompte antérieur (E3B91)</t>
+        </is>
+      </c>
+      <c r="B8" s="25" t="n">
+        <v>1714499</v>
+      </c>
+      <c r="C8" s="25" t="n">
+        <v>1714499</v>
+      </c>
+      <c r="D8" s="35" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Précompte à reporter (E3B99)</t>
+        </is>
+      </c>
+      <c r="B9" s="25" t="n">
+        <v>1714499</v>
+      </c>
+      <c r="C9" s="25" t="n">
+        <v>1714499</v>
+      </c>
+      <c r="D9" s="35" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>Précompte au compte 44550 au 31/12/2025 (comptabilité)</t>
+        </is>
+      </c>
+      <c r="B10" s="6">
+        <f>'Balance 2024-2025'!D49</f>
+        <v/>
+      </c>
+      <c r="C10" s="6">
+        <f>'Balance 2024-2025'!D49</f>
+        <v/>
+      </c>
+      <c r="D10" s="35" t="inlineStr">
+        <is>
+          <t>Identique : crédit reporté depuis 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>IRG salaires — base déclarée</t>
+        </is>
+      </c>
+      <c r="B11" s="25" t="n">
+        <v>91763</v>
+      </c>
+      <c r="C11" s="25" t="n">
+        <v>42190</v>
+      </c>
+      <c r="D11" s="35" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>IRG salaires — base paie TPM (R650) du mois</t>
+        </is>
+      </c>
+      <c r="B12" s="6">
+        <f>'Paie TPM'!I24</f>
+        <v/>
+      </c>
+      <c r="C12" s="6">
+        <f>'Paie TPM'!J24</f>
+        <v/>
+      </c>
+      <c r="D12" s="35" t="inlineStr">
+        <is>
+          <t>Lien paie</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>IRG salaires — montant déclaré</t>
+        </is>
+      </c>
+      <c r="B13" s="25" t="n">
+        <v>9375</v>
+      </c>
+      <c r="C13" s="25" t="n">
+        <v>3690</v>
+      </c>
+      <c r="D13" s="35" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>IRG salaires — retenu en paie TPM (R660) du mois</t>
+        </is>
+      </c>
+      <c r="B14" s="6">
+        <f>'Paie TPM'!I25</f>
+        <v/>
+      </c>
+      <c r="C14" s="6">
+        <f>'Paie TPM'!J25</f>
+        <v/>
+      </c>
+      <c r="D14" s="35" t="inlineStr">
+        <is>
+          <t>Lien paie</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Écart IRG déclaré − paie</t>
+        </is>
+      </c>
+      <c r="B15" s="30">
+        <f>B13-B14</f>
+        <v/>
+      </c>
+      <c r="C15" s="30">
+        <f>C13-C14</f>
+        <v/>
+      </c>
+      <c r="D15" s="35" t="inlineStr">
+        <is>
+          <t>Juillet : la G50 reprend l'IRG d'avril/mai</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>Pour mémoire : IRG paie TPM avril / mai</t>
+        </is>
+      </c>
+      <c r="B16" s="6">
+        <f>'Paie TPM'!F25</f>
+        <v/>
+      </c>
+      <c r="C16" s="6">
+        <f>'Paie TPM'!G25</f>
+        <v/>
+      </c>
+      <c r="D16" s="35" t="inlineStr">
+        <is>
+          <t>Lien paie</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>Taxe d'apprentissage — base</t>
+        </is>
+      </c>
+      <c r="B17" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="25" t="n">
+        <v>680900</v>
+      </c>
+      <c r="D17" s="35" t="inlineStr">
+        <is>
+          <t>Base à justifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>Taxe d'apprentissage — montant</t>
+        </is>
+      </c>
+      <c r="B18" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="25" t="n">
+        <v>6809</v>
+      </c>
+      <c r="D18" s="35" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Total à payer déclaré</t>
+        </is>
+      </c>
+      <c r="B19" s="25" t="n">
+        <v>9375</v>
+      </c>
+      <c r="C19" s="25" t="n">
+        <v>10499</v>
+      </c>
+      <c r="D19" s="35" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Total recalculé (TVA + IRG + TA)</t>
+        </is>
+      </c>
+      <c r="B20" s="30">
+        <f>MAX(0,B7-B8)+B13+B18</f>
+        <v/>
+      </c>
+      <c r="C20" s="30">
+        <f>MAX(0,C7-C8)+C13+C18</f>
+        <v/>
+      </c>
+      <c r="D20" s="35" t="inlineStr">
+        <is>
+          <t>Calcul</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Écart total</t>
+        </is>
+      </c>
+      <c r="B21" s="30">
+        <f>B19-B20</f>
+        <v/>
+      </c>
+      <c r="C21" s="30">
+        <f>C19-C20</f>
+        <v/>
+      </c>
+      <c r="D21" s="35" t="inlineStr">
+        <is>
+          <t>Doit être 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Modèle G50 TPM : la feuille « Recap-TVA » porte encore la G50 de décembre 2025 (factures BOBOR PNEUS) et « Feuil1 » un extrait de journal 2019 ; à nettoyer avant dépôt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>G50 TPM de janvier à juin 2026 non fournies : IRG TPM retenu sur cette période à vérifier (voir anomalie A19).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4718,7 +5113,7 @@
           <t>A01</t>
         </is>
       </c>
-      <c r="B5" s="38" t="n">
+      <c r="B5" s="39" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="29" t="inlineStr">
@@ -4736,7 +5131,7 @@
           <t>Déclaration CNAS de février 2026 non fournie (assiette paie 952 475,81 ; 7 STC payés).</t>
         </is>
       </c>
-      <c r="F5" s="39">
+      <c r="F5" s="40">
         <f>'Rappro CNAS'!J6</f>
         <v/>
       </c>
@@ -4745,8 +5140,8 @@
           <t>Fournir la déclaration de février + EMS avec 7 sorties ; à défaut, la déposer (pénalités de retard).</t>
         </is>
       </c>
-      <c r="H5" s="40" t="n"/>
-      <c r="I5" s="40" t="inlineStr">
+      <c r="H5" s="41" t="n"/>
+      <c r="I5" s="41" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -4758,7 +5153,7 @@
           <t>A02</t>
         </is>
       </c>
-      <c r="B6" s="38" t="n">
+      <c r="B6" s="39" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="29" t="inlineStr">
@@ -4776,7 +5171,7 @@
           <t>Centralisateur de mars 2026 absent (onglet vide) alors que la CNAS de mars déclare 368 389,93 d'assiette, 5 salariés.</t>
         </is>
       </c>
-      <c r="F6" s="39">
+      <c r="F6" s="40">
         <f>'Rappro CNAS'!K7</f>
         <v/>
       </c>
@@ -4785,8 +5180,8 @@
           <t>Obtenir le livre de paie de mars et le saisir dans « Paie IMPORT » col. E ; comptabiliser la paie de mars.</t>
         </is>
       </c>
-      <c r="H6" s="40" t="n"/>
-      <c r="I6" s="40" t="inlineStr">
+      <c r="H6" s="41" t="n"/>
+      <c r="I6" s="41" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -4798,7 +5193,7 @@
           <t>A03</t>
         </is>
       </c>
-      <c r="B7" s="38" t="n">
+      <c r="B7" s="39" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="29" t="inlineStr">
@@ -4816,7 +5211,7 @@
           <t>Prime de ponctualité (R540) imposée à l'IRG mais exclue du salaire de poste (assiette CNAS) chaque mois.</t>
         </is>
       </c>
-      <c r="F7" s="39">
+      <c r="F7" s="40">
         <f>'Rappro CNAS'!V13</f>
         <v/>
       </c>
@@ -4825,8 +5220,8 @@
           <t>Vérifier le paramétrage de la rubrique R540 (soumise SS) ; régulariser les déclarations concernées.</t>
         </is>
       </c>
-      <c r="H7" s="40" t="n"/>
-      <c r="I7" s="40" t="inlineStr">
+      <c r="H7" s="41" t="n"/>
+      <c r="I7" s="41" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -4838,7 +5233,7 @@
           <t>A04</t>
         </is>
       </c>
-      <c r="B8" s="41" t="n">
+      <c r="B8" s="42" t="n">
         <v>2</v>
       </c>
       <c r="C8" s="29" t="inlineStr">
@@ -4856,14 +5251,14 @@
           <t>Effectif déclaré au T1 = 2 alors que 3 salariés sont inscrits ; T2 déclare 1 sortie et un effectif final de 2 ⇒ T1 aurait dû être 3.</t>
         </is>
       </c>
-      <c r="F8" s="42" t="n"/>
+      <c r="F8" s="43" t="n"/>
       <c r="G8" s="29" t="inlineStr">
         <is>
           <t>Rectifier l'effectif du T1 auprès de la CNAS.</t>
         </is>
       </c>
-      <c r="H8" s="40" t="n"/>
-      <c r="I8" s="40" t="inlineStr">
+      <c r="H8" s="41" t="n"/>
+      <c r="I8" s="41" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -4875,7 +5270,7 @@
           <t>A05</t>
         </is>
       </c>
-      <c r="B9" s="41" t="n">
+      <c r="B9" s="42" t="n">
         <v>2</v>
       </c>
       <c r="C9" s="29" t="inlineStr">
@@ -4893,14 +5288,14 @@
           <t>Salarié totalement absent (non rémunéré) en juillet, disparu de la paie en août sans STC ni sortie déclarée.</t>
         </is>
       </c>
-      <c r="F9" s="42" t="n"/>
+      <c r="F9" s="43" t="n"/>
       <c r="G9" s="29" t="inlineStr">
         <is>
           <t>Établir le STC et déclarer la sortie dans l'EMS du T3 (échéance 30/10/2026).</t>
         </is>
       </c>
-      <c r="H9" s="40" t="n"/>
-      <c r="I9" s="40" t="inlineStr">
+      <c r="H9" s="41" t="n"/>
+      <c r="I9" s="41" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -4912,7 +5307,7 @@
           <t>A06</t>
         </is>
       </c>
-      <c r="B10" s="41" t="n">
+      <c r="B10" s="42" t="n">
         <v>2</v>
       </c>
       <c r="C10" s="29" t="inlineStr">
@@ -4930,14 +5325,14 @@
           <t>STC de 2 237,40 en août : une sortie à déclarer au T3.</t>
         </is>
       </c>
-      <c r="F10" s="42" t="n"/>
+      <c r="F10" s="43" t="n"/>
       <c r="G10" s="29" t="inlineStr">
         <is>
           <t>Déclarer la sortie dans l'EMS du T3.</t>
         </is>
       </c>
-      <c r="H10" s="40" t="n"/>
-      <c r="I10" s="40" t="inlineStr">
+      <c r="H10" s="41" t="n"/>
+      <c r="I10" s="41" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -4949,7 +5344,7 @@
           <t>A07</t>
         </is>
       </c>
-      <c r="B11" s="41" t="n">
+      <c r="B11" s="42" t="n">
         <v>2</v>
       </c>
       <c r="C11" s="29" t="inlineStr">
@@ -4967,7 +5362,7 @@
           <t>Déclarations T3 2026 (juil–sept) à établir ; paie de septembre non fournie.</t>
         </is>
       </c>
-      <c r="F11" s="39">
+      <c r="F11" s="40">
         <f>'Rappro CNAS'!J9+'Rappro CNAS'!J12</f>
         <v/>
       </c>
@@ -4976,8 +5371,8 @@
           <t>Transmettre les centralisateurs de septembre ; déposer et payer avant le 30/10/2026.</t>
         </is>
       </c>
-      <c r="H11" s="40" t="n"/>
-      <c r="I11" s="40" t="inlineStr">
+      <c r="H11" s="41" t="n"/>
+      <c r="I11" s="41" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -4989,7 +5384,7 @@
           <t>A08</t>
         </is>
       </c>
-      <c r="B12" s="43" t="n">
+      <c r="B12" s="44" t="n">
         <v>3</v>
       </c>
       <c r="C12" s="29" t="inlineStr">
@@ -5007,14 +5402,14 @@
           <t>Avril = mai et juillet = août strictement identiques (mêmes absences, heures sup., IRG) : variables probablement non saisies.</t>
         </is>
       </c>
-      <c r="F12" s="42" t="n"/>
+      <c r="F12" s="43" t="n"/>
       <c r="G12" s="29" t="inlineStr">
         <is>
           <t>Contrôler les pointages et bulletins de mai et août.</t>
         </is>
       </c>
-      <c r="H12" s="40" t="n"/>
-      <c r="I12" s="40" t="inlineStr">
+      <c r="H12" s="41" t="n"/>
+      <c r="I12" s="41" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5026,7 +5421,7 @@
           <t>A09</t>
         </is>
       </c>
-      <c r="B13" s="43" t="n">
+      <c r="B13" s="44" t="n">
         <v>3</v>
       </c>
       <c r="C13" s="29" t="inlineStr">
@@ -5044,7 +5439,7 @@
           <t>Frais de mission élevés (avril 41 615 ; mai 49 115, soit 47–55 % de l'assiette), non soumis à cotisations.</t>
         </is>
       </c>
-      <c r="F13" s="39">
+      <c r="F13" s="40">
         <f>'Paie TPM'!K26</f>
         <v/>
       </c>
@@ -5053,8 +5448,8 @@
           <t>Conserver ordres de mission et justificatifs ; risque de requalification en salaire.</t>
         </is>
       </c>
-      <c r="H13" s="40" t="n"/>
-      <c r="I13" s="40" t="inlineStr">
+      <c r="H13" s="41" t="n"/>
+      <c r="I13" s="41" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5066,7 +5461,7 @@
           <t>A10</t>
         </is>
       </c>
-      <c r="B14" s="43" t="n">
+      <c r="B14" s="44" t="n">
         <v>3</v>
       </c>
       <c r="C14" s="29" t="inlineStr">
@@ -5084,14 +5479,14 @@
           <t>Prime de responsabilité de 5,00 DA (janv.) et 1,14 DA (févr.) : paramètre vraisemblablement erroné (5 au lieu de 5 %).</t>
         </is>
       </c>
-      <c r="F14" s="42" t="n"/>
+      <c r="F14" s="43" t="n"/>
       <c r="G14" s="29" t="inlineStr">
         <is>
           <t>Corriger le paramètre B291 ; régulariser le rappel éventuel.</t>
         </is>
       </c>
-      <c r="H14" s="40" t="n"/>
-      <c r="I14" s="40" t="inlineStr">
+      <c r="H14" s="41" t="n"/>
+      <c r="I14" s="41" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5103,7 +5498,7 @@
           <t>A11</t>
         </is>
       </c>
-      <c r="B15" s="41" t="n">
+      <c r="B15" s="42" t="n">
         <v>2</v>
       </c>
       <c r="C15" s="29" t="inlineStr">
@@ -5121,7 +5516,7 @@
           <t>Bordereaux de versement CNAS à « 0,00 » : aucune preuve de paiement des cotisations dans le dossier.</t>
         </is>
       </c>
-      <c r="F15" s="39">
+      <c r="F15" s="40">
         <f>'Rappro CNAS'!K13</f>
         <v/>
       </c>
@@ -5130,8 +5525,8 @@
           <t>Joindre les quittances CNAS / avis de virement ; comptabiliser les règlements (débit 431).</t>
         </is>
       </c>
-      <c r="H15" s="40" t="n"/>
-      <c r="I15" s="40" t="inlineStr">
+      <c r="H15" s="41" t="n"/>
+      <c r="I15" s="41" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5143,7 +5538,7 @@
           <t>A12</t>
         </is>
       </c>
-      <c r="B16" s="41" t="n">
+      <c r="B16" s="42" t="n">
         <v>2</v>
       </c>
       <c r="C16" s="29" t="inlineStr">
@@ -5158,20 +5553,20 @@
       </c>
       <c r="E16" s="29" t="inlineStr">
         <is>
-          <t>IRG IMPORT : G50 d'avril à août conformes à la paie (écarts d'arrondi ≤ 3 DA ; juillet : 2,30 DA retenus non reversés). Mars non vérifiable (paie absente). G50 janv.–févr. IMPORT et toutes les G50 TPM non fournies.</t>
-        </is>
-      </c>
-      <c r="F16" s="39">
+          <t>IRG IMPORT : G50 de janvier à août conformes à la paie (écarts d'arrondi ≤ 3 DA ; juillet : 2,30 DA retenus non reversés). Mars non vérifiable (paie absente).</t>
+        </is>
+      </c>
+      <c r="F16" s="40">
         <f>'Échéancier IRG-CNAS'!G13</f>
         <v/>
       </c>
       <c r="G16" s="29" t="inlineStr">
         <is>
-          <t>Fournir les G50 manquantes et compléter la colonne I de l'échéancier.</t>
-        </is>
-      </c>
-      <c r="H16" s="40" t="n"/>
-      <c r="I16" s="40" t="inlineStr">
+          <t>Reverser l'IRG retenu au dinar près ; fournir la paie de mars.</t>
+        </is>
+      </c>
+      <c r="H16" s="41" t="n"/>
+      <c r="I16" s="41" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5183,7 +5578,7 @@
           <t>A13</t>
         </is>
       </c>
-      <c r="B17" s="43" t="n">
+      <c r="B17" s="44" t="n">
         <v>3</v>
       </c>
       <c r="C17" s="29" t="inlineStr">
@@ -5201,14 +5596,14 @@
           <t>Paie paramétrée CACOBATPH (taux X504) mais aucune déclaration CACOBATPH (congés payés / intempéries) dans le dossier.</t>
         </is>
       </c>
-      <c r="F17" s="42" t="n"/>
+      <c r="F17" s="43" t="n"/>
       <c r="G17" s="29" t="inlineStr">
         <is>
           <t>Fournir les déclarations et paiements CACOBATPH 2026.</t>
         </is>
       </c>
-      <c r="H17" s="40" t="n"/>
-      <c r="I17" s="40" t="inlineStr">
+      <c r="H17" s="41" t="n"/>
+      <c r="I17" s="41" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5220,7 +5615,7 @@
           <t>A14</t>
         </is>
       </c>
-      <c r="B18" s="43" t="n">
+      <c r="B18" s="44" t="n">
         <v>3</v>
       </c>
       <c r="C18" s="29" t="inlineStr">
@@ -5238,14 +5633,14 @@
           <t>Libellés divergents : « D.P.R.COMPAGNY » / « DPR COMPAGNY » ; en-tête de paie TPM à l'adresse VGE TIZI alors que l'affiliation TPM est à TISSA.</t>
         </is>
       </c>
-      <c r="F18" s="42" t="n"/>
+      <c r="F18" s="43" t="n"/>
       <c r="G18" s="29" t="inlineStr">
         <is>
           <t>Harmoniser raison sociale et adresse dans le logiciel de paie.</t>
         </is>
       </c>
-      <c r="H18" s="40" t="n"/>
-      <c r="I18" s="40" t="inlineStr">
+      <c r="H18" s="41" t="n"/>
+      <c r="I18" s="41" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5257,7 +5652,7 @@
           <t>A15</t>
         </is>
       </c>
-      <c r="B19" s="43" t="n">
+      <c r="B19" s="44" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="29" t="inlineStr">
@@ -5275,14 +5670,14 @@
           <t>Périodicité mixte : déclarations mensuelles (janv., mars) puis trimestrielle (T2).</t>
         </is>
       </c>
-      <c r="F19" s="42" t="n"/>
+      <c r="F19" s="43" t="n"/>
       <c r="G19" s="29" t="inlineStr">
         <is>
           <t>Confirmer auprès de la CNAS le passage au trimestriel après la baisse d'effectif (12 → 5).</t>
         </is>
       </c>
-      <c r="H19" s="40" t="n"/>
-      <c r="I19" s="40" t="inlineStr">
+      <c r="H19" s="41" t="n"/>
+      <c r="I19" s="41" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5294,7 +5689,7 @@
           <t>A16</t>
         </is>
       </c>
-      <c r="B20" s="43" t="n">
+      <c r="B20" s="44" t="n">
         <v>3</v>
       </c>
       <c r="C20" s="29" t="inlineStr">
@@ -5312,14 +5707,14 @@
           <t>IRG non vérifiable salarié par salarié (centralisateurs uniquement).</t>
         </is>
       </c>
-      <c r="F20" s="42" t="n"/>
+      <c r="F20" s="43" t="n"/>
       <c r="G20" s="29" t="inlineStr">
         <is>
           <t>Fournir le livre de paie individuel / bulletins.</t>
         </is>
       </c>
-      <c r="H20" s="40" t="n"/>
-      <c r="I20" s="40" t="inlineStr">
+      <c r="H20" s="41" t="n"/>
+      <c r="I20" s="41" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5331,7 +5726,7 @@
           <t>A17</t>
         </is>
       </c>
-      <c r="B21" s="38" t="n">
+      <c r="B21" s="39" t="n">
         <v>1</v>
       </c>
       <c r="C21" s="29" t="inlineStr">
@@ -5346,10 +5741,10 @@
       </c>
       <c r="E21" s="29" t="inlineStr">
         <is>
-          <t>TVA collectée TPM (44537) et location (44527) jamais soldées : 58,9 M DA cumulés au 31/12/2025. En 2025, 4 839 300 de TVA TPM générée, seuls 391 208 passés en G50 (déc.).</t>
-        </is>
-      </c>
-      <c r="F21" s="39">
+          <t>TVA collectée TPM (44537) et location (44527) jamais soldées : 58,9 M DA cumulés au 31/12/2025. En 2025, 4 839 300 de TVA TPM générée, seuls 391 208 passés en G50 (déc.). Les G50 TPM 2026 (juil., août) ne déclarent aucun CA et reportent un précompte de 1 714 499 (= compte 44550).</t>
+        </is>
+      </c>
+      <c r="F21" s="40">
         <f>-('Balance 2024-2025'!D48+'Balance 2024-2025'!D47)</f>
         <v/>
       </c>
@@ -5358,8 +5753,8 @@
           <t>Rapprocher avec les G50 TPM 2023–2025 ; si TVA non déclarée, régulariser ; sinon passer les écritures de G50 manquantes.</t>
         </is>
       </c>
-      <c r="H21" s="40" t="n"/>
-      <c r="I21" s="40" t="inlineStr">
+      <c r="H21" s="41" t="n"/>
+      <c r="I21" s="41" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5371,7 +5766,7 @@
           <t>A18</t>
         </is>
       </c>
-      <c r="B22" s="38" t="n">
+      <c r="B22" s="39" t="n">
         <v>1</v>
       </c>
       <c r="C22" s="29" t="inlineStr">
@@ -5389,7 +5784,7 @@
           <t>CA de mars 2026 réalisé 27 006 870 (annotation G50), mais seulement 3 445 200 déclarés en mars « pour manque TVA à récupérer » : 23 561 670 de CA reportés sur avril–août. En avril, le CA annoté (13 157 894,74) est calculé pour obtenir 2 500 000 de TVA. Le CA déclaré mensuellement est ajusté à la TVA déductible disponible.</t>
         </is>
       </c>
-      <c r="F22" s="39">
+      <c r="F22" s="40">
         <f>'G50 2026'!B40</f>
         <v/>
       </c>
@@ -5398,8 +5793,8 @@
           <t>Déclarer le CA au titre du mois de réalisation ; rapprocher le CA déclaré du journal des ventes 2026 ; chiffrer les pénalités de retard sur la TVA différée.</t>
         </is>
       </c>
-      <c r="H22" s="40" t="n"/>
-      <c r="I22" s="40" t="inlineStr">
+      <c r="H22" s="41" t="n"/>
+      <c r="I22" s="41" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5411,7 +5806,7 @@
           <t>A19</t>
         </is>
       </c>
-      <c r="B23" s="41" t="n">
+      <c r="B23" s="42" t="n">
         <v>2</v>
       </c>
       <c r="C23" s="29" t="inlineStr">
@@ -5426,20 +5821,20 @@
       </c>
       <c r="E23" s="29" t="inlineStr">
         <is>
-          <t>IRG retenu sur les salariés TPM (mars–août) absent des G50 IMPORT.</t>
-        </is>
-      </c>
-      <c r="F23" s="39">
-        <f>'G50 2026'!H22</f>
+          <t>G50 TPM de juillet : mois imprimé « AVRIL » et IRG déclaré 9 375 (montant d'avril/mai) au lieu de 3 691,30 retenus en juillet ; août conforme (3 690). G50 TPM de janvier à juin non fournies.</t>
+        </is>
+      </c>
+      <c r="F23" s="40">
+        <f>SUM('Paie TPM'!C25:H25)</f>
         <v/>
       </c>
       <c r="G23" s="29" t="inlineStr">
         <is>
-          <t>Fournir les G50 TPM 2026 ou régulariser.</t>
-        </is>
-      </c>
-      <c r="H23" s="40" t="n"/>
-      <c r="I23" s="40" t="inlineStr">
+          <t>Fournir les G50 TPM janv.–juin ; corriger ou justifier la G50 de juillet (régularisation de l'écart 5 683,70).</t>
+        </is>
+      </c>
+      <c r="H23" s="41" t="n"/>
+      <c r="I23" s="41" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5451,7 +5846,7 @@
           <t>A20</t>
         </is>
       </c>
-      <c r="B24" s="41" t="n">
+      <c r="B24" s="42" t="n">
         <v>2</v>
       </c>
       <c r="C24" s="29" t="inlineStr">
@@ -5469,7 +5864,7 @@
           <t>Écriture du 31/12/2025 « POUR SOLDE PRCT EXE 2025 » passée en sens inverse (D 44410 / C 444, 3 074 299) : dette IBS 9,79 M et acomptes 6,15 M au lieu d'un net de 3 642 951.</t>
         </is>
       </c>
-      <c r="F24" s="39" t="n">
+      <c r="F24" s="40" t="n">
         <v>3074299</v>
       </c>
       <c r="G24" s="29" t="inlineStr">
@@ -5477,8 +5872,8 @@
           <t>Contrepasser et compenser (D 444 / C 44410) ; vérifier le paiement du solde IBS 2025 en 2026.</t>
         </is>
       </c>
-      <c r="H24" s="40" t="n"/>
-      <c r="I24" s="40" t="inlineStr">
+      <c r="H24" s="41" t="n"/>
+      <c r="I24" s="41" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5490,7 +5885,7 @@
           <t>A21</t>
         </is>
       </c>
-      <c r="B25" s="41" t="n">
+      <c r="B25" s="42" t="n">
         <v>2</v>
       </c>
       <c r="C25" s="29" t="inlineStr">
@@ -5508,7 +5903,7 @@
           <t>Solde IBS 2024 réglé le 03/07/2025 ; IBS 2025 net à liquider de 3 642 951 (précomptes douane déduits).</t>
         </is>
       </c>
-      <c r="F25" s="39" t="n">
+      <c r="F25" s="40" t="n">
         <v>3642951</v>
       </c>
       <c r="G25" s="29" t="inlineStr">
@@ -5516,8 +5911,8 @@
           <t>Vérifier les dates d'échéance de liquidation, les pénalités éventuelles et la preuve de paiement 2026.</t>
         </is>
       </c>
-      <c r="H25" s="40" t="n"/>
-      <c r="I25" s="40" t="inlineStr">
+      <c r="H25" s="41" t="n"/>
+      <c r="I25" s="41" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5529,7 +5924,7 @@
           <t>A22</t>
         </is>
       </c>
-      <c r="B26" s="41" t="n">
+      <c r="B26" s="42" t="n">
         <v>2</v>
       </c>
       <c r="C26" s="29" t="inlineStr">
@@ -5547,7 +5942,7 @@
           <t>Caisse de 12,1 M au 31/12/2025 (pic de 22,5 M) ; remboursement en espèces de 6 800 000 à SARL DPR AXXAM le 06/12/2025.</t>
         </is>
       </c>
-      <c r="F26" s="39">
+      <c r="F26" s="40">
         <f>'Balance 2024-2025'!D67</f>
         <v/>
       </c>
@@ -5556,8 +5951,8 @@
           <t>PV de caisse au 31/12 ; respecter l'obligation de paiement scriptural au-delà des seuils réglementaires.</t>
         </is>
       </c>
-      <c r="H26" s="40" t="n"/>
-      <c r="I26" s="40" t="inlineStr">
+      <c r="H26" s="41" t="n"/>
+      <c r="I26" s="41" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5569,7 +5964,7 @@
           <t>A23</t>
         </is>
       </c>
-      <c r="B27" s="41" t="n">
+      <c r="B27" s="42" t="n">
         <v>2</v>
       </c>
       <c r="C27" s="29" t="inlineStr">
@@ -5587,7 +5982,7 @@
           <t>100 % du CA TPM 2025 (25,47 M) facturé à SARL DPR AXXAM BRIQUETERIE ; aucune facturation TPM d'oct. à déc. 2025 alors que du personnel TPM reste payé.</t>
         </is>
       </c>
-      <c r="F27" s="39">
+      <c r="F27" s="40">
         <f>-'Balance 2024-2025'!D100</f>
         <v/>
       </c>
@@ -5596,8 +5991,8 @@
           <t>Documenter les conventions intra-groupe et la facturation d'oct.–déc. 2025.</t>
         </is>
       </c>
-      <c r="H27" s="40" t="n"/>
-      <c r="I27" s="40" t="inlineStr">
+      <c r="H27" s="41" t="n"/>
+      <c r="I27" s="41" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5609,7 +6004,7 @@
           <t>A24</t>
         </is>
       </c>
-      <c r="B28" s="41" t="n">
+      <c r="B28" s="42" t="n">
         <v>2</v>
       </c>
       <c r="C28" s="29" t="inlineStr">
@@ -5627,7 +6022,7 @@
           <t>Compte d'attente 47000 non soldé (« SARL FAHAS ?? », « TRESORERIE BEJAIA ?? », chèques).</t>
         </is>
       </c>
-      <c r="F28" s="39">
+      <c r="F28" s="40">
         <f>'Balance 2024-2025'!D59</f>
         <v/>
       </c>
@@ -5636,8 +6031,8 @@
           <t>Identifier et apurer avant clôture.</t>
         </is>
       </c>
-      <c r="H28" s="40" t="n"/>
-      <c r="I28" s="40" t="inlineStr">
+      <c r="H28" s="41" t="n"/>
+      <c r="I28" s="41" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5649,7 +6044,7 @@
           <t>A25</t>
         </is>
       </c>
-      <c r="B29" s="41" t="n">
+      <c r="B29" s="42" t="n">
         <v>2</v>
       </c>
       <c r="C29" s="29" t="inlineStr">
@@ -5667,7 +6062,7 @@
           <t>Compte 63120 « prime imposable » non soumise à cotisation : 957 406 en 2025 et 1 139 275 en 2024 (même mécanisme que A03).</t>
         </is>
       </c>
-      <c r="F29" s="39">
+      <c r="F29" s="40">
         <f>'États 2024-2025'!C24+'États 2024-2025'!D24</f>
         <v/>
       </c>
@@ -5676,8 +6071,8 @@
           <t>Analyser les primes concernées ; régulariser si elles sont cotisables.</t>
         </is>
       </c>
-      <c r="H29" s="40" t="n"/>
-      <c r="I29" s="40" t="inlineStr">
+      <c r="H29" s="41" t="n"/>
+      <c r="I29" s="41" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5689,7 +6084,7 @@
           <t>A26</t>
         </is>
       </c>
-      <c r="B30" s="43" t="n">
+      <c r="B30" s="44" t="n">
         <v>3</v>
       </c>
       <c r="C30" s="29" t="inlineStr">
@@ -5707,7 +6102,7 @@
           <t>Banque CPA El Kseur (51220) créditrice de 12,43 M au 31/12/2025 : découvert présenté en banque.</t>
         </is>
       </c>
-      <c r="F30" s="39">
+      <c r="F30" s="40">
         <f>ABS('Balance 2024-2025'!D63)</f>
         <v/>
       </c>
@@ -5716,8 +6111,8 @@
           <t>Reclasser en 519 ; vérifier les agios (aucune charge 661 en 2025).</t>
         </is>
       </c>
-      <c r="H30" s="40" t="n"/>
-      <c r="I30" s="40" t="inlineStr">
+      <c r="H30" s="41" t="n"/>
+      <c r="I30" s="41" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5729,7 +6124,7 @@
           <t>A27</t>
         </is>
       </c>
-      <c r="B31" s="43" t="n">
+      <c r="B31" s="44" t="n">
         <v>3</v>
       </c>
       <c r="C31" s="29" t="inlineStr">
@@ -5747,7 +6142,7 @@
           <t>Reversements IRG 2025 parfois partiels (févr., juin) et rattrapés le mois suivant ; amendes 2025 : douane 100 000, CNAS 1 746.</t>
         </is>
       </c>
-      <c r="F31" s="39">
+      <c r="F31" s="40">
         <f>'Balance 2024-2025'!D93</f>
         <v/>
       </c>
@@ -5756,8 +6151,8 @@
           <t>Reverser l'IRG en totalité chaque mois.</t>
         </is>
       </c>
-      <c r="H31" s="40" t="n"/>
-      <c r="I31" s="40" t="inlineStr">
+      <c r="H31" s="41" t="n"/>
+      <c r="I31" s="41" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5769,7 +6164,7 @@
           <t>A28</t>
         </is>
       </c>
-      <c r="B32" s="43" t="n">
+      <c r="B32" s="44" t="n">
         <v>3</v>
       </c>
       <c r="C32" s="29" t="inlineStr">
@@ -5784,17 +6179,17 @@
       </c>
       <c r="E32" s="29" t="inlineStr">
         <is>
-          <t>Modèle G50 non mis à jour : dates de signature imprimées de 2021–2022 sur toutes les G50 2026, onglet de saisie figé (mai, TVA 17 %) ; libellés de comptes de TVA à 17 %.</t>
-        </is>
-      </c>
-      <c r="F32" s="42" t="n"/>
+          <t>Modèles G50 non mis à jour : dates de signature de 2021–2022 sur toutes les G50 2026, onglet de saisie figé (mai, TVA 17 %), G50 TPM contenant le récap TVA de déc. 2025 et un extrait de journal 2019 ; libellés de comptes de TVA à 17 %.</t>
+        </is>
+      </c>
+      <c r="F32" s="43" t="n"/>
       <c r="G32" s="29" t="inlineStr">
         <is>
           <t>Mettre à jour le modèle et les libellés (TVA 19 %).</t>
         </is>
       </c>
-      <c r="H32" s="40" t="n"/>
-      <c r="I32" s="40" t="inlineStr">
+      <c r="H32" s="41" t="n"/>
+      <c r="I32" s="41" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5806,12 +6201,12 @@
           <t>A29</t>
         </is>
       </c>
-      <c r="B33" s="43" t="n">
+      <c r="B33" s="44" t="n">
         <v>3</v>
       </c>
       <c r="C33" s="29" t="inlineStr">
         <is>
-          <t>IMPORT</t>
+          <t>Les deux</t>
         </is>
       </c>
       <c r="D33" s="29" t="inlineStr">
@@ -5821,20 +6216,20 @@
       </c>
       <c r="E33" s="29" t="inlineStr">
         <is>
-          <t>Taxe d'apprentissage de 44 091 (août 2026) sur une base de 4 409 079 à justifier.</t>
-        </is>
-      </c>
-      <c r="F33" s="39">
-        <f>'G50 2026'!G26</f>
+          <t>Taxe d'apprentissage payée deux fois en 2026 : février (87 828 sur 8 782 828) et août (44 091 IMPORT sur 4 409 079 + 6 809 TPM sur 680 900).</t>
+        </is>
+      </c>
+      <c r="F33" s="40">
+        <f>'G50 2026'!J26+'G50 TPM 2026'!C18</f>
         <v/>
       </c>
       <c r="G33" s="29" t="inlineStr">
         <is>
-          <t>Justifier la base (1 % de la masse salariale de référence).</t>
-        </is>
-      </c>
-      <c r="H33" s="40" t="n"/>
-      <c r="I33" s="40" t="inlineStr">
+          <t>Justifier les bases et la période couverte par chaque paiement (risque de double paiement).</t>
+        </is>
+      </c>
+      <c r="H33" s="41" t="n"/>
+      <c r="I33" s="41" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5846,7 +6241,7 @@
           <t>A30</t>
         </is>
       </c>
-      <c r="B34" s="43" t="n">
+      <c r="B34" s="44" t="n">
         <v>3</v>
       </c>
       <c r="C34" s="29" t="inlineStr">
@@ -5861,11 +6256,11 @@
       </c>
       <c r="E34" s="29" t="inlineStr">
         <is>
-          <t>Droit de timbre : même base (177 058) en avril et mai, mais 8 944 puis 3 173 ; aucun timbre les autres mois.</t>
-        </is>
-      </c>
-      <c r="F34" s="39">
-        <f>'G50 2026'!H24</f>
+          <t>Droit de timbre : taux apparents incohérents (janv. 2,0 %, févr. 1,0 %, avr. 5,05 %, mai 1,79 %) ; même base en avril et mai ; aucun timbre en mars et de juin à août.</t>
+        </is>
+      </c>
+      <c r="F34" s="40">
+        <f>'G50 2026'!J24</f>
         <v/>
       </c>
       <c r="G34" s="29" t="inlineStr">
@@ -5873,8 +6268,8 @@
           <t>Justifier la base (ventes en espèces) et le taux appliqué.</t>
         </is>
       </c>
-      <c r="H34" s="40" t="n"/>
-      <c r="I34" s="40" t="inlineStr">
+      <c r="H34" s="41" t="n"/>
+      <c r="I34" s="41" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5886,7 +6281,7 @@
           <t>A31</t>
         </is>
       </c>
-      <c r="B35" s="43" t="n">
+      <c r="B35" s="44" t="n">
         <v>3</v>
       </c>
       <c r="C35" s="29" t="inlineStr">
@@ -5904,14 +6299,14 @@
           <t>Clients débiteurs 387,1 M et avances clients 314,6 M ; fournisseurs débiteurs 46,2 M au 31/12/2025.</t>
         </is>
       </c>
-      <c r="F35" s="42" t="n"/>
+      <c r="F35" s="43" t="n"/>
       <c r="G35" s="29" t="inlineStr">
         <is>
           <t>Lettrer les comptes clients/fournisseurs et compenser les avances soldées.</t>
         </is>
       </c>
-      <c r="H35" s="40" t="n"/>
-      <c r="I35" s="40" t="inlineStr">
+      <c r="H35" s="41" t="n"/>
+      <c r="I35" s="41" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5931,13 +6326,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6013,7 +6408,7 @@
           <t>Janv–août 2026</t>
         </is>
       </c>
-      <c r="E5" s="44" t="inlineStr">
+      <c r="E5" s="45" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6043,7 +6438,7 @@
           <t>Janv–août 2026</t>
         </is>
       </c>
-      <c r="E6" s="44" t="inlineStr">
+      <c r="E6" s="45" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6069,7 +6464,7 @@
           <t>Janvier 2026</t>
         </is>
       </c>
-      <c r="E7" s="44" t="inlineStr">
+      <c r="E7" s="45" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6099,7 +6494,7 @@
           <t>Mars 2026</t>
         </is>
       </c>
-      <c r="E8" s="44" t="inlineStr">
+      <c r="E8" s="45" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6129,7 +6524,7 @@
           <t>T2 2026</t>
         </is>
       </c>
-      <c r="E9" s="44" t="inlineStr">
+      <c r="E9" s="45" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6159,7 +6554,7 @@
           <t>T1 2026</t>
         </is>
       </c>
-      <c r="E10" s="44" t="inlineStr">
+      <c r="E10" s="45" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6189,7 +6584,7 @@
           <t>T2 2026</t>
         </is>
       </c>
-      <c r="E11" s="44" t="inlineStr">
+      <c r="E11" s="45" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6219,7 +6614,7 @@
           <t>Février 2026</t>
         </is>
       </c>
-      <c r="E12" s="45" t="inlineStr">
+      <c r="E12" s="46" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
@@ -6249,7 +6644,7 @@
           <t>Mars 2026</t>
         </is>
       </c>
-      <c r="E13" s="45" t="inlineStr">
+      <c r="E13" s="46" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
@@ -6275,7 +6670,7 @@
           <t>Septembre 2026</t>
         </is>
       </c>
-      <c r="E14" s="45" t="inlineStr">
+      <c r="E14" s="46" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
@@ -6305,7 +6700,7 @@
           <t>T3 2026</t>
         </is>
       </c>
-      <c r="E15" s="45" t="inlineStr">
+      <c r="E15" s="46" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
@@ -6335,7 +6730,7 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="E16" s="45" t="inlineStr">
+      <c r="E16" s="46" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
@@ -6365,7 +6760,7 @@
           <t>Juin 2026</t>
         </is>
       </c>
-      <c r="E17" s="44" t="inlineStr">
+      <c r="E17" s="45" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6395,7 +6790,7 @@
           <t>Août 2026</t>
         </is>
       </c>
-      <c r="E18" s="44" t="inlineStr">
+      <c r="E18" s="45" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6425,7 +6820,7 @@
           <t>Exercice 2024</t>
         </is>
       </c>
-      <c r="E19" s="44" t="inlineStr">
+      <c r="E19" s="45" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6455,7 +6850,7 @@
           <t>Exercice 2025</t>
         </is>
       </c>
-      <c r="E20" s="44" t="inlineStr">
+      <c r="E20" s="45" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6485,7 +6880,7 @@
           <t>Mars, avril, mai, juillet 2026</t>
         </is>
       </c>
-      <c r="E21" s="44" t="inlineStr">
+      <c r="E21" s="45" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6502,7 +6897,7 @@
       </c>
       <c r="B22" s="12" t="inlineStr">
         <is>
-          <t>G50 IMPORT janvier, février et septembre 2026</t>
+          <t>G50_ARL_DPR_COMPANY_IMPORT_01/02-2026.xls</t>
         </is>
       </c>
       <c r="C22" s="12" t="inlineStr">
@@ -6512,15 +6907,19 @@
       </c>
       <c r="D22" s="12" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>Janvier, février 2026</t>
         </is>
       </c>
       <c r="E22" s="45" t="inlineStr">
         <is>
-          <t>Manquante</t>
-        </is>
-      </c>
-      <c r="F22" s="12" t="inlineStr"/>
+          <t>Reçue</t>
+        </is>
+      </c>
+      <c r="F22" s="12" t="inlineStr">
+        <is>
+          <t>Série janv.–août complète</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="12" t="n">
@@ -6528,27 +6927,27 @@
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>Journal des ventes / factures 2026</t>
+          <t>G50_07/08-2026_TPM_ET_LOCATION_CONSOLIDE.xls</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>IMPORT</t>
+          <t>TPM</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>Juillet, août 2026</t>
         </is>
       </c>
       <c r="E23" s="45" t="inlineStr">
         <is>
-          <t>Manquante</t>
+          <t>Reçue</t>
         </is>
       </c>
       <c r="F23" s="12" t="inlineStr">
         <is>
-          <t>Voir A18 : CA réel par mois</t>
+          <t>Juillet : mois imprimé AVRIL</t>
         </is>
       </c>
     </row>
@@ -6558,7 +6957,7 @@
       </c>
       <c r="B24" s="12" t="inlineStr">
         <is>
-          <t>G50 TPM 2026 (et rapprochement TVA TPM 2023–2025)</t>
+          <t>G50 TPM et location janvier à juin 2026</t>
         </is>
       </c>
       <c r="C24" s="12" t="inlineStr">
@@ -6568,17 +6967,17 @@
       </c>
       <c r="D24" s="12" t="inlineStr">
         <is>
-          <t>2023–2026</t>
-        </is>
-      </c>
-      <c r="E24" s="45" t="inlineStr">
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E24" s="46" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
       </c>
       <c r="F24" s="12" t="inlineStr">
         <is>
-          <t>Voir A17, A19</t>
+          <t>Voir A19</t>
         </is>
       </c>
     </row>
@@ -6588,27 +6987,27 @@
       </c>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>Journal comptable 2026 (PCCOMPTA)</t>
+          <t>G50 IMPORT et TPM septembre 2026</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>Société</t>
+          <t>Les deux</t>
         </is>
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="E25" s="45" t="inlineStr">
+          <t>Sept. 2026</t>
+        </is>
+      </c>
+      <c r="E25" s="46" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
       </c>
       <c r="F25" s="12" t="inlineStr">
         <is>
-          <t>Pour rapprocher paie et G50 avec la comptabilité</t>
+          <t>Échéance 20/10/2026</t>
         </is>
       </c>
     </row>
@@ -6618,27 +7017,27 @@
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>Liasse fiscale / bilan 2025 déposé et preuve de paiement IBS</t>
+          <t>Journal des ventes / factures 2026</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>Société</t>
+          <t>IMPORT</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
         <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="E26" s="45" t="inlineStr">
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E26" s="46" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
       </c>
       <c r="F26" s="12" t="inlineStr">
         <is>
-          <t>Voir A20, A21</t>
+          <t>Voir A18 : CA réel par mois</t>
         </is>
       </c>
     </row>
@@ -6648,27 +7047,27 @@
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>PV de caisse au 31/12/2025</t>
+          <t>G50 TPM 2023–2025 (rapprochement TVA collectée TPM)</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>Société</t>
+          <t>TPM</t>
         </is>
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="E27" s="45" t="inlineStr">
+          <t>2023–2025</t>
+        </is>
+      </c>
+      <c r="E27" s="46" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
       </c>
       <c r="F27" s="12" t="inlineStr">
         <is>
-          <t>Voir A22</t>
+          <t>Voir A17</t>
         </is>
       </c>
     </row>
@@ -6678,12 +7077,12 @@
       </c>
       <c r="B28" s="12" t="inlineStr">
         <is>
-          <t>Déclarations et paiements CACOBATPH</t>
+          <t>Journal comptable 2026 (PCCOMPTA)</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
         <is>
-          <t>Les deux</t>
+          <t>Société</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
@@ -6691,12 +7090,16 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="E28" s="45" t="inlineStr">
+      <c r="E28" s="46" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
       </c>
-      <c r="F28" s="12" t="inlineStr"/>
+      <c r="F28" s="12" t="inlineStr">
+        <is>
+          <t>Pour rapprocher paie et G50 avec la comptabilité</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="12" t="n">
@@ -6704,27 +7107,27 @@
       </c>
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>Livre de paie individuel / bulletins</t>
+          <t>Liasse fiscale / bilan 2025 déposé et preuve de paiement IBS</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>Les deux</t>
+          <t>Société</t>
         </is>
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="E29" s="45" t="inlineStr">
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E29" s="46" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
       </c>
       <c r="F29" s="12" t="inlineStr">
         <is>
-          <t>Pour contrôle IRG</t>
+          <t>Voir A20, A21</t>
         </is>
       </c>
     </row>
@@ -6734,27 +7137,27 @@
       </c>
       <c r="B30" s="12" t="inlineStr">
         <is>
-          <t>Ordres de mission et justificatifs de frais</t>
+          <t>PV de caisse au 31/12/2025</t>
         </is>
       </c>
       <c r="C30" s="12" t="inlineStr">
         <is>
-          <t>TPM</t>
+          <t>Société</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="E30" s="45" t="inlineStr">
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E30" s="46" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
       </c>
       <c r="F30" s="12" t="inlineStr">
         <is>
-          <t>Frais de mission élevés</t>
+          <t>Voir A22</t>
         </is>
       </c>
     </row>
@@ -6764,25 +7167,111 @@
       </c>
       <c r="B31" s="12" t="inlineStr">
         <is>
+          <t>Déclarations et paiements CACOBATPH</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>Les deux</t>
+        </is>
+      </c>
+      <c r="D31" s="12" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E31" s="46" t="inlineStr">
+        <is>
+          <t>Manquante</t>
+        </is>
+      </c>
+      <c r="F31" s="12" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>Livre de paie individuel / bulletins</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="inlineStr">
+        <is>
+          <t>Les deux</t>
+        </is>
+      </c>
+      <c r="D32" s="12" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E32" s="46" t="inlineStr">
+        <is>
+          <t>Manquante</t>
+        </is>
+      </c>
+      <c r="F32" s="12" t="inlineStr">
+        <is>
+          <t>Pour contrôle IRG</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>Ordres de mission et justificatifs de frais</t>
+        </is>
+      </c>
+      <c r="C33" s="12" t="inlineStr">
+        <is>
+          <t>TPM</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E33" s="46" t="inlineStr">
+        <is>
+          <t>Manquante</t>
+        </is>
+      </c>
+      <c r="F33" s="12" t="inlineStr">
+        <is>
+          <t>Frais de mission élevés</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="12" t="inlineStr">
+        <is>
           <t>Relevés bancaires — virements de salaires</t>
         </is>
       </c>
-      <c r="C31" s="12" t="inlineStr">
+      <c r="C34" s="12" t="inlineStr">
         <is>
           <t>Les deux</t>
         </is>
       </c>
-      <c r="D31" s="12" t="inlineStr">
+      <c r="D34" s="12" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="E31" s="45" t="inlineStr">
+      <c r="E34" s="46" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
       </c>
-      <c r="F31" s="12" t="inlineStr">
+      <c r="F34" s="12" t="inlineStr">
         <is>
           <t>Pour lettrage du 421</t>
         </is>
@@ -15633,7 +16122,10 @@
           <t>20/02/2026</t>
         </is>
       </c>
-      <c r="I5" s="33" t="n"/>
+      <c r="I5" s="6">
+        <f>'G50 2026'!B19</f>
+        <v/>
+      </c>
       <c r="J5" s="30">
         <f>IF(I5="","",IF(E5=0,"paie absente",I5-E5))</f>
         <v/>
@@ -15690,7 +16182,10 @@
           <t>20/03/2026</t>
         </is>
       </c>
-      <c r="I6" s="33" t="n"/>
+      <c r="I6" s="6">
+        <f>'G50 2026'!C19</f>
+        <v/>
+      </c>
       <c r="J6" s="30">
         <f>IF(I6="","",IF(E6=0,"paie absente",I6-E6))</f>
         <v/>
@@ -15748,7 +16243,7 @@
         </is>
       </c>
       <c r="I7" s="6">
-        <f>'G50 2026'!B19</f>
+        <f>'G50 2026'!D19</f>
         <v/>
       </c>
       <c r="J7" s="30">
@@ -15808,7 +16303,7 @@
         </is>
       </c>
       <c r="I8" s="6">
-        <f>'G50 2026'!C19</f>
+        <f>'G50 2026'!E19</f>
         <v/>
       </c>
       <c r="J8" s="30">
@@ -15868,7 +16363,7 @@
         </is>
       </c>
       <c r="I9" s="6">
-        <f>'G50 2026'!D19</f>
+        <f>'G50 2026'!F19</f>
         <v/>
       </c>
       <c r="J9" s="30">
@@ -15928,7 +16423,7 @@
         </is>
       </c>
       <c r="I10" s="6">
-        <f>'G50 2026'!E19</f>
+        <f>'G50 2026'!G19</f>
         <v/>
       </c>
       <c r="J10" s="30">
@@ -15988,7 +16483,7 @@
         </is>
       </c>
       <c r="I11" s="6">
-        <f>'G50 2026'!F19</f>
+        <f>'G50 2026'!H19</f>
         <v/>
       </c>
       <c r="J11" s="30">
@@ -16048,7 +16543,7 @@
         </is>
       </c>
       <c r="I12" s="6">
-        <f>'G50 2026'!G19</f>
+        <f>'G50 2026'!I19</f>
         <v/>
       </c>
       <c r="J12" s="30">
@@ -16118,7 +16613,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Colonne I : G50 IMPORT mars à août reçues (liées à « G50 2026 ») ; janvier et février en jaune à compléter. Écart IRG = G50 − IRG paie IMPORT. L'IRG TPM (colonne F) doit figurer sur une G50 TPM distincte (non fournie).</t>
+          <t>Colonne I : G50 IMPORT janvier à août reçues (liées à « G50 2026 »). Écart IRG = G50 − IRG paie IMPORT. L'IRG TPM (colonne F) doit figurer sur une G50 TPM distincte (non fournie).</t>
         </is>
       </c>
     </row>
@@ -16134,7 +16629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:K49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -16145,7 +16640,9 @@
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="55" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="55" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -16158,7 +16655,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Sources : fichiers G50_ARL_DPR_COMPANY_IMPORT_03 à 08-2026.xls (feuilles G.50-1/2/3). Valeurs en bleu = lues sur les G50.</t>
+          <t>Sources : fichiers G50_ARL_DPR_COMPANY_IMPORT_01 à 08-2026.xls (feuilles G.50-1/2/3). Valeurs en bleu = lues sur les G50.</t>
         </is>
       </c>
     </row>
@@ -16185,40 +16682,50 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
+          <t>Janv 2026</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>Févr 2026</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
           <t>Mars 2026</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>Avr 2026</t>
         </is>
       </c>
-      <c r="D6" s="11" t="inlineStr">
+      <c r="F6" s="11" t="inlineStr">
         <is>
           <t>Mai 2026</t>
         </is>
       </c>
-      <c r="E6" s="11" t="inlineStr">
+      <c r="G6" s="11" t="inlineStr">
         <is>
           <t>Juin 2026</t>
         </is>
       </c>
-      <c r="F6" s="11" t="inlineStr">
+      <c r="H6" s="11" t="inlineStr">
         <is>
           <t>Juil 2026</t>
         </is>
       </c>
-      <c r="G6" s="11" t="inlineStr">
+      <c r="I6" s="11" t="inlineStr">
         <is>
           <t>Août 2026</t>
         </is>
       </c>
-      <c r="H6" s="11" t="inlineStr">
+      <c r="J6" s="11" t="inlineStr">
         <is>
           <t>Cumul</t>
         </is>
       </c>
-      <c r="I6" s="11" t="inlineStr">
+      <c r="K6" s="11" t="inlineStr">
         <is>
           <t>Commentaire</t>
         </is>
@@ -16231,28 +16738,34 @@
         </is>
       </c>
       <c r="B7" s="25" t="n">
+        <v>11994522</v>
+      </c>
+      <c r="C7" s="25" t="n">
+        <v>27783649</v>
+      </c>
+      <c r="D7" s="25" t="n">
         <v>3445200</v>
       </c>
-      <c r="C7" s="25" t="n">
+      <c r="E7" s="25" t="n">
         <v>23988307</v>
       </c>
-      <c r="D7" s="25" t="n">
+      <c r="F7" s="25" t="n">
         <v>16671298</v>
       </c>
-      <c r="E7" s="25" t="n">
+      <c r="G7" s="25" t="n">
         <v>10479294</v>
       </c>
-      <c r="F7" s="25" t="n">
+      <c r="H7" s="25" t="n">
         <v>7604135</v>
       </c>
-      <c r="G7" s="25" t="n">
+      <c r="I7" s="25" t="n">
         <v>4413684</v>
       </c>
-      <c r="H7" s="7">
-        <f>SUM(B7:G7)</f>
-        <v/>
-      </c>
-      <c r="I7" s="35" t="inlineStr">
+      <c r="J7" s="7">
+        <f>SUM(B7:I7)</f>
+        <v/>
+      </c>
+      <c r="K7" s="35" t="inlineStr">
         <is>
           <t>Revente en l'état</t>
         </is>
@@ -16265,28 +16778,34 @@
         </is>
       </c>
       <c r="B8" s="25" t="n">
+        <v>2278959</v>
+      </c>
+      <c r="C8" s="25" t="n">
+        <v>5278893</v>
+      </c>
+      <c r="D8" s="25" t="n">
         <v>654588</v>
       </c>
-      <c r="C8" s="25" t="n">
+      <c r="E8" s="25" t="n">
         <v>4557778</v>
       </c>
-      <c r="D8" s="25" t="n">
+      <c r="F8" s="25" t="n">
         <v>3167547</v>
       </c>
-      <c r="E8" s="25" t="n">
+      <c r="G8" s="25" t="n">
         <v>1991066</v>
       </c>
-      <c r="F8" s="25" t="n">
+      <c r="H8" s="25" t="n">
         <v>1444786</v>
       </c>
-      <c r="G8" s="25" t="n">
+      <c r="I8" s="25" t="n">
         <v>838600</v>
       </c>
-      <c r="H8" s="7">
-        <f>SUM(B8:G8)</f>
-        <v/>
-      </c>
-      <c r="I8" s="35" t="inlineStr"/>
+      <c r="J8" s="7">
+        <f>SUM(B8:I8)</f>
+        <v/>
+      </c>
+      <c r="K8" s="35" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -16318,11 +16837,19 @@
         <f>ROUND(G7*$B$4,0)</f>
         <v/>
       </c>
-      <c r="H9" s="7">
-        <f>SUM(B9:G9)</f>
-        <v/>
-      </c>
-      <c r="I9" s="35" t="inlineStr">
+      <c r="H9" s="30">
+        <f>ROUND(H7*$B$4,0)</f>
+        <v/>
+      </c>
+      <c r="I9" s="30">
+        <f>ROUND(I7*$B$4,0)</f>
+        <v/>
+      </c>
+      <c r="J9" s="7">
+        <f>SUM(B9:I9)</f>
+        <v/>
+      </c>
+      <c r="K9" s="35" t="inlineStr">
         <is>
           <t>Calcul</t>
         </is>
@@ -16358,11 +16885,19 @@
         <f>G8-G9</f>
         <v/>
       </c>
-      <c r="H10" s="7">
-        <f>SUM(B10:G10)</f>
-        <v/>
-      </c>
-      <c r="I10" s="35" t="inlineStr">
+      <c r="H10" s="30">
+        <f>H8-H9</f>
+        <v/>
+      </c>
+      <c r="I10" s="30">
+        <f>I8-I9</f>
+        <v/>
+      </c>
+      <c r="J10" s="7">
+        <f>SUM(B10:I10)</f>
+        <v/>
+      </c>
+      <c r="K10" s="35" t="inlineStr">
         <is>
           <t>Arrondi admis ±1</t>
         </is>
@@ -16384,19 +16919,25 @@
         <v>0</v>
       </c>
       <c r="E11" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="25" t="n">
         <v>386205</v>
       </c>
-      <c r="F11" s="25" t="n">
+      <c r="H11" s="25" t="n">
         <v>178353</v>
       </c>
-      <c r="G11" s="25" t="n">
+      <c r="I11" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H11" s="7">
-        <f>SUM(B11:G11)</f>
-        <v/>
-      </c>
-      <c r="I11" s="35" t="inlineStr"/>
+      <c r="J11" s="7">
+        <f>SUM(B11:I11)</f>
+        <v/>
+      </c>
+      <c r="K11" s="35" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
@@ -16405,28 +16946,34 @@
         </is>
       </c>
       <c r="B12" s="25" t="n">
+        <v>1150880</v>
+      </c>
+      <c r="C12" s="25" t="n">
+        <v>2199941</v>
+      </c>
+      <c r="D12" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="C12" s="25" t="n">
+      <c r="E12" s="25" t="n">
         <v>3919465</v>
       </c>
-      <c r="D12" s="25" t="n">
+      <c r="F12" s="25" t="n">
         <v>3553752</v>
       </c>
-      <c r="E12" s="25" t="n">
+      <c r="G12" s="25" t="n">
         <v>1783214</v>
       </c>
-      <c r="F12" s="25" t="n">
+      <c r="H12" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="G12" s="25" t="n">
+      <c r="I12" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="7">
-        <f>SUM(B12:G12)</f>
-        <v/>
-      </c>
-      <c r="I12" s="35" t="inlineStr"/>
+      <c r="J12" s="7">
+        <f>SUM(B12:I12)</f>
+        <v/>
+      </c>
+      <c r="K12" s="35" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -16458,11 +17005,19 @@
         <f>G11+G12</f>
         <v/>
       </c>
-      <c r="H13" s="7">
-        <f>SUM(B13:G13)</f>
-        <v/>
-      </c>
-      <c r="I13" s="35" t="inlineStr">
+      <c r="H13" s="30">
+        <f>H11+H12</f>
+        <v/>
+      </c>
+      <c r="I13" s="30">
+        <f>I11+I12</f>
+        <v/>
+      </c>
+      <c r="J13" s="7">
+        <f>SUM(B13:I13)</f>
+        <v/>
+      </c>
+      <c r="K13" s="35" t="inlineStr">
         <is>
           <t>Calcul</t>
         </is>
@@ -16498,11 +17053,19 @@
         <f>MAX(0,G8-G13)</f>
         <v/>
       </c>
-      <c r="H14" s="7">
-        <f>SUM(B14:G14)</f>
-        <v/>
-      </c>
-      <c r="I14" s="35" t="inlineStr">
+      <c r="H14" s="30">
+        <f>MAX(0,H8-H13)</f>
+        <v/>
+      </c>
+      <c r="I14" s="30">
+        <f>MAX(0,I8-I13)</f>
+        <v/>
+      </c>
+      <c r="J14" s="7">
+        <f>SUM(B14:I14)</f>
+        <v/>
+      </c>
+      <c r="K14" s="35" t="inlineStr">
         <is>
           <t>Calcul</t>
         </is>
@@ -16538,8 +17101,16 @@
         <f>MAX(0,G13-G8)</f>
         <v/>
       </c>
-      <c r="H15" s="27" t="n"/>
-      <c r="I15" s="35" t="inlineStr">
+      <c r="H15" s="30">
+        <f>MAX(0,H13-H8)</f>
+        <v/>
+      </c>
+      <c r="I15" s="30">
+        <f>MAX(0,I13-I8)</f>
+        <v/>
+      </c>
+      <c r="J15" s="27" t="n"/>
+      <c r="K15" s="35" t="inlineStr">
         <is>
           <t>Calcul</t>
         </is>
@@ -16572,8 +17143,16 @@
         <f>G11-F15</f>
         <v/>
       </c>
-      <c r="H16" s="27" t="n"/>
-      <c r="I16" s="35" t="inlineStr">
+      <c r="H16" s="30">
+        <f>H11-G15</f>
+        <v/>
+      </c>
+      <c r="I16" s="30">
+        <f>I11-H15</f>
+        <v/>
+      </c>
+      <c r="J16" s="27" t="n"/>
+      <c r="K16" s="35" t="inlineStr">
         <is>
           <t>Doit être 0 (chaîne mai → juin → juillet)</t>
         </is>
@@ -16586,28 +17165,34 @@
         </is>
       </c>
       <c r="B17" s="25" t="n">
+        <v>819091</v>
+      </c>
+      <c r="C17" s="25" t="n">
+        <v>905752</v>
+      </c>
+      <c r="D17" s="25" t="n">
         <v>365763</v>
       </c>
-      <c r="C17" s="25" t="n">
+      <c r="E17" s="25" t="n">
         <v>404385</v>
       </c>
-      <c r="D17" s="25" t="n">
+      <c r="F17" s="25" t="n">
         <v>426576</v>
       </c>
-      <c r="E17" s="25" t="n">
+      <c r="G17" s="25" t="n">
         <v>325645</v>
       </c>
-      <c r="F17" s="25" t="n">
+      <c r="H17" s="25" t="n">
         <v>286954</v>
       </c>
-      <c r="G17" s="25" t="n">
+      <c r="I17" s="25" t="n">
         <v>300000</v>
       </c>
-      <c r="H17" s="7">
-        <f>SUM(B17:G17)</f>
-        <v/>
-      </c>
-      <c r="I17" s="35" t="inlineStr"/>
+      <c r="J17" s="7">
+        <f>SUM(B17:I17)</f>
+        <v/>
+      </c>
+      <c r="K17" s="35" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
@@ -16616,34 +17201,42 @@
         </is>
       </c>
       <c r="B18" s="6">
+        <f>'Paie IMPORT'!C24</f>
+        <v/>
+      </c>
+      <c r="C18" s="6">
+        <f>'Paie IMPORT'!D24</f>
+        <v/>
+      </c>
+      <c r="D18" s="6">
         <f>'Paie IMPORT'!E24</f>
         <v/>
       </c>
-      <c r="C18" s="6">
+      <c r="E18" s="6">
         <f>'Paie IMPORT'!F24</f>
         <v/>
       </c>
-      <c r="D18" s="6">
+      <c r="F18" s="6">
         <f>'Paie IMPORT'!G24</f>
         <v/>
       </c>
-      <c r="E18" s="6">
+      <c r="G18" s="6">
         <f>'Paie IMPORT'!H24</f>
         <v/>
       </c>
-      <c r="F18" s="6">
+      <c r="H18" s="6">
         <f>'Paie IMPORT'!I24</f>
         <v/>
       </c>
-      <c r="G18" s="6">
+      <c r="I18" s="6">
         <f>'Paie IMPORT'!J24</f>
         <v/>
       </c>
-      <c r="H18" s="7">
-        <f>SUM(B18:G18)</f>
-        <v/>
-      </c>
-      <c r="I18" s="35" t="inlineStr">
+      <c r="J18" s="7">
+        <f>SUM(B18:I18)</f>
+        <v/>
+      </c>
+      <c r="K18" s="35" t="inlineStr">
         <is>
           <t>Lien paie (mars : centralisateur absent)</t>
         </is>
@@ -16656,28 +17249,34 @@
         </is>
       </c>
       <c r="B19" s="25" t="n">
+        <v>132616</v>
+      </c>
+      <c r="C19" s="25" t="n">
+        <v>162286</v>
+      </c>
+      <c r="D19" s="25" t="n">
         <v>60932</v>
       </c>
-      <c r="C19" s="25" t="n">
+      <c r="E19" s="25" t="n">
         <v>72478</v>
       </c>
-      <c r="D19" s="25" t="n">
+      <c r="F19" s="25" t="n">
         <v>79138</v>
       </c>
-      <c r="E19" s="25" t="n">
+      <c r="G19" s="25" t="n">
         <v>59018</v>
       </c>
-      <c r="F19" s="25" t="n">
+      <c r="H19" s="25" t="n">
         <v>42610</v>
       </c>
-      <c r="G19" s="25" t="n">
+      <c r="I19" s="25" t="n">
         <v>49670</v>
       </c>
-      <c r="H19" s="7">
-        <f>SUM(B19:G19)</f>
-        <v/>
-      </c>
-      <c r="I19" s="35" t="inlineStr"/>
+      <c r="J19" s="7">
+        <f>SUM(B19:I19)</f>
+        <v/>
+      </c>
+      <c r="K19" s="35" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
@@ -16686,34 +17285,42 @@
         </is>
       </c>
       <c r="B20" s="6">
+        <f>'Paie IMPORT'!C25</f>
+        <v/>
+      </c>
+      <c r="C20" s="6">
+        <f>'Paie IMPORT'!D25</f>
+        <v/>
+      </c>
+      <c r="D20" s="6">
         <f>'Paie IMPORT'!E25</f>
         <v/>
       </c>
-      <c r="C20" s="6">
+      <c r="E20" s="6">
         <f>'Paie IMPORT'!F25</f>
         <v/>
       </c>
-      <c r="D20" s="6">
+      <c r="F20" s="6">
         <f>'Paie IMPORT'!G25</f>
         <v/>
       </c>
-      <c r="E20" s="6">
+      <c r="G20" s="6">
         <f>'Paie IMPORT'!H25</f>
         <v/>
       </c>
-      <c r="F20" s="6">
+      <c r="H20" s="6">
         <f>'Paie IMPORT'!I25</f>
         <v/>
       </c>
-      <c r="G20" s="6">
+      <c r="I20" s="6">
         <f>'Paie IMPORT'!J25</f>
         <v/>
       </c>
-      <c r="H20" s="7">
-        <f>SUM(B20:G20)</f>
-        <v/>
-      </c>
-      <c r="I20" s="35" t="inlineStr">
+      <c r="J20" s="7">
+        <f>SUM(B20:I20)</f>
+        <v/>
+      </c>
+      <c r="K20" s="35" t="inlineStr">
         <is>
           <t>Lien paie</t>
         </is>
@@ -16749,8 +17356,16 @@
         <f>IF(G20=0,"paie absente",G19-G20)</f>
         <v/>
       </c>
-      <c r="H21" s="27" t="n"/>
-      <c r="I21" s="35" t="inlineStr">
+      <c r="H21" s="30">
+        <f>IF(H20=0,"paie absente",H19-H20)</f>
+        <v/>
+      </c>
+      <c r="I21" s="30">
+        <f>IF(I20=0,"paie absente",I19-I20)</f>
+        <v/>
+      </c>
+      <c r="J21" s="27" t="n"/>
+      <c r="K21" s="35" t="inlineStr">
         <is>
           <t>Négatif = IRG retenu non reversé</t>
         </is>
@@ -16759,40 +17374,48 @@
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>IRG retenu en paie TPM (non repris sur ces G50)</t>
+          <t>IRG retenu en paie TPM (déclaré sur G50 TPM, voir onglet G50 TPM)</t>
         </is>
       </c>
       <c r="B22" s="6">
+        <f>'Paie TPM'!C25</f>
+        <v/>
+      </c>
+      <c r="C22" s="6">
+        <f>'Paie TPM'!D25</f>
+        <v/>
+      </c>
+      <c r="D22" s="6">
         <f>'Paie TPM'!E25</f>
         <v/>
       </c>
-      <c r="C22" s="6">
+      <c r="E22" s="6">
         <f>'Paie TPM'!F25</f>
         <v/>
       </c>
-      <c r="D22" s="6">
+      <c r="F22" s="6">
         <f>'Paie TPM'!G25</f>
         <v/>
       </c>
-      <c r="E22" s="6">
+      <c r="G22" s="6">
         <f>'Paie TPM'!H25</f>
         <v/>
       </c>
-      <c r="F22" s="6">
+      <c r="H22" s="6">
         <f>'Paie TPM'!I25</f>
         <v/>
       </c>
-      <c r="G22" s="6">
+      <c r="I22" s="6">
         <f>'Paie TPM'!J25</f>
         <v/>
       </c>
-      <c r="H22" s="7">
-        <f>SUM(B22:G22)</f>
-        <v/>
-      </c>
-      <c r="I22" s="35" t="inlineStr">
-        <is>
-          <t>À déclarer sur une G50 TPM (non fournie)</t>
+      <c r="J22" s="7">
+        <f>SUM(B22:I22)</f>
+        <v/>
+      </c>
+      <c r="K22" s="35" t="inlineStr">
+        <is>
+          <t>G50 TPM fournies : juillet et août seulement</t>
         </is>
       </c>
     </row>
@@ -16803,28 +17426,34 @@
         </is>
       </c>
       <c r="B23" s="25" t="n">
+        <v>1526130</v>
+      </c>
+      <c r="C23" s="25" t="n">
+        <v>6372000</v>
+      </c>
+      <c r="D23" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="C23" s="25" t="n">
+      <c r="E23" s="25" t="n">
         <v>177058</v>
       </c>
-      <c r="D23" s="25" t="n">
+      <c r="F23" s="25" t="n">
         <v>177058</v>
-      </c>
-      <c r="E23" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" s="25" t="n">
-        <v>0</v>
       </c>
       <c r="G23" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H23" s="7">
-        <f>SUM(B23:G23)</f>
-        <v/>
-      </c>
-      <c r="I23" s="35" t="inlineStr"/>
+      <c r="H23" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" s="7">
+        <f>SUM(B23:I23)</f>
+        <v/>
+      </c>
+      <c r="K23" s="35" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
@@ -16833,30 +17462,36 @@
         </is>
       </c>
       <c r="B24" s="25" t="n">
+        <v>30525</v>
+      </c>
+      <c r="C24" s="25" t="n">
+        <v>63720</v>
+      </c>
+      <c r="D24" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="C24" s="25" t="n">
+      <c r="E24" s="25" t="n">
         <v>8944</v>
       </c>
-      <c r="D24" s="25" t="n">
+      <c r="F24" s="25" t="n">
         <v>3173</v>
-      </c>
-      <c r="E24" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" s="25" t="n">
-        <v>0</v>
       </c>
       <c r="G24" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="H24" s="7">
-        <f>SUM(B24:G24)</f>
-        <v/>
-      </c>
-      <c r="I24" s="35" t="inlineStr">
-        <is>
-          <t>Même base, montants différents : à justifier</t>
+      <c r="H24" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="7">
+        <f>SUM(B24:I24)</f>
+        <v/>
+      </c>
+      <c r="K24" s="35" t="inlineStr">
+        <is>
+          <t>Taux apparents incohérents (ligne 31)</t>
         </is>
       </c>
     </row>
@@ -16870,7 +17505,7 @@
         <v>0</v>
       </c>
       <c r="C25" s="25" t="n">
-        <v>0</v>
+        <v>8782828</v>
       </c>
       <c r="D25" s="25" t="n">
         <v>0</v>
@@ -16882,13 +17517,19 @@
         <v>0</v>
       </c>
       <c r="G25" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" s="25" t="n">
         <v>4409079</v>
       </c>
-      <c r="H25" s="7">
-        <f>SUM(B25:G25)</f>
-        <v/>
-      </c>
-      <c r="I25" s="35" t="inlineStr"/>
+      <c r="J25" s="7">
+        <f>SUM(B25:I25)</f>
+        <v/>
+      </c>
+      <c r="K25" s="35" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
@@ -16900,7 +17541,7 @@
         <v>0</v>
       </c>
       <c r="C26" s="25" t="n">
-        <v>0</v>
+        <v>87828</v>
       </c>
       <c r="D26" s="25" t="n">
         <v>0</v>
@@ -16912,15 +17553,21 @@
         <v>0</v>
       </c>
       <c r="G26" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" s="25" t="n">
         <v>44091</v>
       </c>
-      <c r="H26" s="7">
-        <f>SUM(B26:G26)</f>
-        <v/>
-      </c>
-      <c r="I26" s="35" t="inlineStr">
-        <is>
-          <t>1 % ; base à justifier</t>
+      <c r="J26" s="7">
+        <f>SUM(B26:I26)</f>
+        <v/>
+      </c>
+      <c r="K26" s="35" t="inlineStr">
+        <is>
+          <t>1 % ; payée en février ET en août : bases à justifier</t>
         </is>
       </c>
     </row>
@@ -16931,28 +17578,34 @@
         </is>
       </c>
       <c r="B27" s="25" t="n">
+        <v>1291220</v>
+      </c>
+      <c r="C27" s="25" t="n">
+        <v>3392786</v>
+      </c>
+      <c r="D27" s="25" t="n">
         <v>715520</v>
       </c>
-      <c r="C27" s="25" t="n">
+      <c r="E27" s="25" t="n">
         <v>719735</v>
       </c>
-      <c r="D27" s="25" t="n">
+      <c r="F27" s="25" t="n">
         <v>82311</v>
       </c>
-      <c r="E27" s="25" t="n">
+      <c r="G27" s="25" t="n">
         <v>59018</v>
       </c>
-      <c r="F27" s="25" t="n">
+      <c r="H27" s="25" t="n">
         <v>1309043</v>
       </c>
-      <c r="G27" s="25" t="n">
+      <c r="I27" s="25" t="n">
         <v>932361</v>
       </c>
-      <c r="H27" s="7">
-        <f>SUM(B27:G27)</f>
-        <v/>
-      </c>
-      <c r="I27" s="35" t="inlineStr"/>
+      <c r="J27" s="7">
+        <f>SUM(B27:I27)</f>
+        <v/>
+      </c>
+      <c r="K27" s="35" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -16984,11 +17637,19 @@
         <f>G14+G19+G24+G26</f>
         <v/>
       </c>
-      <c r="H28" s="7">
-        <f>SUM(B28:G28)</f>
-        <v/>
-      </c>
-      <c r="I28" s="35" t="inlineStr">
+      <c r="H28" s="30">
+        <f>H14+H19+H24+H26</f>
+        <v/>
+      </c>
+      <c r="I28" s="30">
+        <f>I14+I19+I24+I26</f>
+        <v/>
+      </c>
+      <c r="J28" s="7">
+        <f>SUM(B28:I28)</f>
+        <v/>
+      </c>
+      <c r="K28" s="35" t="inlineStr">
         <is>
           <t>Calcul</t>
         </is>
@@ -17024,11 +17685,19 @@
         <f>G27-G28</f>
         <v/>
       </c>
-      <c r="H29" s="7">
-        <f>SUM(B29:G29)</f>
-        <v/>
-      </c>
-      <c r="I29" s="35" t="inlineStr">
+      <c r="H29" s="30">
+        <f>H27-H28</f>
+        <v/>
+      </c>
+      <c r="I29" s="30">
+        <f>I27-I28</f>
+        <v/>
+      </c>
+      <c r="J29" s="7">
+        <f>SUM(B29:I29)</f>
+        <v/>
+      </c>
+      <c r="K29" s="35" t="inlineStr">
         <is>
           <t>Doit être 0</t>
         </is>
@@ -17042,38 +17711,92 @@
       </c>
       <c r="B30" s="22" t="inlineStr">
         <is>
+          <t>18/02/2022</t>
+        </is>
+      </c>
+      <c r="C30" s="22" t="inlineStr">
+        <is>
+          <t>19/03/2022</t>
+        </is>
+      </c>
+      <c r="D30" s="22" t="inlineStr">
+        <is>
           <t>17/04/2021</t>
         </is>
       </c>
-      <c r="C30" s="22" t="inlineStr">
+      <c r="E30" s="22" t="inlineStr">
         <is>
           <t>18/05/2022</t>
         </is>
       </c>
-      <c r="D30" s="22" t="inlineStr">
+      <c r="F30" s="22" t="inlineStr">
         <is>
           <t>18/06/2022</t>
         </is>
       </c>
-      <c r="E30" s="22" t="inlineStr">
+      <c r="G30" s="22" t="inlineStr">
         <is>
           <t>28/07/2022</t>
         </is>
       </c>
-      <c r="F30" s="22" t="inlineStr">
+      <c r="H30" s="22" t="inlineStr">
         <is>
           <t>19/08/2022</t>
         </is>
       </c>
-      <c r="G30" s="22" t="inlineStr">
+      <c r="I30" s="22" t="inlineStr">
         <is>
           <t>19/08/2022</t>
         </is>
       </c>
-      <c r="H30" s="27" t="n"/>
-      <c r="I30" s="35" t="inlineStr">
+      <c r="J30" s="27" t="n"/>
+      <c r="K30" s="35" t="inlineStr">
         <is>
           <t>Dates obsolètes : modèle non mis à jour</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>Taux apparent du droit de timbre (montant / base)</t>
+        </is>
+      </c>
+      <c r="B31" s="36">
+        <f>IF(B23=0,"",B24/B23)</f>
+        <v/>
+      </c>
+      <c r="C31" s="36">
+        <f>IF(C23=0,"",C24/C23)</f>
+        <v/>
+      </c>
+      <c r="D31" s="36">
+        <f>IF(D23=0,"",D24/D23)</f>
+        <v/>
+      </c>
+      <c r="E31" s="36">
+        <f>IF(E23=0,"",E24/E23)</f>
+        <v/>
+      </c>
+      <c r="F31" s="36">
+        <f>IF(F23=0,"",F24/F23)</f>
+        <v/>
+      </c>
+      <c r="G31" s="36">
+        <f>IF(G23=0,"",G24/G23)</f>
+        <v/>
+      </c>
+      <c r="H31" s="36">
+        <f>IF(H23=0,"",H24/H23)</f>
+        <v/>
+      </c>
+      <c r="I31" s="36">
+        <f>IF(I23=0,"",I24/I23)</f>
+        <v/>
+      </c>
+      <c r="K31" s="21" t="inlineStr">
+        <is>
+          <t>Taux appliqués différents d'un mois à l'autre</t>
         </is>
       </c>
     </row>
@@ -17101,7 +17824,9 @@
       <c r="F34" s="11" t="inlineStr"/>
       <c r="G34" s="11" t="inlineStr"/>
       <c r="H34" s="11" t="inlineStr"/>
-      <c r="I34" s="11" t="inlineStr">
+      <c r="I34" s="11" t="inlineStr"/>
+      <c r="J34" s="11" t="inlineStr"/>
+      <c r="K34" s="11" t="inlineStr">
         <is>
           <t>Commentaire</t>
         </is>
@@ -17116,7 +17841,7 @@
       <c r="B35" s="25" t="n">
         <v>27006870</v>
       </c>
-      <c r="I35" s="35" t="inlineStr">
+      <c r="K35" s="35" t="inlineStr">
         <is>
           <t>Annotation G50 mars et avril</t>
         </is>
@@ -17131,7 +17856,7 @@
       <c r="B36" s="25" t="n">
         <v>5131305</v>
       </c>
-      <c r="I36" s="35" t="inlineStr"/>
+      <c r="K36" s="35" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="29" t="inlineStr">
@@ -17143,7 +17868,7 @@
         <f>ROUND(B35*$B$4,0)</f>
         <v/>
       </c>
-      <c r="I37" s="35" t="inlineStr">
+      <c r="K37" s="35" t="inlineStr">
         <is>
           <t>Contrôle</t>
         </is>
@@ -17156,10 +17881,10 @@
         </is>
       </c>
       <c r="B38" s="30">
-        <f>B7</f>
-        <v/>
-      </c>
-      <c r="I38" s="35" t="inlineStr">
+        <f>D7</f>
+        <v/>
+      </c>
+      <c r="K38" s="35" t="inlineStr">
         <is>
           <t>G50 mars</t>
         </is>
@@ -17171,11 +17896,11 @@
           <t>CA de mars reporté sur les mois suivants</t>
         </is>
       </c>
-      <c r="B39" s="36">
+      <c r="B39" s="37">
         <f>B35-B38</f>
         <v/>
       </c>
-      <c r="I39" s="35" t="inlineStr">
+      <c r="K39" s="35" t="inlineStr">
         <is>
           <t>Annoté « RESTE A DECLARER CA » 23 561 670</t>
         </is>
@@ -17187,11 +17912,11 @@
           <t>TVA de mars payée en retard</t>
         </is>
       </c>
-      <c r="B40" s="36">
+      <c r="B40" s="37">
         <f>ROUND(B39*$B$4,0)</f>
         <v/>
       </c>
-      <c r="I40" s="35" t="inlineStr">
+      <c r="K40" s="35" t="inlineStr">
         <is>
           <t>Annoté « RESTE A DECLARER TVA » 4 476 717</t>
         </is>
@@ -17206,7 +17931,7 @@
       <c r="B41" s="25" t="n">
         <v>13157894.74</v>
       </c>
-      <c r="I41" s="35" t="inlineStr">
+      <c r="K41" s="35" t="inlineStr">
         <is>
           <t>Soit 2 500 000 / 19 % : CA calculé à partir d'un objectif de TVA</t>
         </is>
@@ -17222,7 +17947,7 @@
         <f>ROUND(B41*$B$4,2)</f>
         <v/>
       </c>
-      <c r="I42" s="35" t="inlineStr">
+      <c r="K42" s="35" t="inlineStr">
         <is>
           <t>Contrôle</t>
         </is>
@@ -17237,7 +17962,7 @@
       <c r="B43" s="25" t="n">
         <v>5417538</v>
       </c>
-      <c r="I43" s="35" t="inlineStr">
+      <c r="K43" s="35" t="inlineStr">
         <is>
           <t>Montant restant selon le suivi interne</t>
         </is>
@@ -17258,40 +17983,50 @@
       </c>
       <c r="B46" s="11" t="inlineStr">
         <is>
+          <t>Janv</t>
+        </is>
+      </c>
+      <c r="C46" s="11" t="inlineStr">
+        <is>
+          <t>Févr</t>
+        </is>
+      </c>
+      <c r="D46" s="11" t="inlineStr">
+        <is>
           <t>Mars</t>
         </is>
       </c>
-      <c r="C46" s="11" t="inlineStr">
+      <c r="E46" s="11" t="inlineStr">
         <is>
           <t>Avr</t>
         </is>
       </c>
-      <c r="D46" s="11" t="inlineStr">
+      <c r="F46" s="11" t="inlineStr">
         <is>
           <t>Mai</t>
         </is>
       </c>
-      <c r="E46" s="11" t="inlineStr">
+      <c r="G46" s="11" t="inlineStr">
         <is>
           <t>Juin</t>
         </is>
       </c>
-      <c r="F46" s="11" t="inlineStr">
+      <c r="H46" s="11" t="inlineStr">
         <is>
           <t>Juil</t>
         </is>
       </c>
-      <c r="G46" s="11" t="inlineStr">
+      <c r="I46" s="11" t="inlineStr">
         <is>
           <t>Août</t>
         </is>
       </c>
-      <c r="H46" s="11" t="inlineStr">
+      <c r="J46" s="11" t="inlineStr">
         <is>
           <t>Cumul</t>
         </is>
       </c>
-      <c r="I46" s="11" t="inlineStr">
+      <c r="K46" s="11" t="inlineStr">
         <is>
           <t>Commentaire</t>
         </is>
@@ -17304,25 +18039,31 @@
         </is>
       </c>
       <c r="B47" s="25" t="n">
+        <v>17864580</v>
+      </c>
+      <c r="C47" s="25" t="n">
+        <v>25568207</v>
+      </c>
+      <c r="D47" s="25" t="n">
         <v>31947529</v>
       </c>
-      <c r="C47" s="25" t="n">
+      <c r="E47" s="25" t="n">
         <v>29534571</v>
       </c>
-      <c r="D47" s="25" t="n">
+      <c r="F47" s="25" t="n">
         <v>41310810</v>
       </c>
-      <c r="E47" s="25" t="n">
+      <c r="G47" s="25" t="n">
         <v>28042831</v>
       </c>
-      <c r="F47" s="25" t="n">
+      <c r="H47" s="25" t="n">
         <v>23178604</v>
       </c>
-      <c r="G47" s="25" t="n">
+      <c r="I47" s="25" t="n">
         <v>15524844</v>
       </c>
-      <c r="H47" s="7">
-        <f>SUM(B47:G47)</f>
+      <c r="J47" s="7">
+        <f>SUM(B47:I47)</f>
         <v/>
       </c>
     </row>
@@ -17356,11 +18097,19 @@
         <f>G7</f>
         <v/>
       </c>
-      <c r="H48" s="7">
-        <f>SUM(B48:G48)</f>
-        <v/>
-      </c>
-      <c r="I48" s="35" t="inlineStr">
+      <c r="H48" s="30">
+        <f>H7</f>
+        <v/>
+      </c>
+      <c r="I48" s="30">
+        <f>I7</f>
+        <v/>
+      </c>
+      <c r="J48" s="7">
+        <f>SUM(B48:I48)</f>
+        <v/>
+      </c>
+      <c r="K48" s="35" t="inlineStr">
         <is>
           <t>Le CA 2026 déclaré mois par mois ne reflète pas le CA réalisé (voir annotations) : rapprocher avec le journal des ventes 2026.</t>
         </is>
@@ -17396,8 +18145,16 @@
         <f>IF(G47=0,"",G48/G47-1)</f>
         <v/>
       </c>
-      <c r="H49" s="37">
-        <f>H48/H47-1</f>
+      <c r="H49" s="19">
+        <f>IF(H47=0,"",H48/H47-1)</f>
+        <v/>
+      </c>
+      <c r="I49" s="19">
+        <f>IF(I47=0,"",I48/I47-1)</f>
+        <v/>
+      </c>
+      <c r="J49" s="38">
+        <f>J48/J47-1</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Dossier comptable : G50 TPM avril-juin 2026 et contrôle du journal 2023
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XYis4EzVZMNdoYCxmLrRh4
</commit_message>
<xml_diff>
--- a/DOSSIER_COMPTABLE_SARL_DPR_COMPAGNY_2026.xlsx
+++ b/DOSSIER_COMPTABLE_SARL_DPR_COMPAGNY_2026.xlsx
@@ -19,13 +19,14 @@
     <sheet name="Balance 2024-2025" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="États 2024-2025" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="G50 TPM 2026" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Anomalies &amp; actions" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Pièces" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Contrôle 2023" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Anomalies &amp; actions" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Pièces" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Journal paie'!$A$4:$G$140</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Balance 2024-2025'!$A$4:$E$104</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Anomalies &amp; actions'!$A$4:$I$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Anomalies &amp; actions'!$A$4:$I$36</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -203,7 +204,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -249,6 +250,7 @@
     <xf numFmtId="10" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -678,7 +680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D60"/>
+  <dimension ref="A1:D61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -985,11 +987,11 @@
         </is>
       </c>
       <c r="B24" s="13">
-        <f>COUNTIF('Anomalies &amp; actions'!B5:B35,1)</f>
+        <f>COUNTIF('Anomalies &amp; actions'!B5:B36,1)</f>
         <v/>
       </c>
       <c r="C24" s="13">
-        <f>COUNTIFS('Anomalies &amp; actions'!B5:B35,1,'Anomalies &amp; actions'!I5:I35,"Ouvert")</f>
+        <f>COUNTIFS('Anomalies &amp; actions'!B5:B36,1,'Anomalies &amp; actions'!I5:I36,"Ouvert")</f>
         <v/>
       </c>
     </row>
@@ -1000,11 +1002,11 @@
         </is>
       </c>
       <c r="B25" s="13">
-        <f>COUNTIF('Anomalies &amp; actions'!B5:B35,2)</f>
+        <f>COUNTIF('Anomalies &amp; actions'!B5:B36,2)</f>
         <v/>
       </c>
       <c r="C25" s="13">
-        <f>COUNTIFS('Anomalies &amp; actions'!B5:B35,2,'Anomalies &amp; actions'!I5:I35,"Ouvert")</f>
+        <f>COUNTIFS('Anomalies &amp; actions'!B5:B36,2,'Anomalies &amp; actions'!I5:I36,"Ouvert")</f>
         <v/>
       </c>
     </row>
@@ -1015,11 +1017,11 @@
         </is>
       </c>
       <c r="B26" s="13">
-        <f>COUNTIF('Anomalies &amp; actions'!B5:B35,3)</f>
+        <f>COUNTIF('Anomalies &amp; actions'!B5:B36,3)</f>
         <v/>
       </c>
       <c r="C26" s="13">
-        <f>COUNTIFS('Anomalies &amp; actions'!B5:B35,3,'Anomalies &amp; actions'!I5:I35,"Ouvert")</f>
+        <f>COUNTIFS('Anomalies &amp; actions'!B5:B36,3,'Anomalies &amp; actions'!I5:I36,"Ouvert")</f>
         <v/>
       </c>
     </row>
@@ -1122,11 +1124,11 @@
     <row r="37">
       <c r="A37" s="12" t="inlineStr">
         <is>
-          <t>G50 TPM juil.–août : totaux</t>
+          <t>G50 TPM avr.–août : totaux</t>
         </is>
       </c>
       <c r="B37" s="4">
-        <f>IF(AND(ABS('G50 TPM 2026'!B21)&lt;1,ABS('G50 TPM 2026'!C21)&lt;1),"OK","ÉCART")</f>
+        <f>IF(ABS('G50 TPM 2026'!G20)&lt;1,"OK","ÉCART")</f>
         <v/>
       </c>
     </row>
@@ -1282,7 +1284,7 @@
       </c>
       <c r="B49" s="12" t="inlineStr">
         <is>
-          <t>Contrôle des G50 TPM et location (juil., août)</t>
+          <t>Contrôle des G50 TPM et location (avr.–août)</t>
         </is>
       </c>
       <c r="C49" s="17" t="n"/>
@@ -1291,12 +1293,12 @@
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>Balance 2024-2025</t>
+          <t>Contrôle 2023</t>
         </is>
       </c>
       <c r="B50" s="12" t="inlineStr">
         <is>
-          <t>Balance générale issue des journaux PCCOMPTA</t>
+          <t>Journal 2023 vs à-nouveaux 2024 ; historique TVA TPM</t>
         </is>
       </c>
       <c r="C50" s="17" t="n"/>
@@ -1305,84 +1307,79 @@
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>États 2024-2025</t>
+          <t>Balance 2024-2025</t>
         </is>
       </c>
       <c r="B51" s="12" t="inlineStr">
         <is>
-          <t>Compte de résultat et bilan simplifiés, indicateurs</t>
+          <t>Balance générale issue des journaux PCCOMPTA</t>
         </is>
       </c>
       <c r="C51" s="17" t="n"/>
       <c r="D51" s="18" t="n"/>
     </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>États 2024-2025</t>
+        </is>
+      </c>
+      <c r="B52" s="12" t="inlineStr">
+        <is>
+          <t>Compte de résultat et bilan simplifiés, indicateurs</t>
+        </is>
+      </c>
+      <c r="C52" s="17" t="n"/>
+      <c r="D52" s="18" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
         <is>
           <t>Légende : bleu = saisie depuis une pièce ; vert = lien vers une autre feuille ; noir = calcul ; fond jaune = à compléter.</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="10" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="10" t="inlineStr">
         <is>
           <t>Exercices comptables</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="11" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="11" t="inlineStr">
         <is>
           <t>Indicateur</t>
         </is>
       </c>
-      <c r="B57" s="11" t="inlineStr">
+      <c r="B58" s="11" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="C57" s="11" t="inlineStr">
+      <c r="C58" s="11" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D57" s="11" t="inlineStr">
+      <c r="D58" s="11" t="inlineStr">
         <is>
           <t>Variation</t>
         </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="4" t="inlineStr">
-        <is>
-          <t>Chiffre d'affaires</t>
-        </is>
-      </c>
-      <c r="B58" s="6">
-        <f>'États 2024-2025'!C5</f>
-        <v/>
-      </c>
-      <c r="C58" s="6">
-        <f>'États 2024-2025'!D5</f>
-        <v/>
-      </c>
-      <c r="D58" s="19">
-        <f>IF(B58=0,"",C58/B58-1)</f>
-        <v/>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>Charges de personnel</t>
+          <t>Chiffre d'affaires</t>
         </is>
       </c>
       <c r="B59" s="6">
-        <f>'États 2024-2025'!C10</f>
+        <f>'États 2024-2025'!C5</f>
         <v/>
       </c>
       <c r="C59" s="6">
-        <f>'États 2024-2025'!D10</f>
+        <f>'États 2024-2025'!D5</f>
         <v/>
       </c>
       <c r="D59" s="19">
@@ -1393,15 +1390,15 @@
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>Résultat net</t>
+          <t>Charges de personnel</t>
         </is>
       </c>
       <c r="B60" s="6">
-        <f>'États 2024-2025'!C16</f>
+        <f>'États 2024-2025'!C10</f>
         <v/>
       </c>
       <c r="C60" s="6">
-        <f>'États 2024-2025'!D16</f>
+        <f>'États 2024-2025'!D10</f>
         <v/>
       </c>
       <c r="D60" s="19">
@@ -1409,8 +1406,27 @@
         <v/>
       </c>
     </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>Résultat net</t>
+        </is>
+      </c>
+      <c r="B61" s="6">
+        <f>'États 2024-2025'!C16</f>
+        <v/>
+      </c>
+      <c r="C61" s="6">
+        <f>'États 2024-2025'!D16</f>
+        <v/>
+      </c>
+      <c r="D61" s="19">
+        <f>IF(B61=0,"",C61/B61-1)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="13">
     <mergeCell ref="B42:D42"/>
     <mergeCell ref="B45:D45"/>
     <mergeCell ref="B46:D46"/>
@@ -1418,6 +1434,7 @@
     <mergeCell ref="B49:D49"/>
     <mergeCell ref="B50:D50"/>
     <mergeCell ref="B40:D40"/>
+    <mergeCell ref="B52:D52"/>
     <mergeCell ref="B44:D44"/>
     <mergeCell ref="B43:D43"/>
     <mergeCell ref="B51:D51"/>
@@ -4665,13 +4682,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="54" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4684,7 +4705,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Sources : G50_07-2026_TPM_ET_LOCATION_CONSOLIDE_-.xls et G50_08-2026_TPM_ET_LOCATION_CONSOLIDE.xls. Activité portée : transport et distribution de toutes marchandises.</t>
+          <t>Sources : G50_04 à 08-2026_TPM_ET_LOCATION_CONSOLIDE.xls. Activité portée : transport et distribution de toutes marchandises.</t>
         </is>
       </c>
     </row>
@@ -4696,15 +4717,35 @@
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
+          <t>Avril 2026</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>Mai 2026</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>Juin 2026</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
           <t>Juillet 2026</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="F4" s="11" t="inlineStr">
         <is>
           <t>Août 2026</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>Cumul</t>
+        </is>
+      </c>
+      <c r="H4" s="11" t="inlineStr">
         <is>
           <t>Commentaire</t>
         </is>
@@ -4723,12 +4764,28 @@
       </c>
       <c r="C5" s="22" t="inlineStr">
         <is>
+          <t>AVRIL</t>
+        </is>
+      </c>
+      <c r="D5" s="22" t="inlineStr">
+        <is>
+          <t>AVRIL</t>
+        </is>
+      </c>
+      <c r="E5" s="22" t="inlineStr">
+        <is>
+          <t>AVRIL</t>
+        </is>
+      </c>
+      <c r="F5" s="22" t="inlineStr">
+        <is>
           <t>AOUT</t>
         </is>
       </c>
-      <c r="D5" s="35" t="inlineStr">
-        <is>
-          <t>Fichier « 07-2026 » mais mois imprimé « AVRIL »</t>
+      <c r="G5" s="27" t="n"/>
+      <c r="H5" s="35" t="inlineStr">
+        <is>
+          <t>Avril à juillet : même G50 recopiée (mois « AVRIL »)</t>
         </is>
       </c>
     </row>
@@ -4744,7 +4801,20 @@
       <c r="C6" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="D6" s="35" t="inlineStr">
+      <c r="D6" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="7">
+        <f>SUM(B6:F6)</f>
+        <v/>
+      </c>
+      <c r="H6" s="35" t="inlineStr">
         <is>
           <t>Aucun CA TPM / location déclaré</t>
         </is>
@@ -4762,7 +4832,20 @@
       <c r="C7" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="D7" s="35" t="inlineStr"/>
+      <c r="D7" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="7">
+        <f>SUM(B7:F7)</f>
+        <v/>
+      </c>
+      <c r="H7" s="35" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
@@ -4776,7 +4859,17 @@
       <c r="C8" s="25" t="n">
         <v>1714499</v>
       </c>
-      <c r="D8" s="35" t="inlineStr"/>
+      <c r="D8" s="25" t="n">
+        <v>1714499</v>
+      </c>
+      <c r="E8" s="25" t="n">
+        <v>1714499</v>
+      </c>
+      <c r="F8" s="25" t="n">
+        <v>1714499</v>
+      </c>
+      <c r="G8" s="27" t="n"/>
+      <c r="H8" s="35" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -4790,7 +4883,17 @@
       <c r="C9" s="25" t="n">
         <v>1714499</v>
       </c>
-      <c r="D9" s="35" t="inlineStr"/>
+      <c r="D9" s="25" t="n">
+        <v>1714499</v>
+      </c>
+      <c r="E9" s="25" t="n">
+        <v>1714499</v>
+      </c>
+      <c r="F9" s="25" t="n">
+        <v>1714499</v>
+      </c>
+      <c r="G9" s="27" t="n"/>
+      <c r="H9" s="35" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
@@ -4806,7 +4909,20 @@
         <f>'Balance 2024-2025'!D49</f>
         <v/>
       </c>
-      <c r="D10" s="35" t="inlineStr">
+      <c r="D10" s="6">
+        <f>'Balance 2024-2025'!D49</f>
+        <v/>
+      </c>
+      <c r="E10" s="6">
+        <f>'Balance 2024-2025'!D49</f>
+        <v/>
+      </c>
+      <c r="F10" s="6">
+        <f>'Balance 2024-2025'!D49</f>
+        <v/>
+      </c>
+      <c r="G10" s="27" t="n"/>
+      <c r="H10" s="35" t="inlineStr">
         <is>
           <t>Identique : crédit reporté depuis 2025</t>
         </is>
@@ -4822,9 +4938,22 @@
         <v>91763</v>
       </c>
       <c r="C11" s="25" t="n">
+        <v>91763</v>
+      </c>
+      <c r="D11" s="25" t="n">
+        <v>91763</v>
+      </c>
+      <c r="E11" s="25" t="n">
+        <v>91763</v>
+      </c>
+      <c r="F11" s="25" t="n">
         <v>42190</v>
       </c>
-      <c r="D11" s="35" t="inlineStr"/>
+      <c r="G11" s="7">
+        <f>SUM(B11:F11)</f>
+        <v/>
+      </c>
+      <c r="H11" s="35" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
@@ -4833,14 +4962,30 @@
         </is>
       </c>
       <c r="B12" s="6">
+        <f>'Paie TPM'!F24</f>
+        <v/>
+      </c>
+      <c r="C12" s="6">
+        <f>'Paie TPM'!G24</f>
+        <v/>
+      </c>
+      <c r="D12" s="6">
+        <f>'Paie TPM'!H24</f>
+        <v/>
+      </c>
+      <c r="E12" s="6">
         <f>'Paie TPM'!I24</f>
         <v/>
       </c>
-      <c r="C12" s="6">
+      <c r="F12" s="6">
         <f>'Paie TPM'!J24</f>
         <v/>
       </c>
-      <c r="D12" s="35" t="inlineStr">
+      <c r="G12" s="7">
+        <f>SUM(B12:F12)</f>
+        <v/>
+      </c>
+      <c r="H12" s="35" t="inlineStr">
         <is>
           <t>Lien paie</t>
         </is>
@@ -4856,9 +5001,22 @@
         <v>9375</v>
       </c>
       <c r="C13" s="25" t="n">
+        <v>9375</v>
+      </c>
+      <c r="D13" s="25" t="n">
+        <v>9375</v>
+      </c>
+      <c r="E13" s="25" t="n">
+        <v>9375</v>
+      </c>
+      <c r="F13" s="25" t="n">
         <v>3690</v>
       </c>
-      <c r="D13" s="35" t="inlineStr"/>
+      <c r="G13" s="7">
+        <f>SUM(B13:F13)</f>
+        <v/>
+      </c>
+      <c r="H13" s="35" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
@@ -4867,14 +5025,30 @@
         </is>
       </c>
       <c r="B14" s="6">
+        <f>'Paie TPM'!F25</f>
+        <v/>
+      </c>
+      <c r="C14" s="6">
+        <f>'Paie TPM'!G25</f>
+        <v/>
+      </c>
+      <c r="D14" s="6">
+        <f>'Paie TPM'!H25</f>
+        <v/>
+      </c>
+      <c r="E14" s="6">
         <f>'Paie TPM'!I25</f>
         <v/>
       </c>
-      <c r="C14" s="6">
+      <c r="F14" s="6">
         <f>'Paie TPM'!J25</f>
         <v/>
       </c>
-      <c r="D14" s="35" t="inlineStr">
+      <c r="G14" s="7">
+        <f>SUM(B14:F14)</f>
+        <v/>
+      </c>
+      <c r="H14" s="35" t="inlineStr">
         <is>
           <t>Lien paie</t>
         </is>
@@ -4894,129 +5068,196 @@
         <f>C13-C14</f>
         <v/>
       </c>
-      <c r="D15" s="35" t="inlineStr">
-        <is>
-          <t>Juillet : la G50 reprend l'IRG d'avril/mai</t>
+      <c r="D15" s="30">
+        <f>D13-D14</f>
+        <v/>
+      </c>
+      <c r="E15" s="30">
+        <f>E13-E14</f>
+        <v/>
+      </c>
+      <c r="F15" s="30">
+        <f>F13-F14</f>
+        <v/>
+      </c>
+      <c r="G15" s="7">
+        <f>SUM(B15:F15)</f>
+        <v/>
+      </c>
+      <c r="H15" s="35" t="inlineStr">
+        <is>
+          <t>Négatif = IRG retenu non reversé</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t>Pour mémoire : IRG paie TPM avril / mai</t>
-        </is>
-      </c>
-      <c r="B16" s="6">
-        <f>'Paie TPM'!F25</f>
-        <v/>
-      </c>
-      <c r="C16" s="6">
-        <f>'Paie TPM'!G25</f>
-        <v/>
-      </c>
-      <c r="D16" s="35" t="inlineStr">
-        <is>
-          <t>Lien paie</t>
+          <t>Taxe d'apprentissage — base</t>
+        </is>
+      </c>
+      <c r="B16" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="25" t="n">
+        <v>680900</v>
+      </c>
+      <c r="G16" s="7">
+        <f>SUM(B16:F16)</f>
+        <v/>
+      </c>
+      <c r="H16" s="35" t="inlineStr">
+        <is>
+          <t>Base à justifier</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>Taxe d'apprentissage — base</t>
+          <t>Taxe d'apprentissage — montant</t>
         </is>
       </c>
       <c r="B17" s="25" t="n">
         <v>0</v>
       </c>
       <c r="C17" s="25" t="n">
-        <v>680900</v>
-      </c>
-      <c r="D17" s="35" t="inlineStr">
-        <is>
-          <t>Base à justifier</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="D17" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="25" t="n">
+        <v>6809</v>
+      </c>
+      <c r="G17" s="7">
+        <f>SUM(B17:F17)</f>
+        <v/>
+      </c>
+      <c r="H17" s="35" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>Taxe d'apprentissage — montant</t>
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Total à payer déclaré</t>
         </is>
       </c>
       <c r="B18" s="25" t="n">
-        <v>0</v>
+        <v>9375</v>
       </c>
       <c r="C18" s="25" t="n">
-        <v>6809</v>
-      </c>
-      <c r="D18" s="35" t="inlineStr"/>
+        <v>9375</v>
+      </c>
+      <c r="D18" s="25" t="n">
+        <v>9375</v>
+      </c>
+      <c r="E18" s="25" t="n">
+        <v>9375</v>
+      </c>
+      <c r="F18" s="25" t="n">
+        <v>10499</v>
+      </c>
+      <c r="G18" s="7">
+        <f>SUM(B18:F18)</f>
+        <v/>
+      </c>
+      <c r="H18" s="35" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Total à payer déclaré</t>
-        </is>
-      </c>
-      <c r="B19" s="25" t="n">
-        <v>9375</v>
-      </c>
-      <c r="C19" s="25" t="n">
-        <v>10499</v>
-      </c>
-      <c r="D19" s="35" t="inlineStr"/>
+          <t>Total recalculé (TVA + IRG + TA)</t>
+        </is>
+      </c>
+      <c r="B19" s="30">
+        <f>MAX(0,B7-B8)+B13+B17</f>
+        <v/>
+      </c>
+      <c r="C19" s="30">
+        <f>MAX(0,C7-C8)+C13+C17</f>
+        <v/>
+      </c>
+      <c r="D19" s="30">
+        <f>MAX(0,D7-D8)+D13+D17</f>
+        <v/>
+      </c>
+      <c r="E19" s="30">
+        <f>MAX(0,E7-E8)+E13+E17</f>
+        <v/>
+      </c>
+      <c r="F19" s="30">
+        <f>MAX(0,F7-F8)+F13+F17</f>
+        <v/>
+      </c>
+      <c r="G19" s="7">
+        <f>SUM(B19:F19)</f>
+        <v/>
+      </c>
+      <c r="H19" s="35" t="inlineStr">
+        <is>
+          <t>Calcul</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Total recalculé (TVA + IRG + TA)</t>
+          <t>Écart total</t>
         </is>
       </c>
       <c r="B20" s="30">
-        <f>MAX(0,B7-B8)+B13+B18</f>
+        <f>B18-B19</f>
         <v/>
       </c>
       <c r="C20" s="30">
-        <f>MAX(0,C7-C8)+C13+C18</f>
-        <v/>
-      </c>
-      <c r="D20" s="35" t="inlineStr">
-        <is>
-          <t>Calcul</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>Écart total</t>
-        </is>
-      </c>
-      <c r="B21" s="30">
-        <f>B19-B20</f>
-        <v/>
-      </c>
-      <c r="C21" s="30">
-        <f>C19-C20</f>
-        <v/>
-      </c>
-      <c r="D21" s="35" t="inlineStr">
+        <f>C18-C19</f>
+        <v/>
+      </c>
+      <c r="D20" s="30">
+        <f>D18-D19</f>
+        <v/>
+      </c>
+      <c r="E20" s="30">
+        <f>E18-E19</f>
+        <v/>
+      </c>
+      <c r="F20" s="30">
+        <f>F18-F19</f>
+        <v/>
+      </c>
+      <c r="G20" s="7">
+        <f>SUM(B20:F20)</f>
+        <v/>
+      </c>
+      <c r="H20" s="35" t="inlineStr">
         <is>
           <t>Doit être 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Modèle G50 TPM : la feuille « Recap-TVA » porte encore la G50 de décembre 2025 (factures BOBOR PNEUS) et « Feuil1 » un extrait de journal 2019 ; à nettoyer avant dépôt.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Modèle G50 TPM : la feuille « Recap-TVA » porte encore la G50 de décembre 2025 (factures BOBOR PNEUS) et « Feuil1 » un extrait de journal 2019 ; à nettoyer avant dépôt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>G50 TPM de janvier à juin 2026 non fournies : IRG TPM retenu sur cette période à vérifier (voir anomalie A19).</t>
+          <t>G50 TPM de janvier à mars 2026 non fournies (IRG paie TPM sur la période : voir « Paie TPM »).</t>
         </is>
       </c>
     </row>
@@ -5032,7 +5273,1107 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:F56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Journal 2023 et historique de la TVA collectée TPM</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Source : DLG_COMPTAZ_SARL_DPR_COMPAGNY_2023.xls (3 365 lignes, équilibré) comparé aux à-nouveaux du journal 2024.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Résultat 2023 selon le journal 2023 fourni</t>
+        </is>
+      </c>
+      <c r="B4" s="25" t="n">
+        <v>18539102.4</v>
+      </c>
+      <c r="C4" s="21" t="inlineStr">
+        <is>
+          <t>Journal 2023 sans écriture d'IBS (69) ni d'inventaire complète ; décembre 2023 : 31 lignes seulement</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Résultat 2023 repris en à-nouveau 2024 (compte 12000)</t>
+        </is>
+      </c>
+      <c r="B5" s="25" t="n">
+        <v>7260903.16</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Écart</t>
+        </is>
+      </c>
+      <c r="B6" s="39">
+        <f>B4-B5</f>
+        <v/>
+      </c>
+      <c r="C6" s="21" t="inlineStr">
+        <is>
+          <t>Le fichier 2023 fourni est une version provisoire, antérieure aux écritures de clôture</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>Compte</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Libellé</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>Solde clôture 2023 (fichier)</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>À-nouveau 2024</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>Écart</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>12000</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>RESULTAT DE L'EXERCICE</t>
+        </is>
+      </c>
+      <c r="C9" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="25" t="n">
+        <v>-7260903.16</v>
+      </c>
+      <c r="E9" s="30">
+        <f>D9-C9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>21805</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>INSTAL GEN,AGENC,AMENAG DIVERS</t>
+        </is>
+      </c>
+      <c r="C10" s="25" t="n">
+        <v>8403329.18</v>
+      </c>
+      <c r="D10" s="25" t="n">
+        <v>9463661.109999999</v>
+      </c>
+      <c r="E10" s="30">
+        <f>D10-C10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>28150</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>AMORT MAT ET OUTILLAGES</t>
+        </is>
+      </c>
+      <c r="C11" s="25" t="n">
+        <v>-1249096.22</v>
+      </c>
+      <c r="D11" s="25" t="n">
+        <v>-1416000.43</v>
+      </c>
+      <c r="E11" s="30">
+        <f>D11-C11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>28185</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>AMORT INST GEN AGENC ET AMENAG</t>
+        </is>
+      </c>
+      <c r="C12" s="25" t="n">
+        <v>-3541844.12</v>
+      </c>
+      <c r="D12" s="25" t="n">
+        <v>-3612465.95</v>
+      </c>
+      <c r="E12" s="30">
+        <f>D12-C12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>30002</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>ST IMPORTATION</t>
+        </is>
+      </c>
+      <c r="C13" s="25" t="n">
+        <v>202015456.47</v>
+      </c>
+      <c r="D13" s="25" t="n">
+        <v>253727049.44</v>
+      </c>
+      <c r="E13" s="30">
+        <f>D13-C13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>32201</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>ST PIECES DE RECHANGE</t>
+        </is>
+      </c>
+      <c r="C14" s="25" t="n">
+        <v>3509934.64</v>
+      </c>
+      <c r="D14" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="30">
+        <f>D14-C14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>37000</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>STOCKS A L'EXTERIEUR</t>
+        </is>
+      </c>
+      <c r="C15" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="25" t="n">
+        <v>47936182.2</v>
+      </c>
+      <c r="E15" s="30">
+        <f>D15-C15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>38002</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>ACHATS IMPORTATION</t>
+        </is>
+      </c>
+      <c r="C16" s="25" t="n">
+        <v>17544780.31</v>
+      </c>
+      <c r="D16" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="30">
+        <f>D16-C16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>40100</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>Fournisseurs de stocks et serv</t>
+        </is>
+      </c>
+      <c r="C17" s="25" t="n">
+        <v>-30009104.62</v>
+      </c>
+      <c r="D17" s="25" t="n">
+        <v>-69749175.87</v>
+      </c>
+      <c r="E17" s="30">
+        <f>D17-C17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>40102</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>FOURNSSEURS ETRANGERS</t>
+        </is>
+      </c>
+      <c r="C18" s="25" t="n">
+        <v>-25535217.72</v>
+      </c>
+      <c r="D18" s="25" t="n">
+        <v>-57476811.5</v>
+      </c>
+      <c r="E18" s="30">
+        <f>D18-C18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>40130</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>FOUR. LOCAUX DE SERVICES</t>
+        </is>
+      </c>
+      <c r="C19" s="25" t="n">
+        <v>-2957587.75</v>
+      </c>
+      <c r="D19" s="25" t="n">
+        <v>-1726194.44</v>
+      </c>
+      <c r="E19" s="30">
+        <f>D19-C19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>40400</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>Fournisseurs d'immobilisations</t>
+        </is>
+      </c>
+      <c r="C20" s="25" t="n">
+        <v>-4045605</v>
+      </c>
+      <c r="D20" s="25" t="n">
+        <v>-5307400</v>
+      </c>
+      <c r="E20" s="30">
+        <f>D20-C20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>40800</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>FOURNIS FACTURES NON PARVENUES</t>
+        </is>
+      </c>
+      <c r="C21" s="25" t="n">
+        <v>-23580</v>
+      </c>
+      <c r="D21" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="30">
+        <f>D21-C21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>40900</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>Fournisseurs débiteurs : avanc</t>
+        </is>
+      </c>
+      <c r="C22" s="25" t="n">
+        <v>344533</v>
+      </c>
+      <c r="D22" s="25" t="n">
+        <v>1175567</v>
+      </c>
+      <c r="E22" s="30">
+        <f>D22-C22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>41100</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="C23" s="25" t="n">
+        <v>353909705.59</v>
+      </c>
+      <c r="D23" s="25" t="n">
+        <v>361308738.12</v>
+      </c>
+      <c r="E23" s="30">
+        <f>D23-C23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>41900</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>Clients créditeurs -avances re</t>
+        </is>
+      </c>
+      <c r="C24" s="25" t="n">
+        <v>-295064234.32</v>
+      </c>
+      <c r="D24" s="25" t="n">
+        <v>-303664234.32</v>
+      </c>
+      <c r="E24" s="30">
+        <f>D24-C24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>42100</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>PERSONNEL,REMUNERATIONS DUES</t>
+        </is>
+      </c>
+      <c r="C25" s="25" t="n">
+        <v>-2778976.78</v>
+      </c>
+      <c r="D25" s="25" t="n">
+        <v>-1061592.31</v>
+      </c>
+      <c r="E25" s="30">
+        <f>D25-C25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>43100</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>SECURITE SOCIALE</t>
+        </is>
+      </c>
+      <c r="C26" s="25" t="n">
+        <v>-247850.03</v>
+      </c>
+      <c r="D26" s="25" t="n">
+        <v>-223067.66</v>
+      </c>
+      <c r="E26" s="30">
+        <f>D26-C26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>43200</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>Autres organismes sociaux</t>
+        </is>
+      </c>
+      <c r="C27" s="25" t="n">
+        <v>-830851.87</v>
+      </c>
+      <c r="D27" s="25" t="n">
+        <v>-610922.03</v>
+      </c>
+      <c r="E27" s="30">
+        <f>D27-C27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>44210</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>RETENUES : IRG</t>
+        </is>
+      </c>
+      <c r="C28" s="25" t="n">
+        <v>-166632.72</v>
+      </c>
+      <c r="D28" s="25" t="n">
+        <v>-112633.4</v>
+      </c>
+      <c r="E28" s="30">
+        <f>D28-C28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>44400</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>Etat, impôts sur les résultats</t>
+        </is>
+      </c>
+      <c r="C29" s="25" t="n">
+        <v>-644330.96</v>
+      </c>
+      <c r="D29" s="25" t="n">
+        <v>-2616744</v>
+      </c>
+      <c r="E29" s="30">
+        <f>D29-C29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>44410</t>
+        </is>
+      </c>
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>AVANCES ET ACOMPTES SUR IBS</t>
+        </is>
+      </c>
+      <c r="C30" s="25" t="n">
+        <v>5120187</v>
+      </c>
+      <c r="D30" s="25" t="n">
+        <v>2921073</v>
+      </c>
+      <c r="E30" s="30">
+        <f>D30-C30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>44430</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>EXCEDENT DE VERSEMENT IMPOTS</t>
+        </is>
+      </c>
+      <c r="C31" s="25" t="n">
+        <v>970465</v>
+      </c>
+      <c r="D31" s="25" t="n">
+        <v>2668106</v>
+      </c>
+      <c r="E31" s="30">
+        <f>D31-C31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t>44510</t>
+        </is>
+      </c>
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>TVA A PAYER</t>
+        </is>
+      </c>
+      <c r="C32" s="25" t="n">
+        <v>-121436</v>
+      </c>
+      <c r="D32" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" s="30">
+        <f>D32-C32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>44517</t>
+        </is>
+      </c>
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>TVA COLLECTEE S/VENTES A 17 %</t>
+        </is>
+      </c>
+      <c r="C33" s="25" t="n">
+        <v>-9377413.710000001</v>
+      </c>
+      <c r="D33" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="30">
+        <f>D33-C33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t>44537</t>
+        </is>
+      </c>
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>TVA COLLECTEE/VENTES TPM</t>
+        </is>
+      </c>
+      <c r="C34" s="25" t="n">
+        <v>-44387281.93</v>
+      </c>
+      <c r="D34" s="25" t="n">
+        <v>-42352540.93</v>
+      </c>
+      <c r="E34" s="30">
+        <f>D34-C34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>44550</t>
+        </is>
+      </c>
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>PRECOMPTE</t>
+        </is>
+      </c>
+      <c r="C35" s="25" t="n">
+        <v>155567.5</v>
+      </c>
+      <c r="D35" s="25" t="n">
+        <v>156920</v>
+      </c>
+      <c r="E35" s="30">
+        <f>D35-C35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t>44557</t>
+        </is>
+      </c>
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>TVA RECUPERABLES</t>
+        </is>
+      </c>
+      <c r="C36" s="25" t="n">
+        <v>3454431.45</v>
+      </c>
+      <c r="D36" s="25" t="n">
+        <v>6048716.84</v>
+      </c>
+      <c r="E36" s="30">
+        <f>D36-C36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t>44710</t>
+        </is>
+      </c>
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t>TAP DUES</t>
+        </is>
+      </c>
+      <c r="C37" s="25" t="n">
+        <v>145841</v>
+      </c>
+      <c r="D37" s="25" t="n">
+        <v>-405176</v>
+      </c>
+      <c r="E37" s="30">
+        <f>D37-C37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="12" t="inlineStr">
+        <is>
+          <t>44720</t>
+        </is>
+      </c>
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>TAXES D'APRENT ET FORM PROFES</t>
+        </is>
+      </c>
+      <c r="C38" s="25" t="n">
+        <v>25960</v>
+      </c>
+      <c r="D38" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" s="30">
+        <f>D38-C38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t>44760</t>
+        </is>
+      </c>
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>TIMBRES DUES</t>
+        </is>
+      </c>
+      <c r="C39" s="25" t="n">
+        <v>-54744.65</v>
+      </c>
+      <c r="D39" s="25" t="n">
+        <v>-15720</v>
+      </c>
+      <c r="E39" s="30">
+        <f>D39-C39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="12" t="inlineStr">
+        <is>
+          <t>45500</t>
+        </is>
+      </c>
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>ASSOCIES-COMPTES COURANTS</t>
+        </is>
+      </c>
+      <c r="C40" s="25" t="n">
+        <v>-14221874.59</v>
+      </c>
+      <c r="D40" s="25" t="n">
+        <v>-21979805.85</v>
+      </c>
+      <c r="E40" s="30">
+        <f>D40-C40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="12" t="inlineStr">
+        <is>
+          <t>48600</t>
+        </is>
+      </c>
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>CHARGES CONSTATEES D'AVANCE</t>
+        </is>
+      </c>
+      <c r="C41" s="25" t="n">
+        <v>631787.84</v>
+      </c>
+      <c r="D41" s="25" t="n">
+        <v>625032.89</v>
+      </c>
+      <c r="E41" s="30">
+        <f>D41-C41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="12" t="inlineStr">
+        <is>
+          <t>51202</t>
+        </is>
+      </c>
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>BANQUE EL BARAKA</t>
+        </is>
+      </c>
+      <c r="C42" s="25" t="n">
+        <v>174036.81</v>
+      </c>
+      <c r="D42" s="25" t="n">
+        <v>168562.81</v>
+      </c>
+      <c r="E42" s="30">
+        <f>D42-C42</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="12" t="inlineStr">
+        <is>
+          <t>51220</t>
+        </is>
+      </c>
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>CPA AGENCE EL KSEUR</t>
+        </is>
+      </c>
+      <c r="C43" s="25" t="n">
+        <v>755588.6800000001</v>
+      </c>
+      <c r="D43" s="25" t="n">
+        <v>-13950322.68</v>
+      </c>
+      <c r="E43" s="30">
+        <f>D43-C43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="12" t="inlineStr">
+        <is>
+          <t>51240</t>
+        </is>
+      </c>
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>CPA 4000015290-18</t>
+        </is>
+      </c>
+      <c r="C44" s="25" t="n">
+        <v>3058279.86</v>
+      </c>
+      <c r="D44" s="25" t="n">
+        <v>93959.14999999999</v>
+      </c>
+      <c r="E44" s="30">
+        <f>D44-C44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="12" t="inlineStr">
+        <is>
+          <t>51900</t>
+        </is>
+      </c>
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>Concours bancaires courants</t>
+        </is>
+      </c>
+      <c r="C45" s="25" t="n">
+        <v>-15504804.53</v>
+      </c>
+      <c r="D45" s="25" t="n">
+        <v>-21161600.16</v>
+      </c>
+      <c r="E45" s="30">
+        <f>D45-C45</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="12" t="inlineStr">
+        <is>
+          <t>53000</t>
+        </is>
+      </c>
+      <c r="B46" s="12" t="inlineStr">
+        <is>
+          <t>CAISSE</t>
+        </is>
+      </c>
+      <c r="C46" s="25" t="n">
+        <v>1432477.99</v>
+      </c>
+      <c r="D46" s="25" t="n">
+        <v>760534.53</v>
+      </c>
+      <c r="E46" s="30">
+        <f>D46-C46</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>Nombre de comptes en écart</t>
+        </is>
+      </c>
+      <c r="C47" s="13">
+        <f>COUNTIF(E9:E46,"&lt;&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>Somme des écarts en valeur absolue</t>
+        </is>
+      </c>
+      <c r="E47" s="7">
+        <f>SUMPRODUCT(ABS(E9:E46))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Historique du compte 44537 « TVA collectée / ventes TPM » (crédit = dette de TVA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="11" t="inlineStr">
+        <is>
+          <t>Exercice</t>
+        </is>
+      </c>
+      <c r="B50" s="11" t="inlineStr">
+        <is>
+          <t>Solde d'ouverture</t>
+        </is>
+      </c>
+      <c r="C50" s="11" t="inlineStr">
+        <is>
+          <t>TVA collectée de l'exercice</t>
+        </is>
+      </c>
+      <c r="D50" s="11" t="inlineStr">
+        <is>
+          <t>Apurée par G50 (débits)</t>
+        </is>
+      </c>
+      <c r="E50" s="11" t="inlineStr">
+        <is>
+          <t>Solde de clôture</t>
+        </is>
+      </c>
+      <c r="F50" s="11" t="inlineStr">
+        <is>
+          <t>Contrôle</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="B51" s="25" t="n">
+        <v>37267981.93</v>
+      </c>
+      <c r="C51" s="25" t="n">
+        <v>7119300</v>
+      </c>
+      <c r="D51" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" s="25" t="n">
+        <v>44387281.93</v>
+      </c>
+      <c r="F51" s="30">
+        <f>ROUND(B51+C51-D51-E51,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="B52" s="25" t="n">
+        <v>42352540.93</v>
+      </c>
+      <c r="C52" s="25" t="n">
+        <v>6521750</v>
+      </c>
+      <c r="D52" s="25" t="n">
+        <v>1147983</v>
+      </c>
+      <c r="E52" s="25" t="n">
+        <v>47726307.93</v>
+      </c>
+      <c r="F52" s="30">
+        <f>ROUND(B52+C52-D52-E52,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="B53" s="25" t="n">
+        <v>47726307.93</v>
+      </c>
+      <c r="C53" s="25" t="n">
+        <v>4839300</v>
+      </c>
+      <c r="D53" s="25" t="n">
+        <v>391208</v>
+      </c>
+      <c r="E53" s="25" t="n">
+        <v>52174399.93</v>
+      </c>
+      <c r="F53" s="30">
+        <f>ROUND(B53+C53-D53-E53,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Total 2023–2025</t>
+        </is>
+      </c>
+      <c r="C54" s="7">
+        <f>SUM(C51:C53)</f>
+        <v/>
+      </c>
+      <c r="D54" s="7">
+        <f>SUM(D51:D53)</f>
+        <v/>
+      </c>
+      <c r="E54" s="38">
+        <f>D54/C54</f>
+        <v/>
+      </c>
+      <c r="F54" s="21" t="inlineStr">
+        <is>
+          <t>← part de la TVA TPM apurée</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Ouverture 2024 (42,35 M) ≠ clôture 2023 du fichier (44,39 M) : écart de 2,03 M, voir tableau ci-dessus. La TVA TPM s'accumule au crédit depuis au moins 2022 (37,27 M à l'ouverture 2023).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:I38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5113,7 +6454,7 @@
           <t>A01</t>
         </is>
       </c>
-      <c r="B5" s="39" t="n">
+      <c r="B5" s="40" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="29" t="inlineStr">
@@ -5131,7 +6472,7 @@
           <t>Déclaration CNAS de février 2026 non fournie (assiette paie 952 475,81 ; 7 STC payés).</t>
         </is>
       </c>
-      <c r="F5" s="40">
+      <c r="F5" s="41">
         <f>'Rappro CNAS'!J6</f>
         <v/>
       </c>
@@ -5140,8 +6481,8 @@
           <t>Fournir la déclaration de février + EMS avec 7 sorties ; à défaut, la déposer (pénalités de retard).</t>
         </is>
       </c>
-      <c r="H5" s="41" t="n"/>
-      <c r="I5" s="41" t="inlineStr">
+      <c r="H5" s="42" t="n"/>
+      <c r="I5" s="42" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5153,7 +6494,7 @@
           <t>A02</t>
         </is>
       </c>
-      <c r="B6" s="39" t="n">
+      <c r="B6" s="40" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="29" t="inlineStr">
@@ -5171,7 +6512,7 @@
           <t>Centralisateur de mars 2026 absent (onglet vide) alors que la CNAS de mars déclare 368 389,93 d'assiette, 5 salariés.</t>
         </is>
       </c>
-      <c r="F6" s="40">
+      <c r="F6" s="41">
         <f>'Rappro CNAS'!K7</f>
         <v/>
       </c>
@@ -5180,8 +6521,8 @@
           <t>Obtenir le livre de paie de mars et le saisir dans « Paie IMPORT » col. E ; comptabiliser la paie de mars.</t>
         </is>
       </c>
-      <c r="H6" s="41" t="n"/>
-      <c r="I6" s="41" t="inlineStr">
+      <c r="H6" s="42" t="n"/>
+      <c r="I6" s="42" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5193,7 +6534,7 @@
           <t>A03</t>
         </is>
       </c>
-      <c r="B7" s="39" t="n">
+      <c r="B7" s="40" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="29" t="inlineStr">
@@ -5211,7 +6552,7 @@
           <t>Prime de ponctualité (R540) imposée à l'IRG mais exclue du salaire de poste (assiette CNAS) chaque mois.</t>
         </is>
       </c>
-      <c r="F7" s="40">
+      <c r="F7" s="41">
         <f>'Rappro CNAS'!V13</f>
         <v/>
       </c>
@@ -5220,8 +6561,8 @@
           <t>Vérifier le paramétrage de la rubrique R540 (soumise SS) ; régulariser les déclarations concernées.</t>
         </is>
       </c>
-      <c r="H7" s="41" t="n"/>
-      <c r="I7" s="41" t="inlineStr">
+      <c r="H7" s="42" t="n"/>
+      <c r="I7" s="42" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5233,7 +6574,7 @@
           <t>A04</t>
         </is>
       </c>
-      <c r="B8" s="42" t="n">
+      <c r="B8" s="43" t="n">
         <v>2</v>
       </c>
       <c r="C8" s="29" t="inlineStr">
@@ -5251,14 +6592,14 @@
           <t>Effectif déclaré au T1 = 2 alors que 3 salariés sont inscrits ; T2 déclare 1 sortie et un effectif final de 2 ⇒ T1 aurait dû être 3.</t>
         </is>
       </c>
-      <c r="F8" s="43" t="n"/>
+      <c r="F8" s="44" t="n"/>
       <c r="G8" s="29" t="inlineStr">
         <is>
           <t>Rectifier l'effectif du T1 auprès de la CNAS.</t>
         </is>
       </c>
-      <c r="H8" s="41" t="n"/>
-      <c r="I8" s="41" t="inlineStr">
+      <c r="H8" s="42" t="n"/>
+      <c r="I8" s="42" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5270,7 +6611,7 @@
           <t>A05</t>
         </is>
       </c>
-      <c r="B9" s="42" t="n">
+      <c r="B9" s="43" t="n">
         <v>2</v>
       </c>
       <c r="C9" s="29" t="inlineStr">
@@ -5288,14 +6629,14 @@
           <t>Salarié totalement absent (non rémunéré) en juillet, disparu de la paie en août sans STC ni sortie déclarée.</t>
         </is>
       </c>
-      <c r="F9" s="43" t="n"/>
+      <c r="F9" s="44" t="n"/>
       <c r="G9" s="29" t="inlineStr">
         <is>
           <t>Établir le STC et déclarer la sortie dans l'EMS du T3 (échéance 30/10/2026).</t>
         </is>
       </c>
-      <c r="H9" s="41" t="n"/>
-      <c r="I9" s="41" t="inlineStr">
+      <c r="H9" s="42" t="n"/>
+      <c r="I9" s="42" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5307,7 +6648,7 @@
           <t>A06</t>
         </is>
       </c>
-      <c r="B10" s="42" t="n">
+      <c r="B10" s="43" t="n">
         <v>2</v>
       </c>
       <c r="C10" s="29" t="inlineStr">
@@ -5325,14 +6666,14 @@
           <t>STC de 2 237,40 en août : une sortie à déclarer au T3.</t>
         </is>
       </c>
-      <c r="F10" s="43" t="n"/>
+      <c r="F10" s="44" t="n"/>
       <c r="G10" s="29" t="inlineStr">
         <is>
           <t>Déclarer la sortie dans l'EMS du T3.</t>
         </is>
       </c>
-      <c r="H10" s="41" t="n"/>
-      <c r="I10" s="41" t="inlineStr">
+      <c r="H10" s="42" t="n"/>
+      <c r="I10" s="42" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5344,7 +6685,7 @@
           <t>A07</t>
         </is>
       </c>
-      <c r="B11" s="42" t="n">
+      <c r="B11" s="43" t="n">
         <v>2</v>
       </c>
       <c r="C11" s="29" t="inlineStr">
@@ -5362,7 +6703,7 @@
           <t>Déclarations T3 2026 (juil–sept) à établir ; paie de septembre non fournie.</t>
         </is>
       </c>
-      <c r="F11" s="40">
+      <c r="F11" s="41">
         <f>'Rappro CNAS'!J9+'Rappro CNAS'!J12</f>
         <v/>
       </c>
@@ -5371,8 +6712,8 @@
           <t>Transmettre les centralisateurs de septembre ; déposer et payer avant le 30/10/2026.</t>
         </is>
       </c>
-      <c r="H11" s="41" t="n"/>
-      <c r="I11" s="41" t="inlineStr">
+      <c r="H11" s="42" t="n"/>
+      <c r="I11" s="42" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5384,7 +6725,7 @@
           <t>A08</t>
         </is>
       </c>
-      <c r="B12" s="44" t="n">
+      <c r="B12" s="45" t="n">
         <v>3</v>
       </c>
       <c r="C12" s="29" t="inlineStr">
@@ -5402,14 +6743,14 @@
           <t>Avril = mai et juillet = août strictement identiques (mêmes absences, heures sup., IRG) : variables probablement non saisies.</t>
         </is>
       </c>
-      <c r="F12" s="43" t="n"/>
+      <c r="F12" s="44" t="n"/>
       <c r="G12" s="29" t="inlineStr">
         <is>
           <t>Contrôler les pointages et bulletins de mai et août.</t>
         </is>
       </c>
-      <c r="H12" s="41" t="n"/>
-      <c r="I12" s="41" t="inlineStr">
+      <c r="H12" s="42" t="n"/>
+      <c r="I12" s="42" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5421,7 +6762,7 @@
           <t>A09</t>
         </is>
       </c>
-      <c r="B13" s="44" t="n">
+      <c r="B13" s="45" t="n">
         <v>3</v>
       </c>
       <c r="C13" s="29" t="inlineStr">
@@ -5439,7 +6780,7 @@
           <t>Frais de mission élevés (avril 41 615 ; mai 49 115, soit 47–55 % de l'assiette), non soumis à cotisations.</t>
         </is>
       </c>
-      <c r="F13" s="40">
+      <c r="F13" s="41">
         <f>'Paie TPM'!K26</f>
         <v/>
       </c>
@@ -5448,8 +6789,8 @@
           <t>Conserver ordres de mission et justificatifs ; risque de requalification en salaire.</t>
         </is>
       </c>
-      <c r="H13" s="41" t="n"/>
-      <c r="I13" s="41" t="inlineStr">
+      <c r="H13" s="42" t="n"/>
+      <c r="I13" s="42" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5461,7 +6802,7 @@
           <t>A10</t>
         </is>
       </c>
-      <c r="B14" s="44" t="n">
+      <c r="B14" s="45" t="n">
         <v>3</v>
       </c>
       <c r="C14" s="29" t="inlineStr">
@@ -5479,14 +6820,14 @@
           <t>Prime de responsabilité de 5,00 DA (janv.) et 1,14 DA (févr.) : paramètre vraisemblablement erroné (5 au lieu de 5 %).</t>
         </is>
       </c>
-      <c r="F14" s="43" t="n"/>
+      <c r="F14" s="44" t="n"/>
       <c r="G14" s="29" t="inlineStr">
         <is>
           <t>Corriger le paramètre B291 ; régulariser le rappel éventuel.</t>
         </is>
       </c>
-      <c r="H14" s="41" t="n"/>
-      <c r="I14" s="41" t="inlineStr">
+      <c r="H14" s="42" t="n"/>
+      <c r="I14" s="42" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5498,7 +6839,7 @@
           <t>A11</t>
         </is>
       </c>
-      <c r="B15" s="42" t="n">
+      <c r="B15" s="43" t="n">
         <v>2</v>
       </c>
       <c r="C15" s="29" t="inlineStr">
@@ -5516,7 +6857,7 @@
           <t>Bordereaux de versement CNAS à « 0,00 » : aucune preuve de paiement des cotisations dans le dossier.</t>
         </is>
       </c>
-      <c r="F15" s="40">
+      <c r="F15" s="41">
         <f>'Rappro CNAS'!K13</f>
         <v/>
       </c>
@@ -5525,8 +6866,8 @@
           <t>Joindre les quittances CNAS / avis de virement ; comptabiliser les règlements (débit 431).</t>
         </is>
       </c>
-      <c r="H15" s="41" t="n"/>
-      <c r="I15" s="41" t="inlineStr">
+      <c r="H15" s="42" t="n"/>
+      <c r="I15" s="42" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5538,7 +6879,7 @@
           <t>A12</t>
         </is>
       </c>
-      <c r="B16" s="42" t="n">
+      <c r="B16" s="43" t="n">
         <v>2</v>
       </c>
       <c r="C16" s="29" t="inlineStr">
@@ -5556,7 +6897,7 @@
           <t>IRG IMPORT : G50 de janvier à août conformes à la paie (écarts d'arrondi ≤ 3 DA ; juillet : 2,30 DA retenus non reversés). Mars non vérifiable (paie absente).</t>
         </is>
       </c>
-      <c r="F16" s="40">
+      <c r="F16" s="41">
         <f>'Échéancier IRG-CNAS'!G13</f>
         <v/>
       </c>
@@ -5565,8 +6906,8 @@
           <t>Reverser l'IRG retenu au dinar près ; fournir la paie de mars.</t>
         </is>
       </c>
-      <c r="H16" s="41" t="n"/>
-      <c r="I16" s="41" t="inlineStr">
+      <c r="H16" s="42" t="n"/>
+      <c r="I16" s="42" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5578,7 +6919,7 @@
           <t>A13</t>
         </is>
       </c>
-      <c r="B17" s="44" t="n">
+      <c r="B17" s="45" t="n">
         <v>3</v>
       </c>
       <c r="C17" s="29" t="inlineStr">
@@ -5596,14 +6937,14 @@
           <t>Paie paramétrée CACOBATPH (taux X504) mais aucune déclaration CACOBATPH (congés payés / intempéries) dans le dossier.</t>
         </is>
       </c>
-      <c r="F17" s="43" t="n"/>
+      <c r="F17" s="44" t="n"/>
       <c r="G17" s="29" t="inlineStr">
         <is>
           <t>Fournir les déclarations et paiements CACOBATPH 2026.</t>
         </is>
       </c>
-      <c r="H17" s="41" t="n"/>
-      <c r="I17" s="41" t="inlineStr">
+      <c r="H17" s="42" t="n"/>
+      <c r="I17" s="42" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5615,7 +6956,7 @@
           <t>A14</t>
         </is>
       </c>
-      <c r="B18" s="44" t="n">
+      <c r="B18" s="45" t="n">
         <v>3</v>
       </c>
       <c r="C18" s="29" t="inlineStr">
@@ -5633,14 +6974,14 @@
           <t>Libellés divergents : « D.P.R.COMPAGNY » / « DPR COMPAGNY » ; en-tête de paie TPM à l'adresse VGE TIZI alors que l'affiliation TPM est à TISSA.</t>
         </is>
       </c>
-      <c r="F18" s="43" t="n"/>
+      <c r="F18" s="44" t="n"/>
       <c r="G18" s="29" t="inlineStr">
         <is>
           <t>Harmoniser raison sociale et adresse dans le logiciel de paie.</t>
         </is>
       </c>
-      <c r="H18" s="41" t="n"/>
-      <c r="I18" s="41" t="inlineStr">
+      <c r="H18" s="42" t="n"/>
+      <c r="I18" s="42" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5652,7 +6993,7 @@
           <t>A15</t>
         </is>
       </c>
-      <c r="B19" s="44" t="n">
+      <c r="B19" s="45" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="29" t="inlineStr">
@@ -5670,14 +7011,14 @@
           <t>Périodicité mixte : déclarations mensuelles (janv., mars) puis trimestrielle (T2).</t>
         </is>
       </c>
-      <c r="F19" s="43" t="n"/>
+      <c r="F19" s="44" t="n"/>
       <c r="G19" s="29" t="inlineStr">
         <is>
           <t>Confirmer auprès de la CNAS le passage au trimestriel après la baisse d'effectif (12 → 5).</t>
         </is>
       </c>
-      <c r="H19" s="41" t="n"/>
-      <c r="I19" s="41" t="inlineStr">
+      <c r="H19" s="42" t="n"/>
+      <c r="I19" s="42" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5689,7 +7030,7 @@
           <t>A16</t>
         </is>
       </c>
-      <c r="B20" s="44" t="n">
+      <c r="B20" s="45" t="n">
         <v>3</v>
       </c>
       <c r="C20" s="29" t="inlineStr">
@@ -5707,14 +7048,14 @@
           <t>IRG non vérifiable salarié par salarié (centralisateurs uniquement).</t>
         </is>
       </c>
-      <c r="F20" s="43" t="n"/>
+      <c r="F20" s="44" t="n"/>
       <c r="G20" s="29" t="inlineStr">
         <is>
           <t>Fournir le livre de paie individuel / bulletins.</t>
         </is>
       </c>
-      <c r="H20" s="41" t="n"/>
-      <c r="I20" s="41" t="inlineStr">
+      <c r="H20" s="42" t="n"/>
+      <c r="I20" s="42" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5726,7 +7067,7 @@
           <t>A17</t>
         </is>
       </c>
-      <c r="B21" s="39" t="n">
+      <c r="B21" s="40" t="n">
         <v>1</v>
       </c>
       <c r="C21" s="29" t="inlineStr">
@@ -5741,10 +7082,10 @@
       </c>
       <c r="E21" s="29" t="inlineStr">
         <is>
-          <t>TVA collectée TPM (44537) et location (44527) jamais soldées : 58,9 M DA cumulés au 31/12/2025. En 2025, 4 839 300 de TVA TPM générée, seuls 391 208 passés en G50 (déc.). Les G50 TPM 2026 (juil., août) ne déclarent aucun CA et reportent un précompte de 1 714 499 (= compte 44550).</t>
-        </is>
-      </c>
-      <c r="F21" s="40">
+          <t>TVA collectée TPM (44537) et location (44527) jamais soldées : 58,9 M DA cumulés au 31/12/2025, accumulés depuis au moins 2022 (37,3 M à l'ouverture 2023) ; 2023–2025 : 18,5 M collectés, 1,5 M apurés. En 2025, 4 839 300 de TVA TPM générée, seuls 391 208 passés en G50 (déc.). Les G50 TPM 2026 (juil., août) ne déclarent aucun CA et reportent un précompte de 1 714 499 (= compte 44550).</t>
+        </is>
+      </c>
+      <c r="F21" s="41">
         <f>-('Balance 2024-2025'!D48+'Balance 2024-2025'!D47)</f>
         <v/>
       </c>
@@ -5753,8 +7094,8 @@
           <t>Rapprocher avec les G50 TPM 2023–2025 ; si TVA non déclarée, régulariser ; sinon passer les écritures de G50 manquantes.</t>
         </is>
       </c>
-      <c r="H21" s="41" t="n"/>
-      <c r="I21" s="41" t="inlineStr">
+      <c r="H21" s="42" t="n"/>
+      <c r="I21" s="42" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5766,7 +7107,7 @@
           <t>A18</t>
         </is>
       </c>
-      <c r="B22" s="39" t="n">
+      <c r="B22" s="40" t="n">
         <v>1</v>
       </c>
       <c r="C22" s="29" t="inlineStr">
@@ -5784,7 +7125,7 @@
           <t>CA de mars 2026 réalisé 27 006 870 (annotation G50), mais seulement 3 445 200 déclarés en mars « pour manque TVA à récupérer » : 23 561 670 de CA reportés sur avril–août. En avril, le CA annoté (13 157 894,74) est calculé pour obtenir 2 500 000 de TVA. Le CA déclaré mensuellement est ajusté à la TVA déductible disponible.</t>
         </is>
       </c>
-      <c r="F22" s="40">
+      <c r="F22" s="41">
         <f>'G50 2026'!B40</f>
         <v/>
       </c>
@@ -5793,8 +7134,8 @@
           <t>Déclarer le CA au titre du mois de réalisation ; rapprocher le CA déclaré du journal des ventes 2026 ; chiffrer les pénalités de retard sur la TVA différée.</t>
         </is>
       </c>
-      <c r="H22" s="41" t="n"/>
-      <c r="I22" s="41" t="inlineStr">
+      <c r="H22" s="42" t="n"/>
+      <c r="I22" s="42" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5806,8 +7147,8 @@
           <t>A19</t>
         </is>
       </c>
-      <c r="B23" s="42" t="n">
-        <v>2</v>
+      <c r="B23" s="40" t="n">
+        <v>1</v>
       </c>
       <c r="C23" s="29" t="inlineStr">
         <is>
@@ -5821,20 +7162,20 @@
       </c>
       <c r="E23" s="29" t="inlineStr">
         <is>
-          <t>G50 TPM de juillet : mois imprimé « AVRIL » et IRG déclaré 9 375 (montant d'avril/mai) au lieu de 3 691,30 retenus en juillet ; août conforme (3 690). G50 TPM de janvier à juin non fournies.</t>
-        </is>
-      </c>
-      <c r="F23" s="40">
-        <f>SUM('Paie TPM'!C25:H25)</f>
+          <t>G50 TPM d'avril à juillet identiques (mois imprimé « AVRIL », IRG 9 375 chaque mois) : juin sous-déclaré de 9 614,90 (18 989,90 retenus), juillet sur-déclaré de 5 683,70 ; août conforme. G50 TPM de janvier à mars non fournies.</t>
+        </is>
+      </c>
+      <c r="F23" s="41">
+        <f>-'G50 TPM 2026'!D15</f>
         <v/>
       </c>
       <c r="G23" s="29" t="inlineStr">
         <is>
-          <t>Fournir les G50 TPM janv.–juin ; corriger ou justifier la G50 de juillet (régularisation de l'écart 5 683,70).</t>
-        </is>
-      </c>
-      <c r="H23" s="41" t="n"/>
-      <c r="I23" s="41" t="inlineStr">
+          <t>Déposer une G50 rectificative pour juin (IRG retenu non reversé) et régulariser juillet ; fournir les G50 TPM janv.–mars.</t>
+        </is>
+      </c>
+      <c r="H23" s="42" t="n"/>
+      <c r="I23" s="42" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5846,7 +7187,7 @@
           <t>A20</t>
         </is>
       </c>
-      <c r="B24" s="42" t="n">
+      <c r="B24" s="43" t="n">
         <v>2</v>
       </c>
       <c r="C24" s="29" t="inlineStr">
@@ -5864,7 +7205,7 @@
           <t>Écriture du 31/12/2025 « POUR SOLDE PRCT EXE 2025 » passée en sens inverse (D 44410 / C 444, 3 074 299) : dette IBS 9,79 M et acomptes 6,15 M au lieu d'un net de 3 642 951.</t>
         </is>
       </c>
-      <c r="F24" s="40" t="n">
+      <c r="F24" s="41" t="n">
         <v>3074299</v>
       </c>
       <c r="G24" s="29" t="inlineStr">
@@ -5872,8 +7213,8 @@
           <t>Contrepasser et compenser (D 444 / C 44410) ; vérifier le paiement du solde IBS 2025 en 2026.</t>
         </is>
       </c>
-      <c r="H24" s="41" t="n"/>
-      <c r="I24" s="41" t="inlineStr">
+      <c r="H24" s="42" t="n"/>
+      <c r="I24" s="42" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5885,7 +7226,7 @@
           <t>A21</t>
         </is>
       </c>
-      <c r="B25" s="42" t="n">
+      <c r="B25" s="43" t="n">
         <v>2</v>
       </c>
       <c r="C25" s="29" t="inlineStr">
@@ -5903,7 +7244,7 @@
           <t>Solde IBS 2024 réglé le 03/07/2025 ; IBS 2025 net à liquider de 3 642 951 (précomptes douane déduits).</t>
         </is>
       </c>
-      <c r="F25" s="40" t="n">
+      <c r="F25" s="41" t="n">
         <v>3642951</v>
       </c>
       <c r="G25" s="29" t="inlineStr">
@@ -5911,8 +7252,8 @@
           <t>Vérifier les dates d'échéance de liquidation, les pénalités éventuelles et la preuve de paiement 2026.</t>
         </is>
       </c>
-      <c r="H25" s="41" t="n"/>
-      <c r="I25" s="41" t="inlineStr">
+      <c r="H25" s="42" t="n"/>
+      <c r="I25" s="42" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5924,7 +7265,7 @@
           <t>A22</t>
         </is>
       </c>
-      <c r="B26" s="42" t="n">
+      <c r="B26" s="43" t="n">
         <v>2</v>
       </c>
       <c r="C26" s="29" t="inlineStr">
@@ -5942,7 +7283,7 @@
           <t>Caisse de 12,1 M au 31/12/2025 (pic de 22,5 M) ; remboursement en espèces de 6 800 000 à SARL DPR AXXAM le 06/12/2025.</t>
         </is>
       </c>
-      <c r="F26" s="40">
+      <c r="F26" s="41">
         <f>'Balance 2024-2025'!D67</f>
         <v/>
       </c>
@@ -5951,8 +7292,8 @@
           <t>PV de caisse au 31/12 ; respecter l'obligation de paiement scriptural au-delà des seuils réglementaires.</t>
         </is>
       </c>
-      <c r="H26" s="41" t="n"/>
-      <c r="I26" s="41" t="inlineStr">
+      <c r="H26" s="42" t="n"/>
+      <c r="I26" s="42" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -5964,7 +7305,7 @@
           <t>A23</t>
         </is>
       </c>
-      <c r="B27" s="42" t="n">
+      <c r="B27" s="43" t="n">
         <v>2</v>
       </c>
       <c r="C27" s="29" t="inlineStr">
@@ -5982,7 +7323,7 @@
           <t>100 % du CA TPM 2025 (25,47 M) facturé à SARL DPR AXXAM BRIQUETERIE ; aucune facturation TPM d'oct. à déc. 2025 alors que du personnel TPM reste payé.</t>
         </is>
       </c>
-      <c r="F27" s="40">
+      <c r="F27" s="41">
         <f>-'Balance 2024-2025'!D100</f>
         <v/>
       </c>
@@ -5991,8 +7332,8 @@
           <t>Documenter les conventions intra-groupe et la facturation d'oct.–déc. 2025.</t>
         </is>
       </c>
-      <c r="H27" s="41" t="n"/>
-      <c r="I27" s="41" t="inlineStr">
+      <c r="H27" s="42" t="n"/>
+      <c r="I27" s="42" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -6004,7 +7345,7 @@
           <t>A24</t>
         </is>
       </c>
-      <c r="B28" s="42" t="n">
+      <c r="B28" s="43" t="n">
         <v>2</v>
       </c>
       <c r="C28" s="29" t="inlineStr">
@@ -6022,7 +7363,7 @@
           <t>Compte d'attente 47000 non soldé (« SARL FAHAS ?? », « TRESORERIE BEJAIA ?? », chèques).</t>
         </is>
       </c>
-      <c r="F28" s="40">
+      <c r="F28" s="41">
         <f>'Balance 2024-2025'!D59</f>
         <v/>
       </c>
@@ -6031,8 +7372,8 @@
           <t>Identifier et apurer avant clôture.</t>
         </is>
       </c>
-      <c r="H28" s="41" t="n"/>
-      <c r="I28" s="41" t="inlineStr">
+      <c r="H28" s="42" t="n"/>
+      <c r="I28" s="42" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -6044,7 +7385,7 @@
           <t>A25</t>
         </is>
       </c>
-      <c r="B29" s="42" t="n">
+      <c r="B29" s="43" t="n">
         <v>2</v>
       </c>
       <c r="C29" s="29" t="inlineStr">
@@ -6062,7 +7403,7 @@
           <t>Compte 63120 « prime imposable » non soumise à cotisation : 957 406 en 2025 et 1 139 275 en 2024 (même mécanisme que A03).</t>
         </is>
       </c>
-      <c r="F29" s="40">
+      <c r="F29" s="41">
         <f>'États 2024-2025'!C24+'États 2024-2025'!D24</f>
         <v/>
       </c>
@@ -6071,8 +7412,8 @@
           <t>Analyser les primes concernées ; régulariser si elles sont cotisables.</t>
         </is>
       </c>
-      <c r="H29" s="41" t="n"/>
-      <c r="I29" s="41" t="inlineStr">
+      <c r="H29" s="42" t="n"/>
+      <c r="I29" s="42" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -6084,7 +7425,7 @@
           <t>A26</t>
         </is>
       </c>
-      <c r="B30" s="44" t="n">
+      <c r="B30" s="45" t="n">
         <v>3</v>
       </c>
       <c r="C30" s="29" t="inlineStr">
@@ -6102,7 +7443,7 @@
           <t>Banque CPA El Kseur (51220) créditrice de 12,43 M au 31/12/2025 : découvert présenté en banque.</t>
         </is>
       </c>
-      <c r="F30" s="40">
+      <c r="F30" s="41">
         <f>ABS('Balance 2024-2025'!D63)</f>
         <v/>
       </c>
@@ -6111,8 +7452,8 @@
           <t>Reclasser en 519 ; vérifier les agios (aucune charge 661 en 2025).</t>
         </is>
       </c>
-      <c r="H30" s="41" t="n"/>
-      <c r="I30" s="41" t="inlineStr">
+      <c r="H30" s="42" t="n"/>
+      <c r="I30" s="42" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -6124,7 +7465,7 @@
           <t>A27</t>
         </is>
       </c>
-      <c r="B31" s="44" t="n">
+      <c r="B31" s="45" t="n">
         <v>3</v>
       </c>
       <c r="C31" s="29" t="inlineStr">
@@ -6142,7 +7483,7 @@
           <t>Reversements IRG 2025 parfois partiels (févr., juin) et rattrapés le mois suivant ; amendes 2025 : douane 100 000, CNAS 1 746.</t>
         </is>
       </c>
-      <c r="F31" s="40">
+      <c r="F31" s="41">
         <f>'Balance 2024-2025'!D93</f>
         <v/>
       </c>
@@ -6151,8 +7492,8 @@
           <t>Reverser l'IRG en totalité chaque mois.</t>
         </is>
       </c>
-      <c r="H31" s="41" t="n"/>
-      <c r="I31" s="41" t="inlineStr">
+      <c r="H31" s="42" t="n"/>
+      <c r="I31" s="42" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -6164,7 +7505,7 @@
           <t>A28</t>
         </is>
       </c>
-      <c r="B32" s="44" t="n">
+      <c r="B32" s="45" t="n">
         <v>3</v>
       </c>
       <c r="C32" s="29" t="inlineStr">
@@ -6182,14 +7523,14 @@
           <t>Modèles G50 non mis à jour : dates de signature de 2021–2022 sur toutes les G50 2026, onglet de saisie figé (mai, TVA 17 %), G50 TPM contenant le récap TVA de déc. 2025 et un extrait de journal 2019 ; libellés de comptes de TVA à 17 %.</t>
         </is>
       </c>
-      <c r="F32" s="43" t="n"/>
+      <c r="F32" s="44" t="n"/>
       <c r="G32" s="29" t="inlineStr">
         <is>
           <t>Mettre à jour le modèle et les libellés (TVA 19 %).</t>
         </is>
       </c>
-      <c r="H32" s="41" t="n"/>
-      <c r="I32" s="41" t="inlineStr">
+      <c r="H32" s="42" t="n"/>
+      <c r="I32" s="42" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -6201,7 +7542,7 @@
           <t>A29</t>
         </is>
       </c>
-      <c r="B33" s="44" t="n">
+      <c r="B33" s="45" t="n">
         <v>3</v>
       </c>
       <c r="C33" s="29" t="inlineStr">
@@ -6219,8 +7560,8 @@
           <t>Taxe d'apprentissage payée deux fois en 2026 : février (87 828 sur 8 782 828) et août (44 091 IMPORT sur 4 409 079 + 6 809 TPM sur 680 900).</t>
         </is>
       </c>
-      <c r="F33" s="40">
-        <f>'G50 2026'!J26+'G50 TPM 2026'!C18</f>
+      <c r="F33" s="41">
+        <f>'G50 2026'!J26+'G50 TPM 2026'!G17</f>
         <v/>
       </c>
       <c r="G33" s="29" t="inlineStr">
@@ -6228,8 +7569,8 @@
           <t>Justifier les bases et la période couverte par chaque paiement (risque de double paiement).</t>
         </is>
       </c>
-      <c r="H33" s="41" t="n"/>
-      <c r="I33" s="41" t="inlineStr">
+      <c r="H33" s="42" t="n"/>
+      <c r="I33" s="42" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -6241,7 +7582,7 @@
           <t>A30</t>
         </is>
       </c>
-      <c r="B34" s="44" t="n">
+      <c r="B34" s="45" t="n">
         <v>3</v>
       </c>
       <c r="C34" s="29" t="inlineStr">
@@ -6259,7 +7600,7 @@
           <t>Droit de timbre : taux apparents incohérents (janv. 2,0 %, févr. 1,0 %, avr. 5,05 %, mai 1,79 %) ; même base en avril et mai ; aucun timbre en mars et de juin à août.</t>
         </is>
       </c>
-      <c r="F34" s="40">
+      <c r="F34" s="41">
         <f>'G50 2026'!J24</f>
         <v/>
       </c>
@@ -6268,8 +7609,8 @@
           <t>Justifier la base (ventes en espèces) et le taux appliqué.</t>
         </is>
       </c>
-      <c r="H34" s="41" t="n"/>
-      <c r="I34" s="41" t="inlineStr">
+      <c r="H34" s="42" t="n"/>
+      <c r="I34" s="42" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
@@ -6278,61 +7619,101 @@
     <row r="35" ht="52" customHeight="1">
       <c r="A35" s="4" t="inlineStr">
         <is>
+          <t>A32</t>
+        </is>
+      </c>
+      <c r="B35" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" s="29" t="inlineStr">
+        <is>
+          <t>Société</t>
+        </is>
+      </c>
+      <c r="D35" s="29" t="inlineStr">
+        <is>
+          <t>Comptabilité</t>
+        </is>
+      </c>
+      <c r="E35" s="29" t="inlineStr">
+        <is>
+          <t>Journal 2023 fourni provisoire : résultat 18,54 M contre 7,26 M repris en à-nouveau 2024 ; 38 comptes en écart avec les ouvertures 2024 (stocks, fournisseurs, banques, IBS, TVA).</t>
+        </is>
+      </c>
+      <c r="F35" s="41">
+        <f>'Contrôle 2023'!B6</f>
+        <v/>
+      </c>
+      <c r="G35" s="29" t="inlineStr">
+        <is>
+          <t>Obtenir le journal 2023 définitif et la liasse fiscale 2023 ; documenter les écritures de clôture.</t>
+        </is>
+      </c>
+      <c r="H35" s="42" t="n"/>
+      <c r="I35" s="42" t="inlineStr">
+        <is>
+          <t>Ouvert</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="52" customHeight="1">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
           <t>A31</t>
         </is>
       </c>
-      <c r="B35" s="44" t="n">
+      <c r="B36" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="C35" s="29" t="inlineStr">
+      <c r="C36" s="29" t="inlineStr">
         <is>
           <t>Les deux</t>
         </is>
       </c>
-      <c r="D35" s="29" t="inlineStr">
+      <c r="D36" s="29" t="inlineStr">
         <is>
           <t>Comptabilité</t>
         </is>
       </c>
-      <c r="E35" s="29" t="inlineStr">
+      <c r="E36" s="29" t="inlineStr">
         <is>
           <t>Clients débiteurs 387,1 M et avances clients 314,6 M ; fournisseurs débiteurs 46,2 M au 31/12/2025.</t>
         </is>
       </c>
-      <c r="F35" s="43" t="n"/>
-      <c r="G35" s="29" t="inlineStr">
+      <c r="F36" s="44" t="n"/>
+      <c r="G36" s="29" t="inlineStr">
         <is>
           <t>Lettrer les comptes clients/fournisseurs et compenser les avances soldées.</t>
         </is>
       </c>
-      <c r="H35" s="41" t="n"/>
-      <c r="I35" s="41" t="inlineStr">
+      <c r="H36" s="42" t="n"/>
+      <c r="I36" s="42" t="inlineStr">
         <is>
           <t>Ouvert</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>Impact : A01 = cotisations calculées de février ; A02 = cotisations de mars déclarées sans justificatif ; A03 = cotisations sur ponctualité ; A07 = cotisations T3 partielles (juil–août) ; A09 = frais de mission TPM cumulés ; A11 = cotisations déclarées sans preuve de paiement ; A12 = IRG cumulé à rapprocher.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I35"/>
+  <autoFilter ref="A4:I36"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6408,7 +7789,7 @@
           <t>Janv–août 2026</t>
         </is>
       </c>
-      <c r="E5" s="45" t="inlineStr">
+      <c r="E5" s="46" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6438,7 +7819,7 @@
           <t>Janv–août 2026</t>
         </is>
       </c>
-      <c r="E6" s="45" t="inlineStr">
+      <c r="E6" s="46" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6464,7 +7845,7 @@
           <t>Janvier 2026</t>
         </is>
       </c>
-      <c r="E7" s="45" t="inlineStr">
+      <c r="E7" s="46" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6494,7 +7875,7 @@
           <t>Mars 2026</t>
         </is>
       </c>
-      <c r="E8" s="45" t="inlineStr">
+      <c r="E8" s="46" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6524,7 +7905,7 @@
           <t>T2 2026</t>
         </is>
       </c>
-      <c r="E9" s="45" t="inlineStr">
+      <c r="E9" s="46" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6554,7 +7935,7 @@
           <t>T1 2026</t>
         </is>
       </c>
-      <c r="E10" s="45" t="inlineStr">
+      <c r="E10" s="46" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6584,7 +7965,7 @@
           <t>T2 2026</t>
         </is>
       </c>
-      <c r="E11" s="45" t="inlineStr">
+      <c r="E11" s="46" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6614,7 +7995,7 @@
           <t>Février 2026</t>
         </is>
       </c>
-      <c r="E12" s="46" t="inlineStr">
+      <c r="E12" s="47" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
@@ -6644,7 +8025,7 @@
           <t>Mars 2026</t>
         </is>
       </c>
-      <c r="E13" s="46" t="inlineStr">
+      <c r="E13" s="47" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
@@ -6670,7 +8051,7 @@
           <t>Septembre 2026</t>
         </is>
       </c>
-      <c r="E14" s="46" t="inlineStr">
+      <c r="E14" s="47" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
@@ -6700,7 +8081,7 @@
           <t>T3 2026</t>
         </is>
       </c>
-      <c r="E15" s="46" t="inlineStr">
+      <c r="E15" s="47" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
@@ -6730,7 +8111,7 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="E16" s="46" t="inlineStr">
+      <c r="E16" s="47" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
@@ -6760,7 +8141,7 @@
           <t>Juin 2026</t>
         </is>
       </c>
-      <c r="E17" s="45" t="inlineStr">
+      <c r="E17" s="46" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6790,7 +8171,7 @@
           <t>Août 2026</t>
         </is>
       </c>
-      <c r="E18" s="45" t="inlineStr">
+      <c r="E18" s="46" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6820,7 +8201,7 @@
           <t>Exercice 2024</t>
         </is>
       </c>
-      <c r="E19" s="45" t="inlineStr">
+      <c r="E19" s="46" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6850,7 +8231,7 @@
           <t>Exercice 2025</t>
         </is>
       </c>
-      <c r="E20" s="45" t="inlineStr">
+      <c r="E20" s="46" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6880,7 +8261,7 @@
           <t>Mars, avril, mai, juillet 2026</t>
         </is>
       </c>
-      <c r="E21" s="45" t="inlineStr">
+      <c r="E21" s="46" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6910,7 +8291,7 @@
           <t>Janvier, février 2026</t>
         </is>
       </c>
-      <c r="E22" s="45" t="inlineStr">
+      <c r="E22" s="46" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6940,7 +8321,7 @@
           <t>Juillet, août 2026</t>
         </is>
       </c>
-      <c r="E23" s="45" t="inlineStr">
+      <c r="E23" s="46" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -6957,7 +8338,7 @@
       </c>
       <c r="B24" s="12" t="inlineStr">
         <is>
-          <t>G50 TPM et location janvier à juin 2026</t>
+          <t>G50_04/05/06-2026_TPM_ET_LOCATION_CONSOLIDE.xls</t>
         </is>
       </c>
       <c r="C24" s="12" t="inlineStr">
@@ -6967,17 +8348,17 @@
       </c>
       <c r="D24" s="12" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>Avril, mai, juin 2026</t>
         </is>
       </c>
       <c r="E24" s="46" t="inlineStr">
         <is>
-          <t>Manquante</t>
+          <t>Reçue</t>
         </is>
       </c>
       <c r="F24" s="12" t="inlineStr">
         <is>
-          <t>Voir A19</t>
+          <t>Identiques entre elles (mois AVRIL)</t>
         </is>
       </c>
     </row>
@@ -6987,27 +8368,27 @@
       </c>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>G50 IMPORT et TPM septembre 2026</t>
+          <t>DLG_COMPTAZ_SARL_DPR_COMPAGNY_2023.xls — journal 2023</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>Les deux</t>
+          <t>Société</t>
         </is>
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>Sept. 2026</t>
+          <t>Exercice 2023</t>
         </is>
       </c>
       <c r="E25" s="46" t="inlineStr">
         <is>
-          <t>Manquante</t>
+          <t>Reçue</t>
         </is>
       </c>
       <c r="F25" s="12" t="inlineStr">
         <is>
-          <t>Échéance 20/10/2026</t>
+          <t>Version provisoire (voir A32)</t>
         </is>
       </c>
     </row>
@@ -7017,12 +8398,12 @@
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>Journal des ventes / factures 2026</t>
+          <t>G50 TPM et location janvier à mars 2026</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>IMPORT</t>
+          <t>TPM</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
@@ -7030,14 +8411,14 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="E26" s="46" t="inlineStr">
+      <c r="E26" s="47" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
       </c>
       <c r="F26" s="12" t="inlineStr">
         <is>
-          <t>Voir A18 : CA réel par mois</t>
+          <t>Voir A19</t>
         </is>
       </c>
     </row>
@@ -7047,27 +8428,27 @@
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>G50 TPM 2023–2025 (rapprochement TVA collectée TPM)</t>
+          <t>Journal 2023 définitif et liasse fiscale 2023</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>TPM</t>
+          <t>Société</t>
         </is>
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
-          <t>2023–2025</t>
-        </is>
-      </c>
-      <c r="E27" s="46" t="inlineStr">
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="E27" s="47" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
       </c>
       <c r="F27" s="12" t="inlineStr">
         <is>
-          <t>Voir A17</t>
+          <t>Voir A32</t>
         </is>
       </c>
     </row>
@@ -7077,27 +8458,27 @@
       </c>
       <c r="B28" s="12" t="inlineStr">
         <is>
-          <t>Journal comptable 2026 (PCCOMPTA)</t>
+          <t>G50 IMPORT et TPM septembre 2026</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
         <is>
-          <t>Société</t>
+          <t>Les deux</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="E28" s="46" t="inlineStr">
+          <t>Sept. 2026</t>
+        </is>
+      </c>
+      <c r="E28" s="47" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
       </c>
       <c r="F28" s="12" t="inlineStr">
         <is>
-          <t>Pour rapprocher paie et G50 avec la comptabilité</t>
+          <t>Échéance 20/10/2026</t>
         </is>
       </c>
     </row>
@@ -7107,27 +8488,27 @@
       </c>
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>Liasse fiscale / bilan 2025 déposé et preuve de paiement IBS</t>
+          <t>Journal des ventes / factures 2026</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>Société</t>
+          <t>IMPORT</t>
         </is>
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="E29" s="46" t="inlineStr">
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E29" s="47" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
       </c>
       <c r="F29" s="12" t="inlineStr">
         <is>
-          <t>Voir A20, A21</t>
+          <t>Voir A18 : CA réel par mois</t>
         </is>
       </c>
     </row>
@@ -7137,27 +8518,27 @@
       </c>
       <c r="B30" s="12" t="inlineStr">
         <is>
-          <t>PV de caisse au 31/12/2025</t>
+          <t>G50 TPM 2023–2025 (rapprochement TVA collectée TPM)</t>
         </is>
       </c>
       <c r="C30" s="12" t="inlineStr">
         <is>
-          <t>Société</t>
+          <t>TPM</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
         <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="E30" s="46" t="inlineStr">
+          <t>2023–2025</t>
+        </is>
+      </c>
+      <c r="E30" s="47" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
       </c>
       <c r="F30" s="12" t="inlineStr">
         <is>
-          <t>Voir A22</t>
+          <t>Voir A17</t>
         </is>
       </c>
     </row>
@@ -7167,12 +8548,12 @@
       </c>
       <c r="B31" s="12" t="inlineStr">
         <is>
-          <t>Déclarations et paiements CACOBATPH</t>
+          <t>Journal comptable 2026 (PCCOMPTA)</t>
         </is>
       </c>
       <c r="C31" s="12" t="inlineStr">
         <is>
-          <t>Les deux</t>
+          <t>Société</t>
         </is>
       </c>
       <c r="D31" s="12" t="inlineStr">
@@ -7180,12 +8561,16 @@
           <t>2026</t>
         </is>
       </c>
-      <c r="E31" s="46" t="inlineStr">
+      <c r="E31" s="47" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
       </c>
-      <c r="F31" s="12" t="inlineStr"/>
+      <c r="F31" s="12" t="inlineStr">
+        <is>
+          <t>Pour rapprocher paie et G50 avec la comptabilité</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="12" t="n">
@@ -7193,27 +8578,27 @@
       </c>
       <c r="B32" s="12" t="inlineStr">
         <is>
-          <t>Livre de paie individuel / bulletins</t>
+          <t>Liasse fiscale / bilan 2025 déposé et preuve de paiement IBS</t>
         </is>
       </c>
       <c r="C32" s="12" t="inlineStr">
         <is>
-          <t>Les deux</t>
+          <t>Société</t>
         </is>
       </c>
       <c r="D32" s="12" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="E32" s="46" t="inlineStr">
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E32" s="47" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
       </c>
       <c r="F32" s="12" t="inlineStr">
         <is>
-          <t>Pour contrôle IRG</t>
+          <t>Voir A20, A21</t>
         </is>
       </c>
     </row>
@@ -7223,27 +8608,27 @@
       </c>
       <c r="B33" s="12" t="inlineStr">
         <is>
-          <t>Ordres de mission et justificatifs de frais</t>
+          <t>PV de caisse au 31/12/2025</t>
         </is>
       </c>
       <c r="C33" s="12" t="inlineStr">
         <is>
-          <t>TPM</t>
+          <t>Société</t>
         </is>
       </c>
       <c r="D33" s="12" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="E33" s="46" t="inlineStr">
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E33" s="47" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
       </c>
       <c r="F33" s="12" t="inlineStr">
         <is>
-          <t>Frais de mission élevés</t>
+          <t>Voir A22</t>
         </is>
       </c>
     </row>
@@ -7253,25 +8638,111 @@
       </c>
       <c r="B34" s="12" t="inlineStr">
         <is>
+          <t>Déclarations et paiements CACOBATPH</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="inlineStr">
+        <is>
+          <t>Les deux</t>
+        </is>
+      </c>
+      <c r="D34" s="12" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E34" s="47" t="inlineStr">
+        <is>
+          <t>Manquante</t>
+        </is>
+      </c>
+      <c r="F34" s="12" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>Livre de paie individuel / bulletins</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="inlineStr">
+        <is>
+          <t>Les deux</t>
+        </is>
+      </c>
+      <c r="D35" s="12" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E35" s="47" t="inlineStr">
+        <is>
+          <t>Manquante</t>
+        </is>
+      </c>
+      <c r="F35" s="12" t="inlineStr">
+        <is>
+          <t>Pour contrôle IRG</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>Ordres de mission et justificatifs de frais</t>
+        </is>
+      </c>
+      <c r="C36" s="12" t="inlineStr">
+        <is>
+          <t>TPM</t>
+        </is>
+      </c>
+      <c r="D36" s="12" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E36" s="47" t="inlineStr">
+        <is>
+          <t>Manquante</t>
+        </is>
+      </c>
+      <c r="F36" s="12" t="inlineStr">
+        <is>
+          <t>Frais de mission élevés</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="12" t="inlineStr">
+        <is>
           <t>Relevés bancaires — virements de salaires</t>
         </is>
       </c>
-      <c r="C34" s="12" t="inlineStr">
+      <c r="C37" s="12" t="inlineStr">
         <is>
           <t>Les deux</t>
         </is>
       </c>
-      <c r="D34" s="12" t="inlineStr">
+      <c r="D37" s="12" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="E34" s="46" t="inlineStr">
+      <c r="E37" s="47" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
       </c>
-      <c r="F34" s="12" t="inlineStr">
+      <c r="F37" s="12" t="inlineStr">
         <is>
           <t>Pour lettrage du 421</t>
         </is>

</xml_diff>

<commit_message>
Dossier comptable : G50 TPM janvier-mars 2026
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XYis4EzVZMNdoYCxmLrRh4
</commit_message>
<xml_diff>
--- a/DOSSIER_COMPTABLE_SARL_DPR_COMPAGNY_2026.xlsx
+++ b/DOSSIER_COMPTABLE_SARL_DPR_COMPAGNY_2026.xlsx
@@ -1124,11 +1124,11 @@
     <row r="37">
       <c r="A37" s="12" t="inlineStr">
         <is>
-          <t>G50 TPM avr.–août : totaux</t>
+          <t>G50 TPM janv.–août : totaux</t>
         </is>
       </c>
       <c r="B37" s="4">
-        <f>IF(ABS('G50 TPM 2026'!G20)&lt;1,"OK","ÉCART")</f>
+        <f>IF(SUMPRODUCT(ABS('G50 TPM 2026'!B20:I20))&lt;1,"OK","ÉCART")</f>
         <v/>
       </c>
     </row>
@@ -1284,7 +1284,7 @@
       </c>
       <c r="B49" s="12" t="inlineStr">
         <is>
-          <t>Contrôle des G50 TPM et location (avr.–août)</t>
+          <t>Contrôle des G50 TPM et location (janv.–août)</t>
         </is>
       </c>
       <c r="C49" s="17" t="n"/>
@@ -4682,17 +4682,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="54" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="48" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4705,7 +4708,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Sources : G50_04 à 08-2026_TPM_ET_LOCATION_CONSOLIDE.xls. Activité portée : transport et distribution de toutes marchandises.</t>
+          <t>Sources : G50_01 à 08-2026_TPM_ET_LOCATION_CONSOLIDE.xls. Activité portée : transport et distribution de toutes marchandises.</t>
         </is>
       </c>
     </row>
@@ -4717,35 +4720,50 @@
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
+          <t>Janv 2026</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>Févr 2026</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>Mars 2026</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
           <t>Avril 2026</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="F4" s="11" t="inlineStr">
         <is>
           <t>Mai 2026</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="G4" s="11" t="inlineStr">
         <is>
           <t>Juin 2026</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
-        <is>
-          <t>Juillet 2026</t>
-        </is>
-      </c>
-      <c r="F4" s="11" t="inlineStr">
+      <c r="H4" s="11" t="inlineStr">
+        <is>
+          <t>Juil 2026</t>
+        </is>
+      </c>
+      <c r="I4" s="11" t="inlineStr">
         <is>
           <t>Août 2026</t>
         </is>
       </c>
-      <c r="G4" s="11" t="inlineStr">
+      <c r="J4" s="11" t="inlineStr">
         <is>
           <t>Cumul</t>
         </is>
       </c>
-      <c r="H4" s="11" t="inlineStr">
+      <c r="K4" s="11" t="inlineStr">
         <is>
           <t>Commentaire</t>
         </is>
@@ -4759,31 +4777,46 @@
       </c>
       <c r="B5" s="22" t="inlineStr">
         <is>
+          <t>JANVIER</t>
+        </is>
+      </c>
+      <c r="C5" s="22" t="inlineStr">
+        <is>
+          <t>FEVRIER</t>
+        </is>
+      </c>
+      <c r="D5" s="22" t="inlineStr">
+        <is>
+          <t>MARS</t>
+        </is>
+      </c>
+      <c r="E5" s="22" t="inlineStr">
+        <is>
           <t>AVRIL</t>
         </is>
       </c>
-      <c r="C5" s="22" t="inlineStr">
+      <c r="F5" s="22" t="inlineStr">
         <is>
           <t>AVRIL</t>
         </is>
       </c>
-      <c r="D5" s="22" t="inlineStr">
+      <c r="G5" s="22" t="inlineStr">
         <is>
           <t>AVRIL</t>
         </is>
       </c>
-      <c r="E5" s="22" t="inlineStr">
+      <c r="H5" s="22" t="inlineStr">
         <is>
           <t>AVRIL</t>
         </is>
       </c>
-      <c r="F5" s="22" t="inlineStr">
+      <c r="I5" s="22" t="inlineStr">
         <is>
           <t>AOUT</t>
         </is>
       </c>
-      <c r="G5" s="27" t="n"/>
-      <c r="H5" s="35" t="inlineStr">
+      <c r="J5" s="27" t="n"/>
+      <c r="K5" s="35" t="inlineStr">
         <is>
           <t>Avril à juillet : même G50 recopiée (mois « AVRIL »)</t>
         </is>
@@ -4810,11 +4843,20 @@
       <c r="F6" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="7">
-        <f>SUM(B6:F6)</f>
-        <v/>
-      </c>
-      <c r="H6" s="35" t="inlineStr">
+      <c r="G6" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="7">
+        <f>SUM(B6:I6)</f>
+        <v/>
+      </c>
+      <c r="K6" s="35" t="inlineStr">
         <is>
           <t>Aucun CA TPM / location déclaré</t>
         </is>
@@ -4841,11 +4883,20 @@
       <c r="F7" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="7">
-        <f>SUM(B7:F7)</f>
-        <v/>
-      </c>
-      <c r="H7" s="35" t="inlineStr"/>
+      <c r="G7" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="7">
+        <f>SUM(B7:I7)</f>
+        <v/>
+      </c>
+      <c r="K7" s="35" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
@@ -4868,8 +4919,17 @@
       <c r="F8" s="25" t="n">
         <v>1714499</v>
       </c>
-      <c r="G8" s="27" t="n"/>
-      <c r="H8" s="35" t="inlineStr"/>
+      <c r="G8" s="25" t="n">
+        <v>1714499</v>
+      </c>
+      <c r="H8" s="25" t="n">
+        <v>1714499</v>
+      </c>
+      <c r="I8" s="25" t="n">
+        <v>1714499</v>
+      </c>
+      <c r="J8" s="27" t="n"/>
+      <c r="K8" s="35" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -4892,8 +4952,17 @@
       <c r="F9" s="25" t="n">
         <v>1714499</v>
       </c>
-      <c r="G9" s="27" t="n"/>
-      <c r="H9" s="35" t="inlineStr"/>
+      <c r="G9" s="25" t="n">
+        <v>1714499</v>
+      </c>
+      <c r="H9" s="25" t="n">
+        <v>1714499</v>
+      </c>
+      <c r="I9" s="25" t="n">
+        <v>1714499</v>
+      </c>
+      <c r="J9" s="27" t="n"/>
+      <c r="K9" s="35" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
@@ -4921,8 +4990,20 @@
         <f>'Balance 2024-2025'!D49</f>
         <v/>
       </c>
-      <c r="G10" s="27" t="n"/>
-      <c r="H10" s="35" t="inlineStr">
+      <c r="G10" s="6">
+        <f>'Balance 2024-2025'!D49</f>
+        <v/>
+      </c>
+      <c r="H10" s="6">
+        <f>'Balance 2024-2025'!D49</f>
+        <v/>
+      </c>
+      <c r="I10" s="6">
+        <f>'Balance 2024-2025'!D49</f>
+        <v/>
+      </c>
+      <c r="J10" s="27" t="n"/>
+      <c r="K10" s="35" t="inlineStr">
         <is>
           <t>Identique : crédit reporté depuis 2025</t>
         </is>
@@ -4935,25 +5016,34 @@
         </is>
       </c>
       <c r="B11" s="25" t="n">
-        <v>91763</v>
+        <v>47391</v>
       </c>
       <c r="C11" s="25" t="n">
-        <v>91763</v>
+        <v>62527</v>
       </c>
       <c r="D11" s="25" t="n">
-        <v>91763</v>
+        <v>85300</v>
       </c>
       <c r="E11" s="25" t="n">
         <v>91763</v>
       </c>
       <c r="F11" s="25" t="n">
+        <v>91763</v>
+      </c>
+      <c r="G11" s="25" t="n">
+        <v>91763</v>
+      </c>
+      <c r="H11" s="25" t="n">
+        <v>91763</v>
+      </c>
+      <c r="I11" s="25" t="n">
         <v>42190</v>
       </c>
-      <c r="G11" s="7">
-        <f>SUM(B11:F11)</f>
-        <v/>
-      </c>
-      <c r="H11" s="35" t="inlineStr"/>
+      <c r="J11" s="7">
+        <f>SUM(B11:I11)</f>
+        <v/>
+      </c>
+      <c r="K11" s="35" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
@@ -4962,30 +5052,42 @@
         </is>
       </c>
       <c r="B12" s="6">
+        <f>'Paie TPM'!C24</f>
+        <v/>
+      </c>
+      <c r="C12" s="6">
+        <f>'Paie TPM'!D24</f>
+        <v/>
+      </c>
+      <c r="D12" s="6">
+        <f>'Paie TPM'!E24</f>
+        <v/>
+      </c>
+      <c r="E12" s="6">
         <f>'Paie TPM'!F24</f>
         <v/>
       </c>
-      <c r="C12" s="6">
+      <c r="F12" s="6">
         <f>'Paie TPM'!G24</f>
         <v/>
       </c>
-      <c r="D12" s="6">
+      <c r="G12" s="6">
         <f>'Paie TPM'!H24</f>
         <v/>
       </c>
-      <c r="E12" s="6">
+      <c r="H12" s="6">
         <f>'Paie TPM'!I24</f>
         <v/>
       </c>
-      <c r="F12" s="6">
+      <c r="I12" s="6">
         <f>'Paie TPM'!J24</f>
         <v/>
       </c>
-      <c r="G12" s="7">
-        <f>SUM(B12:F12)</f>
-        <v/>
-      </c>
-      <c r="H12" s="35" t="inlineStr">
+      <c r="J12" s="7">
+        <f>SUM(B12:I12)</f>
+        <v/>
+      </c>
+      <c r="K12" s="35" t="inlineStr">
         <is>
           <t>Lien paie</t>
         </is>
@@ -4998,25 +5100,34 @@
         </is>
       </c>
       <c r="B13" s="25" t="n">
-        <v>9375</v>
+        <v>3330</v>
       </c>
       <c r="C13" s="25" t="n">
-        <v>9375</v>
+        <v>3330</v>
       </c>
       <c r="D13" s="25" t="n">
-        <v>9375</v>
+        <v>7757</v>
       </c>
       <c r="E13" s="25" t="n">
         <v>9375</v>
       </c>
       <c r="F13" s="25" t="n">
+        <v>9375</v>
+      </c>
+      <c r="G13" s="25" t="n">
+        <v>9375</v>
+      </c>
+      <c r="H13" s="25" t="n">
+        <v>9375</v>
+      </c>
+      <c r="I13" s="25" t="n">
         <v>3690</v>
       </c>
-      <c r="G13" s="7">
-        <f>SUM(B13:F13)</f>
-        <v/>
-      </c>
-      <c r="H13" s="35" t="inlineStr"/>
+      <c r="J13" s="7">
+        <f>SUM(B13:I13)</f>
+        <v/>
+      </c>
+      <c r="K13" s="35" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
@@ -5025,30 +5136,42 @@
         </is>
       </c>
       <c r="B14" s="6">
+        <f>'Paie TPM'!C25</f>
+        <v/>
+      </c>
+      <c r="C14" s="6">
+        <f>'Paie TPM'!D25</f>
+        <v/>
+      </c>
+      <c r="D14" s="6">
+        <f>'Paie TPM'!E25</f>
+        <v/>
+      </c>
+      <c r="E14" s="6">
         <f>'Paie TPM'!F25</f>
         <v/>
       </c>
-      <c r="C14" s="6">
+      <c r="F14" s="6">
         <f>'Paie TPM'!G25</f>
         <v/>
       </c>
-      <c r="D14" s="6">
+      <c r="G14" s="6">
         <f>'Paie TPM'!H25</f>
         <v/>
       </c>
-      <c r="E14" s="6">
+      <c r="H14" s="6">
         <f>'Paie TPM'!I25</f>
         <v/>
       </c>
-      <c r="F14" s="6">
+      <c r="I14" s="6">
         <f>'Paie TPM'!J25</f>
         <v/>
       </c>
-      <c r="G14" s="7">
-        <f>SUM(B14:F14)</f>
-        <v/>
-      </c>
-      <c r="H14" s="35" t="inlineStr">
+      <c r="J14" s="7">
+        <f>SUM(B14:I14)</f>
+        <v/>
+      </c>
+      <c r="K14" s="35" t="inlineStr">
         <is>
           <t>Lien paie</t>
         </is>
@@ -5080,11 +5203,23 @@
         <f>F13-F14</f>
         <v/>
       </c>
-      <c r="G15" s="7">
-        <f>SUM(B15:F15)</f>
-        <v/>
-      </c>
-      <c r="H15" s="35" t="inlineStr">
+      <c r="G15" s="30">
+        <f>G13-G14</f>
+        <v/>
+      </c>
+      <c r="H15" s="30">
+        <f>H13-H14</f>
+        <v/>
+      </c>
+      <c r="I15" s="30">
+        <f>I13-I14</f>
+        <v/>
+      </c>
+      <c r="J15" s="7">
+        <f>SUM(B15:I15)</f>
+        <v/>
+      </c>
+      <c r="K15" s="35" t="inlineStr">
         <is>
           <t>Négatif = IRG retenu non reversé</t>
         </is>
@@ -5100,7 +5235,7 @@
         <v>0</v>
       </c>
       <c r="C16" s="25" t="n">
-        <v>0</v>
+        <v>985118</v>
       </c>
       <c r="D16" s="25" t="n">
         <v>0</v>
@@ -5109,15 +5244,24 @@
         <v>0</v>
       </c>
       <c r="F16" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="25" t="n">
         <v>680900</v>
       </c>
-      <c r="G16" s="7">
-        <f>SUM(B16:F16)</f>
-        <v/>
-      </c>
-      <c r="H16" s="35" t="inlineStr">
-        <is>
-          <t>Base à justifier</t>
+      <c r="J16" s="7">
+        <f>SUM(B16:I16)</f>
+        <v/>
+      </c>
+      <c r="K16" s="35" t="inlineStr">
+        <is>
+          <t>Payée en février et en août : bases à justifier</t>
         </is>
       </c>
     </row>
@@ -5131,7 +5275,7 @@
         <v>0</v>
       </c>
       <c r="C17" s="25" t="n">
-        <v>0</v>
+        <v>9851</v>
       </c>
       <c r="D17" s="25" t="n">
         <v>0</v>
@@ -5140,13 +5284,22 @@
         <v>0</v>
       </c>
       <c r="F17" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="25" t="n">
         <v>6809</v>
       </c>
-      <c r="G17" s="7">
-        <f>SUM(B17:F17)</f>
-        <v/>
-      </c>
-      <c r="H17" s="35" t="inlineStr"/>
+      <c r="J17" s="7">
+        <f>SUM(B17:I17)</f>
+        <v/>
+      </c>
+      <c r="K17" s="35" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -5155,25 +5308,34 @@
         </is>
       </c>
       <c r="B18" s="25" t="n">
-        <v>9375</v>
+        <v>3330</v>
       </c>
       <c r="C18" s="25" t="n">
-        <v>9375</v>
+        <v>13181</v>
       </c>
       <c r="D18" s="25" t="n">
-        <v>9375</v>
+        <v>7757</v>
       </c>
       <c r="E18" s="25" t="n">
         <v>9375</v>
       </c>
       <c r="F18" s="25" t="n">
+        <v>9375</v>
+      </c>
+      <c r="G18" s="25" t="n">
+        <v>9375</v>
+      </c>
+      <c r="H18" s="25" t="n">
+        <v>9375</v>
+      </c>
+      <c r="I18" s="25" t="n">
         <v>10499</v>
       </c>
-      <c r="G18" s="7">
-        <f>SUM(B18:F18)</f>
-        <v/>
-      </c>
-      <c r="H18" s="35" t="inlineStr"/>
+      <c r="J18" s="7">
+        <f>SUM(B18:I18)</f>
+        <v/>
+      </c>
+      <c r="K18" s="35" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -5201,11 +5363,23 @@
         <f>MAX(0,F7-F8)+F13+F17</f>
         <v/>
       </c>
-      <c r="G19" s="7">
-        <f>SUM(B19:F19)</f>
-        <v/>
-      </c>
-      <c r="H19" s="35" t="inlineStr">
+      <c r="G19" s="30">
+        <f>MAX(0,G7-G8)+G13+G17</f>
+        <v/>
+      </c>
+      <c r="H19" s="30">
+        <f>MAX(0,H7-H8)+H13+H17</f>
+        <v/>
+      </c>
+      <c r="I19" s="30">
+        <f>MAX(0,I7-I8)+I13+I17</f>
+        <v/>
+      </c>
+      <c r="J19" s="7">
+        <f>SUM(B19:I19)</f>
+        <v/>
+      </c>
+      <c r="K19" s="35" t="inlineStr">
         <is>
           <t>Calcul</t>
         </is>
@@ -5237,11 +5411,23 @@
         <f>F18-F19</f>
         <v/>
       </c>
-      <c r="G20" s="7">
-        <f>SUM(B20:F20)</f>
-        <v/>
-      </c>
-      <c r="H20" s="35" t="inlineStr">
+      <c r="G20" s="30">
+        <f>G18-G19</f>
+        <v/>
+      </c>
+      <c r="H20" s="30">
+        <f>H18-H19</f>
+        <v/>
+      </c>
+      <c r="I20" s="30">
+        <f>I18-I19</f>
+        <v/>
+      </c>
+      <c r="J20" s="7">
+        <f>SUM(B20:I20)</f>
+        <v/>
+      </c>
+      <c r="K20" s="35" t="inlineStr">
         <is>
           <t>Doit être 0</t>
         </is>
@@ -5257,7 +5443,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>G50 TPM de janvier à mars 2026 non fournies (IRG paie TPM sur la période : voir « Paie TPM »).</t>
+          <t>Janvier à mars : G50 conformes à la paie TPM (écarts d'arrondi &lt; 1 DA).</t>
         </is>
       </c>
     </row>
@@ -7162,16 +7348,16 @@
       </c>
       <c r="E23" s="29" t="inlineStr">
         <is>
-          <t>G50 TPM d'avril à juillet identiques (mois imprimé « AVRIL », IRG 9 375 chaque mois) : juin sous-déclaré de 9 614,90 (18 989,90 retenus), juillet sur-déclaré de 5 683,70 ; août conforme. G50 TPM de janvier à mars non fournies.</t>
+          <t>G50 TPM d'avril à juillet identiques (mois imprimé « AVRIL », IRG 9 375 chaque mois) : juin sous-déclaré de 9 614,90 (18 989,90 retenus), juillet sur-déclaré de 5 683,70. Janvier–mars et août conformes.</t>
         </is>
       </c>
       <c r="F23" s="41">
-        <f>-'G50 TPM 2026'!D15</f>
+        <f>-'G50 TPM 2026'!G15</f>
         <v/>
       </c>
       <c r="G23" s="29" t="inlineStr">
         <is>
-          <t>Déposer une G50 rectificative pour juin (IRG retenu non reversé) et régulariser juillet ; fournir les G50 TPM janv.–mars.</t>
+          <t>Déposer une G50 rectificative pour juin (IRG retenu non reversé) et régulariser juillet.</t>
         </is>
       </c>
       <c r="H23" s="42" t="n"/>
@@ -7557,11 +7743,11 @@
       </c>
       <c r="E33" s="29" t="inlineStr">
         <is>
-          <t>Taxe d'apprentissage payée deux fois en 2026 : février (87 828 sur 8 782 828) et août (44 091 IMPORT sur 4 409 079 + 6 809 TPM sur 680 900).</t>
+          <t>Taxe d'apprentissage payée deux fois en 2026 : février (87 828 IMPORT sur 8 782 828 + 9 851 TPM sur 985 118) et août (44 091 IMPORT sur 4 409 079 + 6 809 TPM sur 680 900).</t>
         </is>
       </c>
       <c r="F33" s="41">
-        <f>'G50 2026'!J26+'G50 TPM 2026'!G17</f>
+        <f>'G50 2026'!J26+'G50 TPM 2026'!J17</f>
         <v/>
       </c>
       <c r="G33" s="29" t="inlineStr">
@@ -8398,7 +8584,7 @@
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>G50 TPM et location janvier à mars 2026</t>
+          <t>G50_01/02/03-2026_TPM_ET_LOCATION_CONSOLIDE.xls</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
@@ -8408,17 +8594,17 @@
       </c>
       <c r="D26" s="12" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="E26" s="47" t="inlineStr">
-        <is>
-          <t>Manquante</t>
+          <t>Janvier, février, mars 2026</t>
+        </is>
+      </c>
+      <c r="E26" s="46" t="inlineStr">
+        <is>
+          <t>Reçue</t>
         </is>
       </c>
       <c r="F26" s="12" t="inlineStr">
         <is>
-          <t>Voir A19</t>
+          <t>Conformes à la paie</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dossier comptable : contrôle de l'extrait du registre de commerce
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XYis4EzVZMNdoYCxmLrRh4
</commit_message>
<xml_diff>
--- a/DOSSIER_COMPTABLE_SARL_DPR_COMPAGNY_2026.xlsx
+++ b/DOSSIER_COMPTABLE_SARL_DPR_COMPAGNY_2026.xlsx
@@ -22,14 +22,15 @@
     <sheet name="Contrôle 2023" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="Clients &amp; fournisseurs" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="Démarrage 2026" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Anomalies &amp; actions" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Pièces" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Registre de commerce" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Anomalies &amp; actions" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Pièces" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Journal paie'!$A$4:$G$140</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Balance 2024-2025'!$A$4:$E$104</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Clients &amp; fournisseurs'!$A$21:$L$243</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Anomalies &amp; actions'!$A$4:$I$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Anomalies &amp; actions'!$A$4:$I$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -37,10 +38,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="#,##0;(#,##0);&quot;-&quot;"/>
     <numFmt numFmtId="166" formatCode="#,##0.00;(#,##0.00);&quot;-&quot;"/>
+    <numFmt numFmtId="167" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -207,7 +209,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -257,6 +259,20 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -684,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D63"/>
+  <dimension ref="A1:D64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -991,11 +1007,11 @@
         </is>
       </c>
       <c r="B24" s="13">
-        <f>COUNTIF('Anomalies &amp; actions'!B5:B40,1)</f>
+        <f>COUNTIF('Anomalies &amp; actions'!B5:B44,1)</f>
         <v/>
       </c>
       <c r="C24" s="13">
-        <f>COUNTIFS('Anomalies &amp; actions'!B5:B40,1,'Anomalies &amp; actions'!I5:I40,"Ouvert")</f>
+        <f>COUNTIFS('Anomalies &amp; actions'!B5:B44,1,'Anomalies &amp; actions'!I5:I44,"Ouvert")</f>
         <v/>
       </c>
     </row>
@@ -1006,11 +1022,11 @@
         </is>
       </c>
       <c r="B25" s="13">
-        <f>COUNTIF('Anomalies &amp; actions'!B5:B40,2)</f>
+        <f>COUNTIF('Anomalies &amp; actions'!B5:B44,2)</f>
         <v/>
       </c>
       <c r="C25" s="13">
-        <f>COUNTIFS('Anomalies &amp; actions'!B5:B40,2,'Anomalies &amp; actions'!I5:I40,"Ouvert")</f>
+        <f>COUNTIFS('Anomalies &amp; actions'!B5:B44,2,'Anomalies &amp; actions'!I5:I44,"Ouvert")</f>
         <v/>
       </c>
     </row>
@@ -1021,11 +1037,11 @@
         </is>
       </c>
       <c r="B26" s="13">
-        <f>COUNTIF('Anomalies &amp; actions'!B5:B40,3)</f>
+        <f>COUNTIF('Anomalies &amp; actions'!B5:B44,3)</f>
         <v/>
       </c>
       <c r="C26" s="13">
-        <f>COUNTIFS('Anomalies &amp; actions'!B5:B40,3,'Anomalies &amp; actions'!I5:I40,"Ouvert")</f>
+        <f>COUNTIFS('Anomalies &amp; actions'!B5:B44,3,'Anomalies &amp; actions'!I5:I44,"Ouvert")</f>
         <v/>
       </c>
     </row>
@@ -1339,12 +1355,12 @@
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>Balance 2024-2025</t>
+          <t>Registre de commerce</t>
         </is>
       </c>
       <c r="B53" s="12" t="inlineStr">
         <is>
-          <t>Balance générale issue des journaux PCCOMPTA</t>
+          <t>Extrait CNRC : activités inscrites, gérants, validité</t>
         </is>
       </c>
       <c r="C53" s="17" t="n"/>
@@ -1353,84 +1369,79 @@
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>États 2024-2025</t>
+          <t>Balance 2024-2025</t>
         </is>
       </c>
       <c r="B54" s="12" t="inlineStr">
         <is>
-          <t>Compte de résultat et bilan simplifiés, indicateurs</t>
+          <t>Balance générale issue des journaux PCCOMPTA</t>
         </is>
       </c>
       <c r="C54" s="17" t="n"/>
       <c r="D54" s="18" t="n"/>
     </row>
-    <row r="57">
-      <c r="A57" s="2" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>États 2024-2025</t>
+        </is>
+      </c>
+      <c r="B55" s="12" t="inlineStr">
+        <is>
+          <t>Compte de résultat et bilan simplifiés, indicateurs</t>
+        </is>
+      </c>
+      <c r="C55" s="17" t="n"/>
+      <c r="D55" s="18" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>Légende : bleu = saisie depuis une pièce ; vert = lien vers une autre feuille ; noir = calcul ; fond jaune = à compléter.</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="10" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="10" t="inlineStr">
         <is>
           <t>Exercices comptables</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="11" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="11" t="inlineStr">
         <is>
           <t>Indicateur</t>
         </is>
       </c>
-      <c r="B60" s="11" t="inlineStr">
+      <c r="B61" s="11" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="C60" s="11" t="inlineStr">
+      <c r="C61" s="11" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="D60" s="11" t="inlineStr">
+      <c r="D61" s="11" t="inlineStr">
         <is>
           <t>Variation</t>
         </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="4" t="inlineStr">
-        <is>
-          <t>Chiffre d'affaires</t>
-        </is>
-      </c>
-      <c r="B61" s="6">
-        <f>'États 2024-2025'!C5</f>
-        <v/>
-      </c>
-      <c r="C61" s="6">
-        <f>'États 2024-2025'!D5</f>
-        <v/>
-      </c>
-      <c r="D61" s="19">
-        <f>IF(B61=0,"",C61/B61-1)</f>
-        <v/>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>Charges de personnel</t>
+          <t>Chiffre d'affaires</t>
         </is>
       </c>
       <c r="B62" s="6">
-        <f>'États 2024-2025'!C10</f>
+        <f>'États 2024-2025'!C5</f>
         <v/>
       </c>
       <c r="C62" s="6">
-        <f>'États 2024-2025'!D10</f>
+        <f>'États 2024-2025'!D5</f>
         <v/>
       </c>
       <c r="D62" s="19">
@@ -1441,15 +1452,15 @@
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>Résultat net</t>
+          <t>Charges de personnel</t>
         </is>
       </c>
       <c r="B63" s="6">
-        <f>'États 2024-2025'!C16</f>
+        <f>'États 2024-2025'!C10</f>
         <v/>
       </c>
       <c r="C63" s="6">
-        <f>'États 2024-2025'!D16</f>
+        <f>'États 2024-2025'!D10</f>
         <v/>
       </c>
       <c r="D63" s="19">
@@ -1457,8 +1468,27 @@
         <v/>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>Résultat net</t>
+        </is>
+      </c>
+      <c r="B64" s="6">
+        <f>'États 2024-2025'!C16</f>
+        <v/>
+      </c>
+      <c r="C64" s="6">
+        <f>'États 2024-2025'!D16</f>
+        <v/>
+      </c>
+      <c r="D64" s="19">
+        <f>IF(B64=0,"",C64/B64-1)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="16">
     <mergeCell ref="B42:D42"/>
     <mergeCell ref="B54:D54"/>
     <mergeCell ref="B45:D45"/>
@@ -1471,6 +1501,7 @@
     <mergeCell ref="B44:D44"/>
     <mergeCell ref="B53:D53"/>
     <mergeCell ref="B43:D43"/>
+    <mergeCell ref="B55:D55"/>
     <mergeCell ref="B51:D51"/>
     <mergeCell ref="B47:D47"/>
     <mergeCell ref="B48:D48"/>
@@ -17479,7 +17510,381 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:C29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Extrait du registre de commerce (CNRC) — contrôle de conformité</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Source : SDOC-607B666B93EEF055F89FE8EC0A5E7DF1-11-30-SI.pdf (scan CamScanner, en arabe), extrait n° de série 700267695 délivré par l'antenne CNRC de Béjaïa le 10/09/2024.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Rubrique</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>Mention de l'extrait (traduction)</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>Contrôle / constat</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Dénomination</t>
+        </is>
+      </c>
+      <c r="B5" s="43" t="inlineStr">
+        <is>
+          <t>D.P.R. COMPAGNY</t>
+        </is>
+      </c>
+      <c r="C5" s="29" t="inlineStr">
+        <is>
+          <t>Conforme aux déclarations CNAS et G50</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Forme juridique</t>
+        </is>
+      </c>
+      <c r="B6" s="43" t="inlineStr">
+        <is>
+          <t>Société à responsabilité limitée (SARL)</t>
+        </is>
+      </c>
+      <c r="C6" s="29" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="32" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>N° du registre de commerce</t>
+        </is>
+      </c>
+      <c r="B7" s="43" t="inlineStr">
+        <is>
+          <t>06/00-0184232 B 03</t>
+        </is>
+      </c>
+      <c r="C7" s="29" t="inlineStr">
+        <is>
+          <t>Le dossier comptable (PCCOMPTA) porte 06/01-0184232B03 : à corriger</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Siège social</t>
+        </is>
+      </c>
+      <c r="B8" s="43" t="inlineStr">
+        <is>
+          <t>Lieu-dit Tizi, commune de Semaoun, wilaya de Béjaïa</t>
+        </is>
+      </c>
+      <c r="C8" s="29" t="inlineStr">
+        <is>
+          <t>Conforme (VGE TIZI). Aucun établissement secondaire inscrit</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Capital social</t>
+        </is>
+      </c>
+      <c r="B9" s="43" t="inlineStr">
+        <is>
+          <t>106 000 000,00 DA</t>
+        </is>
+      </c>
+      <c r="C9" s="29">
+        <f>IF(ABS(-'Balance 2024-2025'!D5-106000000)&lt;1,"Conforme au compte 10100","Écart avec le compte 10100")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Date de début d'activité</t>
+        </is>
+      </c>
+      <c r="B10" s="43" t="inlineStr">
+        <is>
+          <t>16/04/2003</t>
+        </is>
+      </c>
+      <c r="C10" s="29" t="inlineStr"/>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Fonds de commerce</t>
+        </is>
+      </c>
+      <c r="B11" s="43" t="inlineStr">
+        <is>
+          <t>Création</t>
+        </is>
+      </c>
+      <c r="C11" s="29" t="inlineStr"/>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Propriétaire du local commercial</t>
+        </is>
+      </c>
+      <c r="B12" s="43" t="inlineStr">
+        <is>
+          <t>DJENNADI Abdelkader</t>
+        </is>
+      </c>
+      <c r="C12" s="29" t="inlineStr">
+        <is>
+          <t>Figure en fournisseur 401 (dette de 2 510 665 sans mouvement en 2025) : bail et loyers à justifier</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Nombre d'établissements secondaires</t>
+        </is>
+      </c>
+      <c r="B13" s="43" t="inlineStr">
+        <is>
+          <t>Néant (non renseigné)</t>
+        </is>
+      </c>
+      <c r="C13" s="29" t="inlineStr">
+        <is>
+          <t>Or affiliation CNAS TPM distincte à TISSA (n° 06736613 53) : établissement secondaire non inscrit</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Gérants associés</t>
+        </is>
+      </c>
+      <c r="B14" s="43" t="inlineStr">
+        <is>
+          <t>DJENNADI Abdelkrim (né le 22/04/1975), DJENNADI Ryad (né le 18/01/1978), DJENNADI Ahcene (né le 08/03/1972), nationalité algérienne</t>
+        </is>
+      </c>
+      <c r="C14" s="29" t="inlineStr">
+        <is>
+          <t>Confirme que leurs soldes en 411 / 419 sont des comptes d'associés (A36)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Secteur d'activité</t>
+        </is>
+      </c>
+      <c r="B15" s="43" t="inlineStr">
+        <is>
+          <t>Importation pour la revente en l'état</t>
+        </is>
+      </c>
+      <c r="C15" s="29" t="inlineStr"/>
+    </row>
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Activité 442101</t>
+        </is>
+      </c>
+      <c r="B16" s="43" t="inlineStr">
+        <is>
+          <t>Importation d'équipements, pièces de rechange et accessoires liés au domaine mécanique</t>
+        </is>
+      </c>
+      <c r="C16" s="29" t="inlineStr"/>
+    </row>
+    <row r="17" ht="32" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Activité 442102</t>
+        </is>
+      </c>
+      <c r="B17" s="43" t="inlineStr">
+        <is>
+          <t>Importation de pièces de rechange et accessoires automobiles</t>
+        </is>
+      </c>
+      <c r="C17" s="29" t="inlineStr"/>
+    </row>
+    <row r="18" ht="32" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Activité 442103</t>
+        </is>
+      </c>
+      <c r="B18" s="43" t="inlineStr">
+        <is>
+          <t>Importation de pneumatiques</t>
+        </is>
+      </c>
+      <c r="C18" s="29" t="inlineStr"/>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Activité 442104</t>
+        </is>
+      </c>
+      <c r="B19" s="43" t="inlineStr">
+        <is>
+          <t>Importation de batteries liées au domaine mécanique</t>
+        </is>
+      </c>
+      <c r="C19" s="29" t="inlineStr"/>
+    </row>
+    <row r="20" ht="32" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Activités exercées NON inscrites</t>
+        </is>
+      </c>
+      <c r="B20" s="43" t="inlineStr">
+        <is>
+          <t>Travaux publics / TPM, location d'engins, transport et distribution de marchandises</t>
+        </is>
+      </c>
+      <c r="C20" s="29" t="inlineStr">
+        <is>
+          <t>Exercées et facturées (70602 : 25,5 M en 2025 ; G50 « TPM et location » ; CNAS TPM) hors objet du registre</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="32" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Date de la dernière modification</t>
+        </is>
+      </c>
+      <c r="B21" s="43" t="inlineStr">
+        <is>
+          <t>10/09/2024</t>
+        </is>
+      </c>
+      <c r="C21" s="29" t="inlineStr"/>
+    </row>
+    <row r="22" ht="32" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Durée de validité de l'extrait</t>
+        </is>
+      </c>
+      <c r="B22" s="43" t="inlineStr">
+        <is>
+          <t>Du 13/02/2024 au 13/02/2026</t>
+        </is>
+      </c>
+      <c r="C22" s="44">
+        <f>IF(B26&gt;0,"EXPIRÉ depuis le 13/02/2026 : renouvellement à faire immédiatement","Valide")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Fin de validité de l'extrait</t>
+        </is>
+      </c>
+      <c r="B24" s="45">
+        <f>DATE(2026,2,13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Date d'arrêté du dossier</t>
+        </is>
+      </c>
+      <c r="B25" s="45">
+        <f>DATE(2026,10,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Jours d'activité depuis l'expiration</t>
+        </is>
+      </c>
+      <c r="B26" s="46">
+        <f>MAX(0,B25-B24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="45" customHeight="1">
+      <c r="A28" s="47" t="inlineStr">
+        <is>
+          <t>Sanctions rappelées au verso de l'extrait (loi n° 04-08 du 14/08/2004 modifiée, art. 31 à 41 bis) : amende de 5 000 à 5 000 000 DA et/ou emprisonnement de 6 mois à 1 an, notamment pour exercice avec un extrait expiré, commerce hors de l'objet du registre et défaut de modification de l'extrait.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="45" customHeight="1">
+      <c r="A29" s="48" t="inlineStr">
+        <is>
+          <t>À vérifier avec un juriste : l'activité d'importation pour la revente en l'état est en principe réservée à des sociétés qui l'exercent à titre exclusif ; l'ajout des activités TPM / location au même registre peut ne pas être possible et imposer une structure distincte.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A28:C28"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -17560,7 +17965,7 @@
           <t>A01</t>
         </is>
       </c>
-      <c r="B5" s="43" t="n">
+      <c r="B5" s="49" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="29" t="inlineStr">
@@ -17578,7 +17983,7 @@
           <t>Déclaration CNAS de février 2026 non fournie (assiette paie 952 475,81 ; 7 STC payés).</t>
         </is>
       </c>
-      <c r="F5" s="44">
+      <c r="F5" s="50">
         <f>'Rappro CNAS'!J6</f>
         <v/>
       </c>
@@ -17600,7 +18005,7 @@
           <t>A02</t>
         </is>
       </c>
-      <c r="B6" s="43" t="n">
+      <c r="B6" s="49" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="29" t="inlineStr">
@@ -17618,7 +18023,7 @@
           <t>Centralisateur de mars 2026 absent (onglet vide) alors que la CNAS de mars déclare 368 389,93 d'assiette, 5 salariés.</t>
         </is>
       </c>
-      <c r="F6" s="44">
+      <c r="F6" s="50">
         <f>'Rappro CNAS'!K7</f>
         <v/>
       </c>
@@ -17640,7 +18045,7 @@
           <t>A03</t>
         </is>
       </c>
-      <c r="B7" s="43" t="n">
+      <c r="B7" s="49" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="29" t="inlineStr">
@@ -17658,7 +18063,7 @@
           <t>Prime de ponctualité (R540) imposée à l'IRG mais exclue du salaire de poste (assiette CNAS) chaque mois.</t>
         </is>
       </c>
-      <c r="F7" s="44">
+      <c r="F7" s="50">
         <f>'Rappro CNAS'!V13</f>
         <v/>
       </c>
@@ -17680,7 +18085,7 @@
           <t>A04</t>
         </is>
       </c>
-      <c r="B8" s="45" t="n">
+      <c r="B8" s="51" t="n">
         <v>2</v>
       </c>
       <c r="C8" s="29" t="inlineStr">
@@ -17698,7 +18103,7 @@
           <t>Effectif déclaré au T1 = 2 alors que 3 salariés sont inscrits ; T2 déclare 1 sortie et un effectif final de 2 ⇒ T1 aurait dû être 3.</t>
         </is>
       </c>
-      <c r="F8" s="46" t="n"/>
+      <c r="F8" s="52" t="n"/>
       <c r="G8" s="29" t="inlineStr">
         <is>
           <t>Rectifier l'effectif du T1 auprès de la CNAS.</t>
@@ -17717,7 +18122,7 @@
           <t>A05</t>
         </is>
       </c>
-      <c r="B9" s="45" t="n">
+      <c r="B9" s="51" t="n">
         <v>2</v>
       </c>
       <c r="C9" s="29" t="inlineStr">
@@ -17735,7 +18140,7 @@
           <t>Salarié totalement absent (non rémunéré) en juillet, disparu de la paie en août sans STC ni sortie déclarée.</t>
         </is>
       </c>
-      <c r="F9" s="46" t="n"/>
+      <c r="F9" s="52" t="n"/>
       <c r="G9" s="29" t="inlineStr">
         <is>
           <t>Établir le STC et déclarer la sortie dans l'EMS du T3 (échéance 30/10/2026).</t>
@@ -17754,7 +18159,7 @@
           <t>A06</t>
         </is>
       </c>
-      <c r="B10" s="45" t="n">
+      <c r="B10" s="51" t="n">
         <v>2</v>
       </c>
       <c r="C10" s="29" t="inlineStr">
@@ -17772,7 +18177,7 @@
           <t>STC de 2 237,40 en août : une sortie à déclarer au T3.</t>
         </is>
       </c>
-      <c r="F10" s="46" t="n"/>
+      <c r="F10" s="52" t="n"/>
       <c r="G10" s="29" t="inlineStr">
         <is>
           <t>Déclarer la sortie dans l'EMS du T3.</t>
@@ -17791,7 +18196,7 @@
           <t>A07</t>
         </is>
       </c>
-      <c r="B11" s="45" t="n">
+      <c r="B11" s="51" t="n">
         <v>2</v>
       </c>
       <c r="C11" s="29" t="inlineStr">
@@ -17809,7 +18214,7 @@
           <t>Déclarations T3 2026 (juil–sept) à établir ; paie de septembre non fournie.</t>
         </is>
       </c>
-      <c r="F11" s="44">
+      <c r="F11" s="50">
         <f>'Rappro CNAS'!J9+'Rappro CNAS'!J12</f>
         <v/>
       </c>
@@ -17831,7 +18236,7 @@
           <t>A08</t>
         </is>
       </c>
-      <c r="B12" s="47" t="n">
+      <c r="B12" s="53" t="n">
         <v>3</v>
       </c>
       <c r="C12" s="29" t="inlineStr">
@@ -17849,7 +18254,7 @@
           <t>Avril = mai et juillet = août strictement identiques (mêmes absences, heures sup., IRG) : variables probablement non saisies.</t>
         </is>
       </c>
-      <c r="F12" s="46" t="n"/>
+      <c r="F12" s="52" t="n"/>
       <c r="G12" s="29" t="inlineStr">
         <is>
           <t>Contrôler les pointages et bulletins de mai et août.</t>
@@ -17868,7 +18273,7 @@
           <t>A09</t>
         </is>
       </c>
-      <c r="B13" s="47" t="n">
+      <c r="B13" s="53" t="n">
         <v>3</v>
       </c>
       <c r="C13" s="29" t="inlineStr">
@@ -17886,7 +18291,7 @@
           <t>Frais de mission élevés (avril 41 615 ; mai 49 115, soit 47–55 % de l'assiette), non soumis à cotisations.</t>
         </is>
       </c>
-      <c r="F13" s="44">
+      <c r="F13" s="50">
         <f>'Paie TPM'!K26</f>
         <v/>
       </c>
@@ -17908,7 +18313,7 @@
           <t>A10</t>
         </is>
       </c>
-      <c r="B14" s="47" t="n">
+      <c r="B14" s="53" t="n">
         <v>3</v>
       </c>
       <c r="C14" s="29" t="inlineStr">
@@ -17926,7 +18331,7 @@
           <t>Prime de responsabilité de 5,00 DA (janv.) et 1,14 DA (févr.) : paramètre vraisemblablement erroné (5 au lieu de 5 %).</t>
         </is>
       </c>
-      <c r="F14" s="46" t="n"/>
+      <c r="F14" s="52" t="n"/>
       <c r="G14" s="29" t="inlineStr">
         <is>
           <t>Corriger le paramètre B291 ; régulariser le rappel éventuel.</t>
@@ -17945,7 +18350,7 @@
           <t>A11</t>
         </is>
       </c>
-      <c r="B15" s="45" t="n">
+      <c r="B15" s="51" t="n">
         <v>2</v>
       </c>
       <c r="C15" s="29" t="inlineStr">
@@ -17963,7 +18368,7 @@
           <t>Bordereaux de versement CNAS à « 0,00 » : aucune preuve de paiement des cotisations dans le dossier.</t>
         </is>
       </c>
-      <c r="F15" s="44">
+      <c r="F15" s="50">
         <f>'Rappro CNAS'!K13</f>
         <v/>
       </c>
@@ -17985,7 +18390,7 @@
           <t>A12</t>
         </is>
       </c>
-      <c r="B16" s="45" t="n">
+      <c r="B16" s="51" t="n">
         <v>2</v>
       </c>
       <c r="C16" s="29" t="inlineStr">
@@ -18003,7 +18408,7 @@
           <t>IRG IMPORT : G50 de janvier à août conformes à la paie (écarts d'arrondi ≤ 3 DA ; juillet : 2,30 DA retenus non reversés). Mars non vérifiable (paie absente).</t>
         </is>
       </c>
-      <c r="F16" s="44">
+      <c r="F16" s="50">
         <f>'Échéancier IRG-CNAS'!G13</f>
         <v/>
       </c>
@@ -18025,7 +18430,7 @@
           <t>A13</t>
         </is>
       </c>
-      <c r="B17" s="47" t="n">
+      <c r="B17" s="53" t="n">
         <v>3</v>
       </c>
       <c r="C17" s="29" t="inlineStr">
@@ -18043,7 +18448,7 @@
           <t>Paie paramétrée CACOBATPH (taux X504) mais aucune déclaration CACOBATPH (congés payés / intempéries) dans le dossier.</t>
         </is>
       </c>
-      <c r="F17" s="46" t="n"/>
+      <c r="F17" s="52" t="n"/>
       <c r="G17" s="29" t="inlineStr">
         <is>
           <t>Fournir les déclarations et paiements CACOBATPH 2026.</t>
@@ -18062,7 +18467,7 @@
           <t>A14</t>
         </is>
       </c>
-      <c r="B18" s="47" t="n">
+      <c r="B18" s="53" t="n">
         <v>3</v>
       </c>
       <c r="C18" s="29" t="inlineStr">
@@ -18080,7 +18485,7 @@
           <t>Libellés divergents : « D.P.R.COMPAGNY » / « DPR COMPAGNY » ; en-tête de paie TPM à l'adresse VGE TIZI alors que l'affiliation TPM est à TISSA.</t>
         </is>
       </c>
-      <c r="F18" s="46" t="n"/>
+      <c r="F18" s="52" t="n"/>
       <c r="G18" s="29" t="inlineStr">
         <is>
           <t>Harmoniser raison sociale et adresse dans le logiciel de paie.</t>
@@ -18099,7 +18504,7 @@
           <t>A15</t>
         </is>
       </c>
-      <c r="B19" s="47" t="n">
+      <c r="B19" s="53" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="29" t="inlineStr">
@@ -18117,7 +18522,7 @@
           <t>Périodicité mixte : déclarations mensuelles (janv., mars) puis trimestrielle (T2).</t>
         </is>
       </c>
-      <c r="F19" s="46" t="n"/>
+      <c r="F19" s="52" t="n"/>
       <c r="G19" s="29" t="inlineStr">
         <is>
           <t>Confirmer auprès de la CNAS le passage au trimestriel après la baisse d'effectif (12 → 5).</t>
@@ -18136,7 +18541,7 @@
           <t>A16</t>
         </is>
       </c>
-      <c r="B20" s="47" t="n">
+      <c r="B20" s="53" t="n">
         <v>3</v>
       </c>
       <c r="C20" s="29" t="inlineStr">
@@ -18154,7 +18559,7 @@
           <t>IRG non vérifiable salarié par salarié (centralisateurs uniquement).</t>
         </is>
       </c>
-      <c r="F20" s="46" t="n"/>
+      <c r="F20" s="52" t="n"/>
       <c r="G20" s="29" t="inlineStr">
         <is>
           <t>Fournir le livre de paie individuel / bulletins.</t>
@@ -18173,7 +18578,7 @@
           <t>A17</t>
         </is>
       </c>
-      <c r="B21" s="43" t="n">
+      <c r="B21" s="49" t="n">
         <v>1</v>
       </c>
       <c r="C21" s="29" t="inlineStr">
@@ -18191,7 +18596,7 @@
           <t>TVA collectée TPM (44537) et location (44527) jamais soldées : 58,9 M DA cumulés au 31/12/2025, accumulés depuis au moins 2022 (37,3 M à l'ouverture 2023) ; 2023–2025 : 18,5 M collectés, 1,5 M apurés. En 2025, 4 839 300 de TVA TPM générée, seuls 391 208 passés en G50 (déc.). Les G50 TPM 2026 (juil., août) ne déclarent aucun CA et reportent un précompte de 1 714 499 (= compte 44550).</t>
         </is>
       </c>
-      <c r="F21" s="44">
+      <c r="F21" s="50">
         <f>-('Balance 2024-2025'!D48+'Balance 2024-2025'!D47)</f>
         <v/>
       </c>
@@ -18213,7 +18618,7 @@
           <t>A18</t>
         </is>
       </c>
-      <c r="B22" s="43" t="n">
+      <c r="B22" s="49" t="n">
         <v>1</v>
       </c>
       <c r="C22" s="29" t="inlineStr">
@@ -18231,7 +18636,7 @@
           <t>CA de mars 2026 réalisé 27 006 870 (annotation G50), mais seulement 3 445 200 déclarés en mars « pour manque TVA à récupérer » : 23 561 670 de CA reportés sur avril–août. En avril, le CA annoté (13 157 894,74) est calculé pour obtenir 2 500 000 de TVA. Le CA déclaré mensuellement est ajusté à la TVA déductible disponible.</t>
         </is>
       </c>
-      <c r="F22" s="44">
+      <c r="F22" s="50">
         <f>'G50 2026'!B40</f>
         <v/>
       </c>
@@ -18253,7 +18658,7 @@
           <t>A19</t>
         </is>
       </c>
-      <c r="B23" s="43" t="n">
+      <c r="B23" s="49" t="n">
         <v>1</v>
       </c>
       <c r="C23" s="29" t="inlineStr">
@@ -18271,7 +18676,7 @@
           <t>G50 TPM d'avril à juillet identiques (mois imprimé « AVRIL », IRG 9 375 chaque mois) : juin sous-déclaré de 9 614,90 (18 989,90 retenus), juillet sur-déclaré de 5 683,70. Janvier–mars et août conformes.</t>
         </is>
       </c>
-      <c r="F23" s="44">
+      <c r="F23" s="50">
         <f>-'G50 TPM 2026'!G15</f>
         <v/>
       </c>
@@ -18293,7 +18698,7 @@
           <t>A20</t>
         </is>
       </c>
-      <c r="B24" s="45" t="n">
+      <c r="B24" s="51" t="n">
         <v>2</v>
       </c>
       <c r="C24" s="29" t="inlineStr">
@@ -18311,7 +18716,7 @@
           <t>Écriture du 31/12/2025 « POUR SOLDE PRCT EXE 2025 » passée en sens inverse (D 44410 / C 444, 3 074 299) : dette IBS 9,79 M et acomptes 6,15 M au lieu d'un net de 3 642 951.</t>
         </is>
       </c>
-      <c r="F24" s="44" t="n">
+      <c r="F24" s="50" t="n">
         <v>3074299</v>
       </c>
       <c r="G24" s="29" t="inlineStr">
@@ -18332,7 +18737,7 @@
           <t>A21</t>
         </is>
       </c>
-      <c r="B25" s="45" t="n">
+      <c r="B25" s="51" t="n">
         <v>2</v>
       </c>
       <c r="C25" s="29" t="inlineStr">
@@ -18350,7 +18755,7 @@
           <t>Solde IBS 2024 réglé le 03/07/2025 ; IBS 2025 net à liquider de 3 642 951 (précomptes douane déduits).</t>
         </is>
       </c>
-      <c r="F25" s="44" t="n">
+      <c r="F25" s="50" t="n">
         <v>3642951</v>
       </c>
       <c r="G25" s="29" t="inlineStr">
@@ -18371,7 +18776,7 @@
           <t>A22</t>
         </is>
       </c>
-      <c r="B26" s="45" t="n">
+      <c r="B26" s="51" t="n">
         <v>2</v>
       </c>
       <c r="C26" s="29" t="inlineStr">
@@ -18389,7 +18794,7 @@
           <t>Caisse de 12,1 M au 31/12/2025 (pic de 22,5 M) ; remboursement en espèces de 6 800 000 à SARL DPR AXXAM le 06/12/2025.</t>
         </is>
       </c>
-      <c r="F26" s="44">
+      <c r="F26" s="50">
         <f>'Balance 2024-2025'!D67</f>
         <v/>
       </c>
@@ -18411,7 +18816,7 @@
           <t>A23</t>
         </is>
       </c>
-      <c r="B27" s="45" t="n">
+      <c r="B27" s="51" t="n">
         <v>2</v>
       </c>
       <c r="C27" s="29" t="inlineStr">
@@ -18429,7 +18834,7 @@
           <t>100 % du CA TPM 2025 (25,47 M) facturé à SARL DPR AXXAM BRIQUETERIE ; aucune facturation TPM d'oct. à déc. 2025 alors que du personnel TPM reste payé.</t>
         </is>
       </c>
-      <c r="F27" s="44">
+      <c r="F27" s="50">
         <f>-'Balance 2024-2025'!D100</f>
         <v/>
       </c>
@@ -18451,7 +18856,7 @@
           <t>A24</t>
         </is>
       </c>
-      <c r="B28" s="45" t="n">
+      <c r="B28" s="51" t="n">
         <v>2</v>
       </c>
       <c r="C28" s="29" t="inlineStr">
@@ -18469,7 +18874,7 @@
           <t>Compte d'attente 47000 non soldé (« SARL FAHAS ?? », « TRESORERIE BEJAIA ?? », chèques).</t>
         </is>
       </c>
-      <c r="F28" s="44">
+      <c r="F28" s="50">
         <f>'Balance 2024-2025'!D59</f>
         <v/>
       </c>
@@ -18491,7 +18896,7 @@
           <t>A25</t>
         </is>
       </c>
-      <c r="B29" s="45" t="n">
+      <c r="B29" s="51" t="n">
         <v>2</v>
       </c>
       <c r="C29" s="29" t="inlineStr">
@@ -18509,7 +18914,7 @@
           <t>Compte 63120 « prime imposable » non soumise à cotisation : 957 406 en 2025 et 1 139 275 en 2024 (même mécanisme que A03).</t>
         </is>
       </c>
-      <c r="F29" s="44">
+      <c r="F29" s="50">
         <f>'États 2024-2025'!C24+'États 2024-2025'!D24</f>
         <v/>
       </c>
@@ -18531,7 +18936,7 @@
           <t>A26</t>
         </is>
       </c>
-      <c r="B30" s="47" t="n">
+      <c r="B30" s="53" t="n">
         <v>3</v>
       </c>
       <c r="C30" s="29" t="inlineStr">
@@ -18549,7 +18954,7 @@
           <t>Banque CPA El Kseur (51220) créditrice de 12,43 M au 31/12/2025 : découvert présenté en banque.</t>
         </is>
       </c>
-      <c r="F30" s="44">
+      <c r="F30" s="50">
         <f>ABS('Balance 2024-2025'!D63)</f>
         <v/>
       </c>
@@ -18571,7 +18976,7 @@
           <t>A27</t>
         </is>
       </c>
-      <c r="B31" s="47" t="n">
+      <c r="B31" s="53" t="n">
         <v>3</v>
       </c>
       <c r="C31" s="29" t="inlineStr">
@@ -18589,7 +18994,7 @@
           <t>Reversements IRG 2025 parfois partiels (févr., juin) et rattrapés le mois suivant ; amendes 2025 : douane 100 000, CNAS 1 746.</t>
         </is>
       </c>
-      <c r="F31" s="44">
+      <c r="F31" s="50">
         <f>'Balance 2024-2025'!D93</f>
         <v/>
       </c>
@@ -18611,7 +19016,7 @@
           <t>A28</t>
         </is>
       </c>
-      <c r="B32" s="47" t="n">
+      <c r="B32" s="53" t="n">
         <v>3</v>
       </c>
       <c r="C32" s="29" t="inlineStr">
@@ -18629,7 +19034,7 @@
           <t>Modèles G50 non mis à jour : dates de signature de 2021–2022 sur toutes les G50 2026, onglet de saisie figé (mai, TVA 17 %), G50 TPM contenant le récap TVA de déc. 2025 et un extrait de journal 2019 ; libellés de comptes de TVA à 17 %.</t>
         </is>
       </c>
-      <c r="F32" s="46" t="n"/>
+      <c r="F32" s="52" t="n"/>
       <c r="G32" s="29" t="inlineStr">
         <is>
           <t>Mettre à jour le modèle et les libellés (TVA 19 %).</t>
@@ -18648,7 +19053,7 @@
           <t>A29</t>
         </is>
       </c>
-      <c r="B33" s="47" t="n">
+      <c r="B33" s="53" t="n">
         <v>3</v>
       </c>
       <c r="C33" s="29" t="inlineStr">
@@ -18666,7 +19071,7 @@
           <t>Taxe d'apprentissage payée deux fois en 2026 : février (87 828 IMPORT sur 8 782 828 + 9 851 TPM sur 985 118) et août (44 091 IMPORT sur 4 409 079 + 6 809 TPM sur 680 900).</t>
         </is>
       </c>
-      <c r="F33" s="44">
+      <c r="F33" s="50">
         <f>'G50 2026'!J26+'G50 TPM 2026'!J17</f>
         <v/>
       </c>
@@ -18688,7 +19093,7 @@
           <t>A30</t>
         </is>
       </c>
-      <c r="B34" s="47" t="n">
+      <c r="B34" s="53" t="n">
         <v>3</v>
       </c>
       <c r="C34" s="29" t="inlineStr">
@@ -18706,7 +19111,7 @@
           <t>Droit de timbre : taux apparents incohérents (janv. 2,0 %, févr. 1,0 %, avr. 5,05 %, mai 1,79 %) ; même base en avril et mai ; aucun timbre en mars et de juin à août.</t>
         </is>
       </c>
-      <c r="F34" s="44">
+      <c r="F34" s="50">
         <f>'G50 2026'!J24</f>
         <v/>
       </c>
@@ -18728,7 +19133,7 @@
           <t>A32</t>
         </is>
       </c>
-      <c r="B35" s="43" t="n">
+      <c r="B35" s="49" t="n">
         <v>1</v>
       </c>
       <c r="C35" s="29" t="inlineStr">
@@ -18746,7 +19151,7 @@
           <t>Journal 2023 fourni provisoire : résultat 18,54 M contre 7,26 M repris en à-nouveau 2024 ; 38 comptes en écart avec les ouvertures 2024 (stocks, fournisseurs, banques, IBS, TVA).</t>
         </is>
       </c>
-      <c r="F35" s="44">
+      <c r="F35" s="50">
         <f>'Contrôle 2023'!B6</f>
         <v/>
       </c>
@@ -18768,7 +19173,7 @@
           <t>A33</t>
         </is>
       </c>
-      <c r="B36" s="43" t="n">
+      <c r="B36" s="49" t="n">
         <v>1</v>
       </c>
       <c r="C36" s="29" t="inlineStr">
@@ -18786,7 +19191,7 @@
           <t>Créance SARL DPR AXXAM BRIQUETERIE : 371,0 M au 31/12/2025 (96 % du poste clients), en hausse continue depuis 2023 (277,7 M) ; 2023–2025 : 115,7 M facturés, 26,2 M encaissés (23 %).</t>
         </is>
       </c>
-      <c r="F36" s="44">
+      <c r="F36" s="50">
         <f>'Démarrage 2026'!E8</f>
         <v/>
       </c>
@@ -18808,7 +19213,7 @@
           <t>A34</t>
         </is>
       </c>
-      <c r="B37" s="43" t="n">
+      <c r="B37" s="49" t="n">
         <v>1</v>
       </c>
       <c r="C37" s="29" t="inlineStr">
@@ -18826,7 +19231,7 @@
           <t>Avances clients (419) dormantes : 229,4 M sur 144 clients, inchangées depuis au moins le 01/01/2023 (hors associés et clients à compenser). Soit livraisons non facturées (CA et TVA non déclarés), soit dettes à rembourser.</t>
         </is>
       </c>
-      <c r="F37" s="44">
+      <c r="F37" s="50">
         <f>'Démarrage 2026'!E35</f>
         <v/>
       </c>
@@ -18848,7 +19253,7 @@
           <t>A35</t>
         </is>
       </c>
-      <c r="B38" s="43" t="n">
+      <c r="B38" s="49" t="n">
         <v>1</v>
       </c>
       <c r="C38" s="29" t="inlineStr">
@@ -18866,7 +19271,7 @@
           <t>SARL DPR AXXAM : 62,5 M versés en 2025 (dont 45,35 M d'avances 409 sans facture) et 6,8 M remboursés en espèces, alors que la briqueterie du même groupe ne paie pas.</t>
         </is>
       </c>
-      <c r="F38" s="44">
+      <c r="F38" s="50">
         <f>'Démarrage 2026'!B21</f>
         <v/>
       </c>
@@ -18888,7 +19293,7 @@
           <t>A36</t>
         </is>
       </c>
-      <c r="B39" s="45" t="n">
+      <c r="B39" s="51" t="n">
         <v>2</v>
       </c>
       <c r="C39" s="29" t="inlineStr">
@@ -18903,10 +19308,10 @@
       </c>
       <c r="E39" s="29" t="inlineStr">
         <is>
-          <t>Associés (famille DJENNADI) logés en comptes clients / fournisseurs : soldes créditeurs en 411, 419 et 401.</t>
-        </is>
-      </c>
-      <c r="F39" s="44">
+          <t>Associés (famille DJENNADI, dont les 3 gérants inscrits au registre de commerce : Abdelkrim, Ryad, Ahcene) logés en comptes clients / fournisseurs : soldes créditeurs en 411, 419 et 401.</t>
+        </is>
+      </c>
+      <c r="F39" s="50">
         <f>'Démarrage 2026'!E26</f>
         <v/>
       </c>
@@ -18925,31 +19330,34 @@
     <row r="40" ht="52" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>A31</t>
-        </is>
-      </c>
-      <c r="B40" s="47" t="n">
-        <v>3</v>
+          <t>A37</t>
+        </is>
+      </c>
+      <c r="B40" s="49" t="n">
+        <v>1</v>
       </c>
       <c r="C40" s="29" t="inlineStr">
         <is>
-          <t>Les deux</t>
+          <t>Société</t>
         </is>
       </c>
       <c r="D40" s="29" t="inlineStr">
         <is>
-          <t>Comptabilité</t>
+          <t>Juridique</t>
         </is>
       </c>
       <c r="E40" s="29" t="inlineStr">
         <is>
-          <t>Clients débiteurs 387,1 M et avances clients 314,6 M ; fournisseurs débiteurs 46,2 M au 31/12/2025.</t>
-        </is>
-      </c>
-      <c r="F40" s="46" t="n"/>
+          <t>Extrait du registre de commerce valable jusqu'au 13/02/2026 seulement : activité poursuivie avec un extrait expiré depuis plus de 7 mois.</t>
+        </is>
+      </c>
+      <c r="F40" s="50">
+        <f>'Registre de commerce'!B26</f>
+        <v/>
+      </c>
       <c r="G40" s="29" t="inlineStr">
         <is>
-          <t>Lettrer les comptes clients/fournisseurs et compenser les avances soldées.</t>
+          <t>Renouveler l'extrait au CNRC sans délai (jours écoulés en impact).</t>
         </is>
       </c>
       <c r="H40" s="41" t="n"/>
@@ -18959,27 +19367,178 @@
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+    <row r="41" ht="52" customHeight="1">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>A38</t>
+        </is>
+      </c>
+      <c r="B41" s="49" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" s="29" t="inlineStr">
+        <is>
+          <t>Société</t>
+        </is>
+      </c>
+      <c r="D41" s="29" t="inlineStr">
+        <is>
+          <t>Juridique / fiscal</t>
+        </is>
+      </c>
+      <c r="E41" s="29" t="inlineStr">
+        <is>
+          <t>Registre limité à l'importation pour revente en l'état (442101 à 442104) ; les activités TPM, location d'engins et transport sont exercées et facturées hors objet du registre.</t>
+        </is>
+      </c>
+      <c r="F41" s="50">
+        <f>-'Balance 2024-2025'!D100</f>
+        <v/>
+      </c>
+      <c r="G41" s="29" t="inlineStr">
+        <is>
+          <t>Modifier le registre ou filialiser les activités TPM / location ; vérifier la compatibilité avec le statut d'importateur.</t>
+        </is>
+      </c>
+      <c r="H41" s="41" t="n"/>
+      <c r="I41" s="41" t="inlineStr">
+        <is>
+          <t>Ouvert</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="52" customHeight="1">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>A39</t>
+        </is>
+      </c>
+      <c r="B42" s="51" t="n">
+        <v>2</v>
+      </c>
+      <c r="C42" s="29" t="inlineStr">
+        <is>
+          <t>TPM</t>
+        </is>
+      </c>
+      <c r="D42" s="29" t="inlineStr">
+        <is>
+          <t>Juridique</t>
+        </is>
+      </c>
+      <c r="E42" s="29" t="inlineStr">
+        <is>
+          <t>Aucun établissement secondaire inscrit au registre, alors que l'activité TPM est affiliée à la CNAS à TISSA sous un numéro distinct.</t>
+        </is>
+      </c>
+      <c r="F42" s="52" t="n"/>
+      <c r="G42" s="29" t="inlineStr">
+        <is>
+          <t>Inscrire l'établissement secondaire ou aligner les affiliations.</t>
+        </is>
+      </c>
+      <c r="H42" s="41" t="n"/>
+      <c r="I42" s="41" t="inlineStr">
+        <is>
+          <t>Ouvert</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="52" customHeight="1">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>A40</t>
+        </is>
+      </c>
+      <c r="B43" s="53" t="n">
+        <v>3</v>
+      </c>
+      <c r="C43" s="29" t="inlineStr">
+        <is>
+          <t>Société</t>
+        </is>
+      </c>
+      <c r="D43" s="29" t="inlineStr">
+        <is>
+          <t>Administratif</t>
+        </is>
+      </c>
+      <c r="E43" s="29" t="inlineStr">
+        <is>
+          <t>N° de registre de commerce différent entre l'extrait (06/00-0184232 B 03) et le dossier comptable PCCOMPTA (06/01-0184232B03) ; local commercial appartenant à un associé (DJENNADI Abdelkader, créancier de 2,51 M en 401).</t>
+        </is>
+      </c>
+      <c r="F43" s="52" t="n"/>
+      <c r="G43" s="29" t="inlineStr">
+        <is>
+          <t>Corriger le n° RC dans PCCOMPTA ; produire le bail et l'état des loyers.</t>
+        </is>
+      </c>
+      <c r="H43" s="41" t="n"/>
+      <c r="I43" s="41" t="inlineStr">
+        <is>
+          <t>Ouvert</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="52" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>A31</t>
+        </is>
+      </c>
+      <c r="B44" s="53" t="n">
+        <v>3</v>
+      </c>
+      <c r="C44" s="29" t="inlineStr">
+        <is>
+          <t>Les deux</t>
+        </is>
+      </c>
+      <c r="D44" s="29" t="inlineStr">
+        <is>
+          <t>Comptabilité</t>
+        </is>
+      </c>
+      <c r="E44" s="29" t="inlineStr">
+        <is>
+          <t>Clients débiteurs 387,1 M et avances clients 314,6 M ; fournisseurs débiteurs 46,2 M au 31/12/2025.</t>
+        </is>
+      </c>
+      <c r="F44" s="52" t="n"/>
+      <c r="G44" s="29" t="inlineStr">
+        <is>
+          <t>Lettrer les comptes clients/fournisseurs et compenser les avances soldées.</t>
+        </is>
+      </c>
+      <c r="H44" s="41" t="n"/>
+      <c r="I44" s="41" t="inlineStr">
+        <is>
+          <t>Ouvert</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>Impact : A01 = cotisations calculées de février ; A02 = cotisations de mars déclarées sans justificatif ; A03 = cotisations sur ponctualité ; A07 = cotisations T3 partielles (juil–août) ; A09 = frais de mission TPM cumulés ; A11 = cotisations déclarées sans preuve de paiement ; A12 = IRG cumulé à rapprocher.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I40"/>
+  <autoFilter ref="A4:I44"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -19055,7 +19614,7 @@
           <t>Janv–août 2026</t>
         </is>
       </c>
-      <c r="E5" s="48" t="inlineStr">
+      <c r="E5" s="54" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -19085,7 +19644,7 @@
           <t>Janv–août 2026</t>
         </is>
       </c>
-      <c r="E6" s="48" t="inlineStr">
+      <c r="E6" s="54" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -19111,7 +19670,7 @@
           <t>Janvier 2026</t>
         </is>
       </c>
-      <c r="E7" s="48" t="inlineStr">
+      <c r="E7" s="54" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -19141,7 +19700,7 @@
           <t>Mars 2026</t>
         </is>
       </c>
-      <c r="E8" s="48" t="inlineStr">
+      <c r="E8" s="54" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -19171,7 +19730,7 @@
           <t>T2 2026</t>
         </is>
       </c>
-      <c r="E9" s="48" t="inlineStr">
+      <c r="E9" s="54" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -19201,7 +19760,7 @@
           <t>T1 2026</t>
         </is>
       </c>
-      <c r="E10" s="48" t="inlineStr">
+      <c r="E10" s="54" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -19231,7 +19790,7 @@
           <t>T2 2026</t>
         </is>
       </c>
-      <c r="E11" s="48" t="inlineStr">
+      <c r="E11" s="54" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -19407,7 +19966,7 @@
           <t>Juin 2026</t>
         </is>
       </c>
-      <c r="E17" s="48" t="inlineStr">
+      <c r="E17" s="54" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -19437,7 +19996,7 @@
           <t>Août 2026</t>
         </is>
       </c>
-      <c r="E18" s="48" t="inlineStr">
+      <c r="E18" s="54" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -19467,7 +20026,7 @@
           <t>Exercice 2024</t>
         </is>
       </c>
-      <c r="E19" s="48" t="inlineStr">
+      <c r="E19" s="54" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -19497,7 +20056,7 @@
           <t>Exercice 2025</t>
         </is>
       </c>
-      <c r="E20" s="48" t="inlineStr">
+      <c r="E20" s="54" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -19527,7 +20086,7 @@
           <t>Mars, avril, mai, juillet 2026</t>
         </is>
       </c>
-      <c r="E21" s="48" t="inlineStr">
+      <c r="E21" s="54" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -19557,7 +20116,7 @@
           <t>Janvier, février 2026</t>
         </is>
       </c>
-      <c r="E22" s="48" t="inlineStr">
+      <c r="E22" s="54" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -19587,7 +20146,7 @@
           <t>Juillet, août 2026</t>
         </is>
       </c>
-      <c r="E23" s="48" t="inlineStr">
+      <c r="E23" s="54" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -19617,7 +20176,7 @@
           <t>Avril, mai, juin 2026</t>
         </is>
       </c>
-      <c r="E24" s="48" t="inlineStr">
+      <c r="E24" s="54" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -19647,7 +20206,7 @@
           <t>Exercice 2023</t>
         </is>
       </c>
-      <c r="E25" s="48" t="inlineStr">
+      <c r="E25" s="54" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -19677,7 +20236,7 @@
           <t>Janvier, février, mars 2026</t>
         </is>
       </c>
-      <c r="E26" s="48" t="inlineStr">
+      <c r="E26" s="54" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -19724,27 +20283,27 @@
       </c>
       <c r="B28" s="12" t="inlineStr">
         <is>
-          <t>G50 IMPORT et TPM septembre 2026</t>
+          <t>Extrait du registre de commerce (scan CNRC)</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
         <is>
-          <t>Les deux</t>
+          <t>Société</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
         <is>
-          <t>Sept. 2026</t>
-        </is>
-      </c>
-      <c r="E28" s="40" t="inlineStr">
-        <is>
-          <t>Manquante</t>
+          <t>Délivré le 10/09/2024</t>
+        </is>
+      </c>
+      <c r="E28" s="54" t="inlineStr">
+        <is>
+          <t>Reçue</t>
         </is>
       </c>
       <c r="F28" s="12" t="inlineStr">
         <is>
-          <t>Échéance 20/10/2026</t>
+          <t>Expiré le 13/02/2026</t>
         </is>
       </c>
     </row>
@@ -19754,12 +20313,12 @@
       </c>
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>Journal des ventes / factures 2026</t>
+          <t>Extrait du registre de commerce renouvelé</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>IMPORT</t>
+          <t>Société</t>
         </is>
       </c>
       <c r="D29" s="12" t="inlineStr">
@@ -19774,7 +20333,7 @@
       </c>
       <c r="F29" s="12" t="inlineStr">
         <is>
-          <t>Voir A18 : CA réel par mois</t>
+          <t>Voir A37, A38</t>
         </is>
       </c>
     </row>
@@ -19784,19 +20343,15 @@
       </c>
       <c r="B30" s="12" t="inlineStr">
         <is>
-          <t>G50 TPM 2023–2025 (rapprochement TVA collectée TPM)</t>
+          <t>Statuts à jour et bail du local (DJENNADI Abdelkader)</t>
         </is>
       </c>
       <c r="C30" s="12" t="inlineStr">
         <is>
-          <t>TPM</t>
-        </is>
-      </c>
-      <c r="D30" s="12" t="inlineStr">
-        <is>
-          <t>2023–2025</t>
-        </is>
-      </c>
+          <t>Société</t>
+        </is>
+      </c>
+      <c r="D30" s="12" t="inlineStr"/>
       <c r="E30" s="40" t="inlineStr">
         <is>
           <t>Manquante</t>
@@ -19804,7 +20359,7 @@
       </c>
       <c r="F30" s="12" t="inlineStr">
         <is>
-          <t>Voir A17</t>
+          <t>Voir A40</t>
         </is>
       </c>
     </row>
@@ -19814,17 +20369,17 @@
       </c>
       <c r="B31" s="12" t="inlineStr">
         <is>
-          <t>Journal comptable 2026 (PCCOMPTA)</t>
+          <t>G50 IMPORT et TPM septembre 2026</t>
         </is>
       </c>
       <c r="C31" s="12" t="inlineStr">
         <is>
-          <t>Société</t>
+          <t>Les deux</t>
         </is>
       </c>
       <c r="D31" s="12" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>Sept. 2026</t>
         </is>
       </c>
       <c r="E31" s="40" t="inlineStr">
@@ -19834,7 +20389,7 @@
       </c>
       <c r="F31" s="12" t="inlineStr">
         <is>
-          <t>Pour rapprocher paie et G50 avec la comptabilité</t>
+          <t>Échéance 20/10/2026</t>
         </is>
       </c>
     </row>
@@ -19844,17 +20399,17 @@
       </c>
       <c r="B32" s="12" t="inlineStr">
         <is>
-          <t>Liasse fiscale / bilan 2025 déposé et preuve de paiement IBS</t>
+          <t>Journal des ventes / factures 2026</t>
         </is>
       </c>
       <c r="C32" s="12" t="inlineStr">
         <is>
-          <t>Société</t>
+          <t>IMPORT</t>
         </is>
       </c>
       <c r="D32" s="12" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="E32" s="40" t="inlineStr">
@@ -19864,7 +20419,7 @@
       </c>
       <c r="F32" s="12" t="inlineStr">
         <is>
-          <t>Voir A20, A21</t>
+          <t>Voir A18 : CA réel par mois</t>
         </is>
       </c>
     </row>
@@ -19874,17 +20429,17 @@
       </c>
       <c r="B33" s="12" t="inlineStr">
         <is>
-          <t>PV de caisse au 31/12/2025</t>
+          <t>G50 TPM 2023–2025 (rapprochement TVA collectée TPM)</t>
         </is>
       </c>
       <c r="C33" s="12" t="inlineStr">
         <is>
-          <t>Société</t>
+          <t>TPM</t>
         </is>
       </c>
       <c r="D33" s="12" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2023–2025</t>
         </is>
       </c>
       <c r="E33" s="40" t="inlineStr">
@@ -19894,7 +20449,7 @@
       </c>
       <c r="F33" s="12" t="inlineStr">
         <is>
-          <t>Voir A22</t>
+          <t>Voir A17</t>
         </is>
       </c>
     </row>
@@ -19904,12 +20459,12 @@
       </c>
       <c r="B34" s="12" t="inlineStr">
         <is>
-          <t>Déclarations et paiements CACOBATPH</t>
+          <t>Journal comptable 2026 (PCCOMPTA)</t>
         </is>
       </c>
       <c r="C34" s="12" t="inlineStr">
         <is>
-          <t>Les deux</t>
+          <t>Société</t>
         </is>
       </c>
       <c r="D34" s="12" t="inlineStr">
@@ -19922,7 +20477,11 @@
           <t>Manquante</t>
         </is>
       </c>
-      <c r="F34" s="12" t="inlineStr"/>
+      <c r="F34" s="12" t="inlineStr">
+        <is>
+          <t>Pour rapprocher paie et G50 avec la comptabilité</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="12" t="n">
@@ -19930,17 +20489,17 @@
       </c>
       <c r="B35" s="12" t="inlineStr">
         <is>
-          <t>Livre de paie individuel / bulletins</t>
+          <t>Liasse fiscale / bilan 2025 déposé et preuve de paiement IBS</t>
         </is>
       </c>
       <c r="C35" s="12" t="inlineStr">
         <is>
-          <t>Les deux</t>
+          <t>Société</t>
         </is>
       </c>
       <c r="D35" s="12" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="E35" s="40" t="inlineStr">
@@ -19950,7 +20509,7 @@
       </c>
       <c r="F35" s="12" t="inlineStr">
         <is>
-          <t>Pour contrôle IRG</t>
+          <t>Voir A20, A21</t>
         </is>
       </c>
     </row>
@@ -19960,17 +20519,17 @@
       </c>
       <c r="B36" s="12" t="inlineStr">
         <is>
-          <t>Ordres de mission et justificatifs de frais</t>
+          <t>PV de caisse au 31/12/2025</t>
         </is>
       </c>
       <c r="C36" s="12" t="inlineStr">
         <is>
-          <t>TPM</t>
+          <t>Société</t>
         </is>
       </c>
       <c r="D36" s="12" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="E36" s="40" t="inlineStr">
@@ -19980,7 +20539,7 @@
       </c>
       <c r="F36" s="12" t="inlineStr">
         <is>
-          <t>Frais de mission élevés</t>
+          <t>Voir A22</t>
         </is>
       </c>
     </row>
@@ -19990,25 +20549,111 @@
       </c>
       <c r="B37" s="12" t="inlineStr">
         <is>
+          <t>Déclarations et paiements CACOBATPH</t>
+        </is>
+      </c>
+      <c r="C37" s="12" t="inlineStr">
+        <is>
+          <t>Les deux</t>
+        </is>
+      </c>
+      <c r="D37" s="12" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E37" s="40" t="inlineStr">
+        <is>
+          <t>Manquante</t>
+        </is>
+      </c>
+      <c r="F37" s="12" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="12" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>Livre de paie individuel / bulletins</t>
+        </is>
+      </c>
+      <c r="C38" s="12" t="inlineStr">
+        <is>
+          <t>Les deux</t>
+        </is>
+      </c>
+      <c r="D38" s="12" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E38" s="40" t="inlineStr">
+        <is>
+          <t>Manquante</t>
+        </is>
+      </c>
+      <c r="F38" s="12" t="inlineStr">
+        <is>
+          <t>Pour contrôle IRG</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>Ordres de mission et justificatifs de frais</t>
+        </is>
+      </c>
+      <c r="C39" s="12" t="inlineStr">
+        <is>
+          <t>TPM</t>
+        </is>
+      </c>
+      <c r="D39" s="12" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E39" s="40" t="inlineStr">
+        <is>
+          <t>Manquante</t>
+        </is>
+      </c>
+      <c r="F39" s="12" t="inlineStr">
+        <is>
+          <t>Frais de mission élevés</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="12" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" s="12" t="inlineStr">
+        <is>
           <t>Relevés bancaires — virements de salaires</t>
         </is>
       </c>
-      <c r="C37" s="12" t="inlineStr">
+      <c r="C40" s="12" t="inlineStr">
         <is>
           <t>Les deux</t>
         </is>
       </c>
-      <c r="D37" s="12" t="inlineStr">
+      <c r="D40" s="12" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="E37" s="40" t="inlineStr">
+      <c r="E40" s="40" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
       </c>
-      <c r="F37" s="12" t="inlineStr">
+      <c r="F40" s="12" t="inlineStr">
         <is>
           <t>Pour lettrage du 421</t>
         </is>

</xml_diff>

<commit_message>
Dossier comptable : extrait du registre de commerce modifié 2026 et augmentation de capital
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XYis4EzVZMNdoYCxmLrRh4
</commit_message>
<xml_diff>
--- a/DOSSIER_COMPTABLE_SARL_DPR_COMPAGNY_2026.xlsx
+++ b/DOSSIER_COMPTABLE_SARL_DPR_COMPAGNY_2026.xlsx
@@ -33,7 +33,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Balance 2024-2025'!$A$4:$E$104</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Clients &amp; fournisseurs'!$A$21:$L$243</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Relevé CPA 2026'!$A$4:$I$466</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'Anomalies &amp; actions'!$A$4:$I$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'Anomalies &amp; actions'!$A$4:$I$48</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -212,7 +212,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -265,15 +265,22 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="167" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="6" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1010,11 +1017,11 @@
         </is>
       </c>
       <c r="B24" s="13">
-        <f>COUNTIF('Anomalies &amp; actions'!B5:B47,1)</f>
+        <f>COUNTIF('Anomalies &amp; actions'!B5:B48,1)</f>
         <v/>
       </c>
       <c r="C24" s="13">
-        <f>COUNTIFS('Anomalies &amp; actions'!B5:B47,1,'Anomalies &amp; actions'!I5:I47,"Ouvert")</f>
+        <f>COUNTIFS('Anomalies &amp; actions'!B5:B48,1,'Anomalies &amp; actions'!I5:I48,"Ouvert")</f>
         <v/>
       </c>
     </row>
@@ -1025,11 +1032,11 @@
         </is>
       </c>
       <c r="B25" s="13">
-        <f>COUNTIF('Anomalies &amp; actions'!B5:B47,2)</f>
+        <f>COUNTIF('Anomalies &amp; actions'!B5:B48,2)</f>
         <v/>
       </c>
       <c r="C25" s="13">
-        <f>COUNTIFS('Anomalies &amp; actions'!B5:B47,2,'Anomalies &amp; actions'!I5:I47,"Ouvert")</f>
+        <f>COUNTIFS('Anomalies &amp; actions'!B5:B48,2,'Anomalies &amp; actions'!I5:I48,"Ouvert")</f>
         <v/>
       </c>
     </row>
@@ -1040,11 +1047,11 @@
         </is>
       </c>
       <c r="B26" s="13">
-        <f>COUNTIF('Anomalies &amp; actions'!B5:B47,3)</f>
+        <f>COUNTIF('Anomalies &amp; actions'!B5:B48,3)</f>
         <v/>
       </c>
       <c r="C26" s="13">
-        <f>COUNTIFS('Anomalies &amp; actions'!B5:B47,3,'Anomalies &amp; actions'!I5:I47,"Ouvert")</f>
+        <f>COUNTIFS('Anomalies &amp; actions'!B5:B48,3,'Anomalies &amp; actions'!I5:I48,"Ouvert")</f>
         <v/>
       </c>
     </row>
@@ -1363,7 +1370,7 @@
       </c>
       <c r="B53" s="12" t="inlineStr">
         <is>
-          <t>Extrait CNRC : activités inscrites, gérants, validité</t>
+          <t>Extraits CNRC 2024 et 2026 : activités, gérants, validité, augmentation de capital</t>
         </is>
       </c>
       <c r="C53" s="17" t="n"/>
@@ -17543,25 +17550,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="62" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Extrait du registre de commerce (CNRC) — contrôle de conformité</t>
+          <t>Extraits du registre de commerce (CNRC) — contrôle de conformité</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Source : SDOC-607B666B93EEF055F89FE8EC0A5E7DF1-11-30-SI.pdf (scan CamScanner, en arabe), extrait n° de série 700267695 délivré par l'antenne CNRC de Béjaïa le 10/09/2024.</t>
+          <t>Sources : extrait n° 700267695 du 10/09/2024 (scan PDF) et extrait modifié n° 700320220 du 29/07/2026 (photo), en arabe, traduits ici.</t>
         </is>
       </c>
     </row>
@@ -17573,338 +17581,511 @@
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>Mention de l'extrait (traduction)</t>
+          <t>Extrait du 10/09/2024</t>
         </is>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>Contrôle / constat</t>
+          <t>Extrait modifié du 29/07/2026</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>Constat</t>
         </is>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Dénomination</t>
+          <t>Dénomination / forme</t>
         </is>
       </c>
       <c r="B5" s="43" t="inlineStr">
         <is>
-          <t>D.P.R. COMPAGNY</t>
-        </is>
-      </c>
-      <c r="C5" s="29" t="inlineStr">
-        <is>
-          <t>Conforme aux déclarations CNAS et G50</t>
+          <t>D.P.R. COMPAGNY — SARL</t>
+        </is>
+      </c>
+      <c r="C5" s="43" t="inlineStr">
+        <is>
+          <t>D.P.R. COMPAGNY — SARL (personne morale)</t>
+        </is>
+      </c>
+      <c r="D5" s="29" t="inlineStr">
+        <is>
+          <t>Inchangé</t>
         </is>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Forme juridique</t>
+          <t>N° du registre de commerce</t>
         </is>
       </c>
       <c r="B6" s="43" t="inlineStr">
         <is>
-          <t>Société à responsabilité limitée (SARL)</t>
-        </is>
-      </c>
-      <c r="C6" s="29" t="inlineStr">
-        <is>
-          <t>Conforme</t>
+          <t>06/00-0184232 B 03</t>
+        </is>
+      </c>
+      <c r="C6" s="43" t="inlineStr">
+        <is>
+          <t>06/00-0184232 B 03</t>
+        </is>
+      </c>
+      <c r="D6" s="29" t="inlineStr">
+        <is>
+          <t>PCCOMPTA porte 06/01-0184232B03 : à corriger</t>
         </is>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>N° du registre de commerce</t>
+          <t>Siège social</t>
         </is>
       </c>
       <c r="B7" s="43" t="inlineStr">
         <is>
-          <t>06/00-0184232 B 03</t>
-        </is>
-      </c>
-      <c r="C7" s="29" t="inlineStr">
-        <is>
-          <t>Le dossier comptable (PCCOMPTA) porte 06/01-0184232B03 : à corriger</t>
+          <t>Lieu-dit Tizi, commune de Semaoun, Béjaïa</t>
+        </is>
+      </c>
+      <c r="C7" s="43" t="inlineStr">
+        <is>
+          <t>Lieu-dit Tizi, commune de Semaoun, Béjaïa</t>
+        </is>
+      </c>
+      <c r="D7" s="29" t="inlineStr">
+        <is>
+          <t>Inchangé</t>
         </is>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Siège social</t>
-        </is>
-      </c>
-      <c r="B8" s="43" t="inlineStr">
-        <is>
-          <t>Lieu-dit Tizi, commune de Semaoun, wilaya de Béjaïa</t>
-        </is>
-      </c>
-      <c r="C8" s="29" t="inlineStr">
-        <is>
-          <t>Conforme (VGE TIZI). Aucun établissement secondaire inscrit</t>
-        </is>
+          <t>Capital social</t>
+        </is>
+      </c>
+      <c r="B8" s="44" t="n">
+        <v>106000000</v>
+      </c>
+      <c r="C8" s="44" t="n">
+        <v>268000000</v>
+      </c>
+      <c r="D8" s="45">
+        <f>IF(C8&gt;B8,"Capital porté à "&amp;TEXT(C8/1000000,"0")&amp;" M DA (+"&amp;TEXT((C8-B8)/1000000,"0")&amp;" M) : voir section B","Inchangé")</f>
+        <v/>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Capital social</t>
+          <t>Date de début d'activité</t>
         </is>
       </c>
       <c r="B9" s="43" t="inlineStr">
         <is>
-          <t>106 000 000,00 DA</t>
-        </is>
-      </c>
-      <c r="C9" s="29">
-        <f>IF(ABS(-'Balance 2024-2025'!D5-106000000)&lt;1,"Conforme au compte 10100","Écart avec le compte 10100")</f>
-        <v/>
-      </c>
+          <t>16/04/2003</t>
+        </is>
+      </c>
+      <c r="C9" s="43" t="inlineStr">
+        <is>
+          <t>16/04/2003</t>
+        </is>
+      </c>
+      <c r="D9" s="29" t="inlineStr"/>
     </row>
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Date de début d'activité</t>
+          <t>Fonds de commerce</t>
         </is>
       </c>
       <c r="B10" s="43" t="inlineStr">
         <is>
-          <t>16/04/2003</t>
-        </is>
-      </c>
-      <c r="C10" s="29" t="inlineStr"/>
+          <t>Création</t>
+        </is>
+      </c>
+      <c r="C10" s="43" t="inlineStr">
+        <is>
+          <t>Création</t>
+        </is>
+      </c>
+      <c r="D10" s="29" t="inlineStr"/>
     </row>
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Fonds de commerce</t>
+          <t>Propriétaire du local commercial</t>
         </is>
       </c>
       <c r="B11" s="43" t="inlineStr">
         <is>
-          <t>Création</t>
-        </is>
-      </c>
-      <c r="C11" s="29" t="inlineStr"/>
+          <t>DJENNADI Abdelkader</t>
+        </is>
+      </c>
+      <c r="C11" s="43" t="inlineStr">
+        <is>
+          <t>DJENNADI Abdelkader</t>
+        </is>
+      </c>
+      <c r="D11" s="29" t="inlineStr">
+        <is>
+          <t>Créancier 401 de 2 510 665 sans mouvement : bail et loyers à justifier</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="32" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Propriétaire du local commercial</t>
+          <t>Établissements secondaires</t>
         </is>
       </c>
       <c r="B12" s="43" t="inlineStr">
         <is>
-          <t>DJENNADI Abdelkader</t>
-        </is>
-      </c>
-      <c r="C12" s="29" t="inlineStr">
-        <is>
-          <t>Figure en fournisseur 401 (dette de 2 510 665 sans mouvement en 2025) : bail et loyers à justifier</t>
+          <t>Néant</t>
+        </is>
+      </c>
+      <c r="C12" s="43" t="inlineStr">
+        <is>
+          <t>Néant</t>
+        </is>
+      </c>
+      <c r="D12" s="29" t="inlineStr">
+        <is>
+          <t>Toujours aucun établissement inscrit alors que l'activité TPM est affiliée à la CNAS à TISSA</t>
         </is>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Nombre d'établissements secondaires</t>
+          <t>Gérants associés</t>
         </is>
       </c>
       <c r="B13" s="43" t="inlineStr">
         <is>
-          <t>Néant (non renseigné)</t>
-        </is>
-      </c>
-      <c r="C13" s="29" t="inlineStr">
-        <is>
-          <t>Or affiliation CNAS TPM distincte à TISSA (n° 06736613 53) : établissement secondaire non inscrit</t>
+          <t>DJENNADI Abdelkrim (22/04/1975), Ryad (18/01/1978), Ahcene (08/03/1972)</t>
+        </is>
+      </c>
+      <c r="C13" s="43" t="inlineStr">
+        <is>
+          <t>Identiques</t>
+        </is>
+      </c>
+      <c r="D13" s="29" t="inlineStr">
+        <is>
+          <t>Leurs soldes en 411 / 419 sont des comptes d'associés (A36)</t>
         </is>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Gérants associés</t>
+          <t>Activités inscrites</t>
         </is>
       </c>
       <c r="B14" s="43" t="inlineStr">
         <is>
-          <t>DJENNADI Abdelkrim (né le 22/04/1975), DJENNADI Ryad (né le 18/01/1978), DJENNADI Ahcene (né le 08/03/1972), nationalité algérienne</t>
-        </is>
-      </c>
-      <c r="C14" s="29" t="inlineStr">
-        <is>
-          <t>Confirme que leurs soldes en 411 / 419 sont des comptes d'associés (A36)</t>
+          <t>Importation pour revente en l'état : 442101, 442102, 442103, 442104</t>
+        </is>
+      </c>
+      <c r="C14" s="43" t="inlineStr">
+        <is>
+          <t>Identiques (442101 à 442104)</t>
+        </is>
+      </c>
+      <c r="D14" s="29" t="inlineStr">
+        <is>
+          <t>Toujours AUCUNE activité TPM, location d'engins ou transport : non régularisé (A38)</t>
         </is>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Secteur d'activité</t>
+          <t>Date d'inscription de la modification</t>
         </is>
       </c>
       <c r="B15" s="43" t="inlineStr">
         <is>
-          <t>Importation pour la revente en l'état</t>
-        </is>
-      </c>
-      <c r="C15" s="29" t="inlineStr"/>
+          <t>10/09/2024</t>
+        </is>
+      </c>
+      <c r="C15" s="43" t="inlineStr">
+        <is>
+          <t>29/07/2026</t>
+        </is>
+      </c>
+      <c r="D15" s="29" t="inlineStr"/>
     </row>
     <row r="16" ht="32" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Activité 442101</t>
+          <t>Validité de l'extrait</t>
         </is>
       </c>
       <c r="B16" s="43" t="inlineStr">
         <is>
-          <t>Importation d'équipements, pièces de rechange et accessoires liés au domaine mécanique</t>
-        </is>
-      </c>
-      <c r="C16" s="29" t="inlineStr"/>
-    </row>
-    <row r="17" ht="32" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>Activité 442102</t>
-        </is>
-      </c>
-      <c r="B17" s="43" t="inlineStr">
-        <is>
-          <t>Importation de pièces de rechange et accessoires automobiles</t>
-        </is>
-      </c>
-      <c r="C17" s="29" t="inlineStr"/>
-    </row>
-    <row r="18" ht="32" customHeight="1">
+          <t>Du 13/02/2024 au 13/02/2026</t>
+        </is>
+      </c>
+      <c r="C16" s="43" t="inlineStr">
+        <is>
+          <t>Du 16/02/2026 au 16/02/2028</t>
+        </is>
+      </c>
+      <c r="D16" s="46">
+        <f>"Extrait remis le 29/07/2026 : "&amp;TEXT(B20,"0")&amp;" jours d'activité entre l'expiration (13/02/2026) et la remise du nouvel extrait"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Activité 442103</t>
-        </is>
-      </c>
-      <c r="B18" s="43" t="inlineStr">
-        <is>
-          <t>Importation de pneumatiques</t>
-        </is>
-      </c>
-      <c r="C18" s="29" t="inlineStr"/>
-    </row>
-    <row r="19" ht="32" customHeight="1">
+          <t>Expiration de l'ancien extrait</t>
+        </is>
+      </c>
+      <c r="B18" s="47">
+        <f>DATE(2026,2,13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Activité 442104</t>
-        </is>
-      </c>
-      <c r="B19" s="43" t="inlineStr">
-        <is>
-          <t>Importation de batteries liées au domaine mécanique</t>
-        </is>
-      </c>
-      <c r="C19" s="29" t="inlineStr"/>
-    </row>
-    <row r="20" ht="32" customHeight="1">
+          <t>Remise de l'extrait modifié</t>
+        </is>
+      </c>
+      <c r="B19" s="47">
+        <f>DATE(2026,7,29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Activités exercées NON inscrites</t>
-        </is>
-      </c>
-      <c r="B20" s="43" t="inlineStr">
-        <is>
-          <t>Travaux publics / TPM, location d'engins, transport et distribution de marchandises</t>
-        </is>
-      </c>
-      <c r="C20" s="29" t="inlineStr">
-        <is>
-          <t>Exercées et facturées (70602 : 25,5 M en 2025 ; G50 « TPM et location » ; CNAS TPM) hors objet du registre</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="32" customHeight="1">
+          <t>Jours sans extrait en cours de validité remis</t>
+        </is>
+      </c>
+      <c r="B20" s="48">
+        <f>MAX(0,B19-B18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Date de la dernière modification</t>
-        </is>
-      </c>
-      <c r="B21" s="43" t="inlineStr">
-        <is>
-          <t>10/09/2024</t>
-        </is>
-      </c>
-      <c r="C21" s="29" t="inlineStr"/>
-    </row>
-    <row r="22" ht="32" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>Durée de validité de l'extrait</t>
-        </is>
-      </c>
-      <c r="B22" s="43" t="inlineStr">
-        <is>
-          <t>Du 13/02/2024 au 13/02/2026</t>
-        </is>
-      </c>
-      <c r="C22" s="44">
-        <f>IF(B26&gt;0,"EXPIRÉ depuis le 13/02/2026 : renouvellement à faire immédiatement","Valide")</f>
-        <v/>
+          <t>Prochaine échéance de renouvellement</t>
+        </is>
+      </c>
+      <c r="B21" s="49">
+        <f>DATE(2028,2,16)</f>
+        <v/>
+      </c>
+      <c r="C21" s="21" t="inlineStr">
+        <is>
+          <t>Lancer le renouvellement au moins 2 mois avant</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>B. Augmentation de capital 2026 — sources possibles au 31/12/2025 (balance)</t>
+        </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>Fin de validité de l'extrait</t>
-        </is>
-      </c>
-      <c r="B24" s="45">
-        <f>DATE(2026,2,13)</f>
-        <v/>
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>Rubrique</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>Comptes</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>Montant (DA)</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>Commentaire</t>
+        </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Date d'arrêté du dossier</t>
-        </is>
-      </c>
-      <c r="B25" s="45">
-        <f>DATE(2026,10,1)</f>
-        <v/>
+          <t>Augmentation de capital à justifier</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>10100</t>
+        </is>
+      </c>
+      <c r="C25" s="7">
+        <f>C8-B8</f>
+        <v/>
+      </c>
+      <c r="D25" s="35" t="inlineStr">
+        <is>
+          <t>Capital extrait 2026 − capital extrait 2024</t>
+        </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>Jours d'activité depuis l'expiration</t>
-        </is>
-      </c>
-      <c r="B26" s="46">
-        <f>MAX(0,B25-B24)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28" ht="45" customHeight="1">
-      <c r="A28" s="47" t="inlineStr">
-        <is>
-          <t>Sanctions rappelées au verso de l'extrait (loi n° 04-08 du 14/08/2004 modifiée, art. 31 à 41 bis) : amende de 5 000 à 5 000 000 DA et/ou emprisonnement de 6 mois à 1 an, notamment pour exercice avec un extrait expiré, commerce hors de l'objet du registre et défaut de modification de l'extrait.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="45" customHeight="1">
-      <c r="A29" s="48" t="inlineStr">
-        <is>
-          <t>À vérifier avec un juriste : l'activité d'importation pour la revente en l'état est en principe réservée à des sociétés qui l'exercent à titre exclusif ; l'ajout des activités TPM / location au même registre peut ne pas être possible et imposer une structure distincte.</t>
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>Réserves et écarts incorporables</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>105, 106</t>
+        </is>
+      </c>
+      <c r="C26" s="6">
+        <f>-(SUMPRODUCT((LEFT('Balance 2024-2025'!$A$5:$A$104,3)="105")*'Balance 2024-2025'!$D$5:$D$104)+SUMPRODUCT((LEFT('Balance 2024-2025'!$A$5:$A$104,3)="106")*'Balance 2024-2025'!$D$5:$D$104))</f>
+        <v/>
+      </c>
+      <c r="D26" s="35" t="inlineStr">
+        <is>
+          <t>Incorporation possible par décision d'AGE</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>Résultat 2025</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>12 (exercice 2025)</t>
+        </is>
+      </c>
+      <c r="C27" s="6">
+        <f>'États 2024-2025'!D16</f>
+        <v/>
+      </c>
+      <c r="D27" s="35" t="inlineStr">
+        <is>
+          <t>Si affecté en 2026 aux réserves puis incorporé</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>Comptes courants d'associés</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>455, 457</t>
+        </is>
+      </c>
+      <c r="C28" s="6">
+        <f>-(SUMPRODUCT((LEFT('Balance 2024-2025'!$A$5:$A$104,3)="455")*'Balance 2024-2025'!$D$5:$D$104)+SUMPRODUCT((LEFT('Balance 2024-2025'!$A$5:$A$104,3)="457")*'Balance 2024-2025'!$D$5:$D$104))</f>
+        <v/>
+      </c>
+      <c r="D28" s="35" t="inlineStr">
+        <is>
+          <t>Conversion de créances des associés en capital</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Total des sources identifiées</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="inlineStr"/>
+      <c r="C29" s="7">
+        <f>SUM(C26:C28)</f>
+        <v/>
+      </c>
+      <c r="D29" s="35" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>Couverture de l'augmentation</t>
+        </is>
+      </c>
+      <c r="B30" s="12" t="inlineStr"/>
+      <c r="C30" s="38">
+        <f>IF(C25=0,"",C29/C25)</f>
+        <v/>
+      </c>
+      <c r="D30" s="35" t="inlineStr">
+        <is>
+          <t>Supérieure à 100 % : l'augmentation peut être financée sans apport en numéraire</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>Réserve légale minimale après augmentation (10 % du capital)</t>
+        </is>
+      </c>
+      <c r="C31" s="30">
+        <f>C8*10%</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t>Réserve légale au 31/12/2025 (10610)</t>
+        </is>
+      </c>
+      <c r="C32" s="6">
+        <f>-'Balance 2024-2025'!D7</f>
+        <v/>
+      </c>
+      <c r="D32" s="21" t="inlineStr">
+        <is>
+          <t>Dotation de 5 % du bénéfice à poursuivre jusqu'au plafond</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="48" customHeight="1">
+      <c r="A34" s="50" t="inlineStr">
+        <is>
+          <t>Pièces à obtenir : PV d'AGE et rapport de gestion, statuts modifiés (acte notarié), publication BOAL, justificatif de libération (incorporation ou apports), enregistrement fiscal. Écriture 2026 attendue : débit 106x / 455-457 (ou 512 si apport en numéraire), crédit 10100 pour 162 000 000 DA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="32" customHeight="1">
+      <c r="A36" s="51" t="inlineStr">
+        <is>
+          <t>Sanctions rappelées au verso (loi n° 04-08 du 14/08/2004 modifiée) : amende de 5 000 à 5 000 000 DA et/ou 6 mois à 1 an d'emprisonnement, notamment pour commerce hors de l'objet du registre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="32" customHeight="1">
+      <c r="A37" s="50" t="inlineStr">
+        <is>
+          <t>À vérifier avec un juriste : l'importation pour la revente en l'état est en principe réservée à des sociétés qui l'exercent à titre exclusif ; les activités TPM / location pourraient devoir être portées par une société distincte.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A29:C29"/>
-    <mergeCell ref="A28:C28"/>
+  <mergeCells count="3">
+    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="A37:D37"/>
+    <mergeCell ref="A36:D36"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
@@ -35025,11 +35206,11 @@
         <f>IF(C24="","",C24-B24)</f>
         <v/>
       </c>
-      <c r="E24" s="45">
+      <c r="E24" s="47">
         <f>DATE(2026,2,20)</f>
         <v/>
       </c>
-      <c r="F24" s="45">
+      <c r="F24" s="47">
         <f>DATE(2026,3,30)</f>
         <v/>
       </c>
@@ -35060,11 +35241,11 @@
         <f>IF(C25="","",C25-B25)</f>
         <v/>
       </c>
-      <c r="E25" s="45">
+      <c r="E25" s="47">
         <f>DATE(2026,3,20)</f>
         <v/>
       </c>
-      <c r="F25" s="45">
+      <c r="F25" s="47">
         <f>DATE(2026,4,7)</f>
         <v/>
       </c>
@@ -35095,11 +35276,11 @@
         <f>IF(C26="","",C26-B26)</f>
         <v/>
       </c>
-      <c r="E26" s="45">
+      <c r="E26" s="47">
         <f>DATE(2026,4,20)</f>
         <v/>
       </c>
-      <c r="F26" s="45">
+      <c r="F26" s="47">
         <f>DATE(2026,4,30)</f>
         <v/>
       </c>
@@ -35130,11 +35311,11 @@
         <f>IF(C27="","",C27-B27)</f>
         <v/>
       </c>
-      <c r="E27" s="45">
+      <c r="E27" s="47">
         <f>DATE(2026,5,20)</f>
         <v/>
       </c>
-      <c r="F27" s="45">
+      <c r="F27" s="47">
         <f>DATE(2026,6,2)</f>
         <v/>
       </c>
@@ -35163,11 +35344,11 @@
         <f>IF(C28="","",C28-B28)</f>
         <v/>
       </c>
-      <c r="E28" s="45">
+      <c r="E28" s="47">
         <f>DATE(2026,6,20)</f>
         <v/>
       </c>
-      <c r="F28" s="45" t="n"/>
+      <c r="F28" s="47" t="n"/>
       <c r="G28" s="13">
         <f>IF(F28="","",F28-E28)</f>
         <v/>
@@ -35195,11 +35376,11 @@
         <f>IF(C29="","",C29-B29)</f>
         <v/>
       </c>
-      <c r="E29" s="45">
+      <c r="E29" s="47">
         <f>DATE(2026,2,28)</f>
         <v/>
       </c>
-      <c r="F29" s="45">
+      <c r="F29" s="47">
         <f>DATE(2026,3,4)</f>
         <v/>
       </c>
@@ -35230,11 +35411,11 @@
         <f>IF(C30="","",C30-B30)</f>
         <v/>
       </c>
-      <c r="E30" s="45">
+      <c r="E30" s="47">
         <f>DATE(2026,3,31)</f>
         <v/>
       </c>
-      <c r="F30" s="45">
+      <c r="F30" s="47">
         <f>DATE(2026,4,6)</f>
         <v/>
       </c>
@@ -35265,11 +35446,11 @@
         <f>IF(C31="","",C31-B31)</f>
         <v/>
       </c>
-      <c r="E31" s="45">
+      <c r="E31" s="47">
         <f>DATE(2026,4,30)</f>
         <v/>
       </c>
-      <c r="F31" s="45">
+      <c r="F31" s="47">
         <f>DATE(2026,5,10)</f>
         <v/>
       </c>
@@ -35300,11 +35481,11 @@
         <f>IF(C32="","",C32-B32)</f>
         <v/>
       </c>
-      <c r="E32" s="45">
+      <c r="E32" s="47">
         <f>DATE(2026,4,30)</f>
         <v/>
       </c>
-      <c r="F32" s="45">
+      <c r="F32" s="47">
         <f>DATE(2026,5,12)</f>
         <v/>
       </c>
@@ -35559,7 +35740,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -35640,7 +35821,7 @@
           <t>A01</t>
         </is>
       </c>
-      <c r="B5" s="49" t="n">
+      <c r="B5" s="52" t="n">
         <v>2</v>
       </c>
       <c r="C5" s="29" t="inlineStr">
@@ -35658,7 +35839,7 @@
           <t>Déclaration CNAS de février 2026 non fournie (assiette paie 952 475,81 ; 7 STC payés). Le relevé CPA montre un paiement de 333 366,53 le 06/04/2026, égal aux cotisations calculées : la déclaration a donc probablement été déposée.</t>
         </is>
       </c>
-      <c r="F5" s="50">
+      <c r="F5" s="53">
         <f>'Rappro CNAS'!J6</f>
         <v/>
       </c>
@@ -35680,7 +35861,7 @@
           <t>A02</t>
         </is>
       </c>
-      <c r="B6" s="51" t="n">
+      <c r="B6" s="54" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="29" t="inlineStr">
@@ -35698,7 +35879,7 @@
           <t>Centralisateur de mars 2026 absent (onglet vide) alors que la CNAS de mars déclare 368 389,93 d'assiette, 5 salariés.</t>
         </is>
       </c>
-      <c r="F6" s="50">
+      <c r="F6" s="53">
         <f>'Rappro CNAS'!K7</f>
         <v/>
       </c>
@@ -35720,7 +35901,7 @@
           <t>A03</t>
         </is>
       </c>
-      <c r="B7" s="51" t="n">
+      <c r="B7" s="54" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="29" t="inlineStr">
@@ -35738,7 +35919,7 @@
           <t>Prime de ponctualité (R540) imposée à l'IRG mais exclue du salaire de poste (assiette CNAS) chaque mois.</t>
         </is>
       </c>
-      <c r="F7" s="50">
+      <c r="F7" s="53">
         <f>'Rappro CNAS'!V13</f>
         <v/>
       </c>
@@ -35760,7 +35941,7 @@
           <t>A04</t>
         </is>
       </c>
-      <c r="B8" s="49" t="n">
+      <c r="B8" s="52" t="n">
         <v>2</v>
       </c>
       <c r="C8" s="29" t="inlineStr">
@@ -35778,7 +35959,7 @@
           <t>Effectif déclaré au T1 = 2 alors que 3 salariés sont inscrits ; T2 déclare 1 sortie et un effectif final de 2 ⇒ T1 aurait dû être 3.</t>
         </is>
       </c>
-      <c r="F8" s="52" t="n"/>
+      <c r="F8" s="55" t="n"/>
       <c r="G8" s="29" t="inlineStr">
         <is>
           <t>Rectifier l'effectif du T1 auprès de la CNAS.</t>
@@ -35797,7 +35978,7 @@
           <t>A05</t>
         </is>
       </c>
-      <c r="B9" s="49" t="n">
+      <c r="B9" s="52" t="n">
         <v>2</v>
       </c>
       <c r="C9" s="29" t="inlineStr">
@@ -35815,7 +35996,7 @@
           <t>Salarié totalement absent (non rémunéré) en juillet, disparu de la paie en août sans STC ni sortie déclarée.</t>
         </is>
       </c>
-      <c r="F9" s="52" t="n"/>
+      <c r="F9" s="55" t="n"/>
       <c r="G9" s="29" t="inlineStr">
         <is>
           <t>Établir le STC et déclarer la sortie dans l'EMS du T3 (échéance 30/10/2026).</t>
@@ -35834,7 +36015,7 @@
           <t>A06</t>
         </is>
       </c>
-      <c r="B10" s="49" t="n">
+      <c r="B10" s="52" t="n">
         <v>2</v>
       </c>
       <c r="C10" s="29" t="inlineStr">
@@ -35852,7 +36033,7 @@
           <t>STC de 2 237,40 en août : une sortie à déclarer au T3.</t>
         </is>
       </c>
-      <c r="F10" s="52" t="n"/>
+      <c r="F10" s="55" t="n"/>
       <c r="G10" s="29" t="inlineStr">
         <is>
           <t>Déclarer la sortie dans l'EMS du T3.</t>
@@ -35871,7 +36052,7 @@
           <t>A07</t>
         </is>
       </c>
-      <c r="B11" s="49" t="n">
+      <c r="B11" s="52" t="n">
         <v>2</v>
       </c>
       <c r="C11" s="29" t="inlineStr">
@@ -35889,7 +36070,7 @@
           <t>Déclarations T3 2026 (juil–sept) à établir ; paie de septembre non fournie.</t>
         </is>
       </c>
-      <c r="F11" s="50">
+      <c r="F11" s="53">
         <f>'Rappro CNAS'!J9+'Rappro CNAS'!J12</f>
         <v/>
       </c>
@@ -35911,7 +36092,7 @@
           <t>A08</t>
         </is>
       </c>
-      <c r="B12" s="53" t="n">
+      <c r="B12" s="56" t="n">
         <v>3</v>
       </c>
       <c r="C12" s="29" t="inlineStr">
@@ -35929,7 +36110,7 @@
           <t>Avril = mai et juillet = août strictement identiques (mêmes absences, heures sup., IRG) : variables probablement non saisies.</t>
         </is>
       </c>
-      <c r="F12" s="52" t="n"/>
+      <c r="F12" s="55" t="n"/>
       <c r="G12" s="29" t="inlineStr">
         <is>
           <t>Contrôler les pointages et bulletins de mai et août.</t>
@@ -35948,7 +36129,7 @@
           <t>A09</t>
         </is>
       </c>
-      <c r="B13" s="53" t="n">
+      <c r="B13" s="56" t="n">
         <v>3</v>
       </c>
       <c r="C13" s="29" t="inlineStr">
@@ -35966,7 +36147,7 @@
           <t>Frais de mission élevés (avril 41 615 ; mai 49 115, soit 47–55 % de l'assiette), non soumis à cotisations.</t>
         </is>
       </c>
-      <c r="F13" s="50">
+      <c r="F13" s="53">
         <f>'Paie TPM'!K26</f>
         <v/>
       </c>
@@ -35988,7 +36169,7 @@
           <t>A10</t>
         </is>
       </c>
-      <c r="B14" s="53" t="n">
+      <c r="B14" s="56" t="n">
         <v>3</v>
       </c>
       <c r="C14" s="29" t="inlineStr">
@@ -36006,7 +36187,7 @@
           <t>Prime de responsabilité de 5,00 DA (janv.) et 1,14 DA (févr.) : paramètre vraisemblablement erroné (5 au lieu de 5 %).</t>
         </is>
       </c>
-      <c r="F14" s="52" t="n"/>
+      <c r="F14" s="55" t="n"/>
       <c r="G14" s="29" t="inlineStr">
         <is>
           <t>Corriger le paramètre B291 ; régulariser le rappel éventuel.</t>
@@ -36025,7 +36206,7 @@
           <t>A11</t>
         </is>
       </c>
-      <c r="B15" s="49" t="n">
+      <c r="B15" s="52" t="n">
         <v>2</v>
       </c>
       <c r="C15" s="29" t="inlineStr">
@@ -36043,7 +36224,7 @@
           <t>Bordereaux de versement CNAS à « 0,00 ». Relevé CPA : paiements retrouvés pour janvier, février, mars IMPORT et T1 TPM (jusqu'à 12 jours après l'échéance) ; T2 à justifier.</t>
         </is>
       </c>
-      <c r="F15" s="50">
+      <c r="F15" s="53">
         <f>'Rappro CNAS'!K13</f>
         <v/>
       </c>
@@ -36065,7 +36246,7 @@
           <t>A12</t>
         </is>
       </c>
-      <c r="B16" s="49" t="n">
+      <c r="B16" s="52" t="n">
         <v>2</v>
       </c>
       <c r="C16" s="29" t="inlineStr">
@@ -36083,7 +36264,7 @@
           <t>IRG IMPORT : G50 de janvier à août conformes à la paie (écarts d'arrondi ≤ 3 DA ; juillet : 2,30 DA retenus non reversés). Mars non vérifiable (paie absente).</t>
         </is>
       </c>
-      <c r="F16" s="50">
+      <c r="F16" s="53">
         <f>'Échéancier IRG-CNAS'!G13</f>
         <v/>
       </c>
@@ -36105,7 +36286,7 @@
           <t>A13</t>
         </is>
       </c>
-      <c r="B17" s="53" t="n">
+      <c r="B17" s="56" t="n">
         <v>3</v>
       </c>
       <c r="C17" s="29" t="inlineStr">
@@ -36123,7 +36304,7 @@
           <t>Paie paramétrée CACOBATPH (taux X504) mais aucune déclaration CACOBATPH (congés payés / intempéries) dans le dossier.</t>
         </is>
       </c>
-      <c r="F17" s="52" t="n"/>
+      <c r="F17" s="55" t="n"/>
       <c r="G17" s="29" t="inlineStr">
         <is>
           <t>Fournir les déclarations et paiements CACOBATPH 2026.</t>
@@ -36142,7 +36323,7 @@
           <t>A14</t>
         </is>
       </c>
-      <c r="B18" s="53" t="n">
+      <c r="B18" s="56" t="n">
         <v>3</v>
       </c>
       <c r="C18" s="29" t="inlineStr">
@@ -36160,7 +36341,7 @@
           <t>Libellés divergents : « D.P.R.COMPAGNY » / « DPR COMPAGNY » ; en-tête de paie TPM à l'adresse VGE TIZI alors que l'affiliation TPM est à TISSA.</t>
         </is>
       </c>
-      <c r="F18" s="52" t="n"/>
+      <c r="F18" s="55" t="n"/>
       <c r="G18" s="29" t="inlineStr">
         <is>
           <t>Harmoniser raison sociale et adresse dans le logiciel de paie.</t>
@@ -36179,7 +36360,7 @@
           <t>A15</t>
         </is>
       </c>
-      <c r="B19" s="53" t="n">
+      <c r="B19" s="56" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="29" t="inlineStr">
@@ -36197,7 +36378,7 @@
           <t>Périodicité mixte : déclarations mensuelles (janv., mars) puis trimestrielle (T2).</t>
         </is>
       </c>
-      <c r="F19" s="52" t="n"/>
+      <c r="F19" s="55" t="n"/>
       <c r="G19" s="29" t="inlineStr">
         <is>
           <t>Confirmer auprès de la CNAS le passage au trimestriel après la baisse d'effectif (12 → 5).</t>
@@ -36216,7 +36397,7 @@
           <t>A16</t>
         </is>
       </c>
-      <c r="B20" s="53" t="n">
+      <c r="B20" s="56" t="n">
         <v>3</v>
       </c>
       <c r="C20" s="29" t="inlineStr">
@@ -36234,7 +36415,7 @@
           <t>IRG non vérifiable salarié par salarié (centralisateurs uniquement).</t>
         </is>
       </c>
-      <c r="F20" s="52" t="n"/>
+      <c r="F20" s="55" t="n"/>
       <c r="G20" s="29" t="inlineStr">
         <is>
           <t>Fournir le livre de paie individuel / bulletins.</t>
@@ -36253,7 +36434,7 @@
           <t>A17</t>
         </is>
       </c>
-      <c r="B21" s="51" t="n">
+      <c r="B21" s="54" t="n">
         <v>1</v>
       </c>
       <c r="C21" s="29" t="inlineStr">
@@ -36271,7 +36452,7 @@
           <t>TVA collectée TPM (44537) et location (44527) jamais soldées : 58,9 M DA cumulés au 31/12/2025, accumulés depuis au moins 2022 (37,3 M à l'ouverture 2023) ; 2023–2025 : 18,5 M collectés, 1,5 M apurés. En 2025, 4 839 300 de TVA TPM générée, seuls 391 208 passés en G50 (déc.). Les G50 TPM 2026 (juil., août) ne déclarent aucun CA et reportent un précompte de 1 714 499 (= compte 44550).</t>
         </is>
       </c>
-      <c r="F21" s="50">
+      <c r="F21" s="53">
         <f>-('Balance 2024-2025'!D48+'Balance 2024-2025'!D47)</f>
         <v/>
       </c>
@@ -36293,7 +36474,7 @@
           <t>A18</t>
         </is>
       </c>
-      <c r="B22" s="51" t="n">
+      <c r="B22" s="54" t="n">
         <v>1</v>
       </c>
       <c r="C22" s="29" t="inlineStr">
@@ -36311,7 +36492,7 @@
           <t>CA de mars 2026 réalisé 27 006 870 (annotation G50), mais seulement 3 445 200 déclarés en mars « pour manque TVA à récupérer » : 23 561 670 de CA reportés sur avril–août. En avril, le CA annoté (13 157 894,74) est calculé pour obtenir 2 500 000 de TVA. Le CA déclaré mensuellement est ajusté à la TVA déductible disponible.</t>
         </is>
       </c>
-      <c r="F22" s="50">
+      <c r="F22" s="53">
         <f>'G50 2026'!B40</f>
         <v/>
       </c>
@@ -36333,7 +36514,7 @@
           <t>A19</t>
         </is>
       </c>
-      <c r="B23" s="51" t="n">
+      <c r="B23" s="54" t="n">
         <v>1</v>
       </c>
       <c r="C23" s="29" t="inlineStr">
@@ -36351,7 +36532,7 @@
           <t>G50 TPM d'avril à juillet identiques (mois imprimé « AVRIL », IRG 9 375 chaque mois) : juin sous-déclaré de 9 614,90 (18 989,90 retenus), juillet sur-déclaré de 5 683,70. Janvier–mars et août conformes.</t>
         </is>
       </c>
-      <c r="F23" s="50">
+      <c r="F23" s="53">
         <f>-'G50 TPM 2026'!G15</f>
         <v/>
       </c>
@@ -36373,7 +36554,7 @@
           <t>A20</t>
         </is>
       </c>
-      <c r="B24" s="49" t="n">
+      <c r="B24" s="52" t="n">
         <v>2</v>
       </c>
       <c r="C24" s="29" t="inlineStr">
@@ -36391,7 +36572,7 @@
           <t>Écriture du 31/12/2025 « POUR SOLDE PRCT EXE 2025 » passée en sens inverse (D 44410 / C 444, 3 074 299) : dette IBS 9,79 M et acomptes 6,15 M au lieu d'un net de 3 642 951.</t>
         </is>
       </c>
-      <c r="F24" s="50" t="n">
+      <c r="F24" s="53" t="n">
         <v>3074299</v>
       </c>
       <c r="G24" s="29" t="inlineStr">
@@ -36412,7 +36593,7 @@
           <t>A21</t>
         </is>
       </c>
-      <c r="B25" s="49" t="n">
+      <c r="B25" s="52" t="n">
         <v>2</v>
       </c>
       <c r="C25" s="29" t="inlineStr">
@@ -36430,7 +36611,7 @@
           <t>Solde IBS 2024 réglé le 03/07/2025 ; IBS 2025 net à liquider de 3 642 951 (précomptes douane déduits).</t>
         </is>
       </c>
-      <c r="F25" s="50" t="n">
+      <c r="F25" s="53" t="n">
         <v>3642951</v>
       </c>
       <c r="G25" s="29" t="inlineStr">
@@ -36451,7 +36632,7 @@
           <t>A22</t>
         </is>
       </c>
-      <c r="B26" s="49" t="n">
+      <c r="B26" s="52" t="n">
         <v>2</v>
       </c>
       <c r="C26" s="29" t="inlineStr">
@@ -36469,7 +36650,7 @@
           <t>Caisse de 12,1 M au 31/12/2025 (pic de 22,5 M) ; remboursement en espèces de 6 800 000 à SARL DPR AXXAM le 06/12/2025.</t>
         </is>
       </c>
-      <c r="F26" s="50">
+      <c r="F26" s="53">
         <f>'Balance 2024-2025'!D67</f>
         <v/>
       </c>
@@ -36491,7 +36672,7 @@
           <t>A23</t>
         </is>
       </c>
-      <c r="B27" s="49" t="n">
+      <c r="B27" s="52" t="n">
         <v>2</v>
       </c>
       <c r="C27" s="29" t="inlineStr">
@@ -36509,7 +36690,7 @@
           <t>100 % du CA TPM 2025 (25,47 M) facturé à SARL DPR AXXAM BRIQUETERIE ; aucune facturation TPM d'oct. à déc. 2025 alors que du personnel TPM reste payé.</t>
         </is>
       </c>
-      <c r="F27" s="50">
+      <c r="F27" s="53">
         <f>-'Balance 2024-2025'!D100</f>
         <v/>
       </c>
@@ -36531,7 +36712,7 @@
           <t>A24</t>
         </is>
       </c>
-      <c r="B28" s="49" t="n">
+      <c r="B28" s="52" t="n">
         <v>2</v>
       </c>
       <c r="C28" s="29" t="inlineStr">
@@ -36549,7 +36730,7 @@
           <t>Compte d'attente 47000 non soldé (« SARL FAHAS ?? », « TRESORERIE BEJAIA ?? », chèques).</t>
         </is>
       </c>
-      <c r="F28" s="50">
+      <c r="F28" s="53">
         <f>'Balance 2024-2025'!D59</f>
         <v/>
       </c>
@@ -36571,7 +36752,7 @@
           <t>A25</t>
         </is>
       </c>
-      <c r="B29" s="49" t="n">
+      <c r="B29" s="52" t="n">
         <v>2</v>
       </c>
       <c r="C29" s="29" t="inlineStr">
@@ -36589,7 +36770,7 @@
           <t>Compte 63120 « prime imposable » non soumise à cotisation : 957 406 en 2025 et 1 139 275 en 2024 (même mécanisme que A03).</t>
         </is>
       </c>
-      <c r="F29" s="50">
+      <c r="F29" s="53">
         <f>'États 2024-2025'!C24+'États 2024-2025'!D24</f>
         <v/>
       </c>
@@ -36611,7 +36792,7 @@
           <t>A26</t>
         </is>
       </c>
-      <c r="B30" s="53" t="n">
+      <c r="B30" s="56" t="n">
         <v>3</v>
       </c>
       <c r="C30" s="29" t="inlineStr">
@@ -36629,7 +36810,7 @@
           <t>Banque CPA El Kseur (51220) créditrice de 12,43 M au 31/12/2025 : découvert présenté en banque.</t>
         </is>
       </c>
-      <c r="F30" s="50">
+      <c r="F30" s="53">
         <f>ABS('Balance 2024-2025'!D63)</f>
         <v/>
       </c>
@@ -36651,7 +36832,7 @@
           <t>A27</t>
         </is>
       </c>
-      <c r="B31" s="53" t="n">
+      <c r="B31" s="56" t="n">
         <v>3</v>
       </c>
       <c r="C31" s="29" t="inlineStr">
@@ -36669,7 +36850,7 @@
           <t>Reversements IRG 2025 parfois partiels (févr., juin) et rattrapés le mois suivant ; amendes 2025 : douane 100 000, CNAS 1 746.</t>
         </is>
       </c>
-      <c r="F31" s="50">
+      <c r="F31" s="53">
         <f>'Balance 2024-2025'!D93</f>
         <v/>
       </c>
@@ -36691,7 +36872,7 @@
           <t>A28</t>
         </is>
       </c>
-      <c r="B32" s="53" t="n">
+      <c r="B32" s="56" t="n">
         <v>3</v>
       </c>
       <c r="C32" s="29" t="inlineStr">
@@ -36709,7 +36890,7 @@
           <t>Modèles G50 non mis à jour : dates de signature de 2021–2022 sur toutes les G50 2026, onglet de saisie figé (mai, TVA 17 %), G50 TPM contenant le récap TVA de déc. 2025 et un extrait de journal 2019 ; libellés de comptes de TVA à 17 %.</t>
         </is>
       </c>
-      <c r="F32" s="52" t="n"/>
+      <c r="F32" s="55" t="n"/>
       <c r="G32" s="29" t="inlineStr">
         <is>
           <t>Mettre à jour le modèle et les libellés (TVA 19 %).</t>
@@ -36728,7 +36909,7 @@
           <t>A29</t>
         </is>
       </c>
-      <c r="B33" s="53" t="n">
+      <c r="B33" s="56" t="n">
         <v>3</v>
       </c>
       <c r="C33" s="29" t="inlineStr">
@@ -36746,7 +36927,7 @@
           <t>Taxe d'apprentissage payée deux fois en 2026 : février (87 828 IMPORT sur 8 782 828 + 9 851 TPM sur 985 118) et août (44 091 IMPORT sur 4 409 079 + 6 809 TPM sur 680 900).</t>
         </is>
       </c>
-      <c r="F33" s="50">
+      <c r="F33" s="53">
         <f>'G50 2026'!J26+'G50 TPM 2026'!J17</f>
         <v/>
       </c>
@@ -36768,7 +36949,7 @@
           <t>A30</t>
         </is>
       </c>
-      <c r="B34" s="53" t="n">
+      <c r="B34" s="56" t="n">
         <v>3</v>
       </c>
       <c r="C34" s="29" t="inlineStr">
@@ -36786,7 +36967,7 @@
           <t>Droit de timbre : taux apparents incohérents (janv. 2,0 %, févr. 1,0 %, avr. 5,05 %, mai 1,79 %) ; même base en avril et mai ; aucun timbre en mars et de juin à août.</t>
         </is>
       </c>
-      <c r="F34" s="50">
+      <c r="F34" s="53">
         <f>'G50 2026'!J24</f>
         <v/>
       </c>
@@ -36808,7 +36989,7 @@
           <t>A32</t>
         </is>
       </c>
-      <c r="B35" s="51" t="n">
+      <c r="B35" s="54" t="n">
         <v>1</v>
       </c>
       <c r="C35" s="29" t="inlineStr">
@@ -36826,7 +37007,7 @@
           <t>Journal 2023 fourni provisoire : résultat 18,54 M contre 7,26 M repris en à-nouveau 2024 ; 38 comptes en écart avec les ouvertures 2024 (stocks, fournisseurs, banques, IBS, TVA).</t>
         </is>
       </c>
-      <c r="F35" s="50">
+      <c r="F35" s="53">
         <f>'Contrôle 2023'!B6</f>
         <v/>
       </c>
@@ -36848,7 +37029,7 @@
           <t>A33</t>
         </is>
       </c>
-      <c r="B36" s="51" t="n">
+      <c r="B36" s="54" t="n">
         <v>1</v>
       </c>
       <c r="C36" s="29" t="inlineStr">
@@ -36866,7 +37047,7 @@
           <t>Créance SARL DPR AXXAM BRIQUETERIE : 371,0 M au 31/12/2025 (96 % du poste clients), en hausse continue depuis 2023 (277,7 M) ; 2023–2025 : 115,7 M facturés, 26,2 M encaissés (23 %).</t>
         </is>
       </c>
-      <c r="F36" s="50">
+      <c r="F36" s="53">
         <f>'Démarrage 2026'!E8</f>
         <v/>
       </c>
@@ -36888,7 +37069,7 @@
           <t>A34</t>
         </is>
       </c>
-      <c r="B37" s="51" t="n">
+      <c r="B37" s="54" t="n">
         <v>1</v>
       </c>
       <c r="C37" s="29" t="inlineStr">
@@ -36906,7 +37087,7 @@
           <t>Avances clients (419) dormantes : 229,4 M sur 144 clients, inchangées depuis au moins le 01/01/2023 (hors associés et clients à compenser). Soit livraisons non facturées (CA et TVA non déclarés), soit dettes à rembourser.</t>
         </is>
       </c>
-      <c r="F37" s="50">
+      <c r="F37" s="53">
         <f>'Démarrage 2026'!E35</f>
         <v/>
       </c>
@@ -36928,7 +37109,7 @@
           <t>A35</t>
         </is>
       </c>
-      <c r="B38" s="51" t="n">
+      <c r="B38" s="54" t="n">
         <v>1</v>
       </c>
       <c r="C38" s="29" t="inlineStr">
@@ -36946,7 +37127,7 @@
           <t>SARL DPR AXXAM : 62,5 M versés en 2025 (dont 45,35 M d'avances 409 sans facture) et 6,8 M remboursés en espèces, alors que la briqueterie du même groupe ne paie pas.</t>
         </is>
       </c>
-      <c r="F38" s="50">
+      <c r="F38" s="53">
         <f>'Démarrage 2026'!B21</f>
         <v/>
       </c>
@@ -36968,7 +37149,7 @@
           <t>A36</t>
         </is>
       </c>
-      <c r="B39" s="49" t="n">
+      <c r="B39" s="52" t="n">
         <v>2</v>
       </c>
       <c r="C39" s="29" t="inlineStr">
@@ -36986,7 +37167,7 @@
           <t>Associés (famille DJENNADI, dont les 3 gérants inscrits au registre de commerce : Abdelkrim, Ryad, Ahcene) logés en comptes clients / fournisseurs : soldes créditeurs en 411, 419 et 401.</t>
         </is>
       </c>
-      <c r="F39" s="50">
+      <c r="F39" s="53">
         <f>'Démarrage 2026'!E26</f>
         <v/>
       </c>
@@ -37008,8 +37189,8 @@
           <t>A37</t>
         </is>
       </c>
-      <c r="B40" s="51" t="n">
-        <v>1</v>
+      <c r="B40" s="56" t="n">
+        <v>3</v>
       </c>
       <c r="C40" s="29" t="inlineStr">
         <is>
@@ -37023,16 +37204,16 @@
       </c>
       <c r="E40" s="29" t="inlineStr">
         <is>
-          <t>Extrait du registre de commerce valable jusqu'au 13/02/2026 seulement : activité poursuivie avec un extrait expiré depuis plus de 7 mois.</t>
-        </is>
-      </c>
-      <c r="F40" s="50">
-        <f>'Registre de commerce'!B26</f>
+          <t>Extrait expiré le 13/02/2026, renouvelé par l'extrait modifié remis le 29/07/2026 (validité 16/02/2026 – 16/02/2028) : 166 jours sans extrait valide remis.</t>
+        </is>
+      </c>
+      <c r="F40" s="53">
+        <f>'Registre de commerce'!B20</f>
         <v/>
       </c>
       <c r="G40" s="29" t="inlineStr">
         <is>
-          <t>Renouveler l'extrait au CNRC sans délai (jours écoulés en impact).</t>
+          <t>Régularisé ; prochain renouvellement avant le 16/02/2028 (impact = jours sans extrait).</t>
         </is>
       </c>
       <c r="H40" s="41" t="n"/>
@@ -37048,7 +37229,7 @@
           <t>A38</t>
         </is>
       </c>
-      <c r="B41" s="51" t="n">
+      <c r="B41" s="54" t="n">
         <v>1</v>
       </c>
       <c r="C41" s="29" t="inlineStr">
@@ -37063,10 +37244,10 @@
       </c>
       <c r="E41" s="29" t="inlineStr">
         <is>
-          <t>Registre limité à l'importation pour revente en l'état (442101 à 442104) ; les activités TPM, location d'engins et transport sont exercées et facturées hors objet du registre.</t>
-        </is>
-      </c>
-      <c r="F41" s="50">
+          <t>Registre limité à l'importation pour revente en l'état (442101 à 442104), y compris dans l'extrait modifié du 29/07/2026 ; les activités TPM, location d'engins et transport sont exercées et facturées hors objet du registre.</t>
+        </is>
+      </c>
+      <c r="F41" s="53">
         <f>-'Balance 2024-2025'!D100</f>
         <v/>
       </c>
@@ -37088,7 +37269,7 @@
           <t>A39</t>
         </is>
       </c>
-      <c r="B42" s="49" t="n">
+      <c r="B42" s="52" t="n">
         <v>2</v>
       </c>
       <c r="C42" s="29" t="inlineStr">
@@ -37106,7 +37287,7 @@
           <t>Aucun établissement secondaire inscrit au registre, alors que l'activité TPM est affiliée à la CNAS à TISSA sous un numéro distinct.</t>
         </is>
       </c>
-      <c r="F42" s="52" t="n"/>
+      <c r="F42" s="55" t="n"/>
       <c r="G42" s="29" t="inlineStr">
         <is>
           <t>Inscrire l'établissement secondaire ou aligner les affiliations.</t>
@@ -37125,7 +37306,7 @@
           <t>A40</t>
         </is>
       </c>
-      <c r="B43" s="53" t="n">
+      <c r="B43" s="56" t="n">
         <v>3</v>
       </c>
       <c r="C43" s="29" t="inlineStr">
@@ -37143,7 +37324,7 @@
           <t>N° de registre de commerce différent entre l'extrait (06/00-0184232 B 03) et le dossier comptable PCCOMPTA (06/01-0184232B03) ; local commercial appartenant à un associé (DJENNADI Abdelkader, créancier de 2,51 M en 401).</t>
         </is>
       </c>
-      <c r="F43" s="52" t="n"/>
+      <c r="F43" s="55" t="n"/>
       <c r="G43" s="29" t="inlineStr">
         <is>
           <t>Corriger le n° RC dans PCCOMPTA ; produire le bail et l'état des loyers.</t>
@@ -37162,7 +37343,7 @@
           <t>A41</t>
         </is>
       </c>
-      <c r="B44" s="51" t="n">
+      <c r="B44" s="54" t="n">
         <v>1</v>
       </c>
       <c r="C44" s="29" t="inlineStr">
@@ -37180,7 +37361,7 @@
           <t>Relevé CPA S1 2026 : 43,5 M virés à SARL DPR AXXAM (6 virements de janvier à avril), après 62,5 M en 2025, alors que le compte est à découvert permanent.</t>
         </is>
       </c>
-      <c r="F44" s="50">
+      <c r="F44" s="53">
         <f>'Banque CPA 2026'!I12</f>
         <v/>
       </c>
@@ -37202,7 +37383,7 @@
           <t>A42</t>
         </is>
       </c>
-      <c r="B45" s="49" t="n">
+      <c r="B45" s="52" t="n">
         <v>2</v>
       </c>
       <c r="C45" s="29" t="inlineStr">
@@ -37220,7 +37401,7 @@
           <t>Compte CPA El Kseur à découvert presque tout le semestre (−19,1 M au 29/06/2026) ; écart de rapprochement au 31/12/2025 entre banque et compte 51220 ; agios non comptabilisés en 2025.</t>
         </is>
       </c>
-      <c r="F45" s="50">
+      <c r="F45" s="53">
         <f>ABS('Banque CPA 2026'!B46)</f>
         <v/>
       </c>
@@ -37242,7 +37423,7 @@
           <t>A43</t>
         </is>
       </c>
-      <c r="B46" s="53" t="n">
+      <c r="B46" s="56" t="n">
         <v>3</v>
       </c>
       <c r="C46" s="29" t="inlineStr">
@@ -37260,7 +37441,7 @@
           <t>Chèques clients rejetés (annulés) sur le relevé CPA en janvier et mars 2026.</t>
         </is>
       </c>
-      <c r="F46" s="50">
+      <c r="F46" s="53">
         <f>'Banque CPA 2026'!I6</f>
         <v/>
       </c>
@@ -37279,31 +37460,34 @@
     <row r="47" ht="52" customHeight="1">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>A31</t>
-        </is>
-      </c>
-      <c r="B47" s="53" t="n">
-        <v>3</v>
+          <t>A44</t>
+        </is>
+      </c>
+      <c r="B47" s="54" t="n">
+        <v>1</v>
       </c>
       <c r="C47" s="29" t="inlineStr">
         <is>
-          <t>Les deux</t>
+          <t>Société</t>
         </is>
       </c>
       <c r="D47" s="29" t="inlineStr">
         <is>
-          <t>Comptabilité</t>
+          <t>Juridique / comptabilité</t>
         </is>
       </c>
       <c r="E47" s="29" t="inlineStr">
         <is>
-          <t>Clients débiteurs 387,1 M et avances clients 314,6 M ; fournisseurs débiteurs 46,2 M au 31/12/2025.</t>
-        </is>
-      </c>
-      <c r="F47" s="52" t="n"/>
+          <t>Capital porté de 106 M à 268 M DA (extrait du 29/07/2026) : +162 M à justifier et à comptabiliser en 2026 ; sources possibles au 31/12/2025 : réserves, résultat 2025, comptes courants d'associés.</t>
+        </is>
+      </c>
+      <c r="F47" s="53">
+        <f>'Registre de commerce'!C25</f>
+        <v/>
+      </c>
       <c r="G47" s="29" t="inlineStr">
         <is>
-          <t>Lettrer les comptes clients/fournisseurs et compenser les avances soldées.</t>
+          <t>Obtenir PV d'AGE, statuts notariés, justificatif de libération ; passer l'écriture 2026 au compte 10100.</t>
         </is>
       </c>
       <c r="H47" s="41" t="n"/>
@@ -37313,15 +37497,52 @@
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
+    <row r="48" ht="52" customHeight="1">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>A31</t>
+        </is>
+      </c>
+      <c r="B48" s="56" t="n">
+        <v>3</v>
+      </c>
+      <c r="C48" s="29" t="inlineStr">
+        <is>
+          <t>Les deux</t>
+        </is>
+      </c>
+      <c r="D48" s="29" t="inlineStr">
+        <is>
+          <t>Comptabilité</t>
+        </is>
+      </c>
+      <c r="E48" s="29" t="inlineStr">
+        <is>
+          <t>Clients débiteurs 387,1 M et avances clients 314,6 M ; fournisseurs débiteurs 46,2 M au 31/12/2025.</t>
+        </is>
+      </c>
+      <c r="F48" s="55" t="n"/>
+      <c r="G48" s="29" t="inlineStr">
+        <is>
+          <t>Lettrer les comptes clients/fournisseurs et compenser les avances soldées.</t>
+        </is>
+      </c>
+      <c r="H48" s="41" t="n"/>
+      <c r="I48" s="41" t="inlineStr">
+        <is>
+          <t>Ouvert</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>Impact : A01 = cotisations calculées de février ; A02 = cotisations de mars déclarées sans justificatif ; A03 = cotisations sur ponctualité ; A07 = cotisations T3 partielles (juil–août) ; A09 = frais de mission TPM cumulés ; A11 = cotisations déclarées sans preuve de paiement ; A12 = IRG cumulé à rapprocher.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I47"/>
+  <autoFilter ref="A4:I48"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>
@@ -37673,7 +37894,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -37749,7 +37970,7 @@
           <t>Janv–août 2026</t>
         </is>
       </c>
-      <c r="E5" s="54" t="inlineStr">
+      <c r="E5" s="57" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -37779,7 +38000,7 @@
           <t>Janv–août 2026</t>
         </is>
       </c>
-      <c r="E6" s="54" t="inlineStr">
+      <c r="E6" s="57" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -37805,7 +38026,7 @@
           <t>Janvier 2026</t>
         </is>
       </c>
-      <c r="E7" s="54" t="inlineStr">
+      <c r="E7" s="57" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -37835,7 +38056,7 @@
           <t>Mars 2026</t>
         </is>
       </c>
-      <c r="E8" s="54" t="inlineStr">
+      <c r="E8" s="57" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -37865,7 +38086,7 @@
           <t>T2 2026</t>
         </is>
       </c>
-      <c r="E9" s="54" t="inlineStr">
+      <c r="E9" s="57" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -37895,7 +38116,7 @@
           <t>T1 2026</t>
         </is>
       </c>
-      <c r="E10" s="54" t="inlineStr">
+      <c r="E10" s="57" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -37925,7 +38146,7 @@
           <t>T2 2026</t>
         </is>
       </c>
-      <c r="E11" s="54" t="inlineStr">
+      <c r="E11" s="57" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -38101,7 +38322,7 @@
           <t>Juin 2026</t>
         </is>
       </c>
-      <c r="E17" s="54" t="inlineStr">
+      <c r="E17" s="57" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -38131,7 +38352,7 @@
           <t>Août 2026</t>
         </is>
       </c>
-      <c r="E18" s="54" t="inlineStr">
+      <c r="E18" s="57" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -38161,7 +38382,7 @@
           <t>Exercice 2024</t>
         </is>
       </c>
-      <c r="E19" s="54" t="inlineStr">
+      <c r="E19" s="57" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -38191,7 +38412,7 @@
           <t>Exercice 2025</t>
         </is>
       </c>
-      <c r="E20" s="54" t="inlineStr">
+      <c r="E20" s="57" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -38221,7 +38442,7 @@
           <t>Mars, avril, mai, juillet 2026</t>
         </is>
       </c>
-      <c r="E21" s="54" t="inlineStr">
+      <c r="E21" s="57" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -38251,7 +38472,7 @@
           <t>Janvier, février 2026</t>
         </is>
       </c>
-      <c r="E22" s="54" t="inlineStr">
+      <c r="E22" s="57" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -38281,7 +38502,7 @@
           <t>Juillet, août 2026</t>
         </is>
       </c>
-      <c r="E23" s="54" t="inlineStr">
+      <c r="E23" s="57" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -38311,7 +38532,7 @@
           <t>Avril, mai, juin 2026</t>
         </is>
       </c>
-      <c r="E24" s="54" t="inlineStr">
+      <c r="E24" s="57" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -38341,7 +38562,7 @@
           <t>Exercice 2023</t>
         </is>
       </c>
-      <c r="E25" s="54" t="inlineStr">
+      <c r="E25" s="57" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -38371,7 +38592,7 @@
           <t>Janvier, février, mars 2026</t>
         </is>
       </c>
-      <c r="E26" s="54" t="inlineStr">
+      <c r="E26" s="57" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -38431,14 +38652,14 @@
           <t>Délivré le 10/09/2024</t>
         </is>
       </c>
-      <c r="E28" s="54" t="inlineStr">
+      <c r="E28" s="57" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
       </c>
       <c r="F28" s="12" t="inlineStr">
         <is>
-          <t>Expiré le 13/02/2026</t>
+          <t>Expiré le 13/02/2026, remplacé</t>
         </is>
       </c>
     </row>
@@ -38448,7 +38669,7 @@
       </c>
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>Extrait du registre de commerce renouvelé</t>
+          <t>Extrait du registre de commerce modifié n° 700320220 (photo)</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
@@ -38458,17 +38679,17 @@
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="E29" s="40" t="inlineStr">
-        <is>
-          <t>Manquante</t>
+          <t>Délivré le 29/07/2026</t>
+        </is>
+      </c>
+      <c r="E29" s="57" t="inlineStr">
+        <is>
+          <t>Reçue</t>
         </is>
       </c>
       <c r="F29" s="12" t="inlineStr">
         <is>
-          <t>Voir A37, A38</t>
+          <t>Valide jusqu'au 16/02/2028 ; capital 268 M</t>
         </is>
       </c>
     </row>
@@ -38478,27 +38699,27 @@
       </c>
       <c r="B30" s="12" t="inlineStr">
         <is>
-          <t>CPA_DPR_COMPANY.xls — relevé CPA El Kseur</t>
+          <t>PV d'AGE, statuts modifiés et justificatif de libération du capital</t>
         </is>
       </c>
       <c r="C30" s="12" t="inlineStr">
         <is>
-          <t>IMPORT</t>
+          <t>Société</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
         <is>
-          <t>31/12/2025 – 29/06/2026</t>
-        </is>
-      </c>
-      <c r="E30" s="54" t="inlineStr">
-        <is>
-          <t>Reçue</t>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E30" s="40" t="inlineStr">
+        <is>
+          <t>Manquante</t>
         </is>
       </c>
       <c r="F30" s="12" t="inlineStr">
         <is>
-          <t>462 opérations</t>
+          <t>Voir A44</t>
         </is>
       </c>
     </row>
@@ -38508,27 +38729,27 @@
       </c>
       <c r="B31" s="12" t="inlineStr">
         <is>
-          <t>Relevés des autres comptes (CPA 4000015290-18, El Baraka, BNA) 2026</t>
+          <t>CPA_DPR_COMPANY.xls — relevé CPA El Kseur</t>
         </is>
       </c>
       <c r="C31" s="12" t="inlineStr">
         <is>
-          <t>Les deux</t>
+          <t>IMPORT</t>
         </is>
       </c>
       <c r="D31" s="12" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="E31" s="40" t="inlineStr">
-        <is>
-          <t>Manquante</t>
+          <t>31/12/2025 – 29/06/2026</t>
+        </is>
+      </c>
+      <c r="E31" s="57" t="inlineStr">
+        <is>
+          <t>Reçue</t>
         </is>
       </c>
       <c r="F31" s="12" t="inlineStr">
         <is>
-          <t>Paiements G50 TPM, salaires</t>
+          <t>462 opérations</t>
         </is>
       </c>
     </row>
@@ -38538,12 +38759,12 @@
       </c>
       <c r="B32" s="12" t="inlineStr">
         <is>
-          <t>Dossiers d'importation (domiciliations PTI, D10, quittances douane)</t>
+          <t>Relevés des autres comptes (CPA 4000015290-18, El Baraka, BNA) 2026</t>
         </is>
       </c>
       <c r="C32" s="12" t="inlineStr">
         <is>
-          <t>IMPORT</t>
+          <t>Les deux</t>
         </is>
       </c>
       <c r="D32" s="12" t="inlineStr">
@@ -38558,7 +38779,7 @@
       </c>
       <c r="F32" s="12" t="inlineStr">
         <is>
-          <t>Justifier règlements et chèques de banque</t>
+          <t>Paiements G50 TPM, salaires</t>
         </is>
       </c>
     </row>
@@ -38568,15 +38789,19 @@
       </c>
       <c r="B33" s="12" t="inlineStr">
         <is>
-          <t>Statuts à jour et bail du local (DJENNADI Abdelkader)</t>
+          <t>Dossiers d'importation (domiciliations PTI, D10, quittances douane)</t>
         </is>
       </c>
       <c r="C33" s="12" t="inlineStr">
         <is>
-          <t>Société</t>
-        </is>
-      </c>
-      <c r="D33" s="12" t="inlineStr"/>
+          <t>IMPORT</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
       <c r="E33" s="40" t="inlineStr">
         <is>
           <t>Manquante</t>
@@ -38584,7 +38809,7 @@
       </c>
       <c r="F33" s="12" t="inlineStr">
         <is>
-          <t>Voir A40</t>
+          <t>Justifier règlements et chèques de banque</t>
         </is>
       </c>
     </row>
@@ -38594,19 +38819,15 @@
       </c>
       <c r="B34" s="12" t="inlineStr">
         <is>
-          <t>G50 IMPORT et TPM septembre 2026</t>
+          <t>Statuts à jour et bail du local (DJENNADI Abdelkader)</t>
         </is>
       </c>
       <c r="C34" s="12" t="inlineStr">
         <is>
-          <t>Les deux</t>
-        </is>
-      </c>
-      <c r="D34" s="12" t="inlineStr">
-        <is>
-          <t>Sept. 2026</t>
-        </is>
-      </c>
+          <t>Société</t>
+        </is>
+      </c>
+      <c r="D34" s="12" t="inlineStr"/>
       <c r="E34" s="40" t="inlineStr">
         <is>
           <t>Manquante</t>
@@ -38614,7 +38835,7 @@
       </c>
       <c r="F34" s="12" t="inlineStr">
         <is>
-          <t>Échéance 20/10/2026</t>
+          <t>Voir A40</t>
         </is>
       </c>
     </row>
@@ -38624,17 +38845,17 @@
       </c>
       <c r="B35" s="12" t="inlineStr">
         <is>
-          <t>Journal des ventes / factures 2026</t>
+          <t>G50 IMPORT et TPM septembre 2026</t>
         </is>
       </c>
       <c r="C35" s="12" t="inlineStr">
         <is>
-          <t>IMPORT</t>
+          <t>Les deux</t>
         </is>
       </c>
       <c r="D35" s="12" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>Sept. 2026</t>
         </is>
       </c>
       <c r="E35" s="40" t="inlineStr">
@@ -38644,7 +38865,7 @@
       </c>
       <c r="F35" s="12" t="inlineStr">
         <is>
-          <t>Voir A18 : CA réel par mois</t>
+          <t>Échéance 20/10/2026</t>
         </is>
       </c>
     </row>
@@ -38654,17 +38875,17 @@
       </c>
       <c r="B36" s="12" t="inlineStr">
         <is>
-          <t>G50 TPM 2023–2025 (rapprochement TVA collectée TPM)</t>
+          <t>Journal des ventes / factures 2026</t>
         </is>
       </c>
       <c r="C36" s="12" t="inlineStr">
         <is>
-          <t>TPM</t>
+          <t>IMPORT</t>
         </is>
       </c>
       <c r="D36" s="12" t="inlineStr">
         <is>
-          <t>2023–2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="E36" s="40" t="inlineStr">
@@ -38674,7 +38895,7 @@
       </c>
       <c r="F36" s="12" t="inlineStr">
         <is>
-          <t>Voir A17</t>
+          <t>Voir A18 : CA réel par mois</t>
         </is>
       </c>
     </row>
@@ -38684,17 +38905,17 @@
       </c>
       <c r="B37" s="12" t="inlineStr">
         <is>
-          <t>Journal comptable 2026 (PCCOMPTA)</t>
+          <t>G50 TPM 2023–2025 (rapprochement TVA collectée TPM)</t>
         </is>
       </c>
       <c r="C37" s="12" t="inlineStr">
         <is>
-          <t>Société</t>
+          <t>TPM</t>
         </is>
       </c>
       <c r="D37" s="12" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2023–2025</t>
         </is>
       </c>
       <c r="E37" s="40" t="inlineStr">
@@ -38704,7 +38925,7 @@
       </c>
       <c r="F37" s="12" t="inlineStr">
         <is>
-          <t>Pour rapprocher paie et G50 avec la comptabilité</t>
+          <t>Voir A17</t>
         </is>
       </c>
     </row>
@@ -38714,7 +38935,7 @@
       </c>
       <c r="B38" s="12" t="inlineStr">
         <is>
-          <t>Liasse fiscale / bilan 2025 déposé et preuve de paiement IBS</t>
+          <t>Journal comptable 2026 (PCCOMPTA)</t>
         </is>
       </c>
       <c r="C38" s="12" t="inlineStr">
@@ -38724,7 +38945,7 @@
       </c>
       <c r="D38" s="12" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="E38" s="40" t="inlineStr">
@@ -38734,7 +38955,7 @@
       </c>
       <c r="F38" s="12" t="inlineStr">
         <is>
-          <t>Voir A20, A21</t>
+          <t>Pour rapprocher paie et G50 avec la comptabilité</t>
         </is>
       </c>
     </row>
@@ -38744,7 +38965,7 @@
       </c>
       <c r="B39" s="12" t="inlineStr">
         <is>
-          <t>PV de caisse au 31/12/2025</t>
+          <t>Liasse fiscale / bilan 2025 déposé et preuve de paiement IBS</t>
         </is>
       </c>
       <c r="C39" s="12" t="inlineStr">
@@ -38764,7 +38985,7 @@
       </c>
       <c r="F39" s="12" t="inlineStr">
         <is>
-          <t>Voir A22</t>
+          <t>Voir A20, A21</t>
         </is>
       </c>
     </row>
@@ -38774,17 +38995,17 @@
       </c>
       <c r="B40" s="12" t="inlineStr">
         <is>
-          <t>Déclarations et paiements CACOBATPH</t>
+          <t>PV de caisse au 31/12/2025</t>
         </is>
       </c>
       <c r="C40" s="12" t="inlineStr">
         <is>
-          <t>Les deux</t>
+          <t>Société</t>
         </is>
       </c>
       <c r="D40" s="12" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="E40" s="40" t="inlineStr">
@@ -38792,7 +39013,11 @@
           <t>Manquante</t>
         </is>
       </c>
-      <c r="F40" s="12" t="inlineStr"/>
+      <c r="F40" s="12" t="inlineStr">
+        <is>
+          <t>Voir A22</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="12" t="n">
@@ -38800,7 +39025,7 @@
       </c>
       <c r="B41" s="12" t="inlineStr">
         <is>
-          <t>Livre de paie individuel / bulletins</t>
+          <t>Déclarations et paiements CACOBATPH</t>
         </is>
       </c>
       <c r="C41" s="12" t="inlineStr">
@@ -38818,11 +39043,7 @@
           <t>Manquante</t>
         </is>
       </c>
-      <c r="F41" s="12" t="inlineStr">
-        <is>
-          <t>Pour contrôle IRG</t>
-        </is>
-      </c>
+      <c r="F41" s="12" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="12" t="n">
@@ -38830,12 +39051,12 @@
       </c>
       <c r="B42" s="12" t="inlineStr">
         <is>
-          <t>Ordres de mission et justificatifs de frais</t>
+          <t>Livre de paie individuel / bulletins</t>
         </is>
       </c>
       <c r="C42" s="12" t="inlineStr">
         <is>
-          <t>TPM</t>
+          <t>Les deux</t>
         </is>
       </c>
       <c r="D42" s="12" t="inlineStr">
@@ -38850,7 +39071,7 @@
       </c>
       <c r="F42" s="12" t="inlineStr">
         <is>
-          <t>Frais de mission élevés</t>
+          <t>Pour contrôle IRG</t>
         </is>
       </c>
     </row>
@@ -38860,25 +39081,55 @@
       </c>
       <c r="B43" s="12" t="inlineStr">
         <is>
+          <t>Ordres de mission et justificatifs de frais</t>
+        </is>
+      </c>
+      <c r="C43" s="12" t="inlineStr">
+        <is>
+          <t>TPM</t>
+        </is>
+      </c>
+      <c r="D43" s="12" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E43" s="40" t="inlineStr">
+        <is>
+          <t>Manquante</t>
+        </is>
+      </c>
+      <c r="F43" s="12" t="inlineStr">
+        <is>
+          <t>Frais de mission élevés</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="12" t="n">
+        <v>40</v>
+      </c>
+      <c r="B44" s="12" t="inlineStr">
+        <is>
           <t>Relevés bancaires — virements de salaires</t>
         </is>
       </c>
-      <c r="C43" s="12" t="inlineStr">
+      <c r="C44" s="12" t="inlineStr">
         <is>
           <t>Les deux</t>
         </is>
       </c>
-      <c r="D43" s="12" t="inlineStr">
+      <c r="D44" s="12" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="E43" s="40" t="inlineStr">
+      <c r="E44" s="40" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
       </c>
-      <c r="F43" s="12" t="inlineStr">
+      <c r="F44" s="12" t="inlineStr">
         <is>
           <t>Pour lettrage du 421</t>
         </is>

</xml_diff>

<commit_message>
Journal des ventes détail (établissement de Fenaia) et dossier administratif
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XYis4EzVZMNdoYCxmLrRh4
</commit_message>
<xml_diff>
--- a/DOSSIER_COMPTABLE_SARL_DPR_COMPAGNY_2026.xlsx
+++ b/DOSSIER_COMPTABLE_SARL_DPR_COMPAGNY_2026.xlsx
@@ -33,7 +33,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Balance 2024-2025'!$A$4:$E$104</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Clients &amp; fournisseurs'!$A$21:$L$243</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Relevé CPA 2026'!$A$4:$L$875</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'Anomalies &amp; actions'!$A$4:$I$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'Anomalies &amp; actions'!$A$4:$I$53</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -212,7 +212,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -283,6 +283,10 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="4" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="6" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1019,11 +1023,11 @@
         </is>
       </c>
       <c r="B24" s="13">
-        <f>COUNTIF('Anomalies &amp; actions'!B5:B51,1)</f>
+        <f>COUNTIF('Anomalies &amp; actions'!B5:B53,1)</f>
         <v/>
       </c>
       <c r="C24" s="13">
-        <f>COUNTIFS('Anomalies &amp; actions'!B5:B51,1,'Anomalies &amp; actions'!I5:I51,"Ouvert")</f>
+        <f>COUNTIFS('Anomalies &amp; actions'!B5:B53,1,'Anomalies &amp; actions'!I5:I53,"Ouvert")</f>
         <v/>
       </c>
     </row>
@@ -1034,11 +1038,11 @@
         </is>
       </c>
       <c r="B25" s="13">
-        <f>COUNTIF('Anomalies &amp; actions'!B5:B51,2)</f>
+        <f>COUNTIF('Anomalies &amp; actions'!B5:B53,2)</f>
         <v/>
       </c>
       <c r="C25" s="13">
-        <f>COUNTIFS('Anomalies &amp; actions'!B5:B51,2,'Anomalies &amp; actions'!I5:I51,"Ouvert")</f>
+        <f>COUNTIFS('Anomalies &amp; actions'!B5:B53,2,'Anomalies &amp; actions'!I5:I53,"Ouvert")</f>
         <v/>
       </c>
     </row>
@@ -1049,11 +1053,11 @@
         </is>
       </c>
       <c r="B26" s="13">
-        <f>COUNTIF('Anomalies &amp; actions'!B5:B51,3)</f>
+        <f>COUNTIF('Anomalies &amp; actions'!B5:B53,3)</f>
         <v/>
       </c>
       <c r="C26" s="13">
-        <f>COUNTIFS('Anomalies &amp; actions'!B5:B51,3,'Anomalies &amp; actions'!I5:I51,"Ouvert")</f>
+        <f>COUNTIFS('Anomalies &amp; actions'!B5:B53,3,'Anomalies &amp; actions'!I5:I53,"Ouvert")</f>
         <v/>
       </c>
     </row>
@@ -17552,7 +17556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -18081,6 +18085,257 @@
         <is>
           <t>À vérifier avec un juriste : l'importation pour la revente en l'état est en principe réservée à des sociétés qui l'exercent à titre exclusif ; les activités TPM / location pourraient devoir être portées par une société distincte.</t>
         </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>C. Établissement secondaire « vente au détail » — Fenaia Il Maten (dossier administratif reçu le 04/10/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="11" t="inlineStr">
+        <is>
+          <t>Rubrique</t>
+        </is>
+      </c>
+      <c r="B41" s="11" t="inlineStr">
+        <is>
+          <t>Mention</t>
+        </is>
+      </c>
+      <c r="C41" s="11" t="inlineStr">
+        <is>
+          <t>Pièce</t>
+        </is>
+      </c>
+      <c r="D41" s="11" t="inlineStr">
+        <is>
+          <t>Constat</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="34" customHeight="1">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Adresse</t>
+        </is>
+      </c>
+      <c r="B42" s="43" t="inlineStr">
+        <is>
+          <t>Lieu-dit Abadou, commune de Fenaia Il Maten, wilaya de Béjaïa</t>
+        </is>
+      </c>
+      <c r="C42" s="35" t="inlineStr">
+        <is>
+          <t>Déclaration d'existence fiscale</t>
+        </is>
+      </c>
+      <c r="D42" s="29" t="inlineStr">
+        <is>
+          <t>Cachet « Pièces détachées et Réparation mécanique »</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="34" customHeight="1">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>N° RC de l'établissement</t>
+        </is>
+      </c>
+      <c r="B43" s="43" t="inlineStr">
+        <is>
+          <t>06/04-0184232 B 03 (inscrit le 10/09/2024)</t>
+        </is>
+      </c>
+      <c r="C43" s="35" t="inlineStr">
+        <is>
+          <t>Extrait n° 920064572 du 11/09/2024</t>
+        </is>
+      </c>
+      <c r="D43" s="29" t="inlineStr">
+        <is>
+          <t>Les extraits du siège portent pourtant « établissements secondaires : néant »</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="34" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Secteur</t>
+        </is>
+      </c>
+      <c r="B44" s="43" t="inlineStr">
+        <is>
+          <t>Services — distribution au détail (sédentaire et non sédentaire)</t>
+        </is>
+      </c>
+      <c r="C44" s="35" t="inlineStr">
+        <is>
+          <t>Extrait RC établissement</t>
+        </is>
+      </c>
+      <c r="D44" s="29" t="inlineStr"/>
+    </row>
+    <row r="45" ht="34" customHeight="1">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Activités</t>
+        </is>
+      </c>
+      <c r="B45" s="43" t="inlineStr">
+        <is>
+          <t>506003 pièces détachées auto ; 506002 outillage ; 506006 pneumatiques ; 506007 batteries ; 506008 huiles et graisses ; 613204 réparation mécanique ; 605024 salle d'exposition</t>
+        </is>
+      </c>
+      <c r="C45" s="35" t="inlineStr">
+        <is>
+          <t>Extrait RC établissement</t>
+        </is>
+      </c>
+      <c r="D45" s="29" t="inlineStr">
+        <is>
+          <t>Nouvelle activité de vente au détail : journal 15001 créé (fichier JOURNAL_VENTES_DETAIL_FENAIA.xlsx)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="34" customHeight="1">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Article d'imposition</t>
+        </is>
+      </c>
+      <c r="B46" s="43" t="inlineStr">
+        <is>
+          <t>06180778071 (IBS)</t>
+        </is>
+      </c>
+      <c r="C46" s="35" t="inlineStr">
+        <is>
+          <t>Déclaration d'existence (série G 2024/08)</t>
+        </is>
+      </c>
+      <c r="D46" s="29" t="inlineStr">
+        <is>
+          <t>Distinct de l'article du siège (06120024511)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="34" customHeight="1">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Début d'activité déclaré</t>
+        </is>
+      </c>
+      <c r="B47" s="43" t="inlineStr">
+        <is>
+          <t>10/09/2024</t>
+        </is>
+      </c>
+      <c r="C47" s="35" t="inlineStr">
+        <is>
+          <t>Déclaration d'existence</t>
+        </is>
+      </c>
+      <c r="D47" s="52">
+        <f>"Déclaration déposée "&amp;TEXT(C53,"0")&amp;" jours après le délai de 30 jours"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48" ht="34" customHeight="1">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Date de la déclaration d'existence</t>
+        </is>
+      </c>
+      <c r="B48" s="43" t="inlineStr">
+        <is>
+          <t>03/03/2026</t>
+        </is>
+      </c>
+      <c r="C48" s="35" t="inlineStr">
+        <is>
+          <t>Déclaration d'existence</t>
+        </is>
+      </c>
+      <c r="D48" s="29" t="inlineStr">
+        <is>
+          <t>Délai légal : 30 jours après le début d'activité</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="34" customHeight="1">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>NIF</t>
+        </is>
+      </c>
+      <c r="B49" s="43" t="inlineStr">
+        <is>
+          <t>000306018423274 (attestation du 09/03/2026, référence 00030601842327406004)</t>
+        </is>
+      </c>
+      <c r="C49" s="35" t="inlineStr">
+        <is>
+          <t>Attestation d'immatriculation fiscale</t>
+        </is>
+      </c>
+      <c r="D49" s="29" t="inlineStr">
+        <is>
+          <t>Conforme au NIF des G50</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="34" customHeight="1">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>NIS (ONS)</t>
+        </is>
+      </c>
+      <c r="B50" s="43" t="inlineStr">
+        <is>
+          <t>0 003 0612 02539 53 — activité principale 5030</t>
+        </is>
+      </c>
+      <c r="C50" s="35" t="inlineStr">
+        <is>
+          <t>Avis d'identification statistique</t>
+        </is>
+      </c>
+      <c r="D50" s="29" t="inlineStr"/>
+    </row>
+    <row r="51" ht="34" customHeight="1">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Déclaration d'existence du siège</t>
+        </is>
+      </c>
+      <c r="B51" s="43" t="inlineStr">
+        <is>
+          <t>10/09/2003 — gérant DJENADI Ahcene ; activité import-export pièces détachées ; comptable BELHADI Lahlou (El Kseur)</t>
+        </is>
+      </c>
+      <c r="C51" s="35" t="inlineStr">
+        <is>
+          <t>Série G 8 (2002)</t>
+        </is>
+      </c>
+      <c r="D51" s="29" t="inlineStr">
+        <is>
+          <t>Historique</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Retard de dépôt de la déclaration d'existence (jours au-delà de 30)</t>
+        </is>
+      </c>
+      <c r="C53" s="53">
+        <f>MAX(0,DATE(2026,3,3)-DATE(2024,9,10)-30)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -60135,7 +60390,7 @@
           <t>Solde final affiché par la banque (−22 070 423,26) − solde calculé</t>
         </is>
       </c>
-      <c r="F878" s="52">
+      <c r="F878" s="54">
         <f>-22070423.26-F875</f>
         <v/>
       </c>
@@ -62135,7 +62390,7 @@
           <t>Écart non expliqué (doit être 0)</t>
         </is>
       </c>
-      <c r="B55" s="53">
+      <c r="B55" s="55">
         <f>ROUND(B52-B53-B54,2)</f>
         <v/>
       </c>
@@ -62246,7 +62501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I53"/>
+  <dimension ref="A1:I55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -62327,7 +62582,7 @@
           <t>A01</t>
         </is>
       </c>
-      <c r="B5" s="54" t="n">
+      <c r="B5" s="56" t="n">
         <v>2</v>
       </c>
       <c r="C5" s="29" t="inlineStr">
@@ -62345,7 +62600,7 @@
           <t>Déclaration CNAS de février 2026 non fournie (assiette paie 952 475,81 ; 7 STC payés). Le relevé CPA montre un paiement de 333 366,53 le 06/04/2026, égal aux cotisations calculées : la déclaration a donc probablement été déposée.</t>
         </is>
       </c>
-      <c r="F5" s="55">
+      <c r="F5" s="57">
         <f>'Rappro CNAS'!J6</f>
         <v/>
       </c>
@@ -62367,7 +62622,7 @@
           <t>A02</t>
         </is>
       </c>
-      <c r="B6" s="56" t="n">
+      <c r="B6" s="58" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="29" t="inlineStr">
@@ -62385,7 +62640,7 @@
           <t>Centralisateur de mars 2026 absent (onglet vide) alors que la CNAS de mars déclare 368 389,93 d'assiette, 5 salariés.</t>
         </is>
       </c>
-      <c r="F6" s="55">
+      <c r="F6" s="57">
         <f>'Rappro CNAS'!K7</f>
         <v/>
       </c>
@@ -62407,7 +62662,7 @@
           <t>A03</t>
         </is>
       </c>
-      <c r="B7" s="56" t="n">
+      <c r="B7" s="58" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="29" t="inlineStr">
@@ -62425,7 +62680,7 @@
           <t>Prime de ponctualité (R540) imposée à l'IRG mais exclue du salaire de poste (assiette CNAS) chaque mois.</t>
         </is>
       </c>
-      <c r="F7" s="55">
+      <c r="F7" s="57">
         <f>'Rappro CNAS'!V13</f>
         <v/>
       </c>
@@ -62447,7 +62702,7 @@
           <t>A04</t>
         </is>
       </c>
-      <c r="B8" s="54" t="n">
+      <c r="B8" s="56" t="n">
         <v>2</v>
       </c>
       <c r="C8" s="29" t="inlineStr">
@@ -62465,7 +62720,7 @@
           <t>Effectif déclaré au T1 = 2 alors que 3 salariés sont inscrits ; T2 déclare 1 sortie et un effectif final de 2 ⇒ T1 aurait dû être 3.</t>
         </is>
       </c>
-      <c r="F8" s="57" t="n"/>
+      <c r="F8" s="59" t="n"/>
       <c r="G8" s="29" t="inlineStr">
         <is>
           <t>Rectifier l'effectif du T1 auprès de la CNAS.</t>
@@ -62484,7 +62739,7 @@
           <t>A05</t>
         </is>
       </c>
-      <c r="B9" s="54" t="n">
+      <c r="B9" s="56" t="n">
         <v>2</v>
       </c>
       <c r="C9" s="29" t="inlineStr">
@@ -62502,7 +62757,7 @@
           <t>Salarié totalement absent (non rémunéré) en juillet, disparu de la paie en août sans STC ni sortie déclarée.</t>
         </is>
       </c>
-      <c r="F9" s="57" t="n"/>
+      <c r="F9" s="59" t="n"/>
       <c r="G9" s="29" t="inlineStr">
         <is>
           <t>Établir le STC et déclarer la sortie dans l'EMS du T3 (échéance 30/10/2026).</t>
@@ -62521,7 +62776,7 @@
           <t>A06</t>
         </is>
       </c>
-      <c r="B10" s="54" t="n">
+      <c r="B10" s="56" t="n">
         <v>2</v>
       </c>
       <c r="C10" s="29" t="inlineStr">
@@ -62539,7 +62794,7 @@
           <t>STC de 2 237,40 en août : une sortie à déclarer au T3.</t>
         </is>
       </c>
-      <c r="F10" s="57" t="n"/>
+      <c r="F10" s="59" t="n"/>
       <c r="G10" s="29" t="inlineStr">
         <is>
           <t>Déclarer la sortie dans l'EMS du T3.</t>
@@ -62558,7 +62813,7 @@
           <t>A07</t>
         </is>
       </c>
-      <c r="B11" s="54" t="n">
+      <c r="B11" s="56" t="n">
         <v>2</v>
       </c>
       <c r="C11" s="29" t="inlineStr">
@@ -62576,7 +62831,7 @@
           <t>Déclarations T3 2026 (juil–sept) à établir ; paie de septembre non fournie.</t>
         </is>
       </c>
-      <c r="F11" s="55">
+      <c r="F11" s="57">
         <f>'Rappro CNAS'!J9+'Rappro CNAS'!J12</f>
         <v/>
       </c>
@@ -62598,7 +62853,7 @@
           <t>A08</t>
         </is>
       </c>
-      <c r="B12" s="58" t="n">
+      <c r="B12" s="60" t="n">
         <v>3</v>
       </c>
       <c r="C12" s="29" t="inlineStr">
@@ -62616,7 +62871,7 @@
           <t>Avril = mai et juillet = août strictement identiques (mêmes absences, heures sup., IRG) : variables probablement non saisies.</t>
         </is>
       </c>
-      <c r="F12" s="57" t="n"/>
+      <c r="F12" s="59" t="n"/>
       <c r="G12" s="29" t="inlineStr">
         <is>
           <t>Contrôler les pointages et bulletins de mai et août.</t>
@@ -62635,7 +62890,7 @@
           <t>A09</t>
         </is>
       </c>
-      <c r="B13" s="58" t="n">
+      <c r="B13" s="60" t="n">
         <v>3</v>
       </c>
       <c r="C13" s="29" t="inlineStr">
@@ -62653,7 +62908,7 @@
           <t>Frais de mission élevés (avril 41 615 ; mai 49 115, soit 47–55 % de l'assiette), non soumis à cotisations.</t>
         </is>
       </c>
-      <c r="F13" s="55">
+      <c r="F13" s="57">
         <f>'Paie TPM'!K26</f>
         <v/>
       </c>
@@ -62675,7 +62930,7 @@
           <t>A10</t>
         </is>
       </c>
-      <c r="B14" s="58" t="n">
+      <c r="B14" s="60" t="n">
         <v>3</v>
       </c>
       <c r="C14" s="29" t="inlineStr">
@@ -62693,7 +62948,7 @@
           <t>Prime de responsabilité de 5,00 DA (janv.) et 1,14 DA (févr.) : paramètre vraisemblablement erroné (5 au lieu de 5 %).</t>
         </is>
       </c>
-      <c r="F14" s="57" t="n"/>
+      <c r="F14" s="59" t="n"/>
       <c r="G14" s="29" t="inlineStr">
         <is>
           <t>Corriger le paramètre B291 ; régulariser le rappel éventuel.</t>
@@ -62712,7 +62967,7 @@
           <t>A11</t>
         </is>
       </c>
-      <c r="B15" s="54" t="n">
+      <c r="B15" s="56" t="n">
         <v>2</v>
       </c>
       <c r="C15" s="29" t="inlineStr">
@@ -62730,7 +62985,7 @@
           <t>Bordereaux de versement CNAS à « 0,00 ». Relevé CPA : paiements retrouvés pour janvier, février, mars IMPORT et T1 TPM (jusqu'à 12 jours après l'échéance) ; T2 à justifier.</t>
         </is>
       </c>
-      <c r="F15" s="55">
+      <c r="F15" s="57">
         <f>'Rappro CNAS'!K13</f>
         <v/>
       </c>
@@ -62752,7 +63007,7 @@
           <t>A12</t>
         </is>
       </c>
-      <c r="B16" s="54" t="n">
+      <c r="B16" s="56" t="n">
         <v>2</v>
       </c>
       <c r="C16" s="29" t="inlineStr">
@@ -62770,7 +63025,7 @@
           <t>IRG IMPORT : G50 de janvier à août conformes à la paie (écarts d'arrondi ≤ 3 DA ; juillet : 2,30 DA retenus non reversés). Mars non vérifiable (paie absente).</t>
         </is>
       </c>
-      <c r="F16" s="55">
+      <c r="F16" s="57">
         <f>'Échéancier IRG-CNAS'!G13</f>
         <v/>
       </c>
@@ -62792,7 +63047,7 @@
           <t>A13</t>
         </is>
       </c>
-      <c r="B17" s="58" t="n">
+      <c r="B17" s="60" t="n">
         <v>3</v>
       </c>
       <c r="C17" s="29" t="inlineStr">
@@ -62810,7 +63065,7 @@
           <t>Paie paramétrée CACOBATPH (taux X504) mais aucune déclaration CACOBATPH (congés payés / intempéries) dans le dossier.</t>
         </is>
       </c>
-      <c r="F17" s="57" t="n"/>
+      <c r="F17" s="59" t="n"/>
       <c r="G17" s="29" t="inlineStr">
         <is>
           <t>Fournir les déclarations et paiements CACOBATPH 2026.</t>
@@ -62829,7 +63084,7 @@
           <t>A14</t>
         </is>
       </c>
-      <c r="B18" s="58" t="n">
+      <c r="B18" s="60" t="n">
         <v>3</v>
       </c>
       <c r="C18" s="29" t="inlineStr">
@@ -62847,7 +63102,7 @@
           <t>Libellés divergents : « D.P.R.COMPAGNY » / « DPR COMPAGNY » ; en-tête de paie TPM à l'adresse VGE TIZI alors que l'affiliation TPM est à TISSA.</t>
         </is>
       </c>
-      <c r="F18" s="57" t="n"/>
+      <c r="F18" s="59" t="n"/>
       <c r="G18" s="29" t="inlineStr">
         <is>
           <t>Harmoniser raison sociale et adresse dans le logiciel de paie.</t>
@@ -62866,7 +63121,7 @@
           <t>A15</t>
         </is>
       </c>
-      <c r="B19" s="58" t="n">
+      <c r="B19" s="60" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="29" t="inlineStr">
@@ -62884,7 +63139,7 @@
           <t>Périodicité mixte : déclarations mensuelles (janv., mars) puis trimestrielle (T2).</t>
         </is>
       </c>
-      <c r="F19" s="57" t="n"/>
+      <c r="F19" s="59" t="n"/>
       <c r="G19" s="29" t="inlineStr">
         <is>
           <t>Confirmer auprès de la CNAS le passage au trimestriel après la baisse d'effectif (12 → 5).</t>
@@ -62903,7 +63158,7 @@
           <t>A16</t>
         </is>
       </c>
-      <c r="B20" s="58" t="n">
+      <c r="B20" s="60" t="n">
         <v>3</v>
       </c>
       <c r="C20" s="29" t="inlineStr">
@@ -62921,7 +63176,7 @@
           <t>IRG non vérifiable salarié par salarié (centralisateurs uniquement).</t>
         </is>
       </c>
-      <c r="F20" s="57" t="n"/>
+      <c r="F20" s="59" t="n"/>
       <c r="G20" s="29" t="inlineStr">
         <is>
           <t>Fournir le livre de paie individuel / bulletins.</t>
@@ -62940,7 +63195,7 @@
           <t>A17</t>
         </is>
       </c>
-      <c r="B21" s="56" t="n">
+      <c r="B21" s="58" t="n">
         <v>1</v>
       </c>
       <c r="C21" s="29" t="inlineStr">
@@ -62958,7 +63213,7 @@
           <t>TVA collectée TPM (44537) et location (44527) jamais soldées : 58,9 M DA cumulés au 31/12/2025, accumulés depuis au moins 2022 (37,3 M à l'ouverture 2023) ; 2023–2025 : 18,5 M collectés, 1,5 M apurés. En 2025, 4 839 300 de TVA TPM générée, seuls 391 208 passés en G50 (déc.). Les G50 TPM 2026 (juil., août) ne déclarent aucun CA et reportent un précompte de 1 714 499 (= compte 44550).</t>
         </is>
       </c>
-      <c r="F21" s="55">
+      <c r="F21" s="57">
         <f>-('Balance 2024-2025'!D48+'Balance 2024-2025'!D47)</f>
         <v/>
       </c>
@@ -62980,7 +63235,7 @@
           <t>A18</t>
         </is>
       </c>
-      <c r="B22" s="56" t="n">
+      <c r="B22" s="58" t="n">
         <v>1</v>
       </c>
       <c r="C22" s="29" t="inlineStr">
@@ -62998,7 +63253,7 @@
           <t>CA de mars 2026 réalisé 27 006 870 (annotation G50), mais seulement 3 445 200 déclarés en mars « pour manque TVA à récupérer » : 23 561 670 de CA reportés sur avril–août. En avril, le CA annoté (13 157 894,74) est calculé pour obtenir 2 500 000 de TVA. Le CA déclaré mensuellement est ajusté à la TVA déductible disponible.</t>
         </is>
       </c>
-      <c r="F22" s="55">
+      <c r="F22" s="57">
         <f>'G50 2026'!B40</f>
         <v/>
       </c>
@@ -63020,7 +63275,7 @@
           <t>A19</t>
         </is>
       </c>
-      <c r="B23" s="56" t="n">
+      <c r="B23" s="58" t="n">
         <v>1</v>
       </c>
       <c r="C23" s="29" t="inlineStr">
@@ -63038,7 +63293,7 @@
           <t>G50 TPM d'avril à juillet identiques (mois imprimé « AVRIL », IRG 9 375 chaque mois) : juin sous-déclaré de 9 614,90 (18 989,90 retenus), juillet sur-déclaré de 5 683,70. Janvier–mars et août conformes.</t>
         </is>
       </c>
-      <c r="F23" s="55">
+      <c r="F23" s="57">
         <f>-'G50 TPM 2026'!G15</f>
         <v/>
       </c>
@@ -63060,7 +63315,7 @@
           <t>A20</t>
         </is>
       </c>
-      <c r="B24" s="54" t="n">
+      <c r="B24" s="56" t="n">
         <v>2</v>
       </c>
       <c r="C24" s="29" t="inlineStr">
@@ -63078,7 +63333,7 @@
           <t>Écriture du 31/12/2025 « POUR SOLDE PRCT EXE 2025 » passée en sens inverse (D 44410 / C 444, 3 074 299) : dette IBS 9,79 M et acomptes 6,15 M au lieu d'un net de 3 642 951.</t>
         </is>
       </c>
-      <c r="F24" s="55" t="n">
+      <c r="F24" s="57" t="n">
         <v>3074299</v>
       </c>
       <c r="G24" s="29" t="inlineStr">
@@ -63099,7 +63354,7 @@
           <t>A21</t>
         </is>
       </c>
-      <c r="B25" s="54" t="n">
+      <c r="B25" s="56" t="n">
         <v>2</v>
       </c>
       <c r="C25" s="29" t="inlineStr">
@@ -63117,7 +63372,7 @@
           <t>Solde IBS 2024 réglé le 03/07/2025 ; IBS 2025 net à liquider de 3 642 951 (précomptes douane déduits).</t>
         </is>
       </c>
-      <c r="F25" s="55" t="n">
+      <c r="F25" s="57" t="n">
         <v>3642951</v>
       </c>
       <c r="G25" s="29" t="inlineStr">
@@ -63138,7 +63393,7 @@
           <t>A22</t>
         </is>
       </c>
-      <c r="B26" s="54" t="n">
+      <c r="B26" s="56" t="n">
         <v>2</v>
       </c>
       <c r="C26" s="29" t="inlineStr">
@@ -63156,7 +63411,7 @@
           <t>Caisse comptable de 12,1 M au 31/12/2025, surévaluée de 10 M : le versement d'espèces à la CPA du 31/12/2025 (10 000 000) n'a pas été sorti de la caisse (caisse réelle ≈ 2,1 M). Remboursement en espèces de 6 800 000 à SARL DPR AXXAM le 06/12/2025.</t>
         </is>
       </c>
-      <c r="F26" s="55">
+      <c r="F26" s="57">
         <f>'Balance 2024-2025'!D67</f>
         <v/>
       </c>
@@ -63178,7 +63433,7 @@
           <t>A23</t>
         </is>
       </c>
-      <c r="B27" s="54" t="n">
+      <c r="B27" s="56" t="n">
         <v>2</v>
       </c>
       <c r="C27" s="29" t="inlineStr">
@@ -63196,7 +63451,7 @@
           <t>100 % du CA TPM 2025 (25,47 M) facturé à SARL DPR AXXAM BRIQUETERIE ; aucune facturation TPM d'oct. à déc. 2025 alors que du personnel TPM reste payé.</t>
         </is>
       </c>
-      <c r="F27" s="55">
+      <c r="F27" s="57">
         <f>-'Balance 2024-2025'!D100</f>
         <v/>
       </c>
@@ -63218,7 +63473,7 @@
           <t>A24</t>
         </is>
       </c>
-      <c r="B28" s="54" t="n">
+      <c r="B28" s="56" t="n">
         <v>2</v>
       </c>
       <c r="C28" s="29" t="inlineStr">
@@ -63236,7 +63491,7 @@
           <t>Compte d'attente 47000 non soldé (« SARL FAHAS ?? », « TRESORERIE BEJAIA ?? », chèques).</t>
         </is>
       </c>
-      <c r="F28" s="55">
+      <c r="F28" s="57">
         <f>'Balance 2024-2025'!D59</f>
         <v/>
       </c>
@@ -63258,7 +63513,7 @@
           <t>A25</t>
         </is>
       </c>
-      <c r="B29" s="54" t="n">
+      <c r="B29" s="56" t="n">
         <v>2</v>
       </c>
       <c r="C29" s="29" t="inlineStr">
@@ -63276,7 +63531,7 @@
           <t>Compte 63120 « prime imposable » non soumise à cotisation : 957 406 en 2025 et 1 139 275 en 2024 (même mécanisme que A03).</t>
         </is>
       </c>
-      <c r="F29" s="55">
+      <c r="F29" s="57">
         <f>'États 2024-2025'!C24+'États 2024-2025'!D24</f>
         <v/>
       </c>
@@ -63298,7 +63553,7 @@
           <t>A26</t>
         </is>
       </c>
-      <c r="B30" s="58" t="n">
+      <c r="B30" s="60" t="n">
         <v>3</v>
       </c>
       <c r="C30" s="29" t="inlineStr">
@@ -63316,7 +63571,7 @@
           <t>Banque CPA El Kseur (51220) créditrice de 12,43 M au 31/12/2025 : découvert présenté en banque.</t>
         </is>
       </c>
-      <c r="F30" s="55">
+      <c r="F30" s="57">
         <f>ABS('Balance 2024-2025'!D63)</f>
         <v/>
       </c>
@@ -63338,7 +63593,7 @@
           <t>A27</t>
         </is>
       </c>
-      <c r="B31" s="58" t="n">
+      <c r="B31" s="60" t="n">
         <v>3</v>
       </c>
       <c r="C31" s="29" t="inlineStr">
@@ -63356,7 +63611,7 @@
           <t>Reversements IRG 2025 parfois partiels (févr., juin) et rattrapés le mois suivant ; amendes 2025 : douane 100 000, CNAS 1 746.</t>
         </is>
       </c>
-      <c r="F31" s="55">
+      <c r="F31" s="57">
         <f>'Balance 2024-2025'!D93</f>
         <v/>
       </c>
@@ -63378,7 +63633,7 @@
           <t>A28</t>
         </is>
       </c>
-      <c r="B32" s="58" t="n">
+      <c r="B32" s="60" t="n">
         <v>3</v>
       </c>
       <c r="C32" s="29" t="inlineStr">
@@ -63396,7 +63651,7 @@
           <t>Modèles G50 non mis à jour : dates de signature de 2021–2022 sur toutes les G50 2026, onglet de saisie figé (mai, TVA 17 %), G50 TPM contenant le récap TVA de déc. 2025 et un extrait de journal 2019 ; libellés de comptes de TVA à 17 %.</t>
         </is>
       </c>
-      <c r="F32" s="57" t="n"/>
+      <c r="F32" s="59" t="n"/>
       <c r="G32" s="29" t="inlineStr">
         <is>
           <t>Mettre à jour le modèle et les libellés (TVA 19 %).</t>
@@ -63415,7 +63670,7 @@
           <t>A29</t>
         </is>
       </c>
-      <c r="B33" s="58" t="n">
+      <c r="B33" s="60" t="n">
         <v>3</v>
       </c>
       <c r="C33" s="29" t="inlineStr">
@@ -63433,7 +63688,7 @@
           <t>Taxe d'apprentissage payée deux fois en 2026 : février (87 828 IMPORT sur 8 782 828 + 9 851 TPM sur 985 118) et août (44 091 IMPORT sur 4 409 079 + 6 809 TPM sur 680 900).</t>
         </is>
       </c>
-      <c r="F33" s="55">
+      <c r="F33" s="57">
         <f>'G50 2026'!J26+'G50 TPM 2026'!J17</f>
         <v/>
       </c>
@@ -63455,7 +63710,7 @@
           <t>A30</t>
         </is>
       </c>
-      <c r="B34" s="58" t="n">
+      <c r="B34" s="60" t="n">
         <v>3</v>
       </c>
       <c r="C34" s="29" t="inlineStr">
@@ -63473,7 +63728,7 @@
           <t>Droit de timbre : taux apparents incohérents (janv. 2,0 %, févr. 1,0 %, avr. 5,05 %, mai 1,79 %) ; même base en avril et mai ; aucun timbre en mars et de juin à août.</t>
         </is>
       </c>
-      <c r="F34" s="55">
+      <c r="F34" s="57">
         <f>'G50 2026'!J24</f>
         <v/>
       </c>
@@ -63495,7 +63750,7 @@
           <t>A32</t>
         </is>
       </c>
-      <c r="B35" s="56" t="n">
+      <c r="B35" s="58" t="n">
         <v>1</v>
       </c>
       <c r="C35" s="29" t="inlineStr">
@@ -63513,7 +63768,7 @@
           <t>Journal 2023 fourni provisoire : résultat 18,54 M contre 7,26 M repris en à-nouveau 2024 ; 38 comptes en écart avec les ouvertures 2024 (stocks, fournisseurs, banques, IBS, TVA).</t>
         </is>
       </c>
-      <c r="F35" s="55">
+      <c r="F35" s="57">
         <f>'Contrôle 2023'!B6</f>
         <v/>
       </c>
@@ -63535,7 +63790,7 @@
           <t>A33</t>
         </is>
       </c>
-      <c r="B36" s="56" t="n">
+      <c r="B36" s="58" t="n">
         <v>1</v>
       </c>
       <c r="C36" s="29" t="inlineStr">
@@ -63553,7 +63808,7 @@
           <t>Créance SARL DPR AXXAM BRIQUETERIE : 371,0 M au 31/12/2025 (96 % du poste clients), en hausse continue depuis 2023 (277,7 M) ; 2023–2025 : 115,7 M facturés, 26,2 M encaissés (23 %).</t>
         </is>
       </c>
-      <c r="F36" s="55">
+      <c r="F36" s="57">
         <f>'Démarrage 2026'!E8</f>
         <v/>
       </c>
@@ -63575,7 +63830,7 @@
           <t>A34</t>
         </is>
       </c>
-      <c r="B37" s="56" t="n">
+      <c r="B37" s="58" t="n">
         <v>1</v>
       </c>
       <c r="C37" s="29" t="inlineStr">
@@ -63593,7 +63848,7 @@
           <t>Avances clients (419) dormantes : 229,4 M sur 144 clients, inchangées depuis au moins le 01/01/2023 (hors associés et clients à compenser). Soit livraisons non facturées (CA et TVA non déclarés), soit dettes à rembourser.</t>
         </is>
       </c>
-      <c r="F37" s="55">
+      <c r="F37" s="57">
         <f>'Démarrage 2026'!E35</f>
         <v/>
       </c>
@@ -63615,7 +63870,7 @@
           <t>A35</t>
         </is>
       </c>
-      <c r="B38" s="56" t="n">
+      <c r="B38" s="58" t="n">
         <v>1</v>
       </c>
       <c r="C38" s="29" t="inlineStr">
@@ -63633,7 +63888,7 @@
           <t>SARL DPR AXXAM : 62,5 M versés en 2025 (dont 45,35 M d'avances 409 sans facture) et 6,8 M remboursés en espèces, alors que la briqueterie du même groupe ne paie pas.</t>
         </is>
       </c>
-      <c r="F38" s="55">
+      <c r="F38" s="57">
         <f>'Démarrage 2026'!B21</f>
         <v/>
       </c>
@@ -63655,7 +63910,7 @@
           <t>A36</t>
         </is>
       </c>
-      <c r="B39" s="54" t="n">
+      <c r="B39" s="56" t="n">
         <v>2</v>
       </c>
       <c r="C39" s="29" t="inlineStr">
@@ -63673,7 +63928,7 @@
           <t>Associés (famille DJENNADI, dont les 3 gérants inscrits au registre de commerce : Abdelkrim, Ryad, Ahcene) logés en comptes clients / fournisseurs : soldes créditeurs en 411, 419 et 401.</t>
         </is>
       </c>
-      <c r="F39" s="55">
+      <c r="F39" s="57">
         <f>'Démarrage 2026'!E26</f>
         <v/>
       </c>
@@ -63695,7 +63950,7 @@
           <t>A37</t>
         </is>
       </c>
-      <c r="B40" s="58" t="n">
+      <c r="B40" s="60" t="n">
         <v>3</v>
       </c>
       <c r="C40" s="29" t="inlineStr">
@@ -63713,7 +63968,7 @@
           <t>Extrait expiré le 13/02/2026, renouvelé par l'extrait modifié remis le 29/07/2026 (validité 16/02/2026 – 16/02/2028) : 166 jours sans extrait valide remis.</t>
         </is>
       </c>
-      <c r="F40" s="55">
+      <c r="F40" s="57">
         <f>'Registre de commerce'!B20</f>
         <v/>
       </c>
@@ -63735,7 +63990,7 @@
           <t>A38</t>
         </is>
       </c>
-      <c r="B41" s="56" t="n">
+      <c r="B41" s="58" t="n">
         <v>1</v>
       </c>
       <c r="C41" s="29" t="inlineStr">
@@ -63750,10 +64005,10 @@
       </c>
       <c r="E41" s="29" t="inlineStr">
         <is>
-          <t>Registre limité à l'importation pour revente en l'état (442101 à 442104), y compris dans l'extrait modifié du 29/07/2026 ; les activités TPM, location d'engins et transport sont exercées et facturées hors objet du registre.</t>
-        </is>
-      </c>
-      <c r="F41" s="55">
+          <t>Registre du siège limité à l'importation pour revente en l'état (442101 à 442104), y compris dans l'extrait modifié du 29/07/2026 ; la vente au détail est inscrite sur l'établissement de Fenaia, mais les activités TPM, location d'engins et transport restent exercées et facturées hors objet du registre.</t>
+        </is>
+      </c>
+      <c r="F41" s="57">
         <f>-'Balance 2024-2025'!D100</f>
         <v/>
       </c>
@@ -63775,7 +64030,7 @@
           <t>A39</t>
         </is>
       </c>
-      <c r="B42" s="54" t="n">
+      <c r="B42" s="56" t="n">
         <v>2</v>
       </c>
       <c r="C42" s="29" t="inlineStr">
@@ -63790,10 +64045,10 @@
       </c>
       <c r="E42" s="29" t="inlineStr">
         <is>
-          <t>Aucun établissement secondaire inscrit au registre, alors que l'activité TPM est affiliée à la CNAS à TISSA sous un numéro distinct.</t>
-        </is>
-      </c>
-      <c r="F42" s="57" t="n"/>
+          <t>Seul établissement secondaire inscrit : le magasin de détail de Fenaia Il Maten (06/04-0184232 B 03). L'activité TPM, affiliée à la CNAS à TISSA sous un numéro distinct, n'a aucun établissement inscrit.</t>
+        </is>
+      </c>
+      <c r="F42" s="59" t="n"/>
       <c r="G42" s="29" t="inlineStr">
         <is>
           <t>Inscrire l'établissement secondaire ou aligner les affiliations.</t>
@@ -63812,7 +64067,7 @@
           <t>A40</t>
         </is>
       </c>
-      <c r="B43" s="58" t="n">
+      <c r="B43" s="60" t="n">
         <v>3</v>
       </c>
       <c r="C43" s="29" t="inlineStr">
@@ -63830,7 +64085,7 @@
           <t>N° de registre de commerce différent entre l'extrait (06/00-0184232 B 03) et le dossier comptable PCCOMPTA (06/01-0184232B03) ; local commercial appartenant à un associé (DJENNADI Abdelkader, créancier de 2,51 M en 401).</t>
         </is>
       </c>
-      <c r="F43" s="57" t="n"/>
+      <c r="F43" s="59" t="n"/>
       <c r="G43" s="29" t="inlineStr">
         <is>
           <t>Corriger le n° RC dans PCCOMPTA ; produire le bail et l'état des loyers.</t>
@@ -63849,7 +64104,7 @@
           <t>A41</t>
         </is>
       </c>
-      <c r="B44" s="56" t="n">
+      <c r="B44" s="58" t="n">
         <v>1</v>
       </c>
       <c r="C44" s="29" t="inlineStr">
@@ -63867,7 +64122,7 @@
           <t>Relevé CPA : du 01/01 au 03/10/2026, 61,75 M virés à SARL DPR AXXAM et 17,7 M reçus d'elle (net 44,05 M) ; sur oct. 2025 – oct. 2026, 68,6 M nets sortis (impact), alors que le compte est à découvert permanent.</t>
         </is>
       </c>
-      <c r="F44" s="55">
+      <c r="F44" s="57">
         <f>'Banque CPA 2026'!O12</f>
         <v/>
       </c>
@@ -63889,7 +64144,7 @@
           <t>A42</t>
         </is>
       </c>
-      <c r="B45" s="54" t="n">
+      <c r="B45" s="56" t="n">
         <v>2</v>
       </c>
       <c r="C45" s="29" t="inlineStr">
@@ -63907,7 +64162,7 @@
           <t>Compte CPA El Kseur à découvert quasi permanent (−22,1 M au 03/10/2026). Écart de 9,47 M au 31/12/2025 entièrement expliqué : 13 opérations du 31/12/2025 non comptabilisées (9,30 M net, dont versement d'espèces de 10 M, agios, provision import) et 0,18 M antérieur au 05/10/2025.</t>
         </is>
       </c>
-      <c r="F45" s="55">
+      <c r="F45" s="57">
         <f>ABS('Banque CPA 2026'!B52)</f>
         <v/>
       </c>
@@ -63929,7 +64184,7 @@
           <t>A43</t>
         </is>
       </c>
-      <c r="B46" s="58" t="n">
+      <c r="B46" s="60" t="n">
         <v>3</v>
       </c>
       <c r="C46" s="29" t="inlineStr">
@@ -63947,7 +64202,7 @@
           <t>Chèques clients rejetés (annulés) sur le relevé CPA en 2026.</t>
         </is>
       </c>
-      <c r="F46" s="55">
+      <c r="F46" s="57">
         <f>'Banque CPA 2026'!O6</f>
         <v/>
       </c>
@@ -63969,7 +64224,7 @@
           <t>A44</t>
         </is>
       </c>
-      <c r="B47" s="56" t="n">
+      <c r="B47" s="58" t="n">
         <v>1</v>
       </c>
       <c r="C47" s="29" t="inlineStr">
@@ -63987,7 +64242,7 @@
           <t>Capital porté de 106 M à 268 M DA (extrait du 29/07/2026) : +162 M à justifier et à comptabiliser en 2026 ; sources possibles au 31/12/2025 : réserves, résultat 2025, comptes courants d'associés.</t>
         </is>
       </c>
-      <c r="F47" s="55">
+      <c r="F47" s="57">
         <f>'Registre de commerce'!C25</f>
         <v/>
       </c>
@@ -64009,7 +64264,7 @@
           <t>A45</t>
         </is>
       </c>
-      <c r="B48" s="54" t="n">
+      <c r="B48" s="56" t="n">
         <v>2</v>
       </c>
       <c r="C48" s="29" t="inlineStr">
@@ -64027,7 +64282,7 @@
           <t>Paiements débités après l'échéance : G50 janvier (+38 j), G50 juillet payée le 01/10/2026 (+42 j, après celle d'août), G50 février (+18 j), CNAS TPM T2 (+9 j).</t>
         </is>
       </c>
-      <c r="F48" s="57" t="n"/>
+      <c r="F48" s="59" t="n"/>
       <c r="G48" s="29" t="inlineStr">
         <is>
           <t>Rapprocher des quittances ; régler chaque G50 avec son dépôt pour éviter les pénalités de retard.</t>
@@ -64046,7 +64301,7 @@
           <t>A46</t>
         </is>
       </c>
-      <c r="B49" s="54" t="n">
+      <c r="B49" s="56" t="n">
         <v>2</v>
       </c>
       <c r="C49" s="29" t="inlineStr">
@@ -64064,7 +64319,7 @@
           <t>Écritures de banque 2026 non tenues : 640 opérations à saisir ; 158 sans tiers identifiable (surtout des remises de chèques clients), proposées en compte d'attente 47000.</t>
         </is>
       </c>
-      <c r="F49" s="55">
+      <c r="F49" s="57">
         <f>'Banque CPA 2026'!C62</f>
         <v/>
       </c>
@@ -64086,7 +64341,7 @@
           <t>A47</t>
         </is>
       </c>
-      <c r="B50" s="58" t="n">
+      <c r="B50" s="60" t="n">
         <v>3</v>
       </c>
       <c r="C50" s="29" t="inlineStr">
@@ -64104,7 +64359,7 @@
           <t>Relevé CPA : solde final affiché (−22 070 423,26) inférieur de 36 068,24 au solde calculé depuis le solde initial annoncé ; écart constant depuis le 06/10/2025.</t>
         </is>
       </c>
-      <c r="F50" s="55" t="n">
+      <c r="F50" s="57" t="n">
         <v>36068.24</v>
       </c>
       <c r="G50" s="29" t="inlineStr">
@@ -64122,31 +64377,34 @@
     <row r="51" ht="52" customHeight="1">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>A31</t>
+          <t>A48</t>
         </is>
       </c>
       <c r="B51" s="58" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C51" s="29" t="inlineStr">
         <is>
-          <t>Les deux</t>
+          <t>Fenaia (détail)</t>
         </is>
       </c>
       <c r="D51" s="29" t="inlineStr">
         <is>
-          <t>Comptabilité</t>
+          <t>Fiscal / comptabilité</t>
         </is>
       </c>
       <c r="E51" s="29" t="inlineStr">
         <is>
-          <t>Clients débiteurs 387,1 M et avances clients 314,6 M ; fournisseurs débiteurs 46,2 M au 31/12/2025.</t>
-        </is>
-      </c>
-      <c r="F51" s="57" t="n"/>
+          <t>Établissement de vente au détail ouvert le 10/09/2024, déclaré aux impôts le 03/03/2026 seulement (article 06180778071) ; aucune vente au détail, aucun stock de magasin ni aucune G50 de cet établissement dans les journaux 2024 et 2025.</t>
+        </is>
+      </c>
+      <c r="F51" s="57">
+        <f>'Registre de commerce'!C53</f>
+        <v/>
+      </c>
       <c r="G51" s="29" t="inlineStr">
         <is>
-          <t>Lettrer les comptes clients/fournisseurs et compenser les avances soldées.</t>
+          <t>Reconstituer les ventes du magasin depuis le 10/09/2024 (factures, tickets, caisse) ; tenir le journal 15001 ; déposer les G50 de l'établissement (impact = jours de retard de la déclaration).</t>
         </is>
       </c>
       <c r="H51" s="41" t="n"/>
@@ -64156,15 +64414,89 @@
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr">
+    <row r="52" ht="52" customHeight="1">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>A49</t>
+        </is>
+      </c>
+      <c r="B52" s="56" t="n">
+        <v>2</v>
+      </c>
+      <c r="C52" s="29" t="inlineStr">
+        <is>
+          <t>Fenaia (détail)</t>
+        </is>
+      </c>
+      <c r="D52" s="29" t="inlineStr">
+        <is>
+          <t>Social</t>
+        </is>
+      </c>
+      <c r="E52" s="29" t="inlineStr">
+        <is>
+          <t>Aucune affiliation CNAS ni paie identifiée pour le personnel du magasin et de l'atelier de Fenaia.</t>
+        </is>
+      </c>
+      <c r="F52" s="59" t="n"/>
+      <c r="G52" s="29" t="inlineStr">
+        <is>
+          <t>Vérifier le personnel affecté au magasin ; l'affilier et le déclarer.</t>
+        </is>
+      </c>
+      <c r="H52" s="41" t="n"/>
+      <c r="I52" s="41" t="inlineStr">
+        <is>
+          <t>Ouvert</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="52" customHeight="1">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>A31</t>
+        </is>
+      </c>
+      <c r="B53" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="C53" s="29" t="inlineStr">
+        <is>
+          <t>Les deux</t>
+        </is>
+      </c>
+      <c r="D53" s="29" t="inlineStr">
+        <is>
+          <t>Comptabilité</t>
+        </is>
+      </c>
+      <c r="E53" s="29" t="inlineStr">
+        <is>
+          <t>Clients débiteurs 387,1 M et avances clients 314,6 M ; fournisseurs débiteurs 46,2 M au 31/12/2025.</t>
+        </is>
+      </c>
+      <c r="F53" s="59" t="n"/>
+      <c r="G53" s="29" t="inlineStr">
+        <is>
+          <t>Lettrer les comptes clients/fournisseurs et compenser les avances soldées.</t>
+        </is>
+      </c>
+      <c r="H53" s="41" t="n"/>
+      <c r="I53" s="41" t="inlineStr">
+        <is>
+          <t>Ouvert</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
         <is>
           <t>Impact : A01 = cotisations calculées de février ; A02 = cotisations de mars déclarées sans justificatif ; A03 = cotisations sur ponctualité ; A07 = cotisations T3 partielles (juil–août) ; A09 = frais de mission TPM cumulés ; A11 = cotisations déclarées sans preuve de paiement ; A12 = IRG cumulé à rapprocher.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I51"/>
+  <autoFilter ref="A4:I53"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>
@@ -64347,15 +64679,32 @@
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
+          <t>NIS (ONS)</t>
+        </is>
+      </c>
+      <c r="B13" s="22" t="inlineStr">
+        <is>
+          <t>000306120253953</t>
+        </is>
+      </c>
+      <c r="C13" s="21" t="inlineStr">
+        <is>
+          <t>Avis d'identification statistique</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
           <t>Date d'arrêté du dossier</t>
         </is>
       </c>
-      <c r="B13" s="22" t="inlineStr">
+      <c r="B14" s="22" t="inlineStr">
         <is>
           <t>01/10/2026</t>
         </is>
       </c>
-      <c r="C13" s="21" t="inlineStr">
+      <c r="C14" s="21" t="inlineStr">
         <is>
           <t>Date de constitution</t>
         </is>
@@ -64516,7 +64865,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -64592,7 +64941,7 @@
           <t>Janv–août 2026</t>
         </is>
       </c>
-      <c r="E5" s="59" t="inlineStr">
+      <c r="E5" s="61" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -64622,7 +64971,7 @@
           <t>Janv–août 2026</t>
         </is>
       </c>
-      <c r="E6" s="59" t="inlineStr">
+      <c r="E6" s="61" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -64648,7 +64997,7 @@
           <t>Janvier 2026</t>
         </is>
       </c>
-      <c r="E7" s="59" t="inlineStr">
+      <c r="E7" s="61" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -64678,7 +65027,7 @@
           <t>Mars 2026</t>
         </is>
       </c>
-      <c r="E8" s="59" t="inlineStr">
+      <c r="E8" s="61" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -64708,7 +65057,7 @@
           <t>T2 2026</t>
         </is>
       </c>
-      <c r="E9" s="59" t="inlineStr">
+      <c r="E9" s="61" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -64738,7 +65087,7 @@
           <t>T1 2026</t>
         </is>
       </c>
-      <c r="E10" s="59" t="inlineStr">
+      <c r="E10" s="61" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -64768,7 +65117,7 @@
           <t>T2 2026</t>
         </is>
       </c>
-      <c r="E11" s="59" t="inlineStr">
+      <c r="E11" s="61" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -64944,7 +65293,7 @@
           <t>Juin 2026</t>
         </is>
       </c>
-      <c r="E17" s="59" t="inlineStr">
+      <c r="E17" s="61" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -64974,7 +65323,7 @@
           <t>Août 2026</t>
         </is>
       </c>
-      <c r="E18" s="59" t="inlineStr">
+      <c r="E18" s="61" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -65004,7 +65353,7 @@
           <t>Exercice 2024</t>
         </is>
       </c>
-      <c r="E19" s="59" t="inlineStr">
+      <c r="E19" s="61" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -65034,7 +65383,7 @@
           <t>Exercice 2025</t>
         </is>
       </c>
-      <c r="E20" s="59" t="inlineStr">
+      <c r="E20" s="61" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -65064,7 +65413,7 @@
           <t>Mars, avril, mai, juillet 2026</t>
         </is>
       </c>
-      <c r="E21" s="59" t="inlineStr">
+      <c r="E21" s="61" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -65094,7 +65443,7 @@
           <t>Janvier, février 2026</t>
         </is>
       </c>
-      <c r="E22" s="59" t="inlineStr">
+      <c r="E22" s="61" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -65124,7 +65473,7 @@
           <t>Juillet, août 2026</t>
         </is>
       </c>
-      <c r="E23" s="59" t="inlineStr">
+      <c r="E23" s="61" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -65154,7 +65503,7 @@
           <t>Avril, mai, juin 2026</t>
         </is>
       </c>
-      <c r="E24" s="59" t="inlineStr">
+      <c r="E24" s="61" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -65184,7 +65533,7 @@
           <t>Exercice 2023</t>
         </is>
       </c>
-      <c r="E25" s="59" t="inlineStr">
+      <c r="E25" s="61" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -65214,7 +65563,7 @@
           <t>Janvier, février, mars 2026</t>
         </is>
       </c>
-      <c r="E26" s="59" t="inlineStr">
+      <c r="E26" s="61" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -65274,7 +65623,7 @@
           <t>Délivré le 10/09/2024</t>
         </is>
       </c>
-      <c r="E28" s="59" t="inlineStr">
+      <c r="E28" s="61" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -65304,7 +65653,7 @@
           <t>Délivré le 29/07/2026</t>
         </is>
       </c>
-      <c r="E29" s="59" t="inlineStr">
+      <c r="E29" s="61" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -65364,7 +65713,7 @@
           <t>31/12/2025 – 29/06/2026</t>
         </is>
       </c>
-      <c r="E31" s="59" t="inlineStr">
+      <c r="E31" s="61" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -65394,7 +65743,7 @@
           <t>06/10/2025 – 03/10/2026</t>
         </is>
       </c>
-      <c r="E32" s="59" t="inlineStr">
+      <c r="E32" s="61" t="inlineStr">
         <is>
           <t>Reçue</t>
         </is>
@@ -65527,27 +65876,27 @@
       </c>
       <c r="B37" s="12" t="inlineStr">
         <is>
-          <t>G50 IMPORT et TPM septembre 2026</t>
+          <t>Déclaration d'existence du siège (10/09/2003) et avis d'identification ONS</t>
         </is>
       </c>
       <c r="C37" s="12" t="inlineStr">
         <is>
-          <t>Les deux</t>
+          <t>Société</t>
         </is>
       </c>
       <c r="D37" s="12" t="inlineStr">
         <is>
-          <t>Sept. 2026</t>
-        </is>
-      </c>
-      <c r="E37" s="40" t="inlineStr">
-        <is>
-          <t>Manquante</t>
+          <t>2003</t>
+        </is>
+      </c>
+      <c r="E37" s="61" t="inlineStr">
+        <is>
+          <t>Reçue</t>
         </is>
       </c>
       <c r="F37" s="12" t="inlineStr">
         <is>
-          <t>Échéance 20/10/2026</t>
+          <t>Dossier administratif</t>
         </is>
       </c>
     </row>
@@ -65557,27 +65906,27 @@
       </c>
       <c r="B38" s="12" t="inlineStr">
         <is>
-          <t>Journal des ventes / factures 2026</t>
+          <t>Extrait RC de l'établissement secondaire de Fenaia (n° 920064572)</t>
         </is>
       </c>
       <c r="C38" s="12" t="inlineStr">
         <is>
-          <t>IMPORT</t>
+          <t>Fenaia</t>
         </is>
       </c>
       <c r="D38" s="12" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="E38" s="40" t="inlineStr">
-        <is>
-          <t>Manquante</t>
+          <t>11/09/2024</t>
+        </is>
+      </c>
+      <c r="E38" s="61" t="inlineStr">
+        <is>
+          <t>Reçue</t>
         </is>
       </c>
       <c r="F38" s="12" t="inlineStr">
         <is>
-          <t>Voir A18 : CA réel par mois</t>
+          <t>Vente au détail et réparation</t>
         </is>
       </c>
     </row>
@@ -65587,27 +65936,27 @@
       </c>
       <c r="B39" s="12" t="inlineStr">
         <is>
-          <t>G50 TPM 2023–2025 (rapprochement TVA collectée TPM)</t>
+          <t>Déclaration d'existence fiscale de l'établissement de Fenaia</t>
         </is>
       </c>
       <c r="C39" s="12" t="inlineStr">
         <is>
-          <t>TPM</t>
+          <t>Fenaia</t>
         </is>
       </c>
       <c r="D39" s="12" t="inlineStr">
         <is>
-          <t>2023–2025</t>
-        </is>
-      </c>
-      <c r="E39" s="40" t="inlineStr">
-        <is>
-          <t>Manquante</t>
+          <t>03/03/2026</t>
+        </is>
+      </c>
+      <c r="E39" s="61" t="inlineStr">
+        <is>
+          <t>Reçue</t>
         </is>
       </c>
       <c r="F39" s="12" t="inlineStr">
         <is>
-          <t>Voir A17</t>
+          <t>Article 06180778071</t>
         </is>
       </c>
     </row>
@@ -65617,7 +65966,7 @@
       </c>
       <c r="B40" s="12" t="inlineStr">
         <is>
-          <t>Journal comptable 2026 (PCCOMPTA)</t>
+          <t>Attestation d'immatriculation fiscale (NIF)</t>
         </is>
       </c>
       <c r="C40" s="12" t="inlineStr">
@@ -65627,19 +65976,15 @@
       </c>
       <c r="D40" s="12" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="E40" s="40" t="inlineStr">
-        <is>
-          <t>Manquante</t>
-        </is>
-      </c>
-      <c r="F40" s="12" t="inlineStr">
-        <is>
-          <t>Pour rapprocher paie et G50 avec la comptabilité</t>
-        </is>
-      </c>
+          <t>09/03/2026</t>
+        </is>
+      </c>
+      <c r="E40" s="61" t="inlineStr">
+        <is>
+          <t>Reçue</t>
+        </is>
+      </c>
+      <c r="F40" s="12" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="12" t="n">
@@ -65647,17 +65992,17 @@
       </c>
       <c r="B41" s="12" t="inlineStr">
         <is>
-          <t>Liasse fiscale / bilan 2025 déposé et preuve de paiement IBS</t>
+          <t>Ventes, stocks et caisse du magasin de Fenaia depuis le 10/09/2024 ; bail du local</t>
         </is>
       </c>
       <c r="C41" s="12" t="inlineStr">
         <is>
-          <t>Société</t>
+          <t>Fenaia</t>
         </is>
       </c>
       <c r="D41" s="12" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024–2026</t>
         </is>
       </c>
       <c r="E41" s="40" t="inlineStr">
@@ -65667,7 +66012,7 @@
       </c>
       <c r="F41" s="12" t="inlineStr">
         <is>
-          <t>Voir A20, A21</t>
+          <t>Voir A48</t>
         </is>
       </c>
     </row>
@@ -65677,17 +66022,17 @@
       </c>
       <c r="B42" s="12" t="inlineStr">
         <is>
-          <t>PV de caisse au 31/12/2025</t>
+          <t>G50 IMPORT et TPM septembre 2026</t>
         </is>
       </c>
       <c r="C42" s="12" t="inlineStr">
         <is>
-          <t>Société</t>
+          <t>Les deux</t>
         </is>
       </c>
       <c r="D42" s="12" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>Sept. 2026</t>
         </is>
       </c>
       <c r="E42" s="40" t="inlineStr">
@@ -65697,7 +66042,7 @@
       </c>
       <c r="F42" s="12" t="inlineStr">
         <is>
-          <t>Voir A22</t>
+          <t>Échéance 20/10/2026</t>
         </is>
       </c>
     </row>
@@ -65707,12 +66052,12 @@
       </c>
       <c r="B43" s="12" t="inlineStr">
         <is>
-          <t>Déclarations et paiements CACOBATPH</t>
+          <t>Journal des ventes / factures 2026</t>
         </is>
       </c>
       <c r="C43" s="12" t="inlineStr">
         <is>
-          <t>Les deux</t>
+          <t>IMPORT</t>
         </is>
       </c>
       <c r="D43" s="12" t="inlineStr">
@@ -65725,7 +66070,11 @@
           <t>Manquante</t>
         </is>
       </c>
-      <c r="F43" s="12" t="inlineStr"/>
+      <c r="F43" s="12" t="inlineStr">
+        <is>
+          <t>Voir A18 : CA réel par mois</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="12" t="n">
@@ -65733,17 +66082,17 @@
       </c>
       <c r="B44" s="12" t="inlineStr">
         <is>
-          <t>Livre de paie individuel / bulletins</t>
+          <t>G50 TPM 2023–2025 (rapprochement TVA collectée TPM)</t>
         </is>
       </c>
       <c r="C44" s="12" t="inlineStr">
         <is>
-          <t>Les deux</t>
+          <t>TPM</t>
         </is>
       </c>
       <c r="D44" s="12" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2023–2025</t>
         </is>
       </c>
       <c r="E44" s="40" t="inlineStr">
@@ -65753,7 +66102,7 @@
       </c>
       <c r="F44" s="12" t="inlineStr">
         <is>
-          <t>Pour contrôle IRG</t>
+          <t>Voir A17</t>
         </is>
       </c>
     </row>
@@ -65763,12 +66112,12 @@
       </c>
       <c r="B45" s="12" t="inlineStr">
         <is>
-          <t>Ordres de mission et justificatifs de frais</t>
+          <t>Journal comptable 2026 (PCCOMPTA)</t>
         </is>
       </c>
       <c r="C45" s="12" t="inlineStr">
         <is>
-          <t>TPM</t>
+          <t>Société</t>
         </is>
       </c>
       <c r="D45" s="12" t="inlineStr">
@@ -65783,7 +66132,7 @@
       </c>
       <c r="F45" s="12" t="inlineStr">
         <is>
-          <t>Frais de mission élevés</t>
+          <t>Pour rapprocher paie et G50 avec la comptabilité</t>
         </is>
       </c>
     </row>
@@ -65793,25 +66142,171 @@
       </c>
       <c r="B46" s="12" t="inlineStr">
         <is>
+          <t>Liasse fiscale / bilan 2025 déposé et preuve de paiement IBS</t>
+        </is>
+      </c>
+      <c r="C46" s="12" t="inlineStr">
+        <is>
+          <t>Société</t>
+        </is>
+      </c>
+      <c r="D46" s="12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E46" s="40" t="inlineStr">
+        <is>
+          <t>Manquante</t>
+        </is>
+      </c>
+      <c r="F46" s="12" t="inlineStr">
+        <is>
+          <t>Voir A20, A21</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="12" t="n">
+        <v>43</v>
+      </c>
+      <c r="B47" s="12" t="inlineStr">
+        <is>
+          <t>PV de caisse au 31/12/2025</t>
+        </is>
+      </c>
+      <c r="C47" s="12" t="inlineStr">
+        <is>
+          <t>Société</t>
+        </is>
+      </c>
+      <c r="D47" s="12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E47" s="40" t="inlineStr">
+        <is>
+          <t>Manquante</t>
+        </is>
+      </c>
+      <c r="F47" s="12" t="inlineStr">
+        <is>
+          <t>Voir A22</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="12" t="n">
+        <v>44</v>
+      </c>
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>Déclarations et paiements CACOBATPH</t>
+        </is>
+      </c>
+      <c r="C48" s="12" t="inlineStr">
+        <is>
+          <t>Les deux</t>
+        </is>
+      </c>
+      <c r="D48" s="12" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E48" s="40" t="inlineStr">
+        <is>
+          <t>Manquante</t>
+        </is>
+      </c>
+      <c r="F48" s="12" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="12" t="n">
+        <v>45</v>
+      </c>
+      <c r="B49" s="12" t="inlineStr">
+        <is>
+          <t>Livre de paie individuel / bulletins</t>
+        </is>
+      </c>
+      <c r="C49" s="12" t="inlineStr">
+        <is>
+          <t>Les deux</t>
+        </is>
+      </c>
+      <c r="D49" s="12" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E49" s="40" t="inlineStr">
+        <is>
+          <t>Manquante</t>
+        </is>
+      </c>
+      <c r="F49" s="12" t="inlineStr">
+        <is>
+          <t>Pour contrôle IRG</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="12" t="n">
+        <v>46</v>
+      </c>
+      <c r="B50" s="12" t="inlineStr">
+        <is>
+          <t>Ordres de mission et justificatifs de frais</t>
+        </is>
+      </c>
+      <c r="C50" s="12" t="inlineStr">
+        <is>
+          <t>TPM</t>
+        </is>
+      </c>
+      <c r="D50" s="12" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E50" s="40" t="inlineStr">
+        <is>
+          <t>Manquante</t>
+        </is>
+      </c>
+      <c r="F50" s="12" t="inlineStr">
+        <is>
+          <t>Frais de mission élevés</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="12" t="n">
+        <v>47</v>
+      </c>
+      <c r="B51" s="12" t="inlineStr">
+        <is>
           <t>Relevés bancaires — virements de salaires</t>
         </is>
       </c>
-      <c r="C46" s="12" t="inlineStr">
+      <c r="C51" s="12" t="inlineStr">
         <is>
           <t>Les deux</t>
         </is>
       </c>
-      <c r="D46" s="12" t="inlineStr">
+      <c r="D51" s="12" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="E46" s="40" t="inlineStr">
+      <c r="E51" s="40" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
       </c>
-      <c r="F46" s="12" t="inlineStr">
+      <c r="F51" s="12" t="inlineStr">
         <is>
           <t>Pour lettrage du 421</t>
         </is>

</xml_diff>

<commit_message>
Écritures de ventes 2026 (gros et détail) et rapprochement avec les G50
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XYis4EzVZMNdoYCxmLrRh4
</commit_message>
<xml_diff>
--- a/DOSSIER_COMPTABLE_SARL_DPR_COMPAGNY_2026.xlsx
+++ b/DOSSIER_COMPTABLE_SARL_DPR_COMPAGNY_2026.xlsx
@@ -33,7 +33,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Balance 2024-2025'!$A$4:$E$104</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Clients &amp; fournisseurs'!$A$21:$L$243</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Relevé CPA 2026'!$A$4:$L$875</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'Anomalies &amp; actions'!$A$4:$I$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'Anomalies &amp; actions'!$A$4:$I$55</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1023,11 +1023,11 @@
         </is>
       </c>
       <c r="B24" s="13">
-        <f>COUNTIF('Anomalies &amp; actions'!B5:B53,1)</f>
+        <f>COUNTIF('Anomalies &amp; actions'!B5:B55,1)</f>
         <v/>
       </c>
       <c r="C24" s="13">
-        <f>COUNTIFS('Anomalies &amp; actions'!B5:B53,1,'Anomalies &amp; actions'!I5:I53,"Ouvert")</f>
+        <f>COUNTIFS('Anomalies &amp; actions'!B5:B55,1,'Anomalies &amp; actions'!I5:I55,"Ouvert")</f>
         <v/>
       </c>
     </row>
@@ -1038,11 +1038,11 @@
         </is>
       </c>
       <c r="B25" s="13">
-        <f>COUNTIF('Anomalies &amp; actions'!B5:B53,2)</f>
+        <f>COUNTIF('Anomalies &amp; actions'!B5:B55,2)</f>
         <v/>
       </c>
       <c r="C25" s="13">
-        <f>COUNTIFS('Anomalies &amp; actions'!B5:B53,2,'Anomalies &amp; actions'!I5:I53,"Ouvert")</f>
+        <f>COUNTIFS('Anomalies &amp; actions'!B5:B55,2,'Anomalies &amp; actions'!I5:I55,"Ouvert")</f>
         <v/>
       </c>
     </row>
@@ -1053,11 +1053,11 @@
         </is>
       </c>
       <c r="B26" s="13">
-        <f>COUNTIF('Anomalies &amp; actions'!B5:B53,3)</f>
+        <f>COUNTIF('Anomalies &amp; actions'!B5:B55,3)</f>
         <v/>
       </c>
       <c r="C26" s="13">
-        <f>COUNTIFS('Anomalies &amp; actions'!B5:B53,3,'Anomalies &amp; actions'!I5:I53,"Ouvert")</f>
+        <f>COUNTIFS('Anomalies &amp; actions'!B5:B55,3,'Anomalies &amp; actions'!I5:I55,"Ouvert")</f>
         <v/>
       </c>
     </row>
@@ -62501,7 +62501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I55"/>
+  <dimension ref="A1:I57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -63240,7 +63240,7 @@
       </c>
       <c r="C22" s="29" t="inlineStr">
         <is>
-          <t>IMPORT</t>
+          <t>Les deux</t>
         </is>
       </c>
       <c r="D22" s="29" t="inlineStr">
@@ -63250,7 +63250,7 @@
       </c>
       <c r="E22" s="29" t="inlineStr">
         <is>
-          <t>CA de mars 2026 réalisé 27 006 870 (annotation G50), mais seulement 3 445 200 déclarés en mars « pour manque TVA à récupérer » : 23 561 670 de CA reportés sur avril–août. En avril, le CA annoté (13 157 894,74) est calculé pour obtenir 2 500 000 de TVA. Le CA déclaré mensuellement est ajusté à la TVA déductible disponible.</t>
+          <t>CA de mars 2026 facturé 27 006 870 (gros 16 281 570 + détail Fenaia 10 725 300, journaux de factures) mais seulement 3 445 200 déclarés en mars « pour manque TVA à récupérer » ; le reste a été déclaré en avril (+13 157 894) et mai (+10 403 776). Fin août, le cumul déclaré rattrape le cumul facturé : la TVA de mars (4 476 717) a été payée avec 1 à 2 mois de retard.</t>
         </is>
       </c>
       <c r="F22" s="57">
@@ -63259,7 +63259,7 @@
       </c>
       <c r="G22" s="29" t="inlineStr">
         <is>
-          <t>Déclarer le CA au titre du mois de réalisation ; rapprocher le CA déclaré du journal des ventes 2026 ; chiffrer les pénalités de retard sur la TVA différée.</t>
+          <t>Déclarer le CA au titre du mois de facturation ; chiffrer les pénalités de retard sur la TVA de mars (fichier ECRITURES_VENTES_2026.xlsx, feuille Rapprochement G50).</t>
         </is>
       </c>
       <c r="H22" s="41" t="n"/>
@@ -64395,7 +64395,7 @@
       </c>
       <c r="E51" s="29" t="inlineStr">
         <is>
-          <t>Établissement de vente au détail ouvert le 10/09/2024, déclaré aux impôts le 03/03/2026 seulement (article 06180778071) ; aucune vente au détail, aucun stock de magasin ni aucune G50 de cet établissement dans les journaux 2024 et 2025.</t>
+          <t>Établissement de vente au détail ouvert le 10/09/2024, déclaré aux impôts le 03/03/2026 seulement (article 06180778071). Ses ventes facturées commencent en mars 2026 (79 factures, 28,64 M HT jusqu'au 04/10/2026) et sont déclarées sur les G50 du siège ; aucune vente, aucun stock de magasin ni G50 propre entre septembre 2024 et février 2026.</t>
         </is>
       </c>
       <c r="F51" s="57">
@@ -64454,31 +64454,33 @@
     <row r="53" ht="52" customHeight="1">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>A31</t>
-        </is>
-      </c>
-      <c r="B53" s="60" t="n">
-        <v>3</v>
+          <t>A50</t>
+        </is>
+      </c>
+      <c r="B53" s="56" t="n">
+        <v>2</v>
       </c>
       <c r="C53" s="29" t="inlineStr">
         <is>
-          <t>Les deux</t>
+          <t>IMPORT</t>
         </is>
       </c>
       <c r="D53" s="29" t="inlineStr">
         <is>
-          <t>Comptabilité</t>
+          <t>Parties liées</t>
         </is>
       </c>
       <c r="E53" s="29" t="inlineStr">
         <is>
-          <t>Clients débiteurs 387,1 M et avances clients 314,6 M ; fournisseurs débiteurs 46,2 M au 31/12/2025.</t>
-        </is>
-      </c>
-      <c r="F53" s="59" t="n"/>
+          <t>Ventes de gros 2026 aux associés-gérants : DJENNADI Abdelkrim (6 factures, 12 739 948 HT) et DJENNADI Reyad (28 factures, 2 051 589 HT), soit 17,6 % du CA de gros facturé.</t>
+        </is>
+      </c>
+      <c r="F53" s="57" t="n">
+        <v>14791537</v>
+      </c>
       <c r="G53" s="29" t="inlineStr">
         <is>
-          <t>Lettrer les comptes clients/fournisseurs et compenser les avances soldées.</t>
+          <t>Documenter les prix pratiqués et le règlement de ces factures ; vérifier qu'elles ne sont pas compensées avec les comptes courants d'associés.</t>
         </is>
       </c>
       <c r="H53" s="41" t="n"/>
@@ -64488,15 +64490,89 @@
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
+    <row r="54" ht="52" customHeight="1">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>A51</t>
+        </is>
+      </c>
+      <c r="B54" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="C54" s="29" t="inlineStr">
+        <is>
+          <t>IMPORT</t>
+        </is>
+      </c>
+      <c r="D54" s="29" t="inlineStr">
+        <is>
+          <t>Facturation</t>
+        </is>
+      </c>
+      <c r="E54" s="29" t="inlineStr">
+        <is>
+          <t>Numérotation des factures de gros 2026 discontinue : n° 2026000128, 129, 141 et 168 absents du journal des factures.</t>
+        </is>
+      </c>
+      <c r="F54" s="59" t="n"/>
+      <c r="G54" s="29" t="inlineStr">
+        <is>
+          <t>Justifier ces numéros (factures annulées, avec l'original et les copies).</t>
+        </is>
+      </c>
+      <c r="H54" s="41" t="n"/>
+      <c r="I54" s="41" t="inlineStr">
+        <is>
+          <t>Ouvert</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="52" customHeight="1">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>A31</t>
+        </is>
+      </c>
+      <c r="B55" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="C55" s="29" t="inlineStr">
+        <is>
+          <t>Les deux</t>
+        </is>
+      </c>
+      <c r="D55" s="29" t="inlineStr">
+        <is>
+          <t>Comptabilité</t>
+        </is>
+      </c>
+      <c r="E55" s="29" t="inlineStr">
+        <is>
+          <t>Clients débiteurs 387,1 M et avances clients 314,6 M ; fournisseurs débiteurs 46,2 M au 31/12/2025.</t>
+        </is>
+      </c>
+      <c r="F55" s="59" t="n"/>
+      <c r="G55" s="29" t="inlineStr">
+        <is>
+          <t>Lettrer les comptes clients/fournisseurs et compenser les avances soldées.</t>
+        </is>
+      </c>
+      <c r="H55" s="41" t="n"/>
+      <c r="I55" s="41" t="inlineStr">
+        <is>
+          <t>Ouvert</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
         <is>
           <t>Impact : A01 = cotisations calculées de février ; A02 = cotisations de mars déclarées sans justificatif ; A03 = cotisations sur ponctualité ; A07 = cotisations T3 partielles (juil–août) ; A09 = frais de mission TPM cumulés ; A11 = cotisations déclarées sans preuve de paiement ; A12 = IRG cumulé à rapprocher.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I53"/>
+  <autoFilter ref="A4:I55"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>
@@ -64865,7 +64941,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -66022,27 +66098,27 @@
       </c>
       <c r="B42" s="12" t="inlineStr">
         <is>
-          <t>G50 IMPORT et TPM septembre 2026</t>
+          <t>Etat Détails Journal Factures gros.xls (siège)</t>
         </is>
       </c>
       <c r="C42" s="12" t="inlineStr">
         <is>
-          <t>Les deux</t>
+          <t>IMPORT</t>
         </is>
       </c>
       <c r="D42" s="12" t="inlineStr">
         <is>
-          <t>Sept. 2026</t>
-        </is>
-      </c>
-      <c r="E42" s="40" t="inlineStr">
-        <is>
-          <t>Manquante</t>
+          <t>01/01 – 04/10/2026</t>
+        </is>
+      </c>
+      <c r="E42" s="61" t="inlineStr">
+        <is>
+          <t>Reçue</t>
         </is>
       </c>
       <c r="F42" s="12" t="inlineStr">
         <is>
-          <t>Échéance 20/10/2026</t>
+          <t>180 factures, 84 355 024,24 HT ; écritures journal 06002</t>
         </is>
       </c>
     </row>
@@ -66052,27 +66128,27 @@
       </c>
       <c r="B43" s="12" t="inlineStr">
         <is>
-          <t>Journal des ventes / factures 2026</t>
+          <t>Etat Détails Journal Factures detail.xls (Fenaia)</t>
         </is>
       </c>
       <c r="C43" s="12" t="inlineStr">
         <is>
-          <t>IMPORT</t>
+          <t>Fenaia</t>
         </is>
       </c>
       <c r="D43" s="12" t="inlineStr">
         <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="E43" s="40" t="inlineStr">
-        <is>
-          <t>Manquante</t>
+          <t>01/01 – 04/10/2026</t>
+        </is>
+      </c>
+      <c r="E43" s="61" t="inlineStr">
+        <is>
+          <t>Reçue</t>
         </is>
       </c>
       <c r="F43" s="12" t="inlineStr">
         <is>
-          <t>Voir A18 : CA réel par mois</t>
+          <t>79 factures, 28 635 000 HT ; écritures journal 15001</t>
         </is>
       </c>
     </row>
@@ -66082,17 +66158,17 @@
       </c>
       <c r="B44" s="12" t="inlineStr">
         <is>
-          <t>G50 TPM 2023–2025 (rapprochement TVA collectée TPM)</t>
+          <t>G50 IMPORT et TPM septembre 2026</t>
         </is>
       </c>
       <c r="C44" s="12" t="inlineStr">
         <is>
-          <t>TPM</t>
+          <t>Les deux</t>
         </is>
       </c>
       <c r="D44" s="12" t="inlineStr">
         <is>
-          <t>2023–2025</t>
+          <t>Sept. 2026</t>
         </is>
       </c>
       <c r="E44" s="40" t="inlineStr">
@@ -66102,7 +66178,7 @@
       </c>
       <c r="F44" s="12" t="inlineStr">
         <is>
-          <t>Voir A17</t>
+          <t>Échéance 20/10/2026</t>
         </is>
       </c>
     </row>
@@ -66112,12 +66188,12 @@
       </c>
       <c r="B45" s="12" t="inlineStr">
         <is>
-          <t>Journal comptable 2026 (PCCOMPTA)</t>
+          <t>Journal des ventes / factures 2026</t>
         </is>
       </c>
       <c r="C45" s="12" t="inlineStr">
         <is>
-          <t>Société</t>
+          <t>IMPORT</t>
         </is>
       </c>
       <c r="D45" s="12" t="inlineStr">
@@ -66132,7 +66208,7 @@
       </c>
       <c r="F45" s="12" t="inlineStr">
         <is>
-          <t>Pour rapprocher paie et G50 avec la comptabilité</t>
+          <t>Voir A18 : CA réel par mois</t>
         </is>
       </c>
     </row>
@@ -66142,17 +66218,17 @@
       </c>
       <c r="B46" s="12" t="inlineStr">
         <is>
-          <t>Liasse fiscale / bilan 2025 déposé et preuve de paiement IBS</t>
+          <t>G50 TPM 2023–2025 (rapprochement TVA collectée TPM)</t>
         </is>
       </c>
       <c r="C46" s="12" t="inlineStr">
         <is>
-          <t>Société</t>
+          <t>TPM</t>
         </is>
       </c>
       <c r="D46" s="12" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2023–2025</t>
         </is>
       </c>
       <c r="E46" s="40" t="inlineStr">
@@ -66162,7 +66238,7 @@
       </c>
       <c r="F46" s="12" t="inlineStr">
         <is>
-          <t>Voir A20, A21</t>
+          <t>Voir A17</t>
         </is>
       </c>
     </row>
@@ -66172,7 +66248,7 @@
       </c>
       <c r="B47" s="12" t="inlineStr">
         <is>
-          <t>PV de caisse au 31/12/2025</t>
+          <t>Journal comptable 2026 (PCCOMPTA)</t>
         </is>
       </c>
       <c r="C47" s="12" t="inlineStr">
@@ -66182,7 +66258,7 @@
       </c>
       <c r="D47" s="12" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="E47" s="40" t="inlineStr">
@@ -66192,7 +66268,7 @@
       </c>
       <c r="F47" s="12" t="inlineStr">
         <is>
-          <t>Voir A22</t>
+          <t>Pour rapprocher paie et G50 avec la comptabilité</t>
         </is>
       </c>
     </row>
@@ -66202,17 +66278,17 @@
       </c>
       <c r="B48" s="12" t="inlineStr">
         <is>
-          <t>Déclarations et paiements CACOBATPH</t>
+          <t>Liasse fiscale / bilan 2025 déposé et preuve de paiement IBS</t>
         </is>
       </c>
       <c r="C48" s="12" t="inlineStr">
         <is>
-          <t>Les deux</t>
+          <t>Société</t>
         </is>
       </c>
       <c r="D48" s="12" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="E48" s="40" t="inlineStr">
@@ -66220,7 +66296,11 @@
           <t>Manquante</t>
         </is>
       </c>
-      <c r="F48" s="12" t="inlineStr"/>
+      <c r="F48" s="12" t="inlineStr">
+        <is>
+          <t>Voir A20, A21</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="12" t="n">
@@ -66228,17 +66308,17 @@
       </c>
       <c r="B49" s="12" t="inlineStr">
         <is>
-          <t>Livre de paie individuel / bulletins</t>
+          <t>PV de caisse au 31/12/2025</t>
         </is>
       </c>
       <c r="C49" s="12" t="inlineStr">
         <is>
-          <t>Les deux</t>
+          <t>Société</t>
         </is>
       </c>
       <c r="D49" s="12" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="E49" s="40" t="inlineStr">
@@ -66248,7 +66328,7 @@
       </c>
       <c r="F49" s="12" t="inlineStr">
         <is>
-          <t>Pour contrôle IRG</t>
+          <t>Voir A22</t>
         </is>
       </c>
     </row>
@@ -66258,12 +66338,12 @@
       </c>
       <c r="B50" s="12" t="inlineStr">
         <is>
-          <t>Ordres de mission et justificatifs de frais</t>
+          <t>Déclarations et paiements CACOBATPH</t>
         </is>
       </c>
       <c r="C50" s="12" t="inlineStr">
         <is>
-          <t>TPM</t>
+          <t>Les deux</t>
         </is>
       </c>
       <c r="D50" s="12" t="inlineStr">
@@ -66276,11 +66356,7 @@
           <t>Manquante</t>
         </is>
       </c>
-      <c r="F50" s="12" t="inlineStr">
-        <is>
-          <t>Frais de mission élevés</t>
-        </is>
-      </c>
+      <c r="F50" s="12" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="12" t="n">
@@ -66288,25 +66364,85 @@
       </c>
       <c r="B51" s="12" t="inlineStr">
         <is>
+          <t>Livre de paie individuel / bulletins</t>
+        </is>
+      </c>
+      <c r="C51" s="12" t="inlineStr">
+        <is>
+          <t>Les deux</t>
+        </is>
+      </c>
+      <c r="D51" s="12" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E51" s="40" t="inlineStr">
+        <is>
+          <t>Manquante</t>
+        </is>
+      </c>
+      <c r="F51" s="12" t="inlineStr">
+        <is>
+          <t>Pour contrôle IRG</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="12" t="n">
+        <v>48</v>
+      </c>
+      <c r="B52" s="12" t="inlineStr">
+        <is>
+          <t>Ordres de mission et justificatifs de frais</t>
+        </is>
+      </c>
+      <c r="C52" s="12" t="inlineStr">
+        <is>
+          <t>TPM</t>
+        </is>
+      </c>
+      <c r="D52" s="12" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E52" s="40" t="inlineStr">
+        <is>
+          <t>Manquante</t>
+        </is>
+      </c>
+      <c r="F52" s="12" t="inlineStr">
+        <is>
+          <t>Frais de mission élevés</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="12" t="n">
+        <v>49</v>
+      </c>
+      <c r="B53" s="12" t="inlineStr">
+        <is>
           <t>Relevés bancaires — virements de salaires</t>
         </is>
       </c>
-      <c r="C51" s="12" t="inlineStr">
+      <c r="C53" s="12" t="inlineStr">
         <is>
           <t>Les deux</t>
         </is>
       </c>
-      <c r="D51" s="12" t="inlineStr">
+      <c r="D53" s="12" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="E51" s="40" t="inlineStr">
+      <c r="E53" s="40" t="inlineStr">
         <is>
           <t>Manquante</t>
         </is>
       </c>
-      <c r="F51" s="12" t="inlineStr">
+      <c r="F53" s="12" t="inlineStr">
         <is>
           <t>Pour lettrage du 421</t>
         </is>

</xml_diff>